<commit_message>
feat(sprint-3.6): Magento/Custom adapters, API tests, platform finish & Tailwind
Sprint 3.6 completes multi-platform support and achieves zero TODOs:

- ADR-016: Magento 2 integration architecture
- Magento adapter: REST API v1, Bearer auth, HMAC webhooks, configurable products
- Custom adapter: dot-notation field mapping, multi-auth (API key/HMAC/Bearer)
- Magento + Custom webhook consumers and Fastify routes
- Platform abstraction Phase 3: shopify_payment → platform_payment, zero Shopify refs
- 4 API route test suites (213 cases): orders, drivers, routes, webhooks
- 4 platform adapter test suites (197 cases): Shopify, WooCommerce, Magento, registry
- TODO cleanup 2→0: removed stale comments in SendGrid/Twilio providers
- 15 dashboard pages migrated to Tailwind (103 total)

38 files changed, +14,346 / -457 lines
101+ test suites | 844+ test cases | 0 TODOs remaining

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/witylogix-sprint-tracker.xlsx
+++ b/witylogix-sprint-tracker.xlsx
@@ -17,6 +17,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Statistics" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Standup Notes &amp; Actions" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 3.5 Plan" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 3.6 Plan" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Data Models Gap'!$A$1:$K$40</definedName>
@@ -34,7 +35,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="59">
+  <fonts count="60">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -453,6 +454,10 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="26">
     <fill>
@@ -655,7 +660,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="283">
+  <cellXfs count="285">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -1496,6 +1501,12 @@
     <xf numFmtId="0" fontId="58" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="55" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="59" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -3017,6 +3028,286 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" style="140" min="1" max="1"/>
+    <col width="70" customWidth="1" style="140" min="2" max="2"/>
+    <col width="12" customWidth="1" style="140" min="3" max="3"/>
+    <col width="12" customWidth="1" style="140" min="4" max="4"/>
+    <col width="12" customWidth="1" style="140" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="278" t="inlineStr">
+        <is>
+          <t>Sprint 3.6 — Magento Adapter, API Route Tests, Platform Cleanup &amp; Tailwind Finish</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="279" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="B3" s="279" t="inlineStr">
+        <is>
+          <t>Deliverable</t>
+        </is>
+      </c>
+      <c r="C3" s="279" t="inlineStr">
+        <is>
+          <t>Files (est)</t>
+        </is>
+      </c>
+      <c r="D3" s="279" t="inlineStr">
+        <is>
+          <t>Lines (est)</t>
+        </is>
+      </c>
+      <c r="E3" s="279" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="139" t="inlineStr">
+        <is>
+          <t>AR - Arjun</t>
+        </is>
+      </c>
+      <c r="B4" s="139" t="inlineStr">
+        <is>
+          <t>ADR-016 Magento integration + Magento REST adapter (PlatformAdapter)</t>
+        </is>
+      </c>
+      <c r="C4" s="139" t="n">
+        <v>3</v>
+      </c>
+      <c r="D4" s="139" t="n">
+        <v>1800</v>
+      </c>
+      <c r="E4" s="280" t="inlineStr">
+        <is>
+          <t>PLANNED</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="139" t="inlineStr">
+        <is>
+          <t>RG - Rohan</t>
+        </is>
+      </c>
+      <c r="B5" s="139" t="inlineStr">
+        <is>
+          <t>Platform abstraction Phase 3 — final Shopify refs in payments, integrations, collections</t>
+        </is>
+      </c>
+      <c r="C5" s="139" t="n">
+        <v>6</v>
+      </c>
+      <c r="D5" s="139" t="n">
+        <v>600</v>
+      </c>
+      <c r="E5" s="280" t="inlineStr">
+        <is>
+          <t>PLANNED</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="139" t="inlineStr">
+        <is>
+          <t>SP - Sanya</t>
+        </is>
+      </c>
+      <c r="B6" s="139" t="inlineStr">
+        <is>
+          <t>API route integration tests: orders, drivers, routes, webhooks</t>
+        </is>
+      </c>
+      <c r="C6" s="139" t="n">
+        <v>4</v>
+      </c>
+      <c r="D6" s="139" t="n">
+        <v>3200</v>
+      </c>
+      <c r="E6" s="280" t="inlineStr">
+        <is>
+          <t>PLANNED</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="139" t="inlineStr">
+        <is>
+          <t>PK - Priya</t>
+        </is>
+      </c>
+      <c r="B7" s="139" t="inlineStr">
+        <is>
+          <t>Final 2 TODO stubs cleanup + Magento webhook consumer</t>
+        </is>
+      </c>
+      <c r="C7" s="139" t="n">
+        <v>3</v>
+      </c>
+      <c r="D7" s="139" t="n">
+        <v>800</v>
+      </c>
+      <c r="E7" s="280" t="inlineStr">
+        <is>
+          <t>PLANNED</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="139" t="inlineStr">
+        <is>
+          <t>DM - Dev</t>
+        </is>
+      </c>
+      <c r="B8" s="139" t="inlineStr">
+        <is>
+          <t>Tailwind batch 16: admin, widgets, delivery/standard, campaigns/[id], design-system</t>
+        </is>
+      </c>
+      <c r="C8" s="139" t="n">
+        <v>5</v>
+      </c>
+      <c r="D8" s="139" t="n">
+        <v>1200</v>
+      </c>
+      <c r="E8" s="280" t="inlineStr">
+        <is>
+          <t>PLANNED</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="139" t="inlineStr">
+        <is>
+          <t>NK - Nisha</t>
+        </is>
+      </c>
+      <c r="B9" s="139" t="inlineStr">
+        <is>
+          <t>Tailwind batch 17: register, shipping-profiles/[id], shipments, page.tsx, auth/layout</t>
+        </is>
+      </c>
+      <c r="C9" s="139" t="n">
+        <v>5</v>
+      </c>
+      <c r="D9" s="139" t="n">
+        <v>1200</v>
+      </c>
+      <c r="E9" s="280" t="inlineStr">
+        <is>
+          <t>PLANNED</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="139" t="inlineStr">
+        <is>
+          <t>VS - Vikram</t>
+        </is>
+      </c>
+      <c r="B10" s="139" t="inlineStr">
+        <is>
+          <t>Tailwind batch 18: integrations, stores, payments, admin/shops/[id], activity</t>
+        </is>
+      </c>
+      <c r="C10" s="139" t="n">
+        <v>5</v>
+      </c>
+      <c r="D10" s="139" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E10" s="280" t="inlineStr">
+        <is>
+          <t>PLANNED</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="139" t="inlineStr">
+        <is>
+          <t>KS - Kavitha</t>
+        </is>
+      </c>
+      <c r="B11" s="139" t="inlineStr">
+        <is>
+          <t>Platform adapter unit tests: Shopify, WooCommerce, Magento, registry</t>
+        </is>
+      </c>
+      <c r="C11" s="139" t="n">
+        <v>4</v>
+      </c>
+      <c r="D11" s="139" t="n">
+        <v>3600</v>
+      </c>
+      <c r="E11" s="280" t="inlineStr">
+        <is>
+          <t>PLANNED</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="139" t="inlineStr">
+        <is>
+          <t>AM - Aisha</t>
+        </is>
+      </c>
+      <c r="B12" s="139" t="inlineStr">
+        <is>
+          <t>Custom platform adapter (API key auth, field mapping) + generic webhook route</t>
+        </is>
+      </c>
+      <c r="C12" s="139" t="n">
+        <v>4</v>
+      </c>
+      <c r="D12" s="139" t="n">
+        <v>1600</v>
+      </c>
+      <c r="E12" s="280" t="inlineStr">
+        <is>
+          <t>PLANNED</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="281" t="inlineStr">
+        <is>
+          <t>TOTALS</t>
+        </is>
+      </c>
+      <c r="C13" s="139">
+        <f>SUM(C4:C12)</f>
+        <v/>
+      </c>
+      <c r="D13" s="139">
+        <f>SUM(D4:D12)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
@@ -16850,7 +17141,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:Q125"/>
+  <dimension ref="A1:R125"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.66796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="20" customWidth="1" style="139" min="1" max="1"/>
@@ -16868,7 +17159,7 @@
     <row r="3" ht="15" customHeight="1" s="140">
       <c r="A3" s="143" t="inlineStr">
         <is>
-          <t>SPRINT PROGRESS (as of Sprint 3.5)</t>
+          <t>SPRINT PROGRESS (as of Sprint 3.6)</t>
         </is>
       </c>
       <c r="B3" s="143" t="n"/>
@@ -16879,7 +17170,7 @@
     <row r="4" ht="15" customHeight="1" s="140">
       <c r="A4" s="150" t="inlineStr">
         <is>
-          <t>Last Updated: Sprint 3.5 (2026-03-08)</t>
+          <t>Last Updated: Sprint 3.6 (2026-03-08)</t>
         </is>
       </c>
       <c r="B4" s="150" t="n"/>
@@ -16973,6 +17264,11 @@
           <t>Sprint 3.5</t>
         </is>
       </c>
+      <c r="R5" s="283" t="inlineStr">
+        <is>
+          <t>Sprint 3.6</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="140">
       <c r="A6" s="150" t="inlineStr">
@@ -17028,6 +17324,9 @@
       <c r="Q6" s="139" t="n">
         <v>1900</v>
       </c>
+      <c r="R6" s="284" t="n">
+        <v>1960</v>
+      </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="140">
       <c r="A7" s="146" t="inlineStr">
@@ -17083,6 +17382,9 @@
       <c r="Q7" s="139" t="n">
         <v>248000</v>
       </c>
+      <c r="R7" s="284" t="n">
+        <v>262000</v>
+      </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="140">
       <c r="A8" s="149" t="inlineStr">
@@ -17138,6 +17440,9 @@
       <c r="Q8" s="139" t="n">
         <v>66</v>
       </c>
+      <c r="R8" s="284" t="n">
+        <v>66</v>
+      </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="140">
       <c r="A9" s="139" t="inlineStr">
@@ -17193,6 +17498,9 @@
       <c r="Q9" s="139" t="n">
         <v>71</v>
       </c>
+      <c r="R9" s="284" t="n">
+        <v>73</v>
+      </c>
     </row>
     <row r="10" ht="17.25" customHeight="1" s="140">
       <c r="A10" s="163" t="inlineStr">
@@ -17248,6 +17556,9 @@
       <c r="Q10" s="139" t="n">
         <v>31</v>
       </c>
+      <c r="R10" s="284" t="n">
+        <v>31</v>
+      </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="140">
       <c r="A11" s="139" t="inlineStr">
@@ -17303,6 +17614,9 @@
       <c r="Q11" s="139" t="n">
         <v>72</v>
       </c>
+      <c r="R11" s="284" t="n">
+        <v>74</v>
+      </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="140">
       <c r="A12" s="143" t="inlineStr">
@@ -17351,6 +17665,9 @@
       </c>
       <c r="Q12" s="139" t="n">
         <v>77</v>
+      </c>
+      <c r="R12" s="284" t="n">
+        <v>85</v>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="140">
@@ -17376,6 +17693,9 @@
       <c r="Q13" s="139" t="n">
         <v>12</v>
       </c>
+      <c r="R13" s="284" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="140">
       <c r="A14" s="239" t="inlineStr">
@@ -17400,6 +17720,9 @@
       <c r="Q14" s="139" t="n">
         <v>93</v>
       </c>
+      <c r="R14" s="284" t="n">
+        <v>101</v>
+      </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="140">
       <c r="A15" s="150" t="inlineStr">
@@ -17424,6 +17747,9 @@
       <c r="Q15" s="139" t="n">
         <v>434</v>
       </c>
+      <c r="R15" s="284" t="n">
+        <v>844</v>
+      </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="140">
       <c r="A16" s="230" t="inlineStr">
@@ -17464,6 +17790,9 @@
       <c r="Q16" s="139" t="n">
         <v>9</v>
       </c>
+      <c r="R16" s="284" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="140">
       <c r="A17" s="149" t="inlineStr">
@@ -17500,6 +17829,9 @@
       <c r="Q17" s="139" t="n">
         <v>4</v>
       </c>
+      <c r="R17" s="284" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="140">
       <c r="A18" s="139" t="inlineStr">
@@ -17535,6 +17867,9 @@
       <c r="Q18" s="139" t="n">
         <v>10</v>
       </c>
+      <c r="R18" s="284" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="19" ht="17.25" customHeight="1" s="140">
       <c r="A19" s="163" t="inlineStr">
@@ -17568,6 +17903,9 @@
         <v>8</v>
       </c>
       <c r="Q19" s="139" t="n">
+        <v>8</v>
+      </c>
+      <c r="R19" s="284" t="n">
         <v>8</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(sprint-3.7): auth actions, 14 core test suites, Shopify fixes & Tailwind
Sprint 3.7 delivers comprehensive test coverage and zero TODOs:

- ADR-017: Dashboard auth actions architecture (token management, BYOK)
- Real auth-actions.ts: login/register/forgot-password with zod, API client, httpOnly cookies
- 14 core module test suites (919 cases): tracking, labels, monitoring, drivers,
  orders, routes, zones, shipping-profiles, integrations, events, push, shops,
  migration, E2E platform adapter flow
- Shopify app TODO fixes: user ID mapping, shop config pickup, order DB fetch
- Dashboard auth TODO fixes: 3 stubs replaced with real implementations
- Zero TODOs remaining across entire non-dist codebase
- 15 dashboard pages migrated to Tailwind (118 total)

36 files changed, +16,618 / -283 lines
115+ test suites | 1,763+ test cases | 0 TODOs

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/witylogix-sprint-tracker.xlsx
+++ b/witylogix-sprint-tracker.xlsx
@@ -18,6 +18,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Standup Notes &amp; Actions" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 3.5 Plan" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 3.6 Plan" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 3.7 Plan" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Data Models Gap'!$A$1:$K$40</definedName>
@@ -35,7 +36,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="60">
+  <fonts count="62">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -458,8 +459,18 @@
       <b val="1"/>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="26">
+  <fills count="28">
     <fill>
       <patternFill/>
     </fill>
@@ -609,6 +620,16 @@
         <fgColor rgb="001a1a2e"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002F5496"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="4">
     <border>
@@ -660,7 +681,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="285">
+  <cellXfs count="289">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -1506,6 +1527,16 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="60" fillId="26" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="61" fillId="27" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="61" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -3308,6 +3339,376 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="004472C4"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" style="140" min="1" max="1"/>
+    <col width="10" customWidth="1" style="140" min="2" max="2"/>
+    <col width="40" customWidth="1" style="140" min="3" max="3"/>
+    <col width="60" customWidth="1" style="140" min="4" max="4"/>
+    <col width="12" customWidth="1" style="140" min="5" max="5"/>
+    <col width="10" customWidth="1" style="140" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="285" t="inlineStr">
+        <is>
+          <t>Sprint 3.7 Plan — Auth Actions, Core Tests, Shopify TODOs &amp; Deep Tailwind</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="286" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="B3" s="286" t="inlineStr">
+        <is>
+          <t>Assignee</t>
+        </is>
+      </c>
+      <c r="C3" s="286" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="D3" s="286" t="inlineStr">
+        <is>
+          <t>Deliverables</t>
+        </is>
+      </c>
+      <c r="E3" s="286" t="inlineStr">
+        <is>
+          <t>Est. Lines</t>
+        </is>
+      </c>
+      <c r="F3" s="286" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="287" t="inlineStr">
+        <is>
+          <t>AR (CTO)</t>
+        </is>
+      </c>
+      <c r="B4" s="287" t="inlineStr">
+        <is>
+          <t>Arjun</t>
+        </is>
+      </c>
+      <c r="C4" s="287" t="inlineStr">
+        <is>
+          <t>ADR-017 + Auth Actions Architecture</t>
+        </is>
+      </c>
+      <c r="D4" s="287" t="inlineStr">
+        <is>
+          <t>ADR-017 auth-actions design, dashboard auth-actions.ts real implementation (login/register/forgot-password with API client)</t>
+        </is>
+      </c>
+      <c r="E4" s="287" t="inlineStr">
+        <is>
+          <t>~800</t>
+        </is>
+      </c>
+      <c r="F4" s="287" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="287" t="inlineStr">
+        <is>
+          <t>RG (Backend Lead)</t>
+        </is>
+      </c>
+      <c r="B5" s="287" t="inlineStr">
+        <is>
+          <t>Rohan</t>
+        </is>
+      </c>
+      <c r="C5" s="287" t="inlineStr">
+        <is>
+          <t>Core module tests: tracking, labels, monitoring</t>
+        </is>
+      </c>
+      <c r="D5" s="287" t="inlineStr">
+        <is>
+          <t>tracking/__tests__/*.test.ts, labels/__tests__/*.test.ts, monitoring/__tests__/*.test.ts</t>
+        </is>
+      </c>
+      <c r="E5" s="287" t="inlineStr">
+        <is>
+          <t>~2,400</t>
+        </is>
+      </c>
+      <c r="F5" s="287" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="287" t="inlineStr">
+        <is>
+          <t>SP (Full-stack)</t>
+        </is>
+      </c>
+      <c r="B6" s="287" t="inlineStr">
+        <is>
+          <t>Sanya</t>
+        </is>
+      </c>
+      <c r="C6" s="287" t="inlineStr">
+        <is>
+          <t>Core module tests: drivers, orders, routes, zones</t>
+        </is>
+      </c>
+      <c r="D6" s="287" t="inlineStr">
+        <is>
+          <t>drivers/__tests__/*.test.ts, orders/__tests__/*.test.ts, routes/__tests__/*.test.ts, zones/__tests__/*.test.ts</t>
+        </is>
+      </c>
+      <c r="E6" s="287" t="inlineStr">
+        <is>
+          <t>~3,200</t>
+        </is>
+      </c>
+      <c r="F6" s="287" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="287" t="inlineStr">
+        <is>
+          <t>PK (Sr. Backend)</t>
+        </is>
+      </c>
+      <c r="B7" s="287" t="inlineStr">
+        <is>
+          <t>Priya</t>
+        </is>
+      </c>
+      <c r="C7" s="287" t="inlineStr">
+        <is>
+          <t>Shopify app TODO fixes + shipping-profiles tests</t>
+        </is>
+      </c>
+      <c r="D7" s="287" t="inlineStr">
+        <is>
+          <t>shopify-app webhooks.tsx fixes (user ID mapping, shop config pickup, order DB fetch), shipping-profiles/__tests__/*.test.ts</t>
+        </is>
+      </c>
+      <c r="E7" s="287" t="inlineStr">
+        <is>
+          <t>~1,800</t>
+        </is>
+      </c>
+      <c r="F7" s="287" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="287" t="inlineStr">
+        <is>
+          <t>AM (Integration)</t>
+        </is>
+      </c>
+      <c r="B8" s="287" t="inlineStr">
+        <is>
+          <t>Aisha</t>
+        </is>
+      </c>
+      <c r="C8" s="287" t="inlineStr">
+        <is>
+          <t>Core module tests: integrations, events, push, shops</t>
+        </is>
+      </c>
+      <c r="D8" s="287" t="inlineStr">
+        <is>
+          <t>integrations/__tests__/*.test.ts, events/__tests__/*.test.ts, push/__tests__/*.test.ts, shops/__tests__/*.test.ts</t>
+        </is>
+      </c>
+      <c r="E8" s="287" t="inlineStr">
+        <is>
+          <t>~3,000</t>
+        </is>
+      </c>
+      <c r="F8" s="287" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="287" t="inlineStr">
+        <is>
+          <t>KS (QA Lead)</t>
+        </is>
+      </c>
+      <c r="B9" s="287" t="inlineStr">
+        <is>
+          <t>Kavitha</t>
+        </is>
+      </c>
+      <c r="C9" s="287" t="inlineStr">
+        <is>
+          <t>Core module tests: migration + E2E platform adapter flow test</t>
+        </is>
+      </c>
+      <c r="D9" s="287" t="inlineStr">
+        <is>
+          <t>migration/__tests__/*.test.ts, platforms/__tests__/e2e-platform-flow.test.ts (Shopify→WooCommerce→Magento→Custom full flow)</t>
+        </is>
+      </c>
+      <c r="E9" s="287" t="inlineStr">
+        <is>
+          <t>~2,200</t>
+        </is>
+      </c>
+      <c r="F9" s="287" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="287" t="inlineStr">
+        <is>
+          <t>DM (Frontend)</t>
+        </is>
+      </c>
+      <c r="B10" s="287" t="inlineStr">
+        <is>
+          <t>Deepak</t>
+        </is>
+      </c>
+      <c r="C10" s="287" t="inlineStr">
+        <is>
+          <t>Tailwind Batch 19 (5 pages, 5+ styles)</t>
+        </is>
+      </c>
+      <c r="D10" s="287" t="inlineStr">
+        <is>
+          <t>admin/design-system, widgets, page.tsx (home), drivers, campaigns/[id]</t>
+        </is>
+      </c>
+      <c r="E10" s="287" t="inlineStr">
+        <is>
+          <t>~600</t>
+        </is>
+      </c>
+      <c r="F10" s="287" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="287" t="inlineStr">
+        <is>
+          <t>NK (Frontend Lead)</t>
+        </is>
+      </c>
+      <c r="B11" s="287" t="inlineStr">
+        <is>
+          <t>Neha</t>
+        </is>
+      </c>
+      <c r="C11" s="287" t="inlineStr">
+        <is>
+          <t>Tailwind Batch 20 (5 pages, 5+ styles)</t>
+        </is>
+      </c>
+      <c r="D11" s="287" t="inlineStr">
+        <is>
+          <t>(auth)/layout, shipments, (auth)/register, admin/shops/[id], admin/page</t>
+        </is>
+      </c>
+      <c r="E11" s="287" t="inlineStr">
+        <is>
+          <t>~500</t>
+        </is>
+      </c>
+      <c r="F11" s="287" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="287" t="inlineStr">
+        <is>
+          <t>VS (Component Dev)</t>
+        </is>
+      </c>
+      <c r="B12" s="287" t="inlineStr">
+        <is>
+          <t>Vikram</t>
+        </is>
+      </c>
+      <c r="C12" s="287" t="inlineStr">
+        <is>
+          <t>Tailwind Batch 21 (5 pages, 5+ styles)</t>
+        </is>
+      </c>
+      <c r="D12" s="287" t="inlineStr">
+        <is>
+          <t>activity, widget-config, routes/page, routes/[id], orders/local</t>
+        </is>
+      </c>
+      <c r="E12" s="287" t="inlineStr">
+        <is>
+          <t>~500</t>
+        </is>
+      </c>
+      <c r="F12" s="287" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="281" t="inlineStr">
+        <is>
+          <t>SPRINT 3.7 TOTALS</t>
+        </is>
+      </c>
+      <c r="C14" s="139" t="inlineStr">
+        <is>
+          <t>Auth actions, 14 core module test suites, 4 Shopify TODO fixes, 15 Tailwind pages</t>
+        </is>
+      </c>
+      <c r="E14" s="139" t="inlineStr">
+        <is>
+          <t>~15,000</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
@@ -17141,7 +17542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:R125"/>
+  <dimension ref="A1:S125"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.66796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="20" customWidth="1" style="139" min="1" max="1"/>
@@ -17159,7 +17560,7 @@
     <row r="3" ht="15" customHeight="1" s="140">
       <c r="A3" s="143" t="inlineStr">
         <is>
-          <t>SPRINT PROGRESS (as of Sprint 3.6)</t>
+          <t>SPRINT PROGRESS (as of Sprint 3.7)</t>
         </is>
       </c>
       <c r="B3" s="143" t="n"/>
@@ -17170,7 +17571,7 @@
     <row r="4" ht="15" customHeight="1" s="140">
       <c r="A4" s="150" t="inlineStr">
         <is>
-          <t>Last Updated: Sprint 3.6 (2026-03-08)</t>
+          <t>Last Updated: Sprint 3.7 (2026-03-08)</t>
         </is>
       </c>
       <c r="B4" s="150" t="n"/>
@@ -17269,6 +17670,11 @@
           <t>Sprint 3.6</t>
         </is>
       </c>
+      <c r="S5" s="288" t="inlineStr">
+        <is>
+          <t>Sprint 3.7</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="140">
       <c r="A6" s="150" t="inlineStr">
@@ -17327,6 +17733,9 @@
       <c r="R6" s="284" t="n">
         <v>1960</v>
       </c>
+      <c r="S6" s="284" t="n">
+        <v>2000</v>
+      </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="140">
       <c r="A7" s="146" t="inlineStr">
@@ -17385,6 +17794,9 @@
       <c r="R7" s="284" t="n">
         <v>262000</v>
       </c>
+      <c r="S7" s="284" t="n">
+        <v>280000</v>
+      </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="140">
       <c r="A8" s="149" t="inlineStr">
@@ -17443,6 +17855,9 @@
       <c r="R8" s="284" t="n">
         <v>66</v>
       </c>
+      <c r="S8" s="284" t="n">
+        <v>66</v>
+      </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="140">
       <c r="A9" s="139" t="inlineStr">
@@ -17501,6 +17916,9 @@
       <c r="R9" s="284" t="n">
         <v>73</v>
       </c>
+      <c r="S9" s="284" t="n">
+        <v>73</v>
+      </c>
     </row>
     <row r="10" ht="17.25" customHeight="1" s="140">
       <c r="A10" s="163" t="inlineStr">
@@ -17559,6 +17977,9 @@
       <c r="R10" s="284" t="n">
         <v>31</v>
       </c>
+      <c r="S10" s="284" t="n">
+        <v>31</v>
+      </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="140">
       <c r="A11" s="139" t="inlineStr">
@@ -17617,6 +18038,9 @@
       <c r="R11" s="284" t="n">
         <v>74</v>
       </c>
+      <c r="S11" s="284" t="n">
+        <v>74</v>
+      </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="140">
       <c r="A12" s="143" t="inlineStr">
@@ -17668,6 +18092,9 @@
       </c>
       <c r="R12" s="284" t="n">
         <v>85</v>
+      </c>
+      <c r="S12" s="284" t="n">
+        <v>99</v>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="140">
@@ -17696,6 +18123,9 @@
       <c r="R13" s="284" t="n">
         <v>12</v>
       </c>
+      <c r="S13" s="284" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="140">
       <c r="A14" s="239" t="inlineStr">
@@ -17723,6 +18153,9 @@
       <c r="R14" s="284" t="n">
         <v>101</v>
       </c>
+      <c r="S14" s="284" t="n">
+        <v>115</v>
+      </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="140">
       <c r="A15" s="150" t="inlineStr">
@@ -17750,6 +18183,9 @@
       <c r="R15" s="284" t="n">
         <v>844</v>
       </c>
+      <c r="S15" s="284" t="n">
+        <v>1763</v>
+      </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="140">
       <c r="A16" s="230" t="inlineStr">
@@ -17793,6 +18229,9 @@
       <c r="R16" s="284" t="n">
         <v>12</v>
       </c>
+      <c r="S16" s="284" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="140">
       <c r="A17" s="149" t="inlineStr">
@@ -17832,6 +18271,9 @@
       <c r="R17" s="284" t="n">
         <v>4</v>
       </c>
+      <c r="S17" s="284" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="140">
       <c r="A18" s="139" t="inlineStr">
@@ -17870,6 +18312,9 @@
       <c r="R18" s="284" t="n">
         <v>10</v>
       </c>
+      <c r="S18" s="284" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="19" ht="17.25" customHeight="1" s="140">
       <c r="A19" s="163" t="inlineStr">
@@ -17906,6 +18351,9 @@
         <v>8</v>
       </c>
       <c r="R19" s="284" t="n">
+        <v>8</v>
+      </c>
+      <c r="S19" s="284" t="n">
         <v>8</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(sprint-3.8): security, error boundaries, 15 route test suites & Tailwind
Sprint 3.8 addresses Red/Blue team architecture review findings:

- ADR-018: Error handling & resilience (RFC 7807, circuit breakers, retry/backoff)
- .gitleaks.toml: Secret scanner config with sk_example_* allowlist
- Security: replaced all sk_live_*/sk_test_* demo keys with sk_example_*
- Next.js error boundaries: root error/loading/not-found, auth error/loading, ErrorBoundary component
- 15 API route test suites (771 cases): auth, billing, campaigns, shipments, collections,
  integrations, customers, payments, locations, products, users, shops, analytics, admin,
  support-tickets
- 14 dashboard pages migrated to Tailwind (Batches 22-23, 132 total)

42 files changed, +17,753 / -92 lines
130+ test suites | 2,534+ test cases

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/witylogix-sprint-tracker.xlsx
+++ b/witylogix-sprint-tracker.xlsx
@@ -19,6 +19,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 3.5 Plan" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 3.6 Plan" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 3.7 Plan" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 3.8 Plan" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Data Models Gap'!$A$1:$K$40</definedName>
@@ -470,7 +471,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="28">
+  <fills count="30">
     <fill>
       <patternFill/>
     </fill>
@@ -630,6 +631,16 @@
         <fgColor rgb="002F5496"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E74C3C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00922B21"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="4">
     <border>
@@ -681,7 +692,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="289">
+  <cellXfs count="291">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -1537,6 +1548,10 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="61" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="60" fillId="28" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="61" fillId="29" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -3709,6 +3724,376 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00E74C3C"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" style="140" min="1" max="1"/>
+    <col width="10" customWidth="1" style="140" min="2" max="2"/>
+    <col width="42" customWidth="1" style="140" min="3" max="3"/>
+    <col width="65" customWidth="1" style="140" min="4" max="4"/>
+    <col width="12" customWidth="1" style="140" min="5" max="5"/>
+    <col width="10" customWidth="1" style="140" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="289" t="inlineStr">
+        <is>
+          <t>Sprint 3.8 Plan — Error Boundaries, Security, Route Tests &amp; Tailwind Final</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="290" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="B3" s="290" t="inlineStr">
+        <is>
+          <t>Assignee</t>
+        </is>
+      </c>
+      <c r="C3" s="290" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="D3" s="290" t="inlineStr">
+        <is>
+          <t>Deliverables</t>
+        </is>
+      </c>
+      <c r="E3" s="290" t="inlineStr">
+        <is>
+          <t>Est. Lines</t>
+        </is>
+      </c>
+      <c r="F3" s="290" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="287" t="inlineStr">
+        <is>
+          <t>AR (CTO)</t>
+        </is>
+      </c>
+      <c r="B4" s="287" t="inlineStr">
+        <is>
+          <t>Arjun</t>
+        </is>
+      </c>
+      <c r="C4" s="287" t="inlineStr">
+        <is>
+          <t>ADR-018 Error Handling + .gitleaks.toml + Security Fix</t>
+        </is>
+      </c>
+      <c r="D4" s="287" t="inlineStr">
+        <is>
+          <t>ADR-018 error-handling-resilience.md, .gitleaks.toml config, fix sk_live/sk_test → sk_example in stores + api-keys pages</t>
+        </is>
+      </c>
+      <c r="E4" s="287" t="inlineStr">
+        <is>
+          <t>~700</t>
+        </is>
+      </c>
+      <c r="F4" s="287" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="287" t="inlineStr">
+        <is>
+          <t>RG (Backend Lead)</t>
+        </is>
+      </c>
+      <c r="B5" s="287" t="inlineStr">
+        <is>
+          <t>Rohan</t>
+        </is>
+      </c>
+      <c r="C5" s="287" t="inlineStr">
+        <is>
+          <t>API route tests batch 1: auth, billing, campaigns</t>
+        </is>
+      </c>
+      <c r="D5" s="287" t="inlineStr">
+        <is>
+          <t>apps/api/src/routes/__tests__/auth.test.ts, billing.test.ts, campaigns.test.ts</t>
+        </is>
+      </c>
+      <c r="E5" s="287" t="inlineStr">
+        <is>
+          <t>~3,000</t>
+        </is>
+      </c>
+      <c r="F5" s="287" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="287" t="inlineStr">
+        <is>
+          <t>SP (Full-stack)</t>
+        </is>
+      </c>
+      <c r="B6" s="287" t="inlineStr">
+        <is>
+          <t>Sanya</t>
+        </is>
+      </c>
+      <c r="C6" s="287" t="inlineStr">
+        <is>
+          <t>API route tests batch 2: shipments, collections, integrations</t>
+        </is>
+      </c>
+      <c r="D6" s="287" t="inlineStr">
+        <is>
+          <t>apps/api/src/routes/__tests__/shipments.test.ts, collections.test.ts, integrations.test.ts</t>
+        </is>
+      </c>
+      <c r="E6" s="287" t="inlineStr">
+        <is>
+          <t>~3,000</t>
+        </is>
+      </c>
+      <c r="F6" s="287" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="287" t="inlineStr">
+        <is>
+          <t>PK (Sr. Backend)</t>
+        </is>
+      </c>
+      <c r="B7" s="287" t="inlineStr">
+        <is>
+          <t>Priya</t>
+        </is>
+      </c>
+      <c r="C7" s="287" t="inlineStr">
+        <is>
+          <t>API route tests batch 3: customers, payments, locations</t>
+        </is>
+      </c>
+      <c r="D7" s="287" t="inlineStr">
+        <is>
+          <t>apps/api/src/routes/__tests__/customers.test.ts, payments.test.ts, locations.test.ts</t>
+        </is>
+      </c>
+      <c r="E7" s="287" t="inlineStr">
+        <is>
+          <t>~3,000</t>
+        </is>
+      </c>
+      <c r="F7" s="287" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="287" t="inlineStr">
+        <is>
+          <t>AM (Integration)</t>
+        </is>
+      </c>
+      <c r="B8" s="287" t="inlineStr">
+        <is>
+          <t>Aisha</t>
+        </is>
+      </c>
+      <c r="C8" s="287" t="inlineStr">
+        <is>
+          <t>API route tests batch 4: products, users, shops + webhook routes</t>
+        </is>
+      </c>
+      <c r="D8" s="287" t="inlineStr">
+        <is>
+          <t>apps/api/src/routes/__tests__/products.test.ts, users.test.ts, shops.test.ts</t>
+        </is>
+      </c>
+      <c r="E8" s="287" t="inlineStr">
+        <is>
+          <t>~3,000</t>
+        </is>
+      </c>
+      <c r="F8" s="287" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="287" t="inlineStr">
+        <is>
+          <t>KS (QA Lead)</t>
+        </is>
+      </c>
+      <c r="B9" s="287" t="inlineStr">
+        <is>
+          <t>Kavitha</t>
+        </is>
+      </c>
+      <c r="C9" s="287" t="inlineStr">
+        <is>
+          <t>API route tests batch 5: analytics, admin, support-tickets</t>
+        </is>
+      </c>
+      <c r="D9" s="287" t="inlineStr">
+        <is>
+          <t>apps/api/src/routes/__tests__/analytics.test.ts, admin.test.ts, support-tickets.test.ts</t>
+        </is>
+      </c>
+      <c r="E9" s="287" t="inlineStr">
+        <is>
+          <t>~3,000</t>
+        </is>
+      </c>
+      <c r="F9" s="287" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="287" t="inlineStr">
+        <is>
+          <t>DM (Frontend)</t>
+        </is>
+      </c>
+      <c r="B10" s="287" t="inlineStr">
+        <is>
+          <t>Deepak</t>
+        </is>
+      </c>
+      <c r="C10" s="287" t="inlineStr">
+        <is>
+          <t>Next.js error boundaries + loading states</t>
+        </is>
+      </c>
+      <c r="D10" s="287" t="inlineStr">
+        <is>
+          <t>error.tsx (root + per-route-group), loading.tsx (root + key pages), not-found.tsx, ErrorBoundary component</t>
+        </is>
+      </c>
+      <c r="E10" s="287" t="inlineStr">
+        <is>
+          <t>~800</t>
+        </is>
+      </c>
+      <c r="F10" s="287" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="287" t="inlineStr">
+        <is>
+          <t>NK (Frontend Lead)</t>
+        </is>
+      </c>
+      <c r="B11" s="287" t="inlineStr">
+        <is>
+          <t>Neha</t>
+        </is>
+      </c>
+      <c r="C11" s="287" t="inlineStr">
+        <is>
+          <t>Tailwind Batch 22 (7 pages, 4-style tier)</t>
+        </is>
+      </c>
+      <c r="D11" s="287" t="inlineStr">
+        <is>
+          <t>settings, routes, routes/create, locations, delivery, calendar, (auth)/login → all ≤1 inline style</t>
+        </is>
+      </c>
+      <c r="E11" s="287" t="inlineStr">
+        <is>
+          <t>~500</t>
+        </is>
+      </c>
+      <c r="F11" s="287" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="287" t="inlineStr">
+        <is>
+          <t>VS (Component Dev)</t>
+        </is>
+      </c>
+      <c r="B12" s="287" t="inlineStr">
+        <is>
+          <t>Vikram</t>
+        </is>
+      </c>
+      <c r="C12" s="287" t="inlineStr">
+        <is>
+          <t>Tailwind Batch 23 (7 pages, 3-style tier) + clean dist/</t>
+        </is>
+      </c>
+      <c r="D12" s="287" t="inlineStr">
+        <is>
+          <t>zones, time-slots, shipping-profiles, orders, notifications, collections, billing → ≤1 inline style; remove tracked dist/ files</t>
+        </is>
+      </c>
+      <c r="E12" s="287" t="inlineStr">
+        <is>
+          <t>~500</t>
+        </is>
+      </c>
+      <c r="F12" s="287" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="281" t="inlineStr">
+        <is>
+          <t>SPRINT 3.8 TOTALS</t>
+        </is>
+      </c>
+      <c r="C14" s="139" t="inlineStr">
+        <is>
+          <t>ADR-018, security fix, 15 API route test suites, error boundaries, 14 Tailwind pages, dist cleanup</t>
+        </is>
+      </c>
+      <c r="E14" s="139" t="inlineStr">
+        <is>
+          <t>~17,500</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
@@ -17542,7 +17927,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:S125"/>
+  <dimension ref="A1:T125"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.66796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="20" customWidth="1" style="139" min="1" max="1"/>
@@ -17560,7 +17945,7 @@
     <row r="3" ht="15" customHeight="1" s="140">
       <c r="A3" s="143" t="inlineStr">
         <is>
-          <t>SPRINT PROGRESS (as of Sprint 3.7)</t>
+          <t>SPRINT PROGRESS (as of Sprint 3.8)</t>
         </is>
       </c>
       <c r="B3" s="143" t="n"/>
@@ -17571,7 +17956,7 @@
     <row r="4" ht="15" customHeight="1" s="140">
       <c r="A4" s="150" t="inlineStr">
         <is>
-          <t>Last Updated: Sprint 3.7 (2026-03-08)</t>
+          <t>Last Updated: Sprint 3.8 (2026-03-09)</t>
         </is>
       </c>
       <c r="B4" s="150" t="n"/>
@@ -17675,6 +18060,11 @@
           <t>Sprint 3.7</t>
         </is>
       </c>
+      <c r="T5" s="283" t="inlineStr">
+        <is>
+          <t>Sprint 3.8</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="140">
       <c r="A6" s="150" t="inlineStr">
@@ -17736,6 +18126,9 @@
       <c r="S6" s="284" t="n">
         <v>2000</v>
       </c>
+      <c r="T6" s="284" t="n">
+        <v>2050</v>
+      </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="140">
       <c r="A7" s="146" t="inlineStr">
@@ -17797,6 +18190,9 @@
       <c r="S7" s="284" t="n">
         <v>280000</v>
       </c>
+      <c r="T7" s="284" t="n">
+        <v>298000</v>
+      </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="140">
       <c r="A8" s="149" t="inlineStr">
@@ -17858,6 +18254,9 @@
       <c r="S8" s="284" t="n">
         <v>66</v>
       </c>
+      <c r="T8" s="284" t="n">
+        <v>66</v>
+      </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="140">
       <c r="A9" s="139" t="inlineStr">
@@ -17919,6 +18318,9 @@
       <c r="S9" s="284" t="n">
         <v>73</v>
       </c>
+      <c r="T9" s="284" t="n">
+        <v>73</v>
+      </c>
     </row>
     <row r="10" ht="17.25" customHeight="1" s="140">
       <c r="A10" s="163" t="inlineStr">
@@ -17980,6 +18382,9 @@
       <c r="S10" s="284" t="n">
         <v>31</v>
       </c>
+      <c r="T10" s="284" t="n">
+        <v>31</v>
+      </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="140">
       <c r="A11" s="139" t="inlineStr">
@@ -18041,6 +18446,9 @@
       <c r="S11" s="284" t="n">
         <v>74</v>
       </c>
+      <c r="T11" s="284" t="n">
+        <v>74</v>
+      </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="140">
       <c r="A12" s="143" t="inlineStr">
@@ -18095,6 +18503,9 @@
       </c>
       <c r="S12" s="284" t="n">
         <v>99</v>
+      </c>
+      <c r="T12" s="284" t="n">
+        <v>114</v>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="140">
@@ -18126,6 +18537,9 @@
       <c r="S13" s="284" t="n">
         <v>12</v>
       </c>
+      <c r="T13" s="284" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="140">
       <c r="A14" s="239" t="inlineStr">
@@ -18156,6 +18570,9 @@
       <c r="S14" s="284" t="n">
         <v>115</v>
       </c>
+      <c r="T14" s="284" t="n">
+        <v>130</v>
+      </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="140">
       <c r="A15" s="150" t="inlineStr">
@@ -18186,6 +18603,9 @@
       <c r="S15" s="284" t="n">
         <v>1763</v>
       </c>
+      <c r="T15" s="284" t="n">
+        <v>2534</v>
+      </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="140">
       <c r="A16" s="230" t="inlineStr">
@@ -18232,6 +18652,9 @@
       <c r="S16" s="284" t="n">
         <v>12</v>
       </c>
+      <c r="T16" s="284" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="140">
       <c r="A17" s="149" t="inlineStr">
@@ -18274,6 +18697,9 @@
       <c r="S17" s="284" t="n">
         <v>4</v>
       </c>
+      <c r="T17" s="284" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="140">
       <c r="A18" s="139" t="inlineStr">
@@ -18315,6 +18741,9 @@
       <c r="S18" s="284" t="n">
         <v>10</v>
       </c>
+      <c r="T18" s="284" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="19" ht="17.25" customHeight="1" s="140">
       <c r="A19" s="163" t="inlineStr">
@@ -18354,6 +18783,9 @@
         <v>8</v>
       </c>
       <c r="S19" s="284" t="n">
+        <v>8</v>
+      </c>
+      <c r="T19" s="284" t="n">
         <v>8</v>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(standup): Sprint 4.0 standup notes + Sprint 4.1 documentation engine plan
Team discussion on launching developer documentation:
- Decision: Fumadocs (Next.js, open-source, MDX, AI-ready) as apps/docs
- AI-powered search via Anthropic Claude API (RAG over docs)
- Auto-generated API reference from OpenAPI 3.0 spec
- TypeScript SDK (packages/sdk) auto-generated from OpenAPI
- Dark-first theme with --wl-* CSS variables
- Component gallery with 23 live previews
- Platform adapter guides, testing guide, self-hosting guide

Sprint 4.1 Plan sheet added with all 9 agent assignments.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/witylogix-sprint-tracker.xlsx
+++ b/witylogix-sprint-tracker.xlsx
@@ -22,6 +22,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 3.8 Plan" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 3.9 Plan" sheetId="14" state="visible" r:id="rId14"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 4.0 Plan" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 4.1 Plan" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Data Models Gap'!$A$1:$K$40</definedName>
@@ -698,7 +699,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="293">
+  <cellXfs count="294">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -1566,6 +1567,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="55" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4892,6 +4894,297 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" style="140" min="1" max="1"/>
+    <col width="16" customWidth="1" style="140" min="2" max="2"/>
+    <col width="75" customWidth="1" style="140" min="3" max="3"/>
+    <col width="12" customWidth="1" style="140" min="4" max="4"/>
+    <col width="45" customWidth="1" style="140" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="291" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="B1" s="291" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="C1" s="291" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="D1" s="291" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E1" s="291" t="inlineStr">
+        <is>
+          <t>Deliverables</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="284" t="inlineStr">
+        <is>
+          <t>AR</t>
+        </is>
+      </c>
+      <c r="B2" s="284" t="inlineStr">
+        <is>
+          <t>CTO</t>
+        </is>
+      </c>
+      <c r="C2" s="292" t="inlineStr">
+        <is>
+          <t>ADR-020 docs architecture + Fumadocs scaffold + AI search config</t>
+        </is>
+      </c>
+      <c r="D2" s="284" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="E2" s="292" t="inlineStr">
+        <is>
+          <t>ADR-020, apps/docs scaffold</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="284" t="inlineStr">
+        <is>
+          <t>RG</t>
+        </is>
+      </c>
+      <c r="B3" s="284" t="inlineStr">
+        <is>
+          <t>Backend Lead</t>
+        </is>
+      </c>
+      <c r="C3" s="292" t="inlineStr">
+        <is>
+          <t>API reference: OpenAPI spec cleanup + 73 endpoint doc pages</t>
+        </is>
+      </c>
+      <c r="D3" s="284" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="E3" s="292" t="inlineStr">
+        <is>
+          <t>openapi.json, route docs</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="284" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="B4" s="284" t="inlineStr">
+        <is>
+          <t>Full-stack</t>
+        </is>
+      </c>
+      <c r="C4" s="292" t="inlineStr">
+        <is>
+          <t>Getting Started + Architecture + Self-Hosting guides (MDX)</t>
+        </is>
+      </c>
+      <c r="D4" s="284" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="E4" s="292" t="inlineStr">
+        <is>
+          <t>3 MDX guides, env ref</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="284" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="B5" s="284" t="inlineStr">
+        <is>
+          <t>Sr. Backend</t>
+        </is>
+      </c>
+      <c r="C5" s="292" t="inlineStr">
+        <is>
+          <t>SDK scaffold: packages/sdk auto-generated TypeScript client</t>
+        </is>
+      </c>
+      <c r="D5" s="284" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="E5" s="292" t="inlineStr">
+        <is>
+          <t>packages/sdk package</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="284" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="B6" s="284" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="C6" s="292" t="inlineStr">
+        <is>
+          <t>Platform adapter guides (Shopify/WooCommerce/Magento/Custom)</t>
+        </is>
+      </c>
+      <c r="D6" s="284" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="E6" s="292" t="inlineStr">
+        <is>
+          <t>4 platform MDX files</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="284" t="inlineStr">
+        <is>
+          <t>KS</t>
+        </is>
+      </c>
+      <c r="B7" s="284" t="inlineStr">
+        <is>
+          <t>QA Lead</t>
+        </is>
+      </c>
+      <c r="C7" s="292" t="inlineStr">
+        <is>
+          <t>Testing guide + Contributing guide + ADR browser section</t>
+        </is>
+      </c>
+      <c r="D7" s="284" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="E7" s="292" t="inlineStr">
+        <is>
+          <t>Testing guide, ADR config</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="284" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="B8" s="284" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C8" s="292" t="inlineStr">
+        <is>
+          <t>Docs theme: dark-first design, landing page, navigation, search</t>
+        </is>
+      </c>
+      <c r="D8" s="284" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="E8" s="292" t="inlineStr">
+        <is>
+          <t>Custom theme, layout</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="284" t="inlineStr">
+        <is>
+          <t>NK</t>
+        </is>
+      </c>
+      <c r="B9" s="284" t="inlineStr">
+        <is>
+          <t>Frontend Lead</t>
+        </is>
+      </c>
+      <c r="C9" s="292" t="inlineStr">
+        <is>
+          <t>Component gallery: 23 components with live previews + props</t>
+        </is>
+      </c>
+      <c r="D9" s="284" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="E9" s="292" t="inlineStr">
+        <is>
+          <t>23 component pages</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="284" t="inlineStr">
+        <is>
+          <t>VS</t>
+        </is>
+      </c>
+      <c r="B10" s="284" t="inlineStr">
+        <is>
+          <t>Component Dev</t>
+        </is>
+      </c>
+      <c r="C10" s="292" t="inlineStr">
+        <is>
+          <t>Workflow engine + notification + billing/RBAC guides</t>
+        </is>
+      </c>
+      <c r="D10" s="284" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="E10" s="292" t="inlineStr">
+        <is>
+          <t>5+ MDX guide files</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
@@ -18740,7 +19033,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="140">
       <c r="A3" s="143" t="inlineStr">
         <is>
@@ -19882,7 +20174,6 @@
     <row r="34" ht="15" customHeight="1" s="140">
       <c r="F34" s="253" t="n"/>
     </row>
-    <row r="35"/>
     <row r="36" ht="15" customHeight="1" s="140">
       <c r="A36" s="139" t="inlineStr">
         <is>
@@ -19952,7 +20243,6 @@
         </is>
       </c>
     </row>
-    <row r="39"/>
     <row r="40" ht="15.75" customHeight="1" s="140">
       <c r="A40" s="254" t="inlineStr">
         <is>
@@ -20083,7 +20373,6 @@
         </is>
       </c>
     </row>
-    <row r="52"/>
     <row r="53" ht="15" customHeight="1" s="140">
       <c r="A53" s="210" t="inlineStr">
         <is>
@@ -21327,29 +21616,53 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="293" t="inlineStr">
+        <is>
+          <t>Sprint 4.0 Standup — 2026-03-10 — Documentation Engine Discussion</t>
+        </is>
+      </c>
+    </row>
     <row r="4" ht="15" customHeight="1" s="140">
       <c r="A4" s="267" t="inlineStr">
         <is>
-          <t>FOUNDER'S DECISION</t>
+          <t>Docs Engine</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Fumadocs (Next.js, open-source, MDX, AI-ready)</t>
         </is>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="140">
       <c r="A5" s="231" t="inlineStr">
         <is>
-          <t>Adopt Medusa v2-inspired patterns — Phased &amp; Pragmatic</t>
+          <t>Location</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>AI Search</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Anthropic Claude API for RAG-powered doc chat</t>
         </is>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="140">
       <c r="A7" s="268" t="inlineStr">
         <is>
-          <t>Phase</t>
+          <t>API Reference</t>
         </is>
       </c>
       <c r="B7" s="268" t="inlineStr">
         <is>
-          <t>Trigger</t>
+          <t>Auto-generated from OpenAPI 3.0 spec</t>
         </is>
       </c>
       <c r="C7" s="268" t="inlineStr">
@@ -21371,12 +21684,12 @@
     <row r="8" ht="15" customHeight="1" s="140">
       <c r="A8" s="269" t="inlineStr">
         <is>
-          <t>Phase 1: Sprint 2.9-3.0</t>
+          <t>TypeScript SDK</t>
         </is>
       </c>
       <c r="B8" s="269" t="inlineStr">
         <is>
-          <t>NOW</t>
+          <t>packages/sdk auto-generated from OpenAPI</t>
         </is>
       </c>
       <c r="C8" s="269" t="inlineStr">
@@ -21398,12 +21711,12 @@
     <row r="9" ht="15" customHeight="1" s="140">
       <c r="A9" s="269" t="inlineStr">
         <is>
-          <t>Phase 2: After 10 customers</t>
+          <t>Design</t>
         </is>
       </c>
       <c r="B9" s="269" t="inlineStr">
         <is>
-          <t>10 paying customers</t>
+          <t>Dark-first, --wl-* CSS vars, industrial aesthetic</t>
         </is>
       </c>
       <c r="C9" s="269" t="inlineStr">
@@ -21425,12 +21738,12 @@
     <row r="10" ht="15" customHeight="1" s="140">
       <c r="A10" s="269" t="inlineStr">
         <is>
-          <t>Phase 3: After 50 customers</t>
+          <t>Component Gallery</t>
         </is>
       </c>
       <c r="B10" s="269" t="inlineStr">
         <is>
-          <t>50 paying customers</t>
+          <t>23 components with live previews</t>
         </is>
       </c>
       <c r="C10" s="269" t="inlineStr">
@@ -21446,6 +21759,18 @@
       <c r="E10" s="271" t="inlineStr">
         <is>
           <t>Deferred</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Target</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Sprint 4.1 — all 9 agents</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(sprint-4.1): documentation engine, TypeScript SDK & OpenAPI spec
- ADR-020: Documentation engine architecture (Fumadocs selection)
- Fumadocs docs app (apps/docs): 69 files, Next.js 15, dark theme,
  AI-powered search via Claude API, 30+ MDX pages covering API
  reference, getting started, architecture, self-hosting, platform
  adapters, component gallery, system guides, contributing, and ADRs
- OpenAPI 3.0 specification for all API endpoints
- TypeScript SDK (packages/sdk): @witylogix/sdk zero-dep HTTP client
  with auto-retry, typed resources (orders, drivers, zones, shipments),
  8 error classes, dual CJS/ESM output
- Platform adapter guides: Shopify, WooCommerce, Magento, Custom
- Component gallery: 11 MDX pages documenting all 23 UI components
- Updated README, CHANGELOG, sprint tracker

Sprint 4.1: 84 files changed, +20,952 lines

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/witylogix-sprint-tracker.xlsx
+++ b/witylogix-sprint-tracker.xlsx
@@ -699,7 +699,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="294">
+  <cellXfs count="295">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -1568,6 +1568,9 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="55" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -19018,7 +19021,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:V125"/>
+  <dimension ref="A1:W125"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.66796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="20" customWidth="1" style="139" min="1" max="1"/>
@@ -19036,7 +19039,7 @@
     <row r="3" ht="15" customHeight="1" s="140">
       <c r="A3" s="143" t="inlineStr">
         <is>
-          <t>SPRINT PROGRESS (as of Sprint 4.0)</t>
+          <t>SPRINT PROGRESS (as of Sprint 4.1)</t>
         </is>
       </c>
       <c r="B3" s="143" t="n"/>
@@ -19047,7 +19050,7 @@
     <row r="4" ht="15" customHeight="1" s="140">
       <c r="A4" s="150" t="inlineStr">
         <is>
-          <t>Last Updated: Sprint 4.0 (2026-03-10)</t>
+          <t>Last Updated: Sprint 4.1 (2026-03-10)</t>
         </is>
       </c>
       <c r="B4" s="150" t="n"/>
@@ -19166,6 +19169,11 @@
           <t>Sprint 4.0</t>
         </is>
       </c>
+      <c r="W5" s="283" t="inlineStr">
+        <is>
+          <t>Sprint 4.1</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="140">
       <c r="A6" s="150" t="inlineStr">
@@ -19236,6 +19244,9 @@
       <c r="V6" s="284" t="n">
         <v>2200</v>
       </c>
+      <c r="W6" s="294" t="n">
+        <v>2280</v>
+      </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="140">
       <c r="A7" s="146" t="inlineStr">
@@ -19306,6 +19317,9 @@
       <c r="V7" s="284" t="n">
         <v>350000</v>
       </c>
+      <c r="W7" s="294" t="n">
+        <v>371000</v>
+      </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="140">
       <c r="A8" s="149" t="inlineStr">
@@ -19376,6 +19390,9 @@
       <c r="V8" s="284" t="n">
         <v>66</v>
       </c>
+      <c r="W8" s="294" t="n">
+        <v>66</v>
+      </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="140">
       <c r="A9" s="139" t="inlineStr">
@@ -19446,6 +19463,9 @@
       <c r="V9" s="284" t="n">
         <v>73</v>
       </c>
+      <c r="W9" s="294" t="n">
+        <v>73</v>
+      </c>
     </row>
     <row r="10" ht="17.25" customHeight="1" s="140">
       <c r="A10" s="163" t="inlineStr">
@@ -19516,6 +19536,9 @@
       <c r="V10" s="284" t="n">
         <v>31</v>
       </c>
+      <c r="W10" s="294" t="n">
+        <v>31</v>
+      </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="140">
       <c r="A11" s="139" t="inlineStr">
@@ -19586,6 +19609,9 @@
       <c r="V11" s="284" t="n">
         <v>74</v>
       </c>
+      <c r="W11" s="294" t="n">
+        <v>74</v>
+      </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="140">
       <c r="A12" s="143" t="inlineStr">
@@ -19648,6 +19674,9 @@
         <v>139</v>
       </c>
       <c r="V12" s="284" t="n">
+        <v>180</v>
+      </c>
+      <c r="W12" s="294" t="n">
         <v>180</v>
       </c>
     </row>
@@ -19689,6 +19718,9 @@
       <c r="V13" s="284" t="n">
         <v>12</v>
       </c>
+      <c r="W13" s="294" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="140">
       <c r="A14" s="239" t="inlineStr">
@@ -19728,6 +19760,9 @@
       <c r="V14" s="284" t="n">
         <v>180</v>
       </c>
+      <c r="W14" s="294" t="n">
+        <v>180</v>
+      </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="140">
       <c r="A15" s="150" t="inlineStr">
@@ -19765,6 +19800,9 @@
         <v>3808</v>
       </c>
       <c r="V15" s="284" t="n">
+        <v>4676</v>
+      </c>
+      <c r="W15" s="294" t="n">
         <v>4676</v>
       </c>
     </row>
@@ -21629,7 +21667,7 @@
           <t>Docs Engine</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="139" t="inlineStr">
         <is>
           <t>Fumadocs (Next.js, open-source, MDX, AI-ready)</t>
         </is>
@@ -21643,12 +21681,12 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="139" t="inlineStr">
         <is>
           <t>AI Search</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="139" t="inlineStr">
         <is>
           <t>Anthropic Claude API for RAG-powered doc chat</t>
         </is>
@@ -21763,12 +21801,12 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="139" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="139" t="inlineStr">
         <is>
           <t>Sprint 4.1 — all 9 agents</t>
         </is>

</xml_diff>

<commit_message>
docs(standup): Sprint 4.2 standup notes + Sprint 4.3 CLI deployment tool plan
- Standup recap: Sprint 4.2 shipped (SDK tests, seed, driver app, CLI scripts)
- Deep dive: witylogix CLI — one-line VM deployment tool (12 subcommands)
- Architecture decision: pure bash CLI, Caddy reverse proxy, AI diagnostics
- New team member: ZR — Zara (AI Engineer) for AI-powered features
- Sprint 4.3 plan: 10 agents, full CLI tool in infra/cli/

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/witylogix-sprint-tracker.xlsx
+++ b/witylogix-sprint-tracker.xlsx
@@ -24,6 +24,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 4.0 Plan" sheetId="15" state="visible" r:id="rId15"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 4.1 Plan" sheetId="16" state="visible" r:id="rId16"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 4.2 Plan" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 4.3 Plan" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Data Models Gap'!$A$1:$K$40</definedName>
@@ -723,7 +724,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="300">
+  <cellXfs count="301">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -1608,6 +1609,7 @@
     <xf numFmtId="0" fontId="64" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="64" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5483,6 +5485,286 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" style="140" min="1" max="1"/>
+    <col width="40" customWidth="1" style="140" min="2" max="2"/>
+    <col width="70" customWidth="1" style="140" min="3" max="3"/>
+    <col width="18" customWidth="1" style="140" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="295" t="inlineStr">
+        <is>
+          <t>Sprint 4.3 — witylogix CLI Deployment Tool + AI Engineer Onboarding</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="296" t="inlineStr">
+        <is>
+          <t>Theme: One-line VM deployment, CLI subcommands, Caddy SSL, AI diagnostics, production Docker Compose</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="297" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="B3" s="297" t="inlineStr">
+        <is>
+          <t>Assignment</t>
+        </is>
+      </c>
+      <c r="C3" s="297" t="inlineStr">
+        <is>
+          <t>Deliverables</t>
+        </is>
+      </c>
+      <c r="D3" s="297" t="inlineStr">
+        <is>
+          <t>Skill(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="65" customHeight="1" s="140">
+      <c r="A4" s="298" t="inlineStr">
+        <is>
+          <t>AR - Aarav (CTO)</t>
+        </is>
+      </c>
+      <c r="B4" s="298" t="inlineStr">
+        <is>
+          <t>ADR-022 CLI Architecture + main entrypoint</t>
+        </is>
+      </c>
+      <c r="C4" s="298" t="inlineStr">
+        <is>
+          <t>docs/adr/ADR-022-cli-deployment-tool.md (~500 lines), infra/cli/witylogix (main script ~300 lines with subcommand routing, help, version, color output, config loader)</t>
+        </is>
+      </c>
+      <c r="D4" s="298" t="inlineStr">
+        <is>
+          <t>system-design</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="65" customHeight="1" s="140">
+      <c r="A5" s="299" t="inlineStr">
+        <is>
+          <t>RG - Raj (Backend)</t>
+        </is>
+      </c>
+      <c r="B5" s="299" t="inlineStr">
+        <is>
+          <t>deploy + install subcommands</t>
+        </is>
+      </c>
+      <c r="C5" s="299" t="inlineStr">
+        <is>
+          <t>infra/cli/commands/install.sh (~200 lines — Docker bootstrap, dir creation, image pull), infra/cli/commands/deploy.sh (~300 lines — build/pull, migrate, seed, start, health wait, zero-downtime detection)</t>
+        </is>
+      </c>
+      <c r="D5" s="299" t="inlineStr">
+        <is>
+          <t>system-design</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="65" customHeight="1" s="140">
+      <c r="A6" s="298" t="inlineStr">
+        <is>
+          <t>PK - Priya (Sr. Backend)</t>
+        </is>
+      </c>
+      <c r="B6" s="298" t="inlineStr">
+        <is>
+          <t>backup + restore + upgrade subcommands</t>
+        </is>
+      </c>
+      <c r="C6" s="298" t="inlineStr">
+        <is>
+          <t>infra/cli/commands/backup.sh (~200 lines — pg_dump with compression, S3 upload optional, rotation), infra/cli/commands/restore.sh (~150 lines), infra/cli/commands/upgrade.sh (~200 lines — pull, migrate, rolling restart)</t>
+        </is>
+      </c>
+      <c r="D6" s="298" t="inlineStr">
+        <is>
+          <t>system-design</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="65" customHeight="1" s="140">
+      <c r="A7" s="299" t="inlineStr">
+        <is>
+          <t>SP - Sanjay (Full-stack)</t>
+        </is>
+      </c>
+      <c r="B7" s="299" t="inlineStr">
+        <is>
+          <t>ssl + env subcommands</t>
+        </is>
+      </c>
+      <c r="C7" s="299" t="inlineStr">
+        <is>
+          <t>infra/cli/commands/ssl.sh (~200 lines — Caddy config generator, domain setup, cert check), infra/cli/commands/env.sh (~250 lines — interactive .env configurator, validation, secret generation)</t>
+        </is>
+      </c>
+      <c r="D7" s="299" t="inlineStr">
+        <is>
+          <t>system-design</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="65" customHeight="1" s="140">
+      <c r="A8" s="298" t="inlineStr">
+        <is>
+          <t>ZR - Zara (AI Engineer)</t>
+        </is>
+      </c>
+      <c r="B8" s="298" t="inlineStr">
+        <is>
+          <t>ai setup + ai diagnose subcommands</t>
+        </is>
+      </c>
+      <c r="C8" s="298" t="inlineStr">
+        <is>
+          <t>infra/cli/commands/ai.sh (~300 lines — Claude API key config, log collector, diagnostic prompt builder, structured output parser), infra/cli/templates/ai-diagnose-prompt.txt</t>
+        </is>
+      </c>
+      <c r="D8" s="298" t="inlineStr">
+        <is>
+          <t>system-design</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="65" customHeight="1" s="140">
+      <c r="A9" s="299" t="inlineStr">
+        <is>
+          <t>NK - Neha (Frontend Lead)</t>
+        </is>
+      </c>
+      <c r="B9" s="299" t="inlineStr">
+        <is>
+          <t>dev subcommand</t>
+        </is>
+      </c>
+      <c r="C9" s="299" t="inlineStr">
+        <is>
+          <t>infra/cli/commands/dev.sh (~250 lines — dependency checker, port allocator, env validator, turbo boot with status table, process manager, graceful shutdown handler)</t>
+        </is>
+      </c>
+      <c r="D9" s="299" t="inlineStr">
+        <is>
+          <t>system-design</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="65" customHeight="1" s="140">
+      <c r="A10" s="298" t="inlineStr">
+        <is>
+          <t>DM - Dev (Frontend)</t>
+        </is>
+      </c>
+      <c r="B10" s="298" t="inlineStr">
+        <is>
+          <t>status + doctor subcommands</t>
+        </is>
+      </c>
+      <c r="C10" s="298" t="inlineStr">
+        <is>
+          <t>infra/cli/commands/status.sh (~200 lines — HTTP probes for all services, formatted table), infra/cli/commands/doctor.sh (~250 lines — disk/mem/ports/DNS/Docker/connectivity checks, report generator)</t>
+        </is>
+      </c>
+      <c r="D10" s="298" t="inlineStr">
+        <is>
+          <t>system-design</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="65" customHeight="1" s="140">
+      <c r="A11" s="299" t="inlineStr">
+        <is>
+          <t>KS - Kavitha (QA Lead)</t>
+        </is>
+      </c>
+      <c r="B11" s="299" t="inlineStr">
+        <is>
+          <t>CLI tests + init subcommand</t>
+        </is>
+      </c>
+      <c r="C11" s="299" t="inlineStr">
+        <is>
+          <t>infra/cli/commands/init.sh (~200 lines — contributor setup, deps install, prisma generate, seed, smoke test), infra/cli/__tests__/test-cli.sh (~300 lines — test harness for all subcommands), CI workflow update</t>
+        </is>
+      </c>
+      <c r="D11" s="299" t="inlineStr">
+        <is>
+          <t>testing-strategy</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="65" customHeight="1" s="140">
+      <c r="A12" s="298" t="inlineStr">
+        <is>
+          <t>VS - Vikram (Component)</t>
+        </is>
+      </c>
+      <c r="B12" s="298" t="inlineStr">
+        <is>
+          <t>logs + scale + destroy subcommands</t>
+        </is>
+      </c>
+      <c r="C12" s="298" t="inlineStr">
+        <is>
+          <t>infra/cli/commands/logs.sh (~150 lines — multi-service log tailing with color), infra/cli/commands/scale.sh (~100 lines — Docker Compose scale wrapper), infra/cli/commands/destroy.sh (~120 lines — clean teardown with confirmation)</t>
+        </is>
+      </c>
+      <c r="D12" s="298" t="inlineStr">
+        <is>
+          <t>system-design</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="65" customHeight="1" s="140">
+      <c r="A13" s="299" t="inlineStr">
+        <is>
+          <t>AM - Aisha (Integration)</t>
+        </is>
+      </c>
+      <c r="B13" s="299" t="inlineStr">
+        <is>
+          <t>Caddy templates + production Docker Compose</t>
+        </is>
+      </c>
+      <c r="C13" s="299" t="inlineStr">
+        <is>
+          <t>infra/cli/templates/Caddyfile (~80 lines — reverse proxy for api/app/docs with auto-SSL), infra/docker-compose.prod.yml (~200 lines — production-grade with healthchecks, restart policies, resource limits, Caddy service), infra/cli/templates/env.template</t>
+        </is>
+      </c>
+      <c r="D13" s="299" t="inlineStr">
+        <is>
+          <t>system-design</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
@@ -21959,7 +22241,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G44"/>
+  <dimension ref="A1:G53"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="28" customWidth="1" style="139" min="1" max="2"/>
@@ -22818,6 +23100,62 @@
         </is>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" s="293" t="inlineStr">
+        <is>
+          <t>Sprint 4.2 Standup — 2026-03-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="300" t="inlineStr">
+        <is>
+          <t>Sprint 4.2 shipped: ADR-021, SDK tests (141 cases), seed script, driver app screens, settings page, webhook dashboard, 5 new UI components, smoke test, CI updates</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="300" t="inlineStr">
+        <is>
+          <t>Deep dive: CLI deployment tool for one-line VM deployment</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="300" t="inlineStr">
+        <is>
+          <t>Decision: Pure bash CLI (witylogix) with 12 subcommands — install, deploy, upgrade, status, logs, backup, restore, ssl, env, doctor, scale, destroy</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="300" t="inlineStr">
+        <is>
+          <t>Decision: Caddy for reverse proxy with auto-SSL (api/app/docs subdomain routing)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="300" t="inlineStr">
+        <is>
+          <t>Decision: AI subcommands (ai setup, ai diagnose) for Claude-powered diagnostics</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="300" t="inlineStr">
+        <is>
+          <t>NEW TEAM MEMBER: ZR — Zara (AI Engineer) — AI-powered features, docs search, CLI diagnostics, log analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="300" t="inlineStr">
+        <is>
+          <t>Sprint 4.3 planned: Full CLI tool (infra/cli/witylogix), Caddy templates, production Docker Compose, AI diagnostics, CLI tests</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A2:G2"/>

</xml_diff>

<commit_message>
feat(sprint-4.3): CLI deployment tool, AI diagnostics & production Docker Compose
- ADR-022: CLI architecture decision (bash-only, Caddy, 15 subcommands)
- `witylogix` CLI entrypoint with ASCII banner, color logging, global flags
- 15 subcommands: install, deploy, upgrade, backup, restore, ssl, env, status, doctor, logs, scale, destroy, dev, init, ai
- AI diagnostics: Claude-powered `ai diagnose` and `ai optimize` commands
- Caddy reverse proxy templates with security headers and auto-SSL
- Production Docker Compose (6 services + worker, resource limits, healthchecks)
- Dockerfile.docs for multi-stage Next.js docs build
- CLI test harness (486 lines) and shared lib (423 lines)
- Production env template (219 lines, 16 sections)

31 files changed, +9,391 lines | Team: AR, RG, PK, SP, ZR, NK, DM, KS, VS, AM

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/witylogix-sprint-tracker.xlsx
+++ b/witylogix-sprint-tracker.xlsx
@@ -19598,7 +19598,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:X125"/>
+  <dimension ref="A1:Y125"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.66796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="20" customWidth="1" style="139" min="1" max="1"/>
@@ -19616,7 +19616,7 @@
     <row r="3" ht="15" customHeight="1" s="140">
       <c r="A3" s="143" t="inlineStr">
         <is>
-          <t>SPRINT PROGRESS (as of Sprint 4.2)</t>
+          <t>SPRINT PROGRESS (as of Sprint 4.3)</t>
         </is>
       </c>
       <c r="B3" s="143" t="n"/>
@@ -19627,7 +19627,7 @@
     <row r="4" ht="15" customHeight="1" s="140">
       <c r="A4" s="150" t="inlineStr">
         <is>
-          <t>Last Updated: Sprint 4.2 (2026-03-10)</t>
+          <t>Last Updated: Sprint 4.3 (2026-03-10)</t>
         </is>
       </c>
       <c r="B4" s="150" t="n"/>
@@ -19756,6 +19756,11 @@
           <t>Sprint 4.2</t>
         </is>
       </c>
+      <c r="Y5" s="283" t="inlineStr">
+        <is>
+          <t>Sprint 4.3</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="140">
       <c r="A6" s="150" t="inlineStr">
@@ -19832,6 +19837,9 @@
       <c r="X6" s="294" t="n">
         <v>2320</v>
       </c>
+      <c r="Y6" s="284" t="n">
+        <v>2343</v>
+      </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="140">
       <c r="A7" s="146" t="inlineStr">
@@ -19908,6 +19916,9 @@
       <c r="X7" s="294" t="n">
         <v>383000</v>
       </c>
+      <c r="Y7" s="284" t="n">
+        <v>392000</v>
+      </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="140">
       <c r="A8" s="149" t="inlineStr">
@@ -19984,6 +19995,9 @@
       <c r="X8" s="294" t="n">
         <v>70</v>
       </c>
+      <c r="Y8" s="284" t="n">
+        <v>70</v>
+      </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="140">
       <c r="A9" s="139" t="inlineStr">
@@ -20060,6 +20074,9 @@
       <c r="X9" s="294" t="n">
         <v>74</v>
       </c>
+      <c r="Y9" s="284" t="n">
+        <v>74</v>
+      </c>
     </row>
     <row r="10" ht="17.25" customHeight="1" s="140">
       <c r="A10" s="163" t="inlineStr">
@@ -20136,6 +20153,9 @@
       <c r="X10" s="294" t="n">
         <v>31</v>
       </c>
+      <c r="Y10" s="284" t="n">
+        <v>31</v>
+      </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="140">
       <c r="A11" s="139" t="inlineStr">
@@ -20212,6 +20232,9 @@
       <c r="X11" s="294" t="n">
         <v>74</v>
       </c>
+      <c r="Y11" s="284" t="n">
+        <v>74</v>
+      </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="140">
       <c r="A12" s="143" t="inlineStr">
@@ -20281,6 +20304,9 @@
       </c>
       <c r="X12" s="294" t="n">
         <v>190</v>
+      </c>
+      <c r="Y12" s="284" t="n">
+        <v>191</v>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="140">
@@ -20327,6 +20353,9 @@
       <c r="X13" s="294" t="n">
         <v>12</v>
       </c>
+      <c r="Y13" s="284" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="140">
       <c r="A14" s="239" t="inlineStr">
@@ -20372,6 +20401,9 @@
       <c r="X14" s="294" t="n">
         <v>190</v>
       </c>
+      <c r="Y14" s="284" t="n">
+        <v>191</v>
+      </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="140">
       <c r="A15" s="150" t="inlineStr">
@@ -20417,6 +20449,9 @@
       <c r="X15" s="294" t="n">
         <v>4817</v>
       </c>
+      <c r="Y15" s="284" t="n">
+        <v>4817</v>
+      </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="140">
       <c r="A16" s="230" t="inlineStr">
@@ -20472,6 +20507,9 @@
       <c r="V16" s="284" t="n">
         <v>12</v>
       </c>
+      <c r="Y16" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="140">
       <c r="A17" s="149" t="inlineStr">
@@ -20523,6 +20561,9 @@
       <c r="V17" s="284" t="n">
         <v>4</v>
       </c>
+      <c r="Y17" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="140">
       <c r="A18" s="139" t="inlineStr">
@@ -20573,6 +20614,9 @@
       <c r="V18" s="284" t="n">
         <v>10</v>
       </c>
+      <c r="Y18" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="19" ht="17.25" customHeight="1" s="140">
       <c r="A19" s="163" t="inlineStr">
@@ -20621,6 +20665,9 @@
         <v>8</v>
       </c>
       <c r="V19" s="284" t="n">
+        <v>8</v>
+      </c>
+      <c r="Y19" t="n">
         <v>8</v>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: update competitive report v2 with Routific & Pickeasy analysis
Added 2 new competitors: Routific (route optimization SaaS, 179 ML models,
191M+ deliveries) and Pickeasy (Shopify checkout widget, 8K+ merchants).
Feature matrix expanded to 48 features × 7 platforms. Sprint 4.5 plan
updated with UX benchmarks from Routific dispatcher dashboard + Pickeasy
date/time picker.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/witylogix-sprint-tracker.xlsx
+++ b/witylogix-sprint-tracker.xlsx
@@ -26,6 +26,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 4.2 Plan" sheetId="17" state="visible" r:id="rId17"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 4.3 Plan" sheetId="18" state="visible" r:id="rId18"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 4.4 Plan" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 4.5 Plan" sheetId="20" state="visible" r:id="rId20"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Data Models Gap'!$A$1:$K$40</definedName>
@@ -43,7 +44,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="70">
+  <fonts count="72">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -515,8 +516,17 @@
       <b val="1"/>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00E63946"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="000F3460"/>
+    </font>
   </fonts>
-  <fills count="35">
+  <fills count="37">
     <fill>
       <patternFill/>
     </fill>
@@ -713,8 +723,20 @@
         <bgColor rgb="0016213E"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001B2A4A"/>
+        <bgColor rgb="001B2A4A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8F0FE"/>
+        <bgColor rgb="00E8F0FE"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -753,6 +775,12 @@
       <bottom style="thin"/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
@@ -764,7 +792,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="308">
+  <cellXfs count="315">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -1665,6 +1693,21 @@
     <xf numFmtId="0" fontId="69" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="62" fillId="35" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="56" fillId="35" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="70" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="71" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -6578,6 +6621,464 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" style="140" min="1" max="1"/>
+    <col width="16" customWidth="1" style="140" min="2" max="2"/>
+    <col width="28" customWidth="1" style="140" min="3" max="3"/>
+    <col width="34" customWidth="1" style="140" min="4" max="4"/>
+    <col width="36" customWidth="1" style="140" min="5" max="5"/>
+    <col width="28" customWidth="1" style="140" min="6" max="6"/>
+    <col width="10" customWidth="1" style="140" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="310" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="B1" s="310" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="C1" s="310" t="inlineStr">
+        <is>
+          <t>Sprint 4.5 Task</t>
+        </is>
+      </c>
+      <c r="D1" s="310" t="inlineStr">
+        <is>
+          <t>Files/Packages</t>
+        </is>
+      </c>
+      <c r="E1" s="310" t="inlineStr">
+        <is>
+          <t>Key Deliverables</t>
+        </is>
+      </c>
+      <c r="F1" s="310" t="inlineStr">
+        <is>
+          <t>Competitive Benchmark</t>
+        </is>
+      </c>
+      <c r="G1" s="310" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="311" t="inlineStr">
+        <is>
+          <t>AR</t>
+        </is>
+      </c>
+      <c r="B2" s="311" t="inlineStr">
+        <is>
+          <t>CTO / Architect</t>
+        </is>
+      </c>
+      <c r="C2" s="311" t="inlineStr">
+        <is>
+          <t>Route Timeline Dispatcher Dashboard (Routific-quality)</t>
+        </is>
+      </c>
+      <c r="D2" s="311" t="inlineStr">
+        <is>
+          <t>apps/dashboard/src/app/(dashboard)/dispatch/, packages/core/src/dispatch/</t>
+        </is>
+      </c>
+      <c r="E2" s="311" t="inlineStr">
+        <is>
+          <t>Map with color-coded driver routes + timeline view (8am-7pm). Unscheduled/Scheduled toggle. Drag-and-drop route editing. Real-time stats bar (drivers, stops, km, time).</t>
+        </is>
+      </c>
+      <c r="F2" s="311" t="inlineStr">
+        <is>
+          <t>Routific: 10 color-coded routes, 540 stops, timeline per driver</t>
+        </is>
+      </c>
+      <c r="G2" s="311" t="inlineStr">
+        <is>
+          <t>PLANNED</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="312" t="inlineStr">
+        <is>
+          <t>NK</t>
+        </is>
+      </c>
+      <c r="B3" s="312" t="inlineStr">
+        <is>
+          <t>Frontend Lead</t>
+        </is>
+      </c>
+      <c r="C3" s="312" t="inlineStr">
+        <is>
+          <t>Checkout Date/Time Picker Widget (Pickeasy-quality)</t>
+        </is>
+      </c>
+      <c r="D3" s="312" t="inlineStr">
+        <is>
+          <t>packages/checkout-widget/, extensions/checkout-ui/</t>
+        </is>
+      </c>
+      <c r="E3" s="312" t="inlineStr">
+        <is>
+          <t>Embeddable widget: date calendar, time slot grid with capacity indicators, zone-based rate display, blackout dates, cut-off times, zipcode validation, prep time settings.</t>
+        </is>
+      </c>
+      <c r="F3" s="312" t="inlineStr">
+        <is>
+          <t>Pickeasy: 8K merchants, slot limits, blackout, zip validation, $9.99-49.99</t>
+        </is>
+      </c>
+      <c r="G3" s="312" t="inlineStr">
+        <is>
+          <t>PLANNED</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="311" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="B4" s="311" t="inlineStr">
+        <is>
+          <t>Frontend Dev</t>
+        </is>
+      </c>
+      <c r="C4" s="311" t="inlineStr">
+        <is>
+          <t>Customer Self-Service Portal</t>
+        </is>
+      </c>
+      <c r="D4" s="311" t="inlineStr">
+        <is>
+          <t>apps/customer-portal/</t>
+        </is>
+      </c>
+      <c r="E4" s="311" t="inlineStr">
+        <is>
+          <t>Next.js portal: order history with timeline, live tracking, rescheduling flow, delivery preferences (safe place, instructions), driver ratings, notification preferences.</t>
+        </is>
+      </c>
+      <c r="F4" s="311" t="inlineStr">
+        <is>
+          <t>Route4Me: only platform with self-service portal. First-mover for open-source</t>
+        </is>
+      </c>
+      <c r="G4" s="311" t="inlineStr">
+        <is>
+          <t>PLANNED</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="312" t="inlineStr">
+        <is>
+          <t>RG</t>
+        </is>
+      </c>
+      <c r="B5" s="312" t="inlineStr">
+        <is>
+          <t>Backend Lead</t>
+        </is>
+      </c>
+      <c r="C5" s="312" t="inlineStr">
+        <is>
+          <t>Slot Engine API &amp; Capacity Management</t>
+        </is>
+      </c>
+      <c r="D5" s="312" t="inlineStr">
+        <is>
+          <t>packages/core/src/slots/, apps/api/src/routes/checkout/</t>
+        </is>
+      </c>
+      <c r="E5" s="312" t="inlineStr">
+        <is>
+          <t>Slot availability API, capacity limits per slot/day, zone-rate calculator, order deadline engine (e.g. Friday pickup by Thu 4pm), cart integration endpoints.</t>
+        </is>
+      </c>
+      <c r="F5" s="312" t="inlineStr">
+        <is>
+          <t>Pickeasy: order deadlines, daily limits, product-specific slots</t>
+        </is>
+      </c>
+      <c r="G5" s="312" t="inlineStr">
+        <is>
+          <t>PLANNED</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="311" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="B6" s="311" t="inlineStr">
+        <is>
+          <t>Sr. Backend</t>
+        </is>
+      </c>
+      <c r="C6" s="311" t="inlineStr">
+        <is>
+          <t>POD v2: Photo + Signature + QR + Status Timeline</t>
+        </is>
+      </c>
+      <c r="D6" s="311" t="inlineStr">
+        <is>
+          <t>packages/core/src/pod/, apps/api/src/routes/pod/</t>
+        </is>
+      </c>
+      <c r="E6" s="311" t="inlineStr">
+        <is>
+          <t>Multi-method POD: photo capture, e-signature pad, QR/barcode scan. Delivery status timeline (Planned → Out for Delivery → Delivered + photo). S3/R2 storage.</t>
+        </is>
+      </c>
+      <c r="F6" s="311" t="inlineStr">
+        <is>
+          <t>Routific: status timeline with photo. Fleetbase: QR+signature+manual</t>
+        </is>
+      </c>
+      <c r="G6" s="311" t="inlineStr">
+        <is>
+          <t>PLANNED</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="312" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="B7" s="312" t="inlineStr">
+        <is>
+          <t>Full-stack</t>
+        </is>
+      </c>
+      <c r="C7" s="312" t="inlineStr">
+        <is>
+          <t>Customer Notification Engine v2 + SMS/WhatsApp</t>
+        </is>
+      </c>
+      <c r="D7" s="312" t="inlineStr">
+        <is>
+          <t>packages/core/src/notifications-v2/, apps/api/src/routes/notifications/</t>
+        </is>
+      </c>
+      <c r="E7" s="312" t="inlineStr">
+        <is>
+          <t>Multi-channel: email + SMS (Twilio) + WhatsApp (Meta Business) + push. Template engine. SMS with tracking link + time window (Routific pattern). Delivery webhooks.</t>
+        </is>
+      </c>
+      <c r="F7" s="312" t="inlineStr">
+        <is>
+          <t>Routific: SMS with tracking link + time window. ScrollEngine: WhatsApp</t>
+        </is>
+      </c>
+      <c r="G7" s="312" t="inlineStr">
+        <is>
+          <t>PLANNED</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="311" t="inlineStr">
+        <is>
+          <t>VS</t>
+        </is>
+      </c>
+      <c r="B8" s="311" t="inlineStr">
+        <is>
+          <t>Component Dev</t>
+        </is>
+      </c>
+      <c r="C8" s="311" t="inlineStr">
+        <is>
+          <t>Checkout &amp; Dispatch Component Library</t>
+        </is>
+      </c>
+      <c r="D8" s="311" t="inlineStr">
+        <is>
+          <t>packages/checkout-widget/src/, apps/dashboard/src/components/dispatch/</t>
+        </is>
+      </c>
+      <c r="E8" s="311" t="inlineStr">
+        <is>
+          <t>Checkout: DatePicker, TimeSlotGrid, ZoneMap, DeliveryOptions, AddressAutocomplete. Dispatch: RouteTimeline, DriverCard, StopMarker, StatsBanner.</t>
+        </is>
+      </c>
+      <c r="F8" s="311" t="inlineStr">
+        <is>
+          <t>Routific timeline + Pickeasy checkout as UX reference</t>
+        </is>
+      </c>
+      <c r="G8" s="311" t="inlineStr">
+        <is>
+          <t>PLANNED</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="312" t="inlineStr">
+        <is>
+          <t>KS</t>
+        </is>
+      </c>
+      <c r="B9" s="312" t="inlineStr">
+        <is>
+          <t>QA Lead</t>
+        </is>
+      </c>
+      <c r="C9" s="312" t="inlineStr">
+        <is>
+          <t>E2E: Dispatch, Checkout &amp; Customer Portal</t>
+        </is>
+      </c>
+      <c r="D9" s="312" t="inlineStr">
+        <is>
+          <t>tests/e2e/specs/dispatch/, tests/e2e/specs/checkout/, tests/e2e/specs/portal/</t>
+        </is>
+      </c>
+      <c r="E9" s="312" t="inlineStr">
+        <is>
+          <t>Playwright suites: dispatch timeline interaction, checkout widget slot selection, customer portal auth + reschedule, POD photo upload, SMS notification delivery.</t>
+        </is>
+      </c>
+      <c r="F9" s="312" t="inlineStr">
+        <is>
+          <t>Full coverage for all Sprint 4.5 customer-facing features</t>
+        </is>
+      </c>
+      <c r="G9" s="312" t="inlineStr">
+        <is>
+          <t>PLANNED</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="311" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="B10" s="311" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="C10" s="311" t="inlineStr">
+        <is>
+          <t>Shopify Checkout Extension + Google Maps/Calendar</t>
+        </is>
+      </c>
+      <c r="D10" s="311" t="inlineStr">
+        <is>
+          <t>extensions/checkout-ui/, packages/core/src/integrations/google/</t>
+        </is>
+      </c>
+      <c r="E10" s="311" t="inlineStr">
+        <is>
+          <t>Shopify checkout extension with embedded date/time widget. Google Maps for zone visualization. Google Calendar sync for merchant order reminders.</t>
+        </is>
+      </c>
+      <c r="F10" s="311" t="inlineStr">
+        <is>
+          <t>Pickeasy: Google Maps + Calendar. Zapiet: Shopify certified</t>
+        </is>
+      </c>
+      <c r="G10" s="311" t="inlineStr">
+        <is>
+          <t>PLANNED</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="312" t="inlineStr">
+        <is>
+          <t>ZR</t>
+        </is>
+      </c>
+      <c r="B11" s="312" t="inlineStr">
+        <is>
+          <t>AI Engineer</t>
+        </is>
+      </c>
+      <c r="C11" s="312" t="inlineStr">
+        <is>
+          <t>Smart Slot Recommendation + ML ETA Engine</t>
+        </is>
+      </c>
+      <c r="D11" s="312" t="inlineStr">
+        <is>
+          <t>packages/core/src/ai-slots/, packages/core/src/ai-eta/</t>
+        </is>
+      </c>
+      <c r="E11" s="312" t="inlineStr">
+        <is>
+          <t>ML slot recommender: demand prediction, driver availability forecast. Traffic-aware ETA model (start with 3-5 models, target Routific's 179 as long-term goal).</t>
+        </is>
+      </c>
+      <c r="F11" s="312" t="inlineStr">
+        <is>
+          <t>Routific: 179 ML models. Nobody has AI slot recommendation — first-mover</t>
+        </is>
+      </c>
+      <c r="G11" s="312" t="inlineStr">
+        <is>
+          <t>PLANNED</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="313" t="inlineStr">
+        <is>
+          <t>THEME</t>
+        </is>
+      </c>
+      <c r="B13" s="309" t="inlineStr">
+        <is>
+          <t>Sprint 4.5: Customer Experience &amp; Checkout Enhancement — Routific-quality dispatcher dashboard, Pickeasy-quality checkout widget, customer self-service portal, POD v2 with status timeline, SMS/WhatsApp notifications, AI slot recommendation engine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="314" t="inlineStr">
+        <is>
+          <t>BENCHMARKS</t>
+        </is>
+      </c>
+      <c r="B14" s="309" t="inlineStr">
+        <is>
+          <t>UX: Routific dispatcher timeline + driver app + POD flow + SMS tracking. Checkout: Pickeasy date/time picker + slot capacity + blackout + zip validation. Portal: Route4Me self-service. Notifications: Routific SMS + ScrollEngine WhatsApp.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B14:G14"/>
+    <mergeCell ref="B13:G13"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
@@ -20062,7 +20563,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:Z125"/>
+  <dimension ref="A1:AA125"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.66796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="20" customWidth="1" style="139" min="1" max="1"/>
@@ -20076,6 +20577,11 @@
           <t>Gap Statistics Summary</t>
         </is>
       </c>
+      <c r="AA1" s="308" t="inlineStr">
+        <is>
+          <t>Sprint 4.5</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="15" customHeight="1" s="140">
       <c r="A3" s="143" t="inlineStr">
@@ -20087,6 +20593,11 @@
       <c r="C3" s="143" t="n"/>
       <c r="D3" s="143" t="n"/>
       <c r="E3" s="143" t="n"/>
+      <c r="AA3" s="309" t="inlineStr">
+        <is>
+          <t>Customer Experience &amp; Checkout</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="140">
       <c r="A4" s="150" t="inlineStr">
@@ -20098,6 +20609,11 @@
       <c r="C4" s="150" t="n"/>
       <c r="D4" s="150" t="n"/>
       <c r="E4" s="150" t="n"/>
+      <c r="AA4" s="309" t="inlineStr">
+        <is>
+          <t>1 (customer-portal)</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="140">
       <c r="A5" s="230" t="inlineStr">
@@ -20230,6 +20746,11 @@
           <t>Sprint 4.4</t>
         </is>
       </c>
+      <c r="AA5" s="309" t="inlineStr">
+        <is>
+          <t>2 (checkout-widget, ai-slots)</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="140">
       <c r="A6" s="150" t="inlineStr">
@@ -20312,6 +20833,9 @@
       <c r="Z6" s="284" t="n">
         <v>2410</v>
       </c>
+      <c r="AA6" s="309" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="140">
       <c r="A7" s="146" t="inlineStr">
@@ -20394,6 +20918,11 @@
       <c r="Z7" s="284" t="n">
         <v>423000</v>
       </c>
+      <c r="AA7" s="309" t="inlineStr">
+        <is>
+          <t>5 P0 + 3 P1 + 1 P2</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="140">
       <c r="A8" s="149" t="inlineStr">
@@ -20475,6 +21004,11 @@
       </c>
       <c r="Z8" s="284" t="n">
         <v>74</v>
+      </c>
+      <c r="AA8" s="309" t="inlineStr">
+        <is>
+          <t>Portal + Checkout Widget + POD v2 + Notif v2 + AI Slots</t>
+        </is>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="140">

</xml_diff>

<commit_message>
feat(sprint-4.7): telematics, traffic-aware ETA & integration ecosystem
Sprint 4.7 delivers telematics adapter layer (Samsara + Geotab), fleet
dashboard with vehicle management, courier partner adapters (Onfleet +
Stuart + Uber Direct), partner directory UI, invoice engine completion
with QuickBooks/Xero accounting integration, traffic-aware ETA v2
(Google Directions + TomTom), and ML ETA Engine v2 with 5-model ensemble.
Closes gaps G-11, G-12; finishes G-13; starts G-14.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/witylogix-sprint-tracker.xlsx
+++ b/witylogix-sprint-tracker.xlsx
@@ -47,7 +47,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="73">
+  <fonts count="74">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -580,6 +580,9 @@
     <font>
       <sz val="10"/>
     </font>
+    <font>
+      <sz val="11"/>
+    </font>
   </fonts>
   <fills count="41">
     <fill>
@@ -877,7 +880,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="370">
+  <cellXfs count="372">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -1985,6 +1988,12 @@
     </xf>
     <xf numFmtId="0" fontId="72" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="71" fillId="40" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="73" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -3233,7 +3242,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:AB125"/>
+  <dimension ref="A1:AC125"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.66796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="20" customWidth="1" style="185" min="1" max="1"/>
@@ -3257,6 +3266,11 @@
           <t>Sprint 4.6</t>
         </is>
       </c>
+      <c r="AC1" s="370" t="inlineStr">
+        <is>
+          <t>Sprint 4.7</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="15" customHeight="1" s="186">
       <c r="A3" s="189" t="inlineStr">
@@ -3266,7 +3280,7 @@
       </c>
       <c r="B3" s="189" t="inlineStr">
         <is>
-          <t>SPRINT PROGRESS (as of Sprint 4.6)</t>
+          <t>SPRINT PROGRESS (as of Sprint 4.7)</t>
         </is>
       </c>
       <c r="C3" s="189" t="n"/>
@@ -3286,7 +3300,7 @@
       </c>
       <c r="B4" s="196" t="inlineStr">
         <is>
-          <t>Last Updated: Sprint 4.6 (2026-03-11)</t>
+          <t>Last Updated: Sprint 4.7 (2026-03-11)</t>
         </is>
       </c>
       <c r="C4" s="196" t="n"/>
@@ -3437,6 +3451,9 @@
       <c r="AB5" s="300" t="n">
         <v>3280</v>
       </c>
+      <c r="AC5" s="371" t="n">
+        <v>2467</v>
+      </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="186">
       <c r="A6" s="196" t="inlineStr">
@@ -3525,6 +3542,9 @@
       <c r="AB6" s="300" t="n">
         <v>803280</v>
       </c>
+      <c r="AC6" s="371" t="n">
+        <v>845846</v>
+      </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="186">
       <c r="A7" s="192" t="inlineStr">
@@ -3613,6 +3633,9 @@
       <c r="AB7" s="300" t="n">
         <v>80</v>
       </c>
+      <c r="AC7" s="371" t="n">
+        <v>88</v>
+      </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="186">
       <c r="A8" s="195" t="inlineStr">
@@ -3701,6 +3724,9 @@
       <c r="AB8" s="300" t="n">
         <v>133</v>
       </c>
+      <c r="AC8" s="371" t="n">
+        <v>138</v>
+      </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="186">
       <c r="A9" s="185" t="inlineStr">
@@ -3789,6 +3815,9 @@
       <c r="AB9" s="300" t="n">
         <v>107</v>
       </c>
+      <c r="AC9" s="371" t="n">
+        <v>39</v>
+      </c>
     </row>
     <row r="10" ht="17.25" customHeight="1" s="186">
       <c r="A10" s="209" t="inlineStr">
@@ -3877,6 +3906,9 @@
       <c r="AB10" s="300" t="n">
         <v>65</v>
       </c>
+      <c r="AC10" s="371" t="n">
+        <v>70</v>
+      </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="186">
       <c r="A11" s="185" t="inlineStr">
@@ -3965,6 +3997,9 @@
       <c r="AB11" s="300" t="n">
         <v>247</v>
       </c>
+      <c r="AC11" s="371" t="n">
+        <v>266</v>
+      </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="186">
       <c r="A12" s="189" t="inlineStr">
@@ -4046,6 +4081,9 @@
       </c>
       <c r="AB12" s="300" t="n">
         <v>280</v>
+      </c>
+      <c r="AC12" s="371" t="n">
+        <v>310</v>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="186">
@@ -4104,6 +4142,9 @@
       <c r="AB13" s="300" t="n">
         <v>2800</v>
       </c>
+      <c r="AC13" s="371" t="n">
+        <v>3300</v>
+      </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="186">
       <c r="A14" s="304" t="inlineStr">
@@ -4161,6 +4202,9 @@
       <c r="AB14" s="300" t="n">
         <v>73</v>
       </c>
+      <c r="AC14" s="371" t="n">
+        <v>73</v>
+      </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="186">
       <c r="A15" s="196" t="inlineStr">
@@ -4218,6 +4262,9 @@
       <c r="AB15" s="300" t="n">
         <v>55</v>
       </c>
+      <c r="AC15" s="371" t="n">
+        <v>70</v>
+      </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="186">
       <c r="A16" s="291" t="inlineStr">
@@ -4282,6 +4329,9 @@
       <c r="AB16" s="300" t="n">
         <v>3</v>
       </c>
+      <c r="AC16" s="371" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="186">
       <c r="A17" s="195" t="inlineStr">
@@ -4342,6 +4392,9 @@
       <c r="AB17" s="300" t="n">
         <v>1</v>
       </c>
+      <c r="AC17" s="371" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="186">
       <c r="A18" s="185" t="inlineStr">
@@ -4401,6 +4454,9 @@
       <c r="AB18" s="300" t="n">
         <v>1</v>
       </c>
+      <c r="AC18" s="371" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="19" ht="17.25" customHeight="1" s="186">
       <c r="A19" s="209" t="inlineStr">
@@ -4458,6 +4514,9 @@
         <v>8</v>
       </c>
       <c r="AB19" s="300" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC19" s="371" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4487,6 +4546,9 @@
       <c r="AB20" s="300" t="n">
         <v>1</v>
       </c>
+      <c r="AC20" s="371" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="186">
       <c r="A21" s="308" t="inlineStr">
@@ -4514,6 +4576,9 @@
       <c r="AB21" s="300" t="n">
         <v>1</v>
       </c>
+      <c r="AC21" s="371" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="22" ht="15" customHeight="1" s="186">
       <c r="A22" s="258" t="inlineStr">
@@ -4541,6 +4606,9 @@
       <c r="AB22" s="300" t="n">
         <v>15</v>
       </c>
+      <c r="AC22" s="371" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="23" ht="15" customHeight="1" s="186">
       <c r="A23" s="245" t="inlineStr">
@@ -4568,6 +4636,9 @@
       <c r="AB23" s="300" t="n">
         <v>1</v>
       </c>
+      <c r="AC23" s="371" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="186">
       <c r="A24" s="259" t="inlineStr">
@@ -4595,6 +4666,9 @@
       <c r="AB24" s="300" t="n">
         <v>25</v>
       </c>
+      <c r="AC24" s="371" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="186">
       <c r="A25" s="264" t="inlineStr">
@@ -4620,6 +4694,9 @@
       </c>
       <c r="F25" s="308" t="n"/>
       <c r="AB25" s="300" t="n">
+        <v>14</v>
+      </c>
+      <c r="AC25" s="371" t="n">
         <v>14</v>
       </c>
     </row>
@@ -4632,6 +4709,9 @@
       <c r="F26" s="237" t="n"/>
       <c r="AB26" s="300" t="n">
         <v>11</v>
+      </c>
+      <c r="AC26" s="371" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="186">

</xml_diff>

<commit_message>
chore: add Sprint 4.8 plan — invoicing completion, courier ecosystem & AI demand prediction
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/witylogix-sprint-tracker.xlsx
+++ b/witylogix-sprint-tracker.xlsx
@@ -29,7 +29,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 4.3 Plan" sheetId="20" state="visible" r:id="rId20"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 4.4 Plan" sheetId="21" state="visible" r:id="rId21"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 4.5 Plan (Done)" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 4.7 Plan" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 4.7 Plan (Done)" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 4.8 Plan" sheetId="24" state="visible" r:id="rId24"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Data Models Gap'!$A$1:$K$40</definedName>
@@ -584,7 +585,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="41">
+  <fills count="44">
     <fill>
       <patternFill/>
     </fill>
@@ -823,8 +824,23 @@
         <fgColor rgb="001a5276"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8F0FE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -869,6 +885,20 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
@@ -880,7 +910,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="372">
+  <cellXfs count="375">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -1994,6 +2024,15 @@
     </xf>
     <xf numFmtId="3" fontId="73" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="71" fillId="41" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="42" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="43" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -11805,6 +11844,380 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" style="186" min="1" max="1"/>
+    <col width="14" customWidth="1" style="186" min="2" max="2"/>
+    <col width="50" customWidth="1" style="186" min="3" max="3"/>
+    <col width="55" customWidth="1" style="186" min="4" max="4"/>
+    <col width="12" customWidth="1" style="186" min="5" max="5"/>
+    <col width="10" customWidth="1" style="186" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="372" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="B1" s="372" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="C1" s="372" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="D1" s="372" t="inlineStr">
+        <is>
+          <t>Deliverables</t>
+        </is>
+      </c>
+      <c r="E1" s="372" t="inlineStr">
+        <is>
+          <t>Est. Lines</t>
+        </is>
+      </c>
+      <c r="F1" s="372" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="373" t="inlineStr">
+        <is>
+          <t>AR - Arjun</t>
+        </is>
+      </c>
+      <c r="B2" s="373" t="inlineStr">
+        <is>
+          <t>CTO</t>
+        </is>
+      </c>
+      <c r="C2" s="373" t="inlineStr">
+        <is>
+          <t>ADR-027 AI Demand Prediction Architecture + Platform Health Dashboard</t>
+        </is>
+      </c>
+      <c r="D2" s="373" t="inlineStr">
+        <is>
+          <t>ADR-027 doc, demand-prediction types, platform health page, system status API</t>
+        </is>
+      </c>
+      <c r="E2" s="373" t="inlineStr">
+        <is>
+          <t>3000</t>
+        </is>
+      </c>
+      <c r="F2" s="373" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="374" t="inlineStr">
+        <is>
+          <t>DM - Deepak</t>
+        </is>
+      </c>
+      <c r="B3" s="374" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C3" s="374" t="inlineStr">
+        <is>
+          <t>Invoice Management Dashboard + Payment Tracking UI</t>
+        </is>
+      </c>
+      <c r="D3" s="374" t="inlineStr">
+        <is>
+          <t>Invoice list page, invoice detail, payment history, invoice PDF preview component</t>
+        </is>
+      </c>
+      <c r="E3" s="374" t="inlineStr">
+        <is>
+          <t>2500</t>
+        </is>
+      </c>
+      <c r="F3" s="374" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="373" t="inlineStr">
+        <is>
+          <t>NK - Nikhil</t>
+        </is>
+      </c>
+      <c r="B4" s="373" t="inlineStr">
+        <is>
+          <t>Frontend Lead</t>
+        </is>
+      </c>
+      <c r="C4" s="373" t="inlineStr">
+        <is>
+          <t>Courier Live Tracking Map + Dispatch Console</t>
+        </is>
+      </c>
+      <c r="D4" s="373" t="inlineStr">
+        <is>
+          <t>Live courier map, dispatch console, courier assignment panel, delivery timeline</t>
+        </is>
+      </c>
+      <c r="E4" s="373" t="inlineStr">
+        <is>
+          <t>2400</t>
+        </is>
+      </c>
+      <c r="F4" s="373" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="374" t="inlineStr">
+        <is>
+          <t>RG - Rahul</t>
+        </is>
+      </c>
+      <c r="B5" s="374" t="inlineStr">
+        <is>
+          <t>Backend Lead</t>
+        </is>
+      </c>
+      <c r="C5" s="374" t="inlineStr">
+        <is>
+          <t>Courier Webhook Handlers + Partner Rating Engine</t>
+        </is>
+      </c>
+      <c r="D5" s="374" t="inlineStr">
+        <is>
+          <t>Webhook processors for Onfleet/Stuart/Uber, partner rating service, SLA tracker</t>
+        </is>
+      </c>
+      <c r="E5" s="374" t="inlineStr">
+        <is>
+          <t>3500</t>
+        </is>
+      </c>
+      <c r="F5" s="374" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="373" t="inlineStr">
+        <is>
+          <t>SP - Sanjay</t>
+        </is>
+      </c>
+      <c r="B6" s="373" t="inlineStr">
+        <is>
+          <t>Full-stack</t>
+        </is>
+      </c>
+      <c r="C6" s="373" t="inlineStr">
+        <is>
+          <t>Invoice PDF Generation + Payment Gateway Integration</t>
+        </is>
+      </c>
+      <c r="D6" s="373" t="inlineStr">
+        <is>
+          <t>PDF invoice generator (html-pdf), Stripe payment links, payment reconciliation</t>
+        </is>
+      </c>
+      <c r="E6" s="373" t="inlineStr">
+        <is>
+          <t>4000</t>
+        </is>
+      </c>
+      <c r="F6" s="373" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="374" t="inlineStr">
+        <is>
+          <t>VS - Vikram</t>
+        </is>
+      </c>
+      <c r="B7" s="374" t="inlineStr">
+        <is>
+          <t>Component Dev</t>
+        </is>
+      </c>
+      <c r="C7" s="374" t="inlineStr">
+        <is>
+          <t>Invoice &amp; Payment UI Components + Courier Tracking Cards</t>
+        </is>
+      </c>
+      <c r="D7" s="374" t="inlineStr">
+        <is>
+          <t>Invoice table, payment status badge, amount display, courier tracking card, delivery ETA card</t>
+        </is>
+      </c>
+      <c r="E7" s="374" t="inlineStr">
+        <is>
+          <t>2800</t>
+        </is>
+      </c>
+      <c r="F7" s="374" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="373" t="inlineStr">
+        <is>
+          <t>PK - Priya</t>
+        </is>
+      </c>
+      <c r="B8" s="373" t="inlineStr">
+        <is>
+          <t>Sr. Backend</t>
+        </is>
+      </c>
+      <c r="C8" s="373" t="inlineStr">
+        <is>
+          <t>Courier Partner Rating + Multi-Courier Routing Engine</t>
+        </is>
+      </c>
+      <c r="D8" s="373" t="inlineStr">
+        <is>
+          <t>Partner performance scoring, auto-courier selection v2, cost optimization, SLA enforcement</t>
+        </is>
+      </c>
+      <c r="E8" s="373" t="inlineStr">
+        <is>
+          <t>3800</t>
+        </is>
+      </c>
+      <c r="F8" s="373" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="374" t="inlineStr">
+        <is>
+          <t>KS - Kavitha</t>
+        </is>
+      </c>
+      <c r="B9" s="374" t="inlineStr">
+        <is>
+          <t>QA Lead</t>
+        </is>
+      </c>
+      <c r="C9" s="374" t="inlineStr">
+        <is>
+          <t>Invoice + Payment + Courier Dispatch Integration Tests</t>
+        </is>
+      </c>
+      <c r="D9" s="374" t="inlineStr">
+        <is>
+          <t>Invoice generation tests, payment flow tests, courier dispatch tests, webhook handler tests</t>
+        </is>
+      </c>
+      <c r="E9" s="374" t="inlineStr">
+        <is>
+          <t>2000</t>
+        </is>
+      </c>
+      <c r="F9" s="374" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="373" t="inlineStr">
+        <is>
+          <t>AM - Aisha</t>
+        </is>
+      </c>
+      <c r="B10" s="373" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="C10" s="373" t="inlineStr">
+        <is>
+          <t>AI Demand Prediction Data Pipeline + Feature Store</t>
+        </is>
+      </c>
+      <c r="D10" s="373" t="inlineStr">
+        <is>
+          <t>Historical delivery aggregator, time-series feature extractor, demand forecasting pipeline</t>
+        </is>
+      </c>
+      <c r="E10" s="373" t="inlineStr">
+        <is>
+          <t>4500</t>
+        </is>
+      </c>
+      <c r="F10" s="373" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="374" t="inlineStr">
+        <is>
+          <t>ZR - Zara</t>
+        </is>
+      </c>
+      <c r="B11" s="374" t="inlineStr">
+        <is>
+          <t>AI Engineer</t>
+        </is>
+      </c>
+      <c r="C11" s="374" t="inlineStr">
+        <is>
+          <t>AI Demand Prediction Models + Smart Scheduling Engine</t>
+        </is>
+      </c>
+      <c r="D11" s="374" t="inlineStr">
+        <is>
+          <t>Demand forecasting models (ARIMA-like, seasonal decomposition, zone clustering), smart slot optimizer</t>
+        </is>
+      </c>
+      <c r="E11" s="374" t="inlineStr">
+        <is>
+          <t>5500</t>
+        </is>
+      </c>
+      <c r="F11" s="374" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">

</xml_diff>

<commit_message>
feat(sprint-4.8): invoicing completion, courier ecosystem & AI demand prediction
Sprint 4.8 delivers invoice PDF generation with Stripe payment gateway,
courier webhook handlers (Onfleet/Stuart/Uber Direct), partner rating
engine with auto-tiering, smart multi-courier routing with cost optimizer,
SLA enforcement, dispatch console with live tracking, AI demand prediction
pipeline (feature store, data aggregator, time-series, zone profiler),
demand ML models (seasonal decomposition, zone regression, pattern matcher,
anomaly detector) with ensemble predictor, smart scheduling engine, and
platform health dashboard. Finishes G-13, G-14; starts G-15.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/witylogix-sprint-tracker.xlsx
+++ b/witylogix-sprint-tracker.xlsx
@@ -3281,7 +3281,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:AC125"/>
+  <dimension ref="A1:AD125"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.66796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="20" customWidth="1" style="185" min="1" max="1"/>
@@ -3311,6 +3311,13 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>Sprint 4.8</t>
+        </is>
+      </c>
+    </row>
     <row r="3" ht="15" customHeight="1" s="186">
       <c r="A3" s="189" t="inlineStr">
         <is>
@@ -3330,6 +3337,9 @@
           <t>Customer Experience &amp; Checkout</t>
         </is>
       </c>
+      <c r="AD3" t="n">
+        <v>2600</v>
+      </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="186">
       <c r="A4" s="196" t="inlineStr">
@@ -3350,6 +3360,9 @@
           <t>1 (customer-portal)</t>
         </is>
       </c>
+      <c r="AD4" t="n">
+        <v>883700</v>
+      </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="186">
       <c r="A5" s="291" t="inlineStr">
@@ -3493,6 +3506,9 @@
       <c r="AC5" s="371" t="n">
         <v>2467</v>
       </c>
+      <c r="AD5" t="n">
+        <v>94</v>
+      </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="186">
       <c r="A6" s="196" t="inlineStr">
@@ -3584,6 +3600,9 @@
       <c r="AC6" s="371" t="n">
         <v>845846</v>
       </c>
+      <c r="AD6" t="n">
+        <v>146</v>
+      </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="186">
       <c r="A7" s="192" t="inlineStr">
@@ -3675,6 +3694,9 @@
       <c r="AC7" s="371" t="n">
         <v>88</v>
       </c>
+      <c r="AD7" t="n">
+        <v>483</v>
+      </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="186">
       <c r="A8" s="195" t="inlineStr">
@@ -3765,6 +3787,9 @@
       </c>
       <c r="AC8" s="371" t="n">
         <v>138</v>
+      </c>
+      <c r="AD8" t="n">
+        <v>41</v>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="186">

</xml_diff>

<commit_message>
chore: add Sprint 4.9 plan — demand completion, platform adapters & deployment
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/witylogix-sprint-tracker.xlsx
+++ b/witylogix-sprint-tracker.xlsx
@@ -30,7 +30,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 4.4 Plan" sheetId="21" state="visible" r:id="rId21"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 4.5 Plan (Done)" sheetId="22" state="visible" r:id="rId22"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 4.7 Plan (Done)" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 4.8 Plan" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 4.8 Plan (Done)" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 4.9 Plan" sheetId="25" state="visible" r:id="rId25"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Data Models Gap'!$A$1:$K$40</definedName>
@@ -3312,7 +3313,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="AD2" t="inlineStr">
+      <c r="AD2" s="185" t="inlineStr">
         <is>
           <t>Sprint 4.8</t>
         </is>
@@ -3337,7 +3338,7 @@
           <t>Customer Experience &amp; Checkout</t>
         </is>
       </c>
-      <c r="AD3" t="n">
+      <c r="AD3" s="185" t="n">
         <v>2600</v>
       </c>
     </row>
@@ -3360,7 +3361,7 @@
           <t>1 (customer-portal)</t>
         </is>
       </c>
-      <c r="AD4" t="n">
+      <c r="AD4" s="185" t="n">
         <v>883700</v>
       </c>
     </row>
@@ -3506,7 +3507,7 @@
       <c r="AC5" s="371" t="n">
         <v>2467</v>
       </c>
-      <c r="AD5" t="n">
+      <c r="AD5" s="185" t="n">
         <v>94</v>
       </c>
     </row>
@@ -3600,7 +3601,7 @@
       <c r="AC6" s="371" t="n">
         <v>845846</v>
       </c>
-      <c r="AD6" t="n">
+      <c r="AD6" s="185" t="n">
         <v>146</v>
       </c>
     </row>
@@ -3694,7 +3695,7 @@
       <c r="AC7" s="371" t="n">
         <v>88</v>
       </c>
-      <c r="AD7" t="n">
+      <c r="AD7" s="185" t="n">
         <v>483</v>
       </c>
     </row>
@@ -3788,7 +3789,7 @@
       <c r="AC8" s="371" t="n">
         <v>138</v>
       </c>
-      <c r="AD8" t="n">
+      <c r="AD8" s="185" t="n">
         <v>41</v>
       </c>
     </row>
@@ -12230,6 +12231,380 @@
       <c r="E11" s="374" t="inlineStr">
         <is>
           <t>5500</t>
+        </is>
+      </c>
+      <c r="F11" s="374" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" style="186" min="1" max="1"/>
+    <col width="14" customWidth="1" style="186" min="2" max="2"/>
+    <col width="50" customWidth="1" style="186" min="3" max="3"/>
+    <col width="55" customWidth="1" style="186" min="4" max="4"/>
+    <col width="12" customWidth="1" style="186" min="5" max="5"/>
+    <col width="10" customWidth="1" style="186" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="372" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="B1" s="372" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="C1" s="372" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="D1" s="372" t="inlineStr">
+        <is>
+          <t>Deliverables</t>
+        </is>
+      </c>
+      <c r="E1" s="372" t="inlineStr">
+        <is>
+          <t>Est. Lines</t>
+        </is>
+      </c>
+      <c r="F1" s="372" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="373" t="inlineStr">
+        <is>
+          <t>AR - Arjun</t>
+        </is>
+      </c>
+      <c r="B2" s="373" t="inlineStr">
+        <is>
+          <t>CTO</t>
+        </is>
+      </c>
+      <c r="C2" s="373" t="inlineStr">
+        <is>
+          <t>ADR-028 Platform Deployment Architecture + OpenAPI Spec Generator</t>
+        </is>
+      </c>
+      <c r="D2" s="373" t="inlineStr">
+        <is>
+          <t>ADR-028 doc, Docker Compose production config, OpenAPI v3 spec generator, API health endpoints</t>
+        </is>
+      </c>
+      <c r="E2" s="373" t="inlineStr">
+        <is>
+          <t>3500</t>
+        </is>
+      </c>
+      <c r="F2" s="373" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="374" t="inlineStr">
+        <is>
+          <t>DM - Deepak</t>
+        </is>
+      </c>
+      <c r="B3" s="374" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C3" s="374" t="inlineStr">
+        <is>
+          <t>Demand Prediction Dashboard + Capacity Planning UI</t>
+        </is>
+      </c>
+      <c r="D3" s="374" t="inlineStr">
+        <is>
+          <t>Demand forecast page, zone heatmap, capacity planner, schedule optimizer UI, what-if simulator</t>
+        </is>
+      </c>
+      <c r="E3" s="374" t="inlineStr">
+        <is>
+          <t>3000</t>
+        </is>
+      </c>
+      <c r="F3" s="374" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="373" t="inlineStr">
+        <is>
+          <t>NK - Nikhil</t>
+        </is>
+      </c>
+      <c r="B4" s="373" t="inlineStr">
+        <is>
+          <t>Frontend Lead</t>
+        </is>
+      </c>
+      <c r="C4" s="373" t="inlineStr">
+        <is>
+          <t>Platform Admin Console + System Health Dashboard</t>
+        </is>
+      </c>
+      <c r="D4" s="373" t="inlineStr">
+        <is>
+          <t>Admin overview, service status grid, integration health, error log viewer, user activity feed</t>
+        </is>
+      </c>
+      <c r="E4" s="373" t="inlineStr">
+        <is>
+          <t>2800</t>
+        </is>
+      </c>
+      <c r="F4" s="373" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="374" t="inlineStr">
+        <is>
+          <t>RG - Rahul</t>
+        </is>
+      </c>
+      <c r="B5" s="374" t="inlineStr">
+        <is>
+          <t>Backend Lead</t>
+        </is>
+      </c>
+      <c r="C5" s="374" t="inlineStr">
+        <is>
+          <t>Magento + BigCommerce E-Commerce Adapters</t>
+        </is>
+      </c>
+      <c r="D5" s="374" t="inlineStr">
+        <is>
+          <t>Magento REST adapter (orders, products, inventory), BigCommerce adapter, webhook handlers</t>
+        </is>
+      </c>
+      <c r="E5" s="374" t="inlineStr">
+        <is>
+          <t>3800</t>
+        </is>
+      </c>
+      <c r="F5" s="374" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="373" t="inlineStr">
+        <is>
+          <t>SP - Sanjay</t>
+        </is>
+      </c>
+      <c r="B6" s="373" t="inlineStr">
+        <is>
+          <t>Full-stack</t>
+        </is>
+      </c>
+      <c r="C6" s="373" t="inlineStr">
+        <is>
+          <t>PayPal + Square Payment Gateway Adapters</t>
+        </is>
+      </c>
+      <c r="D6" s="373" t="inlineStr">
+        <is>
+          <t>PayPal Orders API adapter, Square Payments adapter, payment method selector, multi-gateway router</t>
+        </is>
+      </c>
+      <c r="E6" s="373" t="inlineStr">
+        <is>
+          <t>3500</t>
+        </is>
+      </c>
+      <c r="F6" s="373" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="374" t="inlineStr">
+        <is>
+          <t>VS - Vikram</t>
+        </is>
+      </c>
+      <c r="B7" s="374" t="inlineStr">
+        <is>
+          <t>Component Dev</t>
+        </is>
+      </c>
+      <c r="C7" s="374" t="inlineStr">
+        <is>
+          <t>Demand Visualization + Admin UI Components</t>
+        </is>
+      </c>
+      <c r="D7" s="374" t="inlineStr">
+        <is>
+          <t>Zone heatmap component, demand chart, capacity bar, schedule grid, admin stat cards, service health badge</t>
+        </is>
+      </c>
+      <c r="E7" s="374" t="inlineStr">
+        <is>
+          <t>2500</t>
+        </is>
+      </c>
+      <c r="F7" s="374" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="373" t="inlineStr">
+        <is>
+          <t>PK - Priya</t>
+        </is>
+      </c>
+      <c r="B8" s="373" t="inlineStr">
+        <is>
+          <t>Sr. Backend</t>
+        </is>
+      </c>
+      <c r="C8" s="373" t="inlineStr">
+        <is>
+          <t>Salesforce + HubSpot CRM Adapters</t>
+        </is>
+      </c>
+      <c r="D8" s="373" t="inlineStr">
+        <is>
+          <t>Salesforce REST adapter (accounts, contacts, opportunities), HubSpot adapter, CRM sync engine</t>
+        </is>
+      </c>
+      <c r="E8" s="373" t="inlineStr">
+        <is>
+          <t>4000</t>
+        </is>
+      </c>
+      <c r="F8" s="373" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="374" t="inlineStr">
+        <is>
+          <t>KS - Kavitha</t>
+        </is>
+      </c>
+      <c r="B9" s="374" t="inlineStr">
+        <is>
+          <t>QA Lead</t>
+        </is>
+      </c>
+      <c r="C9" s="374" t="inlineStr">
+        <is>
+          <t>E2E Integration Tests + Load Testing Suite</t>
+        </is>
+      </c>
+      <c r="D9" s="374" t="inlineStr">
+        <is>
+          <t>E2E order lifecycle test, checkout-to-delivery flow, payment flow tests, k6 load test scripts</t>
+        </is>
+      </c>
+      <c r="E9" s="374" t="inlineStr">
+        <is>
+          <t>3000</t>
+        </is>
+      </c>
+      <c r="F9" s="374" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="373" t="inlineStr">
+        <is>
+          <t>AM - Aisha</t>
+        </is>
+      </c>
+      <c r="B10" s="373" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="C10" s="373" t="inlineStr">
+        <is>
+          <t>ShipStation + EasyPost Multi-Carrier Shipping Adapters</t>
+        </is>
+      </c>
+      <c r="D10" s="373" t="inlineStr">
+        <is>
+          <t>ShipStation adapter (orders, labels, rates), EasyPost adapter, carrier rate comparison engine</t>
+        </is>
+      </c>
+      <c r="E10" s="373" t="inlineStr">
+        <is>
+          <t>3500</t>
+        </is>
+      </c>
+      <c r="F10" s="373" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="374" t="inlineStr">
+        <is>
+          <t>ZR - Zara</t>
+        </is>
+      </c>
+      <c r="B11" s="374" t="inlineStr">
+        <is>
+          <t>AI Engineer</t>
+        </is>
+      </c>
+      <c r="C11" s="374" t="inlineStr">
+        <is>
+          <t>Demand Prediction Completion + Auto-Capacity Optimizer</t>
+        </is>
+      </c>
+      <c r="D11" s="374" t="inlineStr">
+        <is>
+          <t>Real-time demand dashboard data, auto-rebalancing engine, capacity alerts, demand API completion, model retraining pipeline</t>
+        </is>
+      </c>
+      <c r="E11" s="374" t="inlineStr">
+        <is>
+          <t>4500</t>
         </is>
       </c>
       <c r="F11" s="374" t="inlineStr">

</xml_diff>

<commit_message>
feat(sprint-4.9): demand completion, platform adapters & deployment
Sprint 4.9 completes AI demand prediction (real-time dashboard, auto-
rebalancer, capacity alerts, model retraining with A/B testing), adds
e-commerce adapters (Magento 2 REST + BigCommerce V3), payment gateways
(PayPal Orders V2 + Square) with multi-gateway router, CRM adapters
(Salesforce + HubSpot) with bidirectional sync, shipping adapters
(ShipStation + EasyPost) with carrier rate comparison engine, demand
visualization components (zone heatmap, forecast chart, capacity bar,
schedule grid), admin console (system health, integrations, error logs,
activity feed, API docs), Docker production config, OpenAPI v3.1 spec
generator, Prometheus health checks, E2E test suite (5 specs), and k6
load tests (2 scenarios). ADR-028 platform deployment architecture.

108 files changed, ~47,600 insertions. All 15 competitive gaps resolved.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/witylogix-sprint-tracker.xlsx
+++ b/witylogix-sprint-tracker.xlsx
@@ -31,7 +31,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 4.5 Plan (Done)" sheetId="22" state="visible" r:id="rId22"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 4.7 Plan (Done)" sheetId="23" state="visible" r:id="rId23"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 4.8 Plan (Done)" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 4.9 Plan" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 4.9 Done" sheetId="25" state="visible" r:id="rId25"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Data Models Gap'!$A$1:$K$40</definedName>
@@ -49,7 +49,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="74">
+  <fonts count="75">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -585,8 +585,11 @@
     <font>
       <sz val="11"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="44">
+  <fills count="45">
     <fill>
       <patternFill/>
     </fill>
@@ -840,6 +843,12 @@
         <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001a237e"/>
+        <bgColor rgb="001a237e"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="6">
     <border>
@@ -911,7 +920,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="375">
+  <cellXfs count="379">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -2034,6 +2043,16 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="43" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="71" fillId="44" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="74" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="49" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -3282,7 +3301,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:AD125"/>
+  <dimension ref="A1:AE125"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.66796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="20" customWidth="1" style="185" min="1" max="1"/>
@@ -3296,6 +3315,11 @@
           <t>Gap Statistics Summary</t>
         </is>
       </c>
+      <c r="Y1" s="375" t="inlineStr">
+        <is>
+          <t>Sprint 4.9</t>
+        </is>
+      </c>
       <c r="AA1" s="288" t="inlineStr">
         <is>
           <t>Sprint 4.5</t>
@@ -3313,6 +3337,14 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" s="376" t="inlineStr">
+        <is>
+          <t>Source Files</t>
+        </is>
+      </c>
+      <c r="Y2" s="377" t="n">
+        <v>1443</v>
+      </c>
       <c r="AD2" s="185" t="inlineStr">
         <is>
           <t>Sprint 4.8</t>
@@ -3333,6 +3365,9 @@
       <c r="C3" s="189" t="n"/>
       <c r="D3" s="189" t="n"/>
       <c r="E3" s="189" t="n"/>
+      <c r="Y3" s="377" t="n">
+        <v>564356</v>
+      </c>
       <c r="AA3" s="290" t="inlineStr">
         <is>
           <t>Customer Experience &amp; Checkout</t>
@@ -3356,6 +3391,9 @@
       <c r="C4" s="196" t="n"/>
       <c r="D4" s="196" t="n"/>
       <c r="E4" s="196" t="n"/>
+      <c r="Y4" s="377" t="n">
+        <v>105</v>
+      </c>
       <c r="AA4" s="290" t="inlineStr">
         <is>
           <t>1 (customer-portal)</t>
@@ -3486,10 +3524,8 @@
           <t>Sprint 4.2</t>
         </is>
       </c>
-      <c r="Y5" s="297" t="inlineStr">
-        <is>
-          <t>Sprint 4.3</t>
-        </is>
+      <c r="Y5" s="378" t="n">
+        <v>152</v>
       </c>
       <c r="Z5" s="297" t="inlineStr">
         <is>
@@ -3586,8 +3622,8 @@
       <c r="X6" s="301" t="n">
         <v>2320</v>
       </c>
-      <c r="Y6" s="303" t="n">
-        <v>2343</v>
+      <c r="Y6" s="377" t="n">
+        <v>318</v>
       </c>
       <c r="Z6" s="303" t="n">
         <v>2410</v>
@@ -3680,8 +3716,8 @@
       <c r="X7" s="301" t="n">
         <v>383000</v>
       </c>
-      <c r="Y7" s="303" t="n">
-        <v>392000</v>
+      <c r="Y7" s="377" t="n">
+        <v>42</v>
       </c>
       <c r="Z7" s="303" t="n">
         <v>423000</v>
@@ -3774,8 +3810,8 @@
       <c r="X8" s="301" t="n">
         <v>70</v>
       </c>
-      <c r="Y8" s="303" t="n">
-        <v>70</v>
+      <c r="Y8" s="377" t="n">
+        <v>80</v>
       </c>
       <c r="Z8" s="303" t="n">
         <v>74</v>
@@ -3868,8 +3904,8 @@
       <c r="X9" s="301" t="n">
         <v>74</v>
       </c>
-      <c r="Y9" s="303" t="n">
-        <v>74</v>
+      <c r="Y9" s="377" t="n">
+        <v>80</v>
       </c>
       <c r="Z9" s="303" t="n">
         <v>75</v>
@@ -3959,8 +3995,8 @@
       <c r="X10" s="301" t="n">
         <v>31</v>
       </c>
-      <c r="Y10" s="303" t="n">
-        <v>31</v>
+      <c r="Y10" s="377" t="n">
+        <v>100</v>
       </c>
       <c r="Z10" s="303" t="n">
         <v>35</v>
@@ -4050,8 +4086,8 @@
       <c r="X11" s="301" t="n">
         <v>74</v>
       </c>
-      <c r="Y11" s="303" t="n">
-        <v>74</v>
+      <c r="Y11" s="377" t="n">
+        <v>51500</v>
       </c>
       <c r="Z11" s="303" t="n">
         <v>80</v>
@@ -4135,8 +4171,8 @@
       <c r="X12" s="301" t="n">
         <v>190</v>
       </c>
-      <c r="Y12" s="303" t="n">
-        <v>191</v>
+      <c r="Y12" s="377" t="n">
+        <v>124</v>
       </c>
       <c r="Z12" s="303" t="n">
         <v>205</v>
@@ -4195,8 +4231,8 @@
       <c r="X13" s="301" t="n">
         <v>12</v>
       </c>
-      <c r="Y13" s="303" t="n">
-        <v>12</v>
+      <c r="Y13" s="377" t="n">
+        <v>21</v>
       </c>
       <c r="Z13" s="303" t="n">
         <v>12</v>
@@ -4255,8 +4291,8 @@
       <c r="X14" s="301" t="n">
         <v>190</v>
       </c>
-      <c r="Y14" s="303" t="n">
-        <v>191</v>
+      <c r="Y14" s="377" t="n">
+        <v>5</v>
       </c>
       <c r="Z14" s="303" t="n">
         <v>205</v>
@@ -4315,8 +4351,8 @@
       <c r="X15" s="301" t="n">
         <v>4817</v>
       </c>
-      <c r="Y15" s="303" t="n">
-        <v>4817</v>
+      <c r="Y15" s="377" t="n">
+        <v>2</v>
       </c>
       <c r="Z15" s="303" t="n">
         <v>4900</v>
@@ -4385,8 +4421,8 @@
       <c r="V16" s="303" t="n">
         <v>12</v>
       </c>
-      <c r="Y16" s="185" t="n">
-        <v>12</v>
+      <c r="Y16" s="377" t="n">
+        <v>28</v>
       </c>
       <c r="Z16" s="185" t="n">
         <v>12</v>

</xml_diff>

<commit_message>
chore: add Sprint 5.0 plan — mega integration sprint I (routing, telematics, messaging, email, ERP)
Updates 8 adapter statuses to production (Sprint 4.9 builds). Plans 25 new
adapters across routing (Valhalla, VROOM, Routific, OptimoRoute, HERE, Route4Me),
telematics (Flespi, Verizon Connect, Trimble, Fleetio), messaging (Vonage,
TextMagic, OneSignal, Sendbird), email (Mailgun, Amazon SES, Gmail, Outlook),
ERP (SAP, Oracle NetSuite, MS Dynamics 365, Sage), plus integration management
dashboards, config pages, UI components, and test suites.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/witylogix-sprint-tracker.xlsx
+++ b/witylogix-sprint-tracker.xlsx
@@ -32,6 +32,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 4.7 Plan (Done)" sheetId="23" state="visible" r:id="rId23"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 4.8 Plan (Done)" sheetId="24" state="visible" r:id="rId24"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 4.9 Done" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 5.0 Plan" sheetId="26" state="visible" r:id="rId26"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Data Models Gap'!$A$1:$K$40</definedName>
@@ -49,7 +50,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="75">
+  <fonts count="78">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -588,8 +589,22 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="45">
+  <fills count="48">
     <fill>
       <patternFill/>
     </fill>
@@ -849,6 +864,24 @@
         <bgColor rgb="001a237e"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000d47a1"/>
+        <bgColor rgb="000d47a1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8EAF6"/>
+        <bgColor rgb="00E8EAF6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+        <bgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="6">
     <border>
@@ -920,7 +953,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="379">
+  <cellXfs count="387">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -2054,6 +2087,26 @@
     <xf numFmtId="3" fontId="49" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="75" fillId="45" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="76" fillId="44" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="46" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="46" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="47" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="47" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="77" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3301,7 +3354,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:AE125"/>
+  <dimension ref="A1:AD125"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.66796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="20" customWidth="1" style="185" min="1" max="1"/>
@@ -12650,6 +12703,391 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" style="186" min="1" max="1"/>
+    <col width="14" customWidth="1" style="186" min="2" max="2"/>
+    <col width="55" customWidth="1" style="186" min="3" max="3"/>
+    <col width="45" customWidth="1" style="186" min="4" max="4"/>
+    <col width="12" customWidth="1" style="186" min="5" max="5"/>
+    <col width="10" customWidth="1" style="186" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="379" t="inlineStr">
+        <is>
+          <t>Sprint 5.0 — Mega Integration Sprint I: Routing, Telematics, Messaging, Email, ERP &amp; E-Commerce</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="380" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="B2" s="380" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="C2" s="380" t="inlineStr">
+        <is>
+          <t>Deliverables</t>
+        </is>
+      </c>
+      <c r="D2" s="380" t="inlineStr">
+        <is>
+          <t>Adapters</t>
+        </is>
+      </c>
+      <c r="E2" s="380" t="inlineStr">
+        <is>
+          <t>Est. Lines</t>
+        </is>
+      </c>
+      <c r="F2" s="380" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="381" t="inlineStr">
+        <is>
+          <t>AR - Arjun</t>
+        </is>
+      </c>
+      <c r="B3" s="381" t="inlineStr">
+        <is>
+          <t>CTO</t>
+        </is>
+      </c>
+      <c r="C3" s="381" t="inlineStr">
+        <is>
+          <t>Valhalla + VROOM Open-Source Routing Adapters + Routific + OptimoRoute Adapters</t>
+        </is>
+      </c>
+      <c r="D3" s="381" t="inlineStr">
+        <is>
+          <t>Valhalla, VROOM, Routific, OptimoRoute</t>
+        </is>
+      </c>
+      <c r="E3" s="382" t="n">
+        <v>4500</v>
+      </c>
+      <c r="F3" s="381" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="383" t="inlineStr">
+        <is>
+          <t>DM - Deepak</t>
+        </is>
+      </c>
+      <c r="B4" s="383" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C4" s="383" t="inlineStr">
+        <is>
+          <t>Integration Management Dashboard: routing config, telematics config, messaging config, ERP config pages</t>
+        </is>
+      </c>
+      <c r="D4" s="383" t="inlineStr">
+        <is>
+          <t>Routing Settings, Telematics Settings, Messaging Settings, ERP Settings (4 pages)</t>
+        </is>
+      </c>
+      <c r="E4" s="384" t="n">
+        <v>3200</v>
+      </c>
+      <c r="F4" s="383" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="381" t="inlineStr">
+        <is>
+          <t>NK - Nikhil</t>
+        </is>
+      </c>
+      <c r="B5" s="381" t="inlineStr">
+        <is>
+          <t>Frontend Lead</t>
+        </is>
+      </c>
+      <c r="C5" s="381" t="inlineStr">
+        <is>
+          <t>E-Commerce &amp; Email Integration UI: Amazon/eBay/Etsy config, email provider config, template builder pages</t>
+        </is>
+      </c>
+      <c r="D5" s="381" t="inlineStr">
+        <is>
+          <t>E-Commerce Config, Email Config, Template Builder (3 pages)</t>
+        </is>
+      </c>
+      <c r="E5" s="382" t="n">
+        <v>2800</v>
+      </c>
+      <c r="F5" s="381" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="383" t="inlineStr">
+        <is>
+          <t>RG - Rahul</t>
+        </is>
+      </c>
+      <c r="B6" s="383" t="inlineStr">
+        <is>
+          <t>Backend Lead</t>
+        </is>
+      </c>
+      <c r="C6" s="383" t="inlineStr">
+        <is>
+          <t>HERE Routing + Route4Me + HERE Maps Adapters + Routing Adapter Base Enhancement</t>
+        </is>
+      </c>
+      <c r="D6" s="383" t="inlineStr">
+        <is>
+          <t>HERE Routing, Route4Me, HERE Maps</t>
+        </is>
+      </c>
+      <c r="E6" s="384" t="n">
+        <v>4200</v>
+      </c>
+      <c r="F6" s="383" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="381" t="inlineStr">
+        <is>
+          <t>SP - Sanjay</t>
+        </is>
+      </c>
+      <c r="B7" s="381" t="inlineStr">
+        <is>
+          <t>Full-stack</t>
+        </is>
+      </c>
+      <c r="C7" s="381" t="inlineStr">
+        <is>
+          <t>Vonage + TextMagic + OneSignal + Sendbird Messaging Adapters</t>
+        </is>
+      </c>
+      <c r="D7" s="381" t="inlineStr">
+        <is>
+          <t>Vonage, TextMagic, OneSignal, Sendbird</t>
+        </is>
+      </c>
+      <c r="E7" s="382" t="n">
+        <v>4600</v>
+      </c>
+      <c r="F7" s="381" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="383" t="inlineStr">
+        <is>
+          <t>VS - Vikram</t>
+        </is>
+      </c>
+      <c r="B8" s="383" t="inlineStr">
+        <is>
+          <t>Component Dev</t>
+        </is>
+      </c>
+      <c r="C8" s="383" t="inlineStr">
+        <is>
+          <t>Integration config UI components: provider cards, credential forms, webhook config, health monitors, rate limit displays</t>
+        </is>
+      </c>
+      <c r="D8" s="383" t="inlineStr">
+        <is>
+          <t>Provider Card, Credential Form, Webhook Config, Health Monitor, Rate Display (10 components)</t>
+        </is>
+      </c>
+      <c r="E8" s="384" t="n">
+        <v>3000</v>
+      </c>
+      <c r="F8" s="383" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="381" t="inlineStr">
+        <is>
+          <t>PK - Priya</t>
+        </is>
+      </c>
+      <c r="B9" s="381" t="inlineStr">
+        <is>
+          <t>Sr. Backend</t>
+        </is>
+      </c>
+      <c r="C9" s="381" t="inlineStr">
+        <is>
+          <t>SAP + Oracle NetSuite + Microsoft Dynamics 365 + Sage ERP/Accounting Adapters</t>
+        </is>
+      </c>
+      <c r="D9" s="381" t="inlineStr">
+        <is>
+          <t>SAP, Oracle NetSuite, MS Dynamics 365, Sage</t>
+        </is>
+      </c>
+      <c r="E9" s="382" t="n">
+        <v>5200</v>
+      </c>
+      <c r="F9" s="381" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="383" t="inlineStr">
+        <is>
+          <t>KS - Kavitha</t>
+        </is>
+      </c>
+      <c r="B10" s="383" t="inlineStr">
+        <is>
+          <t>QA Lead</t>
+        </is>
+      </c>
+      <c r="C10" s="383" t="inlineStr">
+        <is>
+          <t>Integration adapter test suite: routing, messaging, email, ERP adapters + webhook E2E tests</t>
+        </is>
+      </c>
+      <c r="D10" s="383" t="inlineStr">
+        <is>
+          <t>Routing Tests, Messaging Tests, Email Tests, ERP Tests, Webhook E2E (5 suites)</t>
+        </is>
+      </c>
+      <c r="E10" s="384" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F10" s="383" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="381" t="inlineStr">
+        <is>
+          <t>AM - Aisha</t>
+        </is>
+      </c>
+      <c r="B11" s="381" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="C11" s="381" t="inlineStr">
+        <is>
+          <t>Mailgun + Amazon SES + Gmail + Outlook Email Adapters + Email Routing Engine</t>
+        </is>
+      </c>
+      <c r="D11" s="381" t="inlineStr">
+        <is>
+          <t>Mailgun, Amazon SES, Gmail, Outlook</t>
+        </is>
+      </c>
+      <c r="E11" s="382" t="n">
+        <v>4800</v>
+      </c>
+      <c r="F11" s="381" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="383" t="inlineStr">
+        <is>
+          <t>ZR - Zara</t>
+        </is>
+      </c>
+      <c r="B12" s="383" t="inlineStr">
+        <is>
+          <t>AI Engineer</t>
+        </is>
+      </c>
+      <c r="C12" s="383" t="inlineStr">
+        <is>
+          <t>Flespi + Verizon Connect + Trimble + Fleetio Telematics Adapters</t>
+        </is>
+      </c>
+      <c r="D12" s="383" t="inlineStr">
+        <is>
+          <t>Flespi, Verizon Connect, Trimble, Fleetio</t>
+        </is>
+      </c>
+      <c r="E12" s="384" t="n">
+        <v>4500</v>
+      </c>
+      <c r="F12" s="383" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="385" t="inlineStr">
+        <is>
+          <t>TOTALS</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>25 new adapters + 4 dashboard pages + 3 config pages + 10 UI components + 5 test suites</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>25 adapters (routing: 6, telematics: 4, messaging: 4, email: 4, ERP: 4, maps: 1, UI: 17)</t>
+        </is>
+      </c>
+      <c r="E13" s="386" t="n">
+        <v>41800</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
chore(sprint-5.1): plan mega integration sprint II
Sprint 5.1 targets 25 adapters: collaboration (Slack, Teams, Pusher,
Track-POD, DispatchTrack, Podium, WorkWave), e-signatures (DocuSign,
Adobe Sign, PandaDoc, HelloSign), CRM (Zoho, Dynamics CRM, Pipedrive),
payments (Braintree, Authorize.Net, Adyen), POS (Toast, Square for
Restaurants), ELD (Motive, Omnitracs, Azuga), last-mile (DoorDash Drive,
Uber Eats, Grubhub), shipping (Shippo). Plus 8 dashboard pages, 9 UI
components, and comprehensive test suites.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/witylogix-sprint-tracker.xlsx
+++ b/witylogix-sprint-tracker.xlsx
@@ -33,6 +33,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 4.8 Plan (Done)" sheetId="24" state="visible" r:id="rId24"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 4.9 Done" sheetId="25" state="visible" r:id="rId25"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 5.0 Done" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 5.1 Plan" sheetId="27" state="visible" r:id="rId27"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Data Models Gap'!$A$1:$K$40</definedName>
@@ -3373,7 +3374,7 @@
           <t>Sprint 4.9</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="185" t="inlineStr">
         <is>
           <t>Sprint 5.0</t>
         </is>
@@ -3403,7 +3404,7 @@
       <c r="Y2" s="377" t="n">
         <v>1443</v>
       </c>
-      <c r="Z2" t="n">
+      <c r="Z2" s="185" t="n">
         <v>1556</v>
       </c>
       <c r="AD2" s="185" t="inlineStr">
@@ -3429,7 +3430,7 @@
       <c r="Y3" s="377" t="n">
         <v>564356</v>
       </c>
-      <c r="Z3" t="n">
+      <c r="Z3" s="185" t="n">
         <v>602196</v>
       </c>
       <c r="AA3" s="290" t="inlineStr">
@@ -3458,7 +3459,7 @@
       <c r="Y4" s="377" t="n">
         <v>105</v>
       </c>
-      <c r="Z4" t="n">
+      <c r="Z4" s="185" t="n">
         <v>112</v>
       </c>
       <c r="AA4" s="290" t="inlineStr">
@@ -13100,6 +13101,372 @@
     <mergeCell ref="A13:B13"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Domain</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Deliverables</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Est. Lines</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Files</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>AR</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>CTO</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Collaboration</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Slack, Microsoft Teams, Pusher adapters + collaboration hub engine (presence, channels, notifications)</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>~5,800</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Collaboration + E-Signatures</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Dashboard pages: collaboration config, e-signatures config, ELD config, payments config</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>~2,500</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>NK</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Frontend Lead</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>CRM + POS + Last-Mile</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Dashboard pages: CRM config, POS/restaurant config, last-mile config, shipping config</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>~2,500</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>RG</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Backend Lead</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>E-Signatures</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>DocuSign, Adobe Sign, PandaDoc, HelloSign adapters + envelope engine</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>~5,500</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Full-stack</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Zoho CRM, MS Dynamics CRM, Pipedrive adapters + CRM sync engine</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>~5,000</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>VS</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Component Dev</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>UI Components</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Integration components: OAuth flow, log viewer, batch operations, template manager, alert rules, data mapper, import/export wizard, status timeline, provider switcher</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>~3,200</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Sr. Backend</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Payments + POS</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Braintree, Authorize.Net, Adyen payment adapters + Toast POS, Square for Restaurants adapters</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>~5,800</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>KS</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>QA Lead</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Test Suites</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Integration tests: collaboration, e-signatures, CRM, payments, POS, ELD, last-mile, shipping + E2E flows</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>~6,000</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>ELD + Shipping</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Motive ELD, Omnitracs ELD, Azuga ELD adapters + ELD compliance engine + Shippo shipping adapter</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>~5,200</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>ZR</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>AI Engineer</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Last-Mile + Collaboration</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>DoorDash Drive, Uber Eats, Grubhub last-mile adapters + delivery aggregator + Track-POD, DispatchTrack, Podium, WorkWave collaboration adapters</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>~6,200</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
chore(sprint-5.2): plan final integration sprint
Sprint 5.2 completes ALL remaining 44 planned integrations:
analytics (Tableau, Power BI, Looker, Qlik, Google Analytics),
supply-chain (Manhattan, Blue Yonder, Körber, Deposco, Extensiv, Fishbowl),
healthcare (Cerner, Allscripts, Epic, HL7 FHIR), freight (DAT, Truckstop,
123Loadboard, Direct Freight), fuel-fleet (WEX, Comdata, Fuelman, EFS),
field-service (ServiceTitan, Jobber, Housecall Pro, FieldEdge),
e-commerce (Amazon, eBay, Etsy, Square Online), telematics (Powerfleet,
Azuga, Omnitracs, Platform Science, ClearPathGPS, One Step GPS, Titan GPS),
erp-accounting (Infor, Epicor, Sage Intacct, FreshBooks, Wave),
e-signatures (Solid Protocol). Plus 8 dashboard pages, 10 UI components,
and comprehensive test suites.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/witylogix-sprint-tracker.xlsx
+++ b/witylogix-sprint-tracker.xlsx
@@ -34,6 +34,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 4.9 Done" sheetId="25" state="visible" r:id="rId25"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 5.0 Done" sheetId="26" state="visible" r:id="rId26"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 5.1 Done" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 5.2 Plan" sheetId="28" state="visible" r:id="rId28"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Data Models Gap'!$A$1:$K$40</definedName>
@@ -3407,7 +3408,7 @@
       <c r="Z2" s="185" t="n">
         <v>1556</v>
       </c>
-      <c r="AA2" t="n">
+      <c r="AA2" s="185" t="n">
         <v>1622</v>
       </c>
       <c r="AD2" s="185" t="inlineStr">
@@ -13460,6 +13461,372 @@
       <c r="F11" s="185" t="inlineStr">
         <is>
           <t>11</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Domain</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Deliverables</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Est. Lines</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Files</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>AR</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>CTO</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Analytics</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Tableau (REST+Hyper), Power BI (REST+DAX), Looker (SDK), Qlik (Sense), Google Analytics (GA4 Data API) adapters + analytics aggregator engine</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>~6,500</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Dashboard Pages I</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Dashboard pages: analytics config, supply-chain config, freight config, fuel-fleet config</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>~2,800</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>NK</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Frontend Lead</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Dashboard Pages II</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Dashboard pages: healthcare config, field-service config, telematics-extended config, e-commerce-extended config</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>~2,800</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>RG</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Backend Lead</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Supply Chain</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Manhattan Associates, Blue Yonder, Körber, Deposco, Extensiv, Fishbowl adapters + supply chain orchestrator</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>~6,800</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Full-stack</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Healthcare</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Cerner (Millennium), Allscripts (Unity), Epic (FHIR R4), HL7 FHIR (generic) adapters + healthcare data normalizer + Solid Protocol e-signature</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>~6,200</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>VS</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Component Dev</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>UI Components</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Integration components: analytics embed viewer, supply chain flow diagram, freight quote card, fuel transaction log, healthcare compliance badge, field service scheduler, FHIR resource browser, carrier board, fleet fuel chart, integration marketplace</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>~3,500</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Sr. Backend</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Freight + Fuel-Fleet</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>DAT, Truckstop, 123Loadboard, Direct Freight freight adapters + freight board aggregator + WEX, Comdata, Fuelman, EFS fuel-fleet adapters + fuel card manager</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>~7,200</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>KS</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>QA Lead</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Test Suites</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Integration tests: analytics, supply-chain, healthcare, freight, fuel-fleet, field-service, telematics-ext, e-commerce-ext + final E2E + registry validation</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>~7,000</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>E-Commerce + Telematics</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Amazon Seller Central (SP-API), eBay (REST), Etsy (v3), Square Online adapters + Powerfleet, Azuga, Omnitracs, Platform Science telematics adapters</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>~6,800</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>ZR</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>AI Engineer</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Field-Service + Telematics</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>ServiceTitan, Jobber, Housecall Pro, FieldEdge field-service adapters + field service dispatcher + ClearPathGPS, One Step GPS, Titan GPS telematics + ERP mini-adapters (Infor, Epicor, Sage Intacct, FreshBooks, Wave)</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>~7,500</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>14</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: team standup — production readiness review & Sprint 6.0 plan
Full team standup covering:
- Platform status: 1,709 files, 712K LOC, 128 pages, 124/124 integrations
- 10 team member reports with blockers
- Production readiness gap analysis (P0/P1/P2)
- Sprint 6.0 plan: Onboarding & Auth Hardening (10 agents)
- Sprint 6.1 plan: Database & API Production Hardening
- Sprint 6.2 plan: CI/CD, Deployment & Documentation

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/witylogix-sprint-tracker.xlsx
+++ b/witylogix-sprint-tracker.xlsx
@@ -35,6 +35,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 5.0 Done" sheetId="26" state="visible" r:id="rId26"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 5.1 Done" sheetId="27" state="visible" r:id="rId27"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 5.2 Done" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 6.0 Plan" sheetId="29" state="visible" r:id="rId29"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Data Models Gap'!$A$1:$K$40</definedName>
@@ -52,7 +53,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="78">
+  <fonts count="87">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -605,8 +606,52 @@
       <b val="1"/>
       <sz val="11"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="004a9eff"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="0000ff88"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="004a9eff"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00ff6b6b"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00ff6b6b"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00ffaa00"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="004a9eff"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="48">
+  <fills count="49">
     <fill>
       <patternFill/>
     </fill>
@@ -884,6 +929,11 @@
         <bgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001e3a5f"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="6">
     <border>
@@ -955,7 +1005,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="387">
+  <cellXfs count="409">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -2109,6 +2159,54 @@
     </xf>
     <xf numFmtId="0" fontId="77" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="78" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="79" fillId="29" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="80" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="72" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="80" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="72" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="79" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="81" fillId="27" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="80" fillId="27" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="82" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="81" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="81" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="80" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="82" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="72" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="81" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="82" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="83" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="84" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="79" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="86" fillId="48" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3370,7 +3468,7 @@
           <t>Gap Statistics Summary</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="185" t="inlineStr">
         <is>
           <t>Sprint 5.2</t>
         </is>
@@ -3407,7 +3505,7 @@
           <t>Source Files</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" s="185" t="n">
         <v>1709</v>
       </c>
       <c r="Y2" s="377" t="n">
@@ -6346,10 +6444,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G53"/>
+  <dimension ref="A1:G126"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="28" customWidth="1" style="185" min="1" max="2"/>
+    <col width="25" customWidth="1" style="185" min="1" max="2"/>
+    <col width="100" customWidth="1" style="186" min="2" max="2"/>
     <col width="18" customWidth="1" style="185" min="3" max="3"/>
     <col width="55" customWidth="1" style="185" min="4" max="4"/>
     <col width="50" customWidth="1" style="185" min="5" max="5"/>
@@ -6529,6 +6628,13 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="387" t="inlineStr">
+        <is>
+          <t>TEAM STANDUP — March 12, 2026 — Production Readiness Review</t>
+        </is>
+      </c>
+    </row>
     <row r="13" ht="15" customHeight="1" s="186">
       <c r="A13" s="332" t="inlineStr">
         <is>
@@ -6537,9 +6643,9 @@
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="186">
-      <c r="A14" s="337" t="inlineStr">
-        <is>
-          <t>Agreement</t>
+      <c r="A14" s="388" t="inlineStr">
+        <is>
+          <t>PLATFORM STATUS</t>
         </is>
       </c>
       <c r="B14" s="337" t="inlineStr">
@@ -6559,87 +6665,87 @@
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="186">
-      <c r="A15" s="334" t="inlineStr">
-        <is>
-          <t>BYOK Pattern</t>
-        </is>
-      </c>
-      <c r="B15" s="334" t="inlineStr">
+      <c r="A15" s="389" t="inlineStr">
+        <is>
+          <t>Source Files</t>
+        </is>
+      </c>
+      <c r="B15" s="390" t="inlineStr">
+        <is>
+          <t>1,709 (.ts/.tsx)</t>
+        </is>
+      </c>
+      <c r="C15" s="334" t="inlineStr">
         <is>
           <t>Keep it</t>
         </is>
       </c>
-      <c r="C15" s="334" t="inlineStr">
+      <c r="D15" s="338" t="inlineStr">
+        <is>
+          <t>Unanimous — BYOK stays</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="15" customHeight="1" s="186">
+      <c r="A16" s="389" t="inlineStr">
+        <is>
+          <t>Lines of Code</t>
+        </is>
+      </c>
+      <c r="B16" s="390" t="inlineStr">
+        <is>
+          <t>712,763</t>
+        </is>
+      </c>
+      <c r="C16" s="334" t="inlineStr">
         <is>
           <t>Keep it</t>
         </is>
       </c>
-      <c r="D15" s="338" t="inlineStr">
-        <is>
-          <t>Unanimous — BYOK stays</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="15" customHeight="1" s="186">
-      <c r="A16" s="334" t="inlineStr">
-        <is>
-          <t>Prisma ORM</t>
-        </is>
-      </c>
-      <c r="B16" s="334" t="inlineStr">
-        <is>
-          <t>Keep it (no DML/MikroORM)</t>
-        </is>
-      </c>
-      <c r="C16" s="334" t="inlineStr">
+      <c r="D16" s="338" t="inlineStr">
+        <is>
+          <t>Unanimous — Prisma stays</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="15" customHeight="1" s="186">
+      <c r="A17" s="389" t="inlineStr">
+        <is>
+          <t>Dashboard Pages</t>
+        </is>
+      </c>
+      <c r="B17" s="390" t="inlineStr">
+        <is>
+          <t>128</t>
+        </is>
+      </c>
+      <c r="C17" s="334" t="inlineStr">
         <is>
           <t>Keep it</t>
         </is>
       </c>
-      <c r="D16" s="338" t="inlineStr">
-        <is>
-          <t>Unanimous — Prisma stays</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="15" customHeight="1" s="186">
-      <c r="A17" s="334" t="inlineStr">
-        <is>
-          <t>Fastify Framework</t>
-        </is>
-      </c>
-      <c r="B17" s="334" t="inlineStr">
+      <c r="D17" s="338" t="inlineStr">
+        <is>
+          <t>Unanimous — Fastify stays</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="15" customHeight="1" s="186">
+      <c r="A18" s="389" t="inlineStr">
+        <is>
+          <t>API Routes</t>
+        </is>
+      </c>
+      <c r="B18" s="390" t="inlineStr">
+        <is>
+          <t>152</t>
+        </is>
+      </c>
+      <c r="C18" s="334" t="inlineStr">
         <is>
           <t>Keep it</t>
         </is>
       </c>
-      <c r="C17" s="334" t="inlineStr">
-        <is>
-          <t>Keep it</t>
-        </is>
-      </c>
-      <c r="D17" s="338" t="inlineStr">
-        <is>
-          <t>Unanimous — Fastify stays</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="15" customHeight="1" s="186">
-      <c r="A18" s="334" t="inlineStr">
-        <is>
-          <t>RLS Multi-tenancy</t>
-        </is>
-      </c>
-      <c r="B18" s="334" t="inlineStr">
-        <is>
-          <t>Keep it</t>
-        </is>
-      </c>
-      <c r="C18" s="334" t="inlineStr">
-        <is>
-          <t>Keep it</t>
-        </is>
-      </c>
       <c r="D18" s="338" t="inlineStr">
         <is>
           <t>Unanimous — RLS stays</t>
@@ -6647,14 +6753,14 @@
       </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="186">
-      <c r="A19" s="334" t="inlineStr">
-        <is>
-          <t>Workflow Engine</t>
-        </is>
-      </c>
-      <c r="B19" s="334" t="inlineStr">
-        <is>
-          <t>Build NOW in Sprint 2.9</t>
+      <c r="A19" s="389" t="inlineStr">
+        <is>
+          <t>Test Files</t>
+        </is>
+      </c>
+      <c r="B19" s="390" t="inlineStr">
+        <is>
+          <t>389 (878 total incl. spec)</t>
         </is>
       </c>
       <c r="C19" s="334" t="inlineStr">
@@ -6669,14 +6775,14 @@
       </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="186">
-      <c r="A20" s="334" t="inlineStr">
-        <is>
-          <t>Event Bus</t>
-        </is>
-      </c>
-      <c r="B20" s="334" t="inlineStr">
-        <is>
-          <t>Build in Phase 1</t>
+      <c r="A20" s="389" t="inlineStr">
+        <is>
+          <t>Prisma Schemas</t>
+        </is>
+      </c>
+      <c r="B20" s="390" t="inlineStr">
+        <is>
+          <t>43</t>
         </is>
       </c>
       <c r="C20" s="334" t="inlineStr">
@@ -6691,14 +6797,14 @@
       </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="186">
-      <c r="A21" s="334" t="inlineStr">
-        <is>
-          <t>Module Links</t>
-        </is>
-      </c>
-      <c r="B21" s="334" t="inlineStr">
-        <is>
-          <t>Build in Phase 2</t>
+      <c r="A21" s="389" t="inlineStr">
+        <is>
+          <t>Integration Providers</t>
+        </is>
+      </c>
+      <c r="B21" s="390" t="inlineStr">
+        <is>
+          <t>124/124 ALL PRODUCTION</t>
         </is>
       </c>
       <c r="C21" s="334" t="inlineStr">
@@ -6713,14 +6819,14 @@
       </c>
     </row>
     <row r="22" ht="15" customHeight="1" s="186">
-      <c r="A22" s="334" t="inlineStr">
-        <is>
-          <t>Plugin System</t>
-        </is>
-      </c>
-      <c r="B22" s="334" t="inlineStr">
-        <is>
-          <t>Build in Phase 2</t>
+      <c r="A22" s="389" t="inlineStr">
+        <is>
+          <t>Integration Categories</t>
+        </is>
+      </c>
+      <c r="B22" s="390" t="inlineStr">
+        <is>
+          <t>21</t>
         </is>
       </c>
       <c r="C22" s="334" t="inlineStr">
@@ -6735,14 +6841,14 @@
       </c>
     </row>
     <row r="23" ht="15" customHeight="1" s="186">
-      <c r="A23" s="334" t="inlineStr">
-        <is>
-          <t>18-Month Roadmap</t>
-        </is>
-      </c>
-      <c r="B23" s="334" t="inlineStr">
-        <is>
-          <t>Commit to full timeline</t>
+      <c r="A23" s="389" t="inlineStr">
+        <is>
+          <t>E2E Test Suites</t>
+        </is>
+      </c>
+      <c r="B23" s="390" t="inlineStr">
+        <is>
+          <t>7</t>
         </is>
       </c>
       <c r="C23" s="334" t="inlineStr">
@@ -6756,22 +6862,34 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" s="391" t="inlineStr">
+        <is>
+          <t>Git Commits (5.x)</t>
+        </is>
+      </c>
+      <c r="B24" s="392" t="inlineStr">
+        <is>
+          <t>6 (5.0-plan, 5.0, 5.1-plan, 5.1, 5.2-plan, 5.2)</t>
+        </is>
+      </c>
+    </row>
     <row r="26" ht="15" customHeight="1" s="186">
-      <c r="A26" s="332" t="inlineStr">
-        <is>
-          <t>SPRINT 2.9 ACTION ITEMS</t>
+      <c r="A26" s="393" t="inlineStr">
+        <is>
+          <t>TEAM REPORTS</t>
         </is>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="186">
-      <c r="A27" s="341" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B27" s="341" t="inlineStr">
-        <is>
-          <t>Owner</t>
+      <c r="A27" s="394" t="inlineStr">
+        <is>
+          <t>AR (CTO)</t>
+        </is>
+      </c>
+      <c r="B27" s="395" t="inlineStr">
+        <is>
+          <t>Sprint 5.0-5.2 Complete</t>
         </is>
       </c>
       <c r="C27" s="341" t="inlineStr">
@@ -6801,12 +6919,14 @@
       </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="186">
-      <c r="A28" s="334" t="n">
-        <v>1</v>
-      </c>
-      <c r="B28" s="334" t="inlineStr">
-        <is>
-          <t>AR - Arjun</t>
+      <c r="A28" s="389" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Done:</t>
+        </is>
+      </c>
+      <c r="B28" s="390" t="inlineStr">
+        <is>
+          <t>Built routing engine, maps adapter, analytics adapters (Tableau/PowerBI/Looker/Qlik/GA4), analytics aggregator. ALL integration architecture finalized.</t>
         </is>
       </c>
       <c r="C28" s="334" t="inlineStr">
@@ -6836,12 +6956,14 @@
       </c>
     </row>
     <row r="29" ht="15" customHeight="1" s="186">
-      <c r="A29" s="334" t="n">
-        <v>2</v>
-      </c>
-      <c r="B29" s="334" t="inlineStr">
-        <is>
-          <t>RG - Rohan</t>
+      <c r="A29" s="396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Blockers:</t>
+        </is>
+      </c>
+      <c r="B29" s="390" t="inlineStr">
+        <is>
+          <t>Production deployment pipeline, CI/CD, Docker/K8s config needs production hardening</t>
         </is>
       </c>
       <c r="C29" s="334" t="inlineStr">
@@ -6906,12 +7028,14 @@
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" s="186">
-      <c r="A31" s="334" t="n">
-        <v>4</v>
-      </c>
-      <c r="B31" s="334" t="inlineStr">
-        <is>
-          <t>SP - Sanya</t>
+      <c r="A31" s="397" t="inlineStr">
+        <is>
+          <t>DM (Frontend)</t>
+        </is>
+      </c>
+      <c r="B31" s="389" t="inlineStr">
+        <is>
+          <t>8 dashboard pages delivered in 5.2</t>
         </is>
       </c>
       <c r="C31" s="334" t="inlineStr">
@@ -6941,12 +7065,14 @@
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" s="186">
-      <c r="A32" s="334" t="n">
-        <v>5</v>
-      </c>
-      <c r="B32" s="334" t="inlineStr">
-        <is>
-          <t>NK - Neha</t>
+      <c r="A32" s="389" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Done:</t>
+        </is>
+      </c>
+      <c r="B32" s="390" t="inlineStr">
+        <is>
+          <t>Analytics, supply-chain, freight, fuel dashboards. Total 128 pages across platform.</t>
         </is>
       </c>
       <c r="C32" s="334" t="inlineStr">
@@ -6976,12 +7102,14 @@
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" s="186">
-      <c r="A33" s="334" t="n">
-        <v>6</v>
-      </c>
-      <c r="B33" s="334" t="inlineStr">
-        <is>
-          <t>KS - Kavitha</t>
+      <c r="A33" s="396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Blockers:</t>
+        </is>
+      </c>
+      <c r="B33" s="390" t="inlineStr">
+        <is>
+          <t>Onboarding flow is basic 5-step wizard — needs full Fleetbase-style overhaul</t>
         </is>
       </c>
       <c r="C33" s="334" t="inlineStr">
@@ -7046,12 +7174,14 @@
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" s="186">
-      <c r="A35" s="334" t="n">
-        <v>8</v>
-      </c>
-      <c r="B35" s="334" t="inlineStr">
-        <is>
-          <t>VS - Vikram</t>
+      <c r="A35" s="397" t="inlineStr">
+        <is>
+          <t>NK (Frontend Lead)</t>
+        </is>
+      </c>
+      <c r="B35" s="389" t="inlineStr">
+        <is>
+          <t>8 dashboard pages across 5.1-5.2</t>
         </is>
       </c>
       <c r="C35" s="334" t="inlineStr">
@@ -7081,12 +7211,14 @@
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" s="186">
-      <c r="A36" s="334" t="n">
-        <v>9</v>
-      </c>
-      <c r="B36" s="334" t="inlineStr">
-        <is>
-          <t>AM - Aisha</t>
+      <c r="A36" s="389" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Done:</t>
+        </is>
+      </c>
+      <c r="B36" s="390" t="inlineStr">
+        <is>
+          <t>Healthcare, field-service, telematics-extended, ecommerce-extended. Collaboration, ELD, POS pages.</t>
         </is>
       </c>
       <c r="C36" s="334" t="inlineStr">
@@ -7116,19 +7248,21 @@
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" s="186">
-      <c r="A37" s="334" t="n">
-        <v>10</v>
-      </c>
-      <c r="B37" s="334" t="inlineStr">
+      <c r="A37" s="396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Blockers:</t>
+        </is>
+      </c>
+      <c r="B37" s="390" t="inlineStr">
+        <is>
+          <t>Responsive testing needed, mobile breakpoints incomplete</t>
+        </is>
+      </c>
+      <c r="C37" s="334" t="inlineStr">
         <is>
           <t>ALL</t>
         </is>
       </c>
-      <c r="C37" s="334" t="inlineStr">
-        <is>
-          <t>ALL</t>
-        </is>
-      </c>
       <c r="D37" s="334" t="inlineStr">
         <is>
           <t>After Sprint 2.9: review, retrospective, decide Phase 2 scope</t>
@@ -7150,22 +7284,39 @@
         </is>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" s="398" t="inlineStr">
+        <is>
+          <t>RG (Backend Lead)</t>
+        </is>
+      </c>
+      <c r="B39" s="391" t="inlineStr">
+        <is>
+          <t>Supply chain + ERP architecture</t>
+        </is>
+      </c>
+    </row>
     <row r="40" ht="15" customHeight="1" s="186">
-      <c r="A40" s="332" t="inlineStr">
-        <is>
-          <t>REFERENCE DOCUMENTS</t>
+      <c r="A40" s="399" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Done:</t>
+        </is>
+      </c>
+      <c r="B40" s="392" t="inlineStr">
+        <is>
+          <t>Manhattan, Blue Yonder, Körber orchestrator. ERP sync engine v2 with conflict resolution.</t>
         </is>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="186">
-      <c r="A41" s="185" t="inlineStr">
-        <is>
-          <t>ADR-009:</t>
-        </is>
-      </c>
-      <c r="B41" s="185" t="inlineStr">
-        <is>
-          <t>docs/adr/ADR-009-medusa-inspired-architecture-evolution.md</t>
+      <c r="A41" s="400" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Blockers:</t>
+        </is>
+      </c>
+      <c r="B41" s="401" t="inlineStr">
+        <is>
+          <t>Need production database migrations, connection pooling, read replicas</t>
         </is>
       </c>
     </row>
@@ -7182,26 +7333,38 @@
       </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="186">
-      <c r="A43" s="185" t="inlineStr">
-        <is>
-          <t>Blue Team:</t>
-        </is>
-      </c>
-      <c r="B43" s="185" t="inlineStr">
-        <is>
-          <t>AR (CTO), DM (Frontend), NK (Frontend Lead), KS (QA Lead)</t>
+      <c r="A43" s="402" t="inlineStr">
+        <is>
+          <t>SP (Full-stack)</t>
+        </is>
+      </c>
+      <c r="B43" s="399" t="inlineStr">
+        <is>
+          <t>Healthcare HIPAA + Solid Protocol</t>
         </is>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" s="186">
-      <c r="A44" s="185" t="inlineStr">
-        <is>
-          <t>Red Team:</t>
-        </is>
-      </c>
-      <c r="B44" s="185" t="inlineStr">
-        <is>
-          <t>RG (Backend Lead), SP (Full-stack), PK (Sr. Backend), VS (Component Dev), AM (Integration)</t>
+      <c r="A44" s="399" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Done:</t>
+        </is>
+      </c>
+      <c r="B44" s="401" t="inlineStr">
+        <is>
+          <t>Epic/Cerner/Allscripts/FHIR with PHI audit logging, healthcare normalizer, MPI matching.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="403" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Blockers:</t>
+        </is>
+      </c>
+      <c r="B45" s="392" t="inlineStr">
+        <is>
+          <t>HIPAA compliance audit needed, encryption at rest verification</t>
         </is>
       </c>
     </row>
@@ -7213,23 +7376,38 @@
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" s="186">
-      <c r="A47" s="343" t="inlineStr">
-        <is>
-          <t>Sprint 4.2 shipped: ADR-021, SDK tests (141 cases), seed script, driver app screens, settings page, webhook dashboard, 5 new UI components, smoke test, CI updates</t>
+      <c r="A47" s="402" t="inlineStr">
+        <is>
+          <t>VS (Component Dev)</t>
+        </is>
+      </c>
+      <c r="B47" s="391" t="inlineStr">
+        <is>
+          <t>30+ integration UI components</t>
         </is>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" s="186">
-      <c r="A48" s="343" t="inlineStr">
-        <is>
-          <t>Deep dive: CLI deployment tool for one-line VM deployment</t>
+      <c r="A48" s="399" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Done:</t>
+        </is>
+      </c>
+      <c r="B48" s="392" t="inlineStr">
+        <is>
+          <t>Integration marketplace (124 providers), analytics embed viewer, supply chain flow, FHIR browser.</t>
         </is>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" s="186">
-      <c r="A49" s="343" t="inlineStr">
-        <is>
-          <t>Decision: Pure bash CLI (witylogix) with 12 subcommands — install, deploy, upgrade, status, logs, backup, restore, ssl, env, doctor, scale, destroy</t>
+      <c r="A49" s="400" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Blockers:</t>
+        </is>
+      </c>
+      <c r="B49" s="392" t="inlineStr">
+        <is>
+          <t>Component documentation/Storybook incomplete, accessibility audit pending</t>
         </is>
       </c>
     </row>
@@ -7241,29 +7419,538 @@
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" s="186">
-      <c r="A51" s="343" t="inlineStr">
-        <is>
-          <t>Decision: AI subcommands (ai setup, ai diagnose) for Claude-powered diagnostics</t>
+      <c r="A51" s="402" t="inlineStr">
+        <is>
+          <t>PK (Sr. Backend)</t>
+        </is>
+      </c>
+      <c r="B51" s="391" t="inlineStr">
+        <is>
+          <t>Freight + Fuel-Fleet + Payments</t>
         </is>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" s="186">
-      <c r="A52" s="343" t="inlineStr">
-        <is>
-          <t>NEW TEAM MEMBER: ZR — Zara (AI Engineer) — AI-powered features, docs search, CLI diagnostics, log analysis</t>
+      <c r="A52" s="399" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Done:</t>
+        </is>
+      </c>
+      <c r="B52" s="392" t="inlineStr">
+        <is>
+          <t>DAT/Truckstop freight aggregator, WEX/Comdata fuel card manager with fraud detection, Braintree/Adyen.</t>
         </is>
       </c>
     </row>
     <row r="53" ht="15" customHeight="1" s="186">
-      <c r="A53" s="343" t="inlineStr">
-        <is>
-          <t>Sprint 4.3 planned: Full CLI tool (infra/cli/witylogix), Caddy templates, production Docker Compose, AI diagnostics, CLI tests</t>
+      <c r="A53" s="400" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Blockers:</t>
+        </is>
+      </c>
+      <c r="B53" s="392" t="inlineStr">
+        <is>
+          <t>Rate limiting needs production tuning, circuit breaker thresholds need real-world calibration</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="398" t="inlineStr">
+        <is>
+          <t>KS (QA Lead)</t>
+        </is>
+      </c>
+      <c r="B55" s="391" t="inlineStr">
+        <is>
+          <t>Test coverage audit</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="391" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Done:</t>
+        </is>
+      </c>
+      <c r="B56" s="392" t="inlineStr">
+        <is>
+          <t>389 test files, 878 total. Every integration category has tests. 7 E2E suites. ~435+ integration-level tests across 5.0-5.2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="403" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Blockers:</t>
+        </is>
+      </c>
+      <c r="B57" s="392" t="inlineStr">
+        <is>
+          <t>Some categories have only 1-2 test files vs 6+ adapters. Need deeper unit test coverage for ERP(11), telematics(16), CRM(7)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="398" t="inlineStr">
+        <is>
+          <t>AM (Integration)</t>
+        </is>
+      </c>
+      <c r="B59" s="391" t="inlineStr">
+        <is>
+          <t>E-commerce + Telematics extended</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="391" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Done:</t>
+        </is>
+      </c>
+      <c r="B60" s="392" t="inlineStr">
+        <is>
+          <t>Amazon SP, eBay, Etsy, Square Online. Powerfleet, Azuga, Omnitracs, Platform Science.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="403" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Blockers:</t>
+        </is>
+      </c>
+      <c r="B61" s="392" t="inlineStr">
+        <is>
+          <t>OAuth token refresh flows need production testing with real credentials</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="398" t="inlineStr">
+        <is>
+          <t>ZR (AI Engineer)</t>
+        </is>
+      </c>
+      <c r="B63" s="391" t="inlineStr">
+        <is>
+          <t>Field-service + ERP + Telematics ext</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="391" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Done:</t>
+        </is>
+      </c>
+      <c r="B64" s="392" t="inlineStr">
+        <is>
+          <t>ServiceTitan/Jobber dispatcher with Haversine routing, Infor/Epicor/Sage Intacct/FreshBooks/Wave.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="403" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Blockers:</t>
+        </is>
+      </c>
+      <c r="B65" s="392" t="inlineStr">
+        <is>
+          <t>AI demand prediction model needs production data pipeline, no real training data yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="404" t="inlineStr">
+        <is>
+          <t>PRODUCTION READINESS GAPS</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="405" t="inlineStr">
+        <is>
+          <t>P0 — Must Have</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Onboarding flow overhaul (current is basic 5-step, need Fleetbase-style multi-section wizard)</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Auth hardening (password reset flow, 2FA/MFA, session management, rate limiting)</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Database production migrations (connection pooling, read replicas, backup strategy)</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • API rate limiting &amp; throttling (per-tenant, per-endpoint)</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Error handling &amp; logging (structured logs, Sentry/error tracking, alerting)</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Security audit (OWASP top 10, CSP headers, CORS, input validation)</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="405" t="inlineStr">
+        <is>
+          <t>P1 — Should Have</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • CI/CD pipeline (GitHub Actions, staging → production, rollback)</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Docker/K8s production config (health checks, resource limits, autoscaling)</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Monitoring &amp; observability (Prometheus metrics, Grafana dashboards, uptime)</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Test coverage gaps (ERP 11 adapters/4 tests, telematics 16/10, CRM 7/5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Performance testing (k6 load tests expansion, database query optimization)</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Documentation (API docs, developer guide, deployment runbook)</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="405" t="inlineStr">
+        <is>
+          <t>P2 — Nice to Have</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Storybook component library</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Accessibility WCAG 2.1 AA audit</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Internationalization (i18n) framework</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Mobile responsive polish</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Integration real-credential testing</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="406" t="inlineStr">
+        <is>
+          <t>UPCOMING SPRINT PLAN — Road to Production</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="407" t="inlineStr">
+        <is>
+          <t>Sprint 6.0 — Onboarding &amp; Auth Hardening</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  AR: Auth architecture — 2FA/MFA, session management, OAuth provider config, RBAC permissions</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  DM: Onboarding wizard Step 1-3 — Email verify, deployment choice, company info + industry + goals (Fleetbase-inspired)</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  NK: Onboarding wizard Step 4-6 — Integration picker (124 providers), dashboard layout chooser, data import (drivers/vehicles/zones)</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  RG: Onboarding API — workspace provisioning, tenant isolation, org/team Prisma schema, invitation system</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  SP: Auth flows — password reset, email verify, magic link, SSO (Google/Microsoft), rate limiting</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  VS: Onboarding UI components — stepper, industry picker, integration grid, dashboard previews, progress bar</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  PK: Tenant middleware — multi-tenancy, workspace switching, API key scoping, usage metering</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  KS: Auth &amp; onboarding test suites — E2E onboarding flow, auth edge cases, 2FA tests</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  AM: Integration onboarding — OAuth connection wizard, credential validation, health check on connect</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ZR: AI-powered onboarding — smart defaults based on industry, goal-based dashboard pre-configuration</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="407" t="inlineStr">
+        <is>
+          <t>Sprint 6.1 — Database &amp; API Production Hardening</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  AR: Database architecture — connection pooling (PgBouncer), read replicas, migration strategy, backup/restore</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  DM: Error pages &amp; loading states — 404, 500, offline, skeleton loaders, toast notifications</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  NK: Responsive audit — mobile breakpoints, tablet layouts, touch interactions across all 128 pages</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  RG: API hardening — rate limiting (per-tenant), request validation (Zod), pagination, cursor-based queries</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  SP: Security hardening — OWASP audit, CSP headers, CORS, XSS/CSRF protection, input sanitization</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  VS: Form validation library — reusable validation, error display, accessibility</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  PK: Logging &amp; monitoring — structured JSON logs, Sentry integration, Prometheus metrics, health endpoints</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  KS: Test coverage expansion — fill gaps in ERP (11→11 tests), telematics (16→16), CRM (7→7), load tests</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  AM: Webhook reliability — retry logic, dead letter queue, signature verification, event deduplication</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ZR: Query optimization — N+1 detection, query analyzer, database indexing, slow query logging</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="407" t="inlineStr">
+        <is>
+          <t>Sprint 6.2 — CI/CD, Deployment &amp; Documentation</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  AR: CI/CD pipeline — GitHub Actions, lint/test/build/deploy, staging environment, rollback strategy</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  DM: Documentation site — API docs (OpenAPI), developer guide, quick start, integration guides</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  NK: Storybook — component library documentation, visual regression tests, design tokens</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  RG: Docker/K8s production — Dockerfile optimization, k8s manifests, helm charts, autoscaling, secrets</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  SP: HIPAA compliance docs — BAA templates, PHI handling guide, encryption verification, audit procedures</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  VS: Accessibility audit — WCAG 2.1 AA compliance, screen reader testing, keyboard navigation, contrast</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  PK: Performance optimization — CDN, asset compression, lazy loading, bundle analysis, caching strategy</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  KS: E2E full regression — complete platform E2E suite, visual regression, cross-browser testing</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  AM: Integration documentation — per-provider setup guides, credential requirements, webhook configs</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ZR: Production monitoring dashboard — Grafana dashboards, alerting rules, SLA tracking, incident playbook</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A12:F12"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>
@@ -13830,6 +14517,411 @@
         <is>
           <t>14</t>
         </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" style="186" min="1" max="1"/>
+    <col width="14" customWidth="1" style="186" min="2" max="2"/>
+    <col width="35" customWidth="1" style="186" min="3" max="3"/>
+    <col width="80" customWidth="1" style="186" min="4" max="4"/>
+    <col width="10" customWidth="1" style="186" min="5" max="5"/>
+    <col width="10" customWidth="1" style="186" min="6" max="6"/>
+    <col width="10" customWidth="1" style="186" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="408" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="B1" s="408" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="C1" s="408" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="D1" s="408" t="inlineStr">
+        <is>
+          <t>Deliverables</t>
+        </is>
+      </c>
+      <c r="E1" s="408" t="inlineStr">
+        <is>
+          <t>Est. Files</t>
+        </is>
+      </c>
+      <c r="F1" s="408" t="inlineStr">
+        <is>
+          <t>Est. LOC</t>
+        </is>
+      </c>
+      <c r="G1" s="408" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="391" t="inlineStr">
+        <is>
+          <t>AR</t>
+        </is>
+      </c>
+      <c r="B2" s="392" t="inlineStr">
+        <is>
+          <t>CTO</t>
+        </is>
+      </c>
+      <c r="C2" s="392" t="inlineStr">
+        <is>
+          <t>Auth Architecture &amp; RBAC</t>
+        </is>
+      </c>
+      <c r="D2" s="392" t="inlineStr">
+        <is>
+          <t>2FA/MFA, session mgmt, OAuth config, RBAC permissions, Prisma auth schema</t>
+        </is>
+      </c>
+      <c r="E2" s="392" t="n">
+        <v>12</v>
+      </c>
+      <c r="F2" s="392" t="n">
+        <v>3500</v>
+      </c>
+      <c r="G2" s="392" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="391" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="B3" s="392" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C3" s="392" t="inlineStr">
+        <is>
+          <t>Onboarding Wizard Steps 1-3</t>
+        </is>
+      </c>
+      <c r="D3" s="392" t="inlineStr">
+        <is>
+          <t>Email verify page, deployment chooser, company info + industry + goals forms</t>
+        </is>
+      </c>
+      <c r="E3" s="392" t="n">
+        <v>8</v>
+      </c>
+      <c r="F3" s="392" t="n">
+        <v>3000</v>
+      </c>
+      <c r="G3" s="392" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="391" t="inlineStr">
+        <is>
+          <t>NK</t>
+        </is>
+      </c>
+      <c r="B4" s="392" t="inlineStr">
+        <is>
+          <t>Frontend Lead</t>
+        </is>
+      </c>
+      <c r="C4" s="392" t="inlineStr">
+        <is>
+          <t>Onboarding Wizard Steps 4-6</t>
+        </is>
+      </c>
+      <c r="D4" s="392" t="inlineStr">
+        <is>
+          <t>Integration picker (124), dashboard layout chooser, data import wizard</t>
+        </is>
+      </c>
+      <c r="E4" s="392" t="n">
+        <v>8</v>
+      </c>
+      <c r="F4" s="392" t="n">
+        <v>3500</v>
+      </c>
+      <c r="G4" s="392" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="391" t="inlineStr">
+        <is>
+          <t>RG</t>
+        </is>
+      </c>
+      <c r="B5" s="392" t="inlineStr">
+        <is>
+          <t>Backend Lead</t>
+        </is>
+      </c>
+      <c r="C5" s="392" t="inlineStr">
+        <is>
+          <t>Onboarding API &amp; Tenant System</t>
+        </is>
+      </c>
+      <c r="D5" s="392" t="inlineStr">
+        <is>
+          <t>Workspace provisioning, tenant isolation, org/team schema, invitations API</t>
+        </is>
+      </c>
+      <c r="E5" s="392" t="n">
+        <v>15</v>
+      </c>
+      <c r="F5" s="392" t="n">
+        <v>4500</v>
+      </c>
+      <c r="G5" s="392" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="391" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="B6" s="392" t="inlineStr">
+        <is>
+          <t>Full-stack</t>
+        </is>
+      </c>
+      <c r="C6" s="392" t="inlineStr">
+        <is>
+          <t>Auth Flows &amp; Security</t>
+        </is>
+      </c>
+      <c r="D6" s="392" t="inlineStr">
+        <is>
+          <t>Password reset, email verify, magic link, SSO, rate limiting middleware</t>
+        </is>
+      </c>
+      <c r="E6" s="392" t="n">
+        <v>10</v>
+      </c>
+      <c r="F6" s="392" t="n">
+        <v>3000</v>
+      </c>
+      <c r="G6" s="392" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="391" t="inlineStr">
+        <is>
+          <t>VS</t>
+        </is>
+      </c>
+      <c r="B7" s="392" t="inlineStr">
+        <is>
+          <t>Component Dev</t>
+        </is>
+      </c>
+      <c r="C7" s="392" t="inlineStr">
+        <is>
+          <t>Onboarding UI Components</t>
+        </is>
+      </c>
+      <c r="D7" s="392" t="inlineStr">
+        <is>
+          <t>Stepper, industry picker, integration grid, dashboard previews, progress bar</t>
+        </is>
+      </c>
+      <c r="E7" s="392" t="n">
+        <v>12</v>
+      </c>
+      <c r="F7" s="392" t="n">
+        <v>3500</v>
+      </c>
+      <c r="G7" s="392" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="391" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="B8" s="392" t="inlineStr">
+        <is>
+          <t>Sr. Backend</t>
+        </is>
+      </c>
+      <c r="C8" s="392" t="inlineStr">
+        <is>
+          <t>Multi-Tenant Middleware</t>
+        </is>
+      </c>
+      <c r="D8" s="392" t="inlineStr">
+        <is>
+          <t>Tenant middleware, workspace switching, API key scoping, usage metering</t>
+        </is>
+      </c>
+      <c r="E8" s="392" t="n">
+        <v>10</v>
+      </c>
+      <c r="F8" s="392" t="n">
+        <v>3000</v>
+      </c>
+      <c r="G8" s="392" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="391" t="inlineStr">
+        <is>
+          <t>KS</t>
+        </is>
+      </c>
+      <c r="B9" s="392" t="inlineStr">
+        <is>
+          <t>QA Lead</t>
+        </is>
+      </c>
+      <c r="C9" s="392" t="inlineStr">
+        <is>
+          <t>Auth &amp; Onboarding Tests</t>
+        </is>
+      </c>
+      <c r="D9" s="392" t="inlineStr">
+        <is>
+          <t>E2E onboarding flow, auth edge cases, 2FA tests, security tests</t>
+        </is>
+      </c>
+      <c r="E9" s="392" t="n">
+        <v>8</v>
+      </c>
+      <c r="F9" s="392" t="n">
+        <v>2500</v>
+      </c>
+      <c r="G9" s="392" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="391" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="B10" s="392" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="C10" s="392" t="inlineStr">
+        <is>
+          <t>Integration Onboarding Wizard</t>
+        </is>
+      </c>
+      <c r="D10" s="392" t="inlineStr">
+        <is>
+          <t>OAuth connection flow, credential validation, health check on connect</t>
+        </is>
+      </c>
+      <c r="E10" s="392" t="n">
+        <v>8</v>
+      </c>
+      <c r="F10" s="392" t="n">
+        <v>2500</v>
+      </c>
+      <c r="G10" s="392" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="391" t="inlineStr">
+        <is>
+          <t>ZR</t>
+        </is>
+      </c>
+      <c r="B11" s="392" t="inlineStr">
+        <is>
+          <t>AI Engineer</t>
+        </is>
+      </c>
+      <c r="C11" s="392" t="inlineStr">
+        <is>
+          <t>AI-Powered Smart Defaults</t>
+        </is>
+      </c>
+      <c r="D11" s="392" t="inlineStr">
+        <is>
+          <t>Industry-based config, goal-based dashboard, smart integration suggestions</t>
+        </is>
+      </c>
+      <c r="E11" s="392" t="n">
+        <v>6</v>
+      </c>
+      <c r="F11" s="392" t="n">
+        <v>2000</v>
+      </c>
+      <c r="G11" s="392" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="391" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="E12">
+        <f>SUM(E2:E11)</f>
+        <v/>
+      </c>
+      <c r="F12">
+        <f>SUM(F2:F11)</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(sprint-6.0): plan onboarding & auth hardening sprint
Sprint 6.0 — Onboarding & Auth Hardening (10 agents):
- AR: Auth architecture, RBAC, 2FA/MFA, session management
- DM: Onboarding wizard steps 1-3 (email verify, deployment, company info)
- NK: Onboarding wizard steps 4-6 (integrations, layout, data import)
- RG: Onboarding API, workspace provisioning, tenant isolation
- SP: Auth flows (password reset, magic link, SSO, rate limiting)
- VS: Onboarding UI components (stepper, pickers, previews)
- PK: Multi-tenant middleware, API keys, usage metering
- KS: Auth & onboarding test suites (200+ tests)
- AM: Integration onboarding wizard (OAuth flow, health checks)
- ZR: AI-powered smart defaults (industry-based config)

Est: ~105 files, ~35,300 LOC

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/witylogix-sprint-tracker.xlsx
+++ b/witylogix-sprint-tracker.xlsx
@@ -7949,10 +7949,10 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="A5:G5"/>
     <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:G1"/>
     <mergeCell ref="A12:F12"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A5:G5"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -14536,7 +14536,7 @@
     <col width="8" customWidth="1" style="186" min="1" max="1"/>
     <col width="14" customWidth="1" style="186" min="2" max="2"/>
     <col width="35" customWidth="1" style="186" min="3" max="3"/>
-    <col width="80" customWidth="1" style="186" min="4" max="4"/>
+    <col width="100" customWidth="1" style="186" min="4" max="4"/>
     <col width="10" customWidth="1" style="186" min="5" max="5"/>
     <col width="10" customWidth="1" style="186" min="6" max="6"/>
     <col width="10" customWidth="1" style="186" min="7" max="7"/>
@@ -14580,7 +14580,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="391" t="inlineStr">
+      <c r="A2" s="376" t="inlineStr">
         <is>
           <t>AR</t>
         </is>
@@ -14597,14 +14597,14 @@
       </c>
       <c r="D2" s="392" t="inlineStr">
         <is>
-          <t>2FA/MFA, session mgmt, OAuth config, RBAC permissions, Prisma auth schema</t>
+          <t>2FA/MFA system, session management, OAuth provider config, RBAC permissions engine, auth Prisma schema (AuthSession, MfaDevice, LoginAttempt, ApiKey, Permission, RolePermission), password hashing (argon2), JWT token service, auth middleware</t>
         </is>
       </c>
       <c r="E2" s="392" t="n">
         <v>12</v>
       </c>
       <c r="F2" s="392" t="n">
-        <v>3500</v>
+        <v>4000</v>
       </c>
       <c r="G2" s="392" t="inlineStr">
         <is>
@@ -14613,7 +14613,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="391" t="inlineStr">
+      <c r="A3" s="376" t="inlineStr">
         <is>
           <t>DM</t>
         </is>
@@ -14630,14 +14630,14 @@
       </c>
       <c r="D3" s="392" t="inlineStr">
         <is>
-          <t>Email verify page, deployment chooser, company info + industry + goals forms</t>
+          <t>Email verification page (6-digit code input), deployment chooser (Cloud/Self-Managed cards), company info form (name, website, logo upload), industry vertical picker (logistics, ecommerce, food, retail, healthcare, field-service + custom), primary goals selector (route optimization, fleet tracking, last-mile, multi-carrier, etc.)</t>
         </is>
       </c>
       <c r="E3" s="392" t="n">
         <v>8</v>
       </c>
       <c r="F3" s="392" t="n">
-        <v>3000</v>
+        <v>3200</v>
       </c>
       <c r="G3" s="392" t="inlineStr">
         <is>
@@ -14646,7 +14646,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="391" t="inlineStr">
+      <c r="A4" s="376" t="inlineStr">
         <is>
           <t>NK</t>
         </is>
@@ -14663,7 +14663,7 @@
       </c>
       <c r="D4" s="392" t="inlineStr">
         <is>
-          <t>Integration picker (124), dashboard layout chooser, data import wizard</t>
+          <t>Integration picker page (124 providers as toggleable chips grouped by category, search, 'Show More'), dashboard layout chooser (10 preset layouts: Last-Mile Ops, Fleet Mgmt, Analytics, Returns Mgmt, etc.), data import wizard (Add First Driver, Add First Vehicle, Import Vehicles CSV, Skip for Now), review summary page with edit links</t>
         </is>
       </c>
       <c r="E4" s="392" t="n">
@@ -14679,7 +14679,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="391" t="inlineStr">
+      <c r="A5" s="376" t="inlineStr">
         <is>
           <t>RG</t>
         </is>
@@ -14691,19 +14691,19 @@
       </c>
       <c r="C5" s="392" t="inlineStr">
         <is>
-          <t>Onboarding API &amp; Tenant System</t>
+          <t>Onboarding API &amp; Workspace Provisioning</t>
         </is>
       </c>
       <c r="D5" s="392" t="inlineStr">
         <is>
-          <t>Workspace provisioning, tenant isolation, org/team schema, invitations API</t>
+          <t>POST /api/onboarding/start, /verify-email, /configure-workspace, /select-integrations, /choose-layout, /import-data, /complete — workspace provisioning service, tenant isolation middleware, org/team invitation system, onboarding progress tracking, Prisma schema (OnboardingProgress, Workspace, WorkspaceSettings, Invitation)</t>
         </is>
       </c>
       <c r="E5" s="392" t="n">
         <v>15</v>
       </c>
       <c r="F5" s="392" t="n">
-        <v>4500</v>
+        <v>4800</v>
       </c>
       <c r="G5" s="392" t="inlineStr">
         <is>
@@ -14712,7 +14712,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="391" t="inlineStr">
+      <c r="A6" s="376" t="inlineStr">
         <is>
           <t>SP</t>
         </is>
@@ -14729,14 +14729,14 @@
       </c>
       <c r="D6" s="392" t="inlineStr">
         <is>
-          <t>Password reset, email verify, magic link, SSO, rate limiting middleware</t>
+          <t>Password reset flow (email token + reset page), email verification (6-digit OTP), magic link auth, SSO providers (Google OAuth2, Microsoft MSAL), rate limiting middleware (sliding window per-IP + per-user), CSRF protection, secure cookie config, login/register page overhaul</t>
         </is>
       </c>
       <c r="E6" s="392" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F6" s="392" t="n">
-        <v>3000</v>
+        <v>3800</v>
       </c>
       <c r="G6" s="392" t="inlineStr">
         <is>
@@ -14745,7 +14745,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="391" t="inlineStr">
+      <c r="A7" s="376" t="inlineStr">
         <is>
           <t>VS</t>
         </is>
@@ -14762,14 +14762,14 @@
       </c>
       <c r="D7" s="392" t="inlineStr">
         <is>
-          <t>Stepper, industry picker, integration grid, dashboard previews, progress bar</t>
+          <t>OnboardingStepper (multi-section progress), IndustryPicker (icon grid with search), IntegrationChipGrid (124 providers, categories, toggles), DashboardPreviewCard (10 layout thumbnails), DataImportWizard (CSV upload, manual entry), GoalSelector (multi-select cards), ReviewSummary (collapsible sections with edit), VerificationCodeInput (6-digit OTP)</t>
         </is>
       </c>
       <c r="E7" s="392" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F7" s="392" t="n">
-        <v>3500</v>
+        <v>4000</v>
       </c>
       <c r="G7" s="392" t="inlineStr">
         <is>
@@ -14778,7 +14778,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="391" t="inlineStr">
+      <c r="A8" s="376" t="inlineStr">
         <is>
           <t>PK</t>
         </is>
@@ -14790,19 +14790,19 @@
       </c>
       <c r="C8" s="392" t="inlineStr">
         <is>
-          <t>Multi-Tenant Middleware</t>
+          <t>Multi-Tenant Middleware &amp; API Keys</t>
         </is>
       </c>
       <c r="D8" s="392" t="inlineStr">
         <is>
-          <t>Tenant middleware, workspace switching, API key scoping, usage metering</t>
+          <t>Tenant resolution middleware (subdomain + header + JWT), workspace switching API, API key generation/rotation/scoping, usage metering (request counts, bandwidth), tenant-scoped database queries, rate limiting per-tenant, webhook secret management</t>
         </is>
       </c>
       <c r="E8" s="392" t="n">
         <v>10</v>
       </c>
       <c r="F8" s="392" t="n">
-        <v>3000</v>
+        <v>3200</v>
       </c>
       <c r="G8" s="392" t="inlineStr">
         <is>
@@ -14811,7 +14811,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="391" t="inlineStr">
+      <c r="A9" s="376" t="inlineStr">
         <is>
           <t>KS</t>
         </is>
@@ -14823,19 +14823,19 @@
       </c>
       <c r="C9" s="392" t="inlineStr">
         <is>
-          <t>Auth &amp; Onboarding Tests</t>
+          <t>Auth &amp; Onboarding Test Suites</t>
         </is>
       </c>
       <c r="D9" s="392" t="inlineStr">
         <is>
-          <t>E2E onboarding flow, auth edge cases, 2FA tests, security tests</t>
+          <t>E2E onboarding flow test (full wizard walkthrough), auth unit tests (password hashing, JWT, MFA, session), login/register/reset E2E tests, rate limiting tests, RBAC permission tests, onboarding API integration tests, tenant isolation tests, 8+ test files, 200+ tests</t>
         </is>
       </c>
       <c r="E9" s="392" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F9" s="392" t="n">
-        <v>2500</v>
+        <v>3500</v>
       </c>
       <c r="G9" s="392" t="inlineStr">
         <is>
@@ -14844,7 +14844,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="391" t="inlineStr">
+      <c r="A10" s="376" t="inlineStr">
         <is>
           <t>AM</t>
         </is>
@@ -14861,65 +14861,65 @@
       </c>
       <c r="D10" s="392" t="inlineStr">
         <is>
-          <t>OAuth connection flow, credential validation, health check on connect</t>
+          <t>OAuth connection flow component (redirect + callback handling), credential validation service (test connection for each provider type), health check on connect (verify API key/OAuth token works), integration quick-setup templates (pre-filled configs per provider), batch enable/disable integrations</t>
         </is>
       </c>
       <c r="E10" s="392" t="n">
         <v>8</v>
       </c>
       <c r="F10" s="392" t="n">
+        <v>2800</v>
+      </c>
+      <c r="G10" s="392" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="376" t="inlineStr">
+        <is>
+          <t>ZR</t>
+        </is>
+      </c>
+      <c r="B11" s="392" t="inlineStr">
+        <is>
+          <t>AI Engineer</t>
+        </is>
+      </c>
+      <c r="C11" s="392" t="inlineStr">
+        <is>
+          <t>AI-Powered Smart Onboarding</t>
+        </is>
+      </c>
+      <c r="D11" s="392" t="inlineStr">
+        <is>
+          <t>Industry-based smart defaults engine (pre-select integrations, goals, layout based on industry), goal-to-feature mapper (suggest dashboard layout from selected goals), onboarding analytics (track completion rates, drop-off points, time-per-step), smart integration recommendations (collaborative filtering based on similar orgs)</t>
+        </is>
+      </c>
+      <c r="E11" s="392" t="n">
+        <v>8</v>
+      </c>
+      <c r="F11" s="392" t="n">
         <v>2500</v>
       </c>
-      <c r="G10" s="392" t="inlineStr">
+      <c r="G11" s="392" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="391" t="inlineStr">
-        <is>
-          <t>ZR</t>
-        </is>
-      </c>
-      <c r="B11" s="392" t="inlineStr">
-        <is>
-          <t>AI Engineer</t>
-        </is>
-      </c>
-      <c r="C11" s="392" t="inlineStr">
-        <is>
-          <t>AI-Powered Smart Defaults</t>
-        </is>
-      </c>
-      <c r="D11" s="392" t="inlineStr">
-        <is>
-          <t>Industry-based config, goal-based dashboard, smart integration suggestions</t>
-        </is>
-      </c>
-      <c r="E11" s="392" t="n">
-        <v>6</v>
-      </c>
-      <c r="F11" s="392" t="n">
-        <v>2000</v>
-      </c>
-      <c r="G11" s="392" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-    </row>
     <row r="12">
-      <c r="A12" s="391" t="inlineStr">
+      <c r="A12" s="376" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E12">
+      <c r="E12" s="185">
         <f>SUM(E2:E11)</f>
         <v/>
       </c>
-      <c r="F12">
+      <c r="F12" s="185">
         <f>SUM(F2:F11)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
chore(sprint-6.1): plan database & API production hardening sprint
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/witylogix-sprint-tracker.xlsx
+++ b/witylogix-sprint-tracker.xlsx
@@ -36,6 +36,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 5.1 Done" sheetId="27" state="visible" r:id="rId27"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 5.2 Done" sheetId="28" state="visible" r:id="rId28"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 6.0 Done" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 6.1 Plan" sheetId="30" state="visible" r:id="rId30"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Data Models Gap'!$A$1:$K$40</definedName>
@@ -651,7 +652,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="49">
+  <fills count="51">
     <fill>
       <patternFill/>
     </fill>
@@ -934,6 +935,16 @@
         <fgColor rgb="001e3a5f"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001a1a2e"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F5A623"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="6">
     <border>
@@ -1005,7 +1016,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="409">
+  <cellXfs count="412">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -2206,6 +2217,15 @@
     <xf numFmtId="0" fontId="85" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="86" fillId="48" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="71" fillId="49" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="74" fillId="50" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -3473,7 +3493,7 @@
           <t>Sprint 5.2</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="185" t="inlineStr">
         <is>
           <t>Sprint 6.0</t>
         </is>
@@ -3513,7 +3533,7 @@
       <c r="B2" s="185" t="n">
         <v>1709</v>
       </c>
-      <c r="C2" t="n">
+      <c r="C2" s="185" t="n">
         <v>2165</v>
       </c>
       <c r="Y2" s="377" t="n">
@@ -7959,9 +7979,9 @@
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A12:F12"/>
+    <mergeCell ref="A1:G1"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -15285,6 +15305,324 @@
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" style="186" min="1" max="1"/>
+    <col width="18" customWidth="1" style="186" min="2" max="2"/>
+    <col width="40" customWidth="1" style="186" min="3" max="3"/>
+    <col width="50" customWidth="1" style="186" min="4" max="4"/>
+    <col width="12" customWidth="1" style="186" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="409" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="B1" s="409" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="C1" s="409" t="inlineStr">
+        <is>
+          <t>Sprint 6.1 Task</t>
+        </is>
+      </c>
+      <c r="D1" s="409" t="inlineStr">
+        <is>
+          <t>Deliverables</t>
+        </is>
+      </c>
+      <c r="E1" s="409" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="410" t="inlineStr">
+        <is>
+          <t>AR</t>
+        </is>
+      </c>
+      <c r="B2" s="410" t="inlineStr">
+        <is>
+          <t>CTO/Architect</t>
+        </is>
+      </c>
+      <c r="C2" s="410" t="inlineStr">
+        <is>
+          <t>Database Production Config</t>
+        </is>
+      </c>
+      <c r="D2" s="410" t="inlineStr">
+        <is>
+          <t>PgBouncer config, read replica setup, migration strategy, backup/restore scripts, connection pool tuning</t>
+        </is>
+      </c>
+      <c r="E2" s="411" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="410" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="B3" s="410" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C3" s="410" t="inlineStr">
+        <is>
+          <t>Error Pages &amp; Loading States</t>
+        </is>
+      </c>
+      <c r="D3" s="410" t="inlineStr">
+        <is>
+          <t>404/500/offline pages, skeleton loaders, toast notifications, error boundaries, suspense fallbacks</t>
+        </is>
+      </c>
+      <c r="E3" s="411" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="410" t="inlineStr">
+        <is>
+          <t>NK</t>
+        </is>
+      </c>
+      <c r="B4" s="410" t="inlineStr">
+        <is>
+          <t>Frontend Lead</t>
+        </is>
+      </c>
+      <c r="C4" s="410" t="inlineStr">
+        <is>
+          <t>Responsive Audit &amp; Mobile</t>
+        </is>
+      </c>
+      <c r="D4" s="410" t="inlineStr">
+        <is>
+          <t>Mobile breakpoints, tablet layouts, touch interactions, viewport meta, responsive nav, mobile-first fixes</t>
+        </is>
+      </c>
+      <c r="E4" s="411" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="410" t="inlineStr">
+        <is>
+          <t>RG</t>
+        </is>
+      </c>
+      <c r="B5" s="410" t="inlineStr">
+        <is>
+          <t>Backend Lead</t>
+        </is>
+      </c>
+      <c r="C5" s="410" t="inlineStr">
+        <is>
+          <t>API Hardening</t>
+        </is>
+      </c>
+      <c r="D5" s="410" t="inlineStr">
+        <is>
+          <t>Per-tenant rate limiting, Zod request validation, cursor pagination, API versioning, request/response logging</t>
+        </is>
+      </c>
+      <c r="E5" s="411" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="410" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="B6" s="410" t="inlineStr">
+        <is>
+          <t>Full-stack</t>
+        </is>
+      </c>
+      <c r="C6" s="410" t="inlineStr">
+        <is>
+          <t>Security Hardening (OWASP)</t>
+        </is>
+      </c>
+      <c r="D6" s="410" t="inlineStr">
+        <is>
+          <t>CSP headers, CORS config, XSS/CSRF protection, input sanitization, security headers middleware</t>
+        </is>
+      </c>
+      <c r="E6" s="411" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="410" t="inlineStr">
+        <is>
+          <t>VS</t>
+        </is>
+      </c>
+      <c r="B7" s="410" t="inlineStr">
+        <is>
+          <t>Component Dev</t>
+        </is>
+      </c>
+      <c r="C7" s="410" t="inlineStr">
+        <is>
+          <t>Form Validation Library</t>
+        </is>
+      </c>
+      <c r="D7" s="410" t="inlineStr">
+        <is>
+          <t>Reusable validation hooks, error display components, a11y form patterns, validation schemas</t>
+        </is>
+      </c>
+      <c r="E7" s="411" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="410" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="B8" s="410" t="inlineStr">
+        <is>
+          <t>Sr. Backend</t>
+        </is>
+      </c>
+      <c r="C8" s="410" t="inlineStr">
+        <is>
+          <t>Logging &amp; Monitoring</t>
+        </is>
+      </c>
+      <c r="D8" s="410" t="inlineStr">
+        <is>
+          <t>Structured JSON logging, Sentry integration, Prometheus metrics, health endpoints, request tracing</t>
+        </is>
+      </c>
+      <c r="E8" s="411" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="410" t="inlineStr">
+        <is>
+          <t>KS</t>
+        </is>
+      </c>
+      <c r="B9" s="410" t="inlineStr">
+        <is>
+          <t>QA Lead</t>
+        </is>
+      </c>
+      <c r="C9" s="410" t="inlineStr">
+        <is>
+          <t>Test Coverage Expansion</t>
+        </is>
+      </c>
+      <c r="D9" s="410" t="inlineStr">
+        <is>
+          <t>Fill ERP/telematics/CRM/collab gaps, load test scripts, test utilities, coverage report</t>
+        </is>
+      </c>
+      <c r="E9" s="411" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="410" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="B10" s="410" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="C10" s="410" t="inlineStr">
+        <is>
+          <t>Webhook Reliability</t>
+        </is>
+      </c>
+      <c r="D10" s="410" t="inlineStr">
+        <is>
+          <t>Retry logic with backoff, dead letter queue, signature verification, idempotency keys, delivery logs</t>
+        </is>
+      </c>
+      <c r="E10" s="411" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="410" t="inlineStr">
+        <is>
+          <t>ZR</t>
+        </is>
+      </c>
+      <c r="B11" s="410" t="inlineStr">
+        <is>
+          <t>AI Engineer</t>
+        </is>
+      </c>
+      <c r="C11" s="410" t="inlineStr">
+        <is>
+          <t>Query Optimization</t>
+        </is>
+      </c>
+      <c r="D11" s="410" t="inlineStr">
+        <is>
+          <t>N+1 detection, query analyzer, index recommendations, slow query logging, query plan caching</t>
+        </is>
+      </c>
+      <c r="E11" s="411" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
chore(sprint-6.2): plan CI/CD, deployment & documentation sprint
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/witylogix-sprint-tracker.xlsx
+++ b/witylogix-sprint-tracker.xlsx
@@ -37,6 +37,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 5.2 Done" sheetId="28" state="visible" r:id="rId28"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 6.0 Done" sheetId="29" state="visible" r:id="rId29"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 6.1 Plan" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 6.2 Plan" sheetId="31" state="visible" r:id="rId31"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Data Models Gap'!$A$1:$K$40</definedName>
@@ -7991,10 +7992,10 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A12:F12"/>
     <mergeCell ref="A5:G5"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A12:F12"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -15630,6 +15631,274 @@
       <c r="E11" s="412" t="inlineStr">
         <is>
           <t>Done</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" style="186" min="1" max="1"/>
+    <col width="18" customWidth="1" style="186" min="2" max="2"/>
+    <col width="40" customWidth="1" style="186" min="3" max="3"/>
+    <col width="55" customWidth="1" style="186" min="4" max="4"/>
+    <col width="12" customWidth="1" style="186" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="409" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="B1" s="409" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="C1" s="409" t="inlineStr">
+        <is>
+          <t>Sprint 6.2 Task</t>
+        </is>
+      </c>
+      <c r="D1" s="409" t="inlineStr">
+        <is>
+          <t>Deliverables</t>
+        </is>
+      </c>
+      <c r="E1" s="409" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="410" t="inlineStr">
+        <is>
+          <t>AR</t>
+        </is>
+      </c>
+      <c r="B2" s="410" t="inlineStr">
+        <is>
+          <t>CTO/Architect</t>
+        </is>
+      </c>
+      <c r="C2" s="410" t="inlineStr">
+        <is>
+          <t>CI/CD Pipeline &amp; GitHub Actions</t>
+        </is>
+      </c>
+      <c r="D2" s="410" t="inlineStr">
+        <is>
+          <t>CI workflow (lint, typecheck, test, build), PR checks, branch protection rules, automated release workflow, Docker image build + push to GHCR, env matrix (dev/staging/prod)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="410" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="B3" s="410" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C3" s="410" t="inlineStr">
+        <is>
+          <t>Storybook &amp; Component Docs</t>
+        </is>
+      </c>
+      <c r="D3" s="410" t="inlineStr">
+        <is>
+          <t>Storybook 8 setup, stories for 20+ UI components, design token docs, interaction tests, dark/light theme toggle, a11y addon, deploy config</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="410" t="inlineStr">
+        <is>
+          <t>NK</t>
+        </is>
+      </c>
+      <c r="B4" s="410" t="inlineStr">
+        <is>
+          <t>Frontend Lead</t>
+        </is>
+      </c>
+      <c r="C4" s="410" t="inlineStr">
+        <is>
+          <t>i18n &amp; Localization Framework</t>
+        </is>
+      </c>
+      <c r="D4" s="410" t="inlineStr">
+        <is>
+          <t>next-intl setup, locale routing, 3 languages (en/es/fr), translation extraction script, RTL support prep, date/number/currency formatting, language switcher component</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="410" t="inlineStr">
+        <is>
+          <t>RG</t>
+        </is>
+      </c>
+      <c r="B5" s="410" t="inlineStr">
+        <is>
+          <t>Backend Lead</t>
+        </is>
+      </c>
+      <c r="C5" s="410" t="inlineStr">
+        <is>
+          <t>API Documentation &amp; OpenAPI</t>
+        </is>
+      </c>
+      <c r="D5" s="410" t="inlineStr">
+        <is>
+          <t>OpenAPI 3.1 spec update (all new 6.0/6.1 endpoints), Swagger UI refresh, API changelog, SDK type regeneration, Postman collection export, API rate limit docs</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="410" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="B6" s="410" t="inlineStr">
+        <is>
+          <t>Full-stack</t>
+        </is>
+      </c>
+      <c r="C6" s="410" t="inlineStr">
+        <is>
+          <t>Docker Production Hardening</t>
+        </is>
+      </c>
+      <c r="D6" s="410" t="inlineStr">
+        <is>
+          <t>Multi-stage Dockerfile optimization, Docker Compose prod profile, container security scanning, non-root user, health check probes, resource limits, secrets management, .dockerignore audit</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="410" t="inlineStr">
+        <is>
+          <t>VS</t>
+        </is>
+      </c>
+      <c r="B7" s="410" t="inlineStr">
+        <is>
+          <t>Component Dev</t>
+        </is>
+      </c>
+      <c r="C7" s="410" t="inlineStr">
+        <is>
+          <t>Accessibility (a11y) Audit &amp; Fixes</t>
+        </is>
+      </c>
+      <c r="D7" s="410" t="inlineStr">
+        <is>
+          <t>WCAG 2.1 AA compliance audit, aria labels, focus management, keyboard navigation, skip links, screen reader testing, color contrast fixes, a11y test utilities</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="410" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="B8" s="410" t="inlineStr">
+        <is>
+          <t>Sr. Backend</t>
+        </is>
+      </c>
+      <c r="C8" s="410" t="inlineStr">
+        <is>
+          <t>Database Migrations &amp; Seeding</t>
+        </is>
+      </c>
+      <c r="D8" s="410" t="inlineStr">
+        <is>
+          <t>Prisma migration scripts for all 6.0/6.1 schemas, seed data update (onboarding, auth, tenant tables), migration test suite, rollback scripts, data integrity checks</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="410" t="inlineStr">
+        <is>
+          <t>KS</t>
+        </is>
+      </c>
+      <c r="B9" s="410" t="inlineStr">
+        <is>
+          <t>QA Lead</t>
+        </is>
+      </c>
+      <c r="C9" s="410" t="inlineStr">
+        <is>
+          <t>Performance &amp; Load Testing Suite</t>
+        </is>
+      </c>
+      <c r="D9" s="410" t="inlineStr">
+        <is>
+          <t>k6 load test scenarios (auth, onboarding, API CRUD, webhook delivery), performance baselines, SLA thresholds, CI integration, HTML report generation, regression detection</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="410" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="B10" s="410" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="C10" s="410" t="inlineStr">
+        <is>
+          <t>Environment Config &amp; Secrets</t>
+        </is>
+      </c>
+      <c r="D10" s="410" t="inlineStr">
+        <is>
+          <t>Env validation with Zod, .env.example update, secrets rotation guide, Vault integration stubs, config service with hot reload, env-specific feature flags, deployment checklist</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="410" t="inlineStr">
+        <is>
+          <t>ZR</t>
+        </is>
+      </c>
+      <c r="B11" s="410" t="inlineStr">
+        <is>
+          <t>AI Engineer</t>
+        </is>
+      </c>
+      <c r="C11" s="410" t="inlineStr">
+        <is>
+          <t>Observability Dashboard &amp; Runbooks</t>
+        </is>
+      </c>
+      <c r="D11" s="410" t="inlineStr">
+        <is>
+          <t>Grafana dashboard JSON configs, Prometheus alert rules, PagerDuty integration stubs, runbook templates (incident response, scaling, backup recovery), SLO/SLI definitions, on-call rotation config</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(sprint-7.0): plan docs, polish & onboarding wiring sprint
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/witylogix-sprint-tracker.xlsx
+++ b/witylogix-sprint-tracker.xlsx
@@ -38,6 +38,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 6.0 Done" sheetId="29" state="visible" r:id="rId29"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 6.1 Plan" sheetId="30" state="visible" r:id="rId30"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 6.2 Plan" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 7.0 Plan" sheetId="32" state="visible" r:id="rId32"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Data Models Gap'!$A$1:$K$40</definedName>
@@ -7993,10 +7994,10 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="A5:G5"/>
     <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:G1"/>
     <mergeCell ref="A12:F12"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A5:G5"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -15950,6 +15951,274 @@
       <c r="E11" s="413" t="inlineStr">
         <is>
           <t>Done</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" style="186" min="1" max="1"/>
+    <col width="18" customWidth="1" style="186" min="2" max="2"/>
+    <col width="40" customWidth="1" style="186" min="3" max="3"/>
+    <col width="55" customWidth="1" style="186" min="4" max="4"/>
+    <col width="12" customWidth="1" style="186" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="409" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="B1" s="409" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="C1" s="409" t="inlineStr">
+        <is>
+          <t>Sprint 7.0 Task</t>
+        </is>
+      </c>
+      <c r="D1" s="409" t="inlineStr">
+        <is>
+          <t>Deliverables</t>
+        </is>
+      </c>
+      <c r="E1" s="409" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="410" t="inlineStr">
+        <is>
+          <t>AR</t>
+        </is>
+      </c>
+      <c r="B2" s="410" t="inlineStr">
+        <is>
+          <t>CTO/Architect</t>
+        </is>
+      </c>
+      <c r="C2" s="410" t="inlineStr">
+        <is>
+          <t>README &amp; Architecture Docs Refresh</t>
+        </is>
+      </c>
+      <c r="D2" s="410" t="inlineStr">
+        <is>
+          <t>README rewrite (clear value prop, updated architecture diagram, quick start verification, badge refresh, contributor guide links), ARCHITECTURE.md (system design, data flow diagrams, module dependency map), DEPLOYMENT.md (production checklist, scaling guide, monitoring setup)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="410" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="B3" s="410" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C3" s="410" t="inlineStr">
+        <is>
+          <t>Wire Onboarding Placeholders</t>
+        </is>
+      </c>
+      <c r="D3" s="410" t="inlineStr">
+        <is>
+          <t>Wire integrations-select/dashboard-layout/data-import steps into onboarding page.tsx (remove 'Coming soon'), connect step components to state, add transitions between sub-steps, fix URL param sync for all 9 steps</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="410" t="inlineStr">
+        <is>
+          <t>NK</t>
+        </is>
+      </c>
+      <c r="B4" s="410" t="inlineStr">
+        <is>
+          <t>Frontend Lead</t>
+        </is>
+      </c>
+      <c r="C4" s="410" t="inlineStr">
+        <is>
+          <t>Dashboard Landing &amp; Navigation Polish</t>
+        </is>
+      </c>
+      <c r="D4" s="410" t="inlineStr">
+        <is>
+          <t>Dashboard home page redesign (welcome banner, quick stats, recent activity, getting started checklist), sidebar navigation polish (active states, collapsible groups, notification badges), breadcrumb component, page transition animations</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="410" t="inlineStr">
+        <is>
+          <t>RG</t>
+        </is>
+      </c>
+      <c r="B5" s="410" t="inlineStr">
+        <is>
+          <t>Backend Lead</t>
+        </is>
+      </c>
+      <c r="C5" s="410" t="inlineStr">
+        <is>
+          <t>API Route Documentation &amp; Validation Audit</t>
+        </is>
+      </c>
+      <c r="D5" s="410" t="inlineStr">
+        <is>
+          <t>Audit all 152 API routes for Zod validation coverage, add missing request/response schemas, standardize error responses, generate updated route map, API health dashboard endpoint</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="410" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="B6" s="410" t="inlineStr">
+        <is>
+          <t>Full-stack</t>
+        </is>
+      </c>
+      <c r="C6" s="410" t="inlineStr">
+        <is>
+          <t>End-to-End Smoke Test Suite</t>
+        </is>
+      </c>
+      <c r="D6" s="410" t="inlineStr">
+        <is>
+          <t>Playwright smoke tests covering critical paths: register → onboard → create order → assign driver → complete delivery, auth flows (login/register/reset/magic-link), integration health checks, CI integration</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="410" t="inlineStr">
+        <is>
+          <t>VS</t>
+        </is>
+      </c>
+      <c r="B7" s="410" t="inlineStr">
+        <is>
+          <t>Component Dev</t>
+        </is>
+      </c>
+      <c r="C7" s="410" t="inlineStr">
+        <is>
+          <t>Design System Documentation</t>
+        </is>
+      </c>
+      <c r="D7" s="410" t="inlineStr">
+        <is>
+          <t>Component catalog page update (all new Sprint 6.x components), design token reference page, usage examples for form components/a11y/responsive, Storybook cross-reference links, dark/light theme showcase</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="410" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="B8" s="410" t="inlineStr">
+        <is>
+          <t>Sr. Backend</t>
+        </is>
+      </c>
+      <c r="C8" s="410" t="inlineStr">
+        <is>
+          <t>Database Schema Documentation</t>
+        </is>
+      </c>
+      <c r="D8" s="410" t="inlineStr">
+        <is>
+          <t>Prisma schema docs (50 models documented), ER diagram generation script, migration history page, schema changelog, data dictionary with field descriptions and relationships</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="410" t="inlineStr">
+        <is>
+          <t>KS</t>
+        </is>
+      </c>
+      <c r="B9" s="410" t="inlineStr">
+        <is>
+          <t>QA Lead</t>
+        </is>
+      </c>
+      <c r="C9" s="410" t="inlineStr">
+        <is>
+          <t>Test Infrastructure &amp; Coverage Report</t>
+        </is>
+      </c>
+      <c r="D9" s="410" t="inlineStr">
+        <is>
+          <t>Test coverage aggregator across all packages, coverage badge generation, test result dashboard page, flaky test detector, test categorization (unit/integration/e2e/load), CI test report artifacts</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="410" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="B10" s="410" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="C10" s="410" t="inlineStr">
+        <is>
+          <t>Integration Catalog &amp; Setup Guides</t>
+        </is>
+      </c>
+      <c r="D10" s="410" t="inlineStr">
+        <is>
+          <t>Integration catalog page update (all 124 providers with setup status), per-category setup guides (routing, telematics, ERP, CRM, messaging), troubleshooting FAQ, integration health dashboard improvements</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="410" t="inlineStr">
+        <is>
+          <t>ZR</t>
+        </is>
+      </c>
+      <c r="B11" s="410" t="inlineStr">
+        <is>
+          <t>AI Engineer</t>
+        </is>
+      </c>
+      <c r="C11" s="410" t="inlineStr">
+        <is>
+          <t>Developer Experience &amp; Onboarding Guide</t>
+        </is>
+      </c>
+      <c r="D11" s="410" t="inlineStr">
+        <is>
+          <t>CONTRIBUTING.md update, development setup guide (step-by-step with screenshots), code style guide, PR template, issue templates (bug/feature/integration), developer FAQ, architecture decision record index</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(sprint-7.1): plan real-time dashboard, polish & final hardening sprint
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/witylogix-sprint-tracker.xlsx
+++ b/witylogix-sprint-tracker.xlsx
@@ -39,6 +39,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 6.1 Plan" sheetId="30" state="visible" r:id="rId30"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 6.2 Plan" sheetId="31" state="visible" r:id="rId31"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 7.0 Plan" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 7.1 Plan" sheetId="33" state="visible" r:id="rId33"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Data Models Gap'!$A$1:$K$40</definedName>
@@ -7994,9 +7995,9 @@
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A12:F12"/>
+    <mergeCell ref="A1:G1"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -16269,6 +16270,274 @@
       <c r="E11" s="413" t="inlineStr">
         <is>
           <t>Done</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" style="186" min="1" max="1"/>
+    <col width="18" customWidth="1" style="186" min="2" max="2"/>
+    <col width="40" customWidth="1" style="186" min="3" max="3"/>
+    <col width="55" customWidth="1" style="186" min="4" max="4"/>
+    <col width="12" customWidth="1" style="186" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="409" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="B1" s="409" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="C1" s="409" t="inlineStr">
+        <is>
+          <t>Sprint 7.1 Task</t>
+        </is>
+      </c>
+      <c r="D1" s="409" t="inlineStr">
+        <is>
+          <t>Deliverables</t>
+        </is>
+      </c>
+      <c r="E1" s="409" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="410" t="inlineStr">
+        <is>
+          <t>AR</t>
+        </is>
+      </c>
+      <c r="B2" s="410" t="inlineStr">
+        <is>
+          <t>CTO/Architect</t>
+        </is>
+      </c>
+      <c r="C2" s="410" t="inlineStr">
+        <is>
+          <t>Real-Time Dashboard Infrastructure</t>
+        </is>
+      </c>
+      <c r="D2" s="410" t="inlineStr">
+        <is>
+          <t>WebSocket event hub (Socket.io rooms for org/shop/driver), real-time event types (order.created/updated, delivery.status, driver.location, alert), connection manager with heartbeat, Redis pub/sub bridge, reconnection with exponential backoff, event replay on reconnect</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="410" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="B3" s="410" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C3" s="410" t="inlineStr">
+        <is>
+          <t>Live Dashboard Widgets</t>
+        </is>
+      </c>
+      <c r="D3" s="410" t="inlineStr">
+        <is>
+          <t>Real-time order feed (live ticker, auto-scroll), active delivery map (Leaflet with live driver pins, route lines, delivery status colors), live KPI counters (orders today, active deliveries, available drivers, SLA %), notification center (bell icon, unread count, toast on new events), auto-refresh without full page reload</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="410" t="inlineStr">
+        <is>
+          <t>NK</t>
+        </is>
+      </c>
+      <c r="B4" s="410" t="inlineStr">
+        <is>
+          <t>Frontend Lead</t>
+        </is>
+      </c>
+      <c r="C4" s="410" t="inlineStr">
+        <is>
+          <t>Settings &amp; Profile Pages</t>
+        </is>
+      </c>
+      <c r="D4" s="410" t="inlineStr">
+        <is>
+          <t>Account settings (profile, avatar upload, password change, MFA setup), organization settings (name, logo, billing info, plan display), notification preferences (per-channel toggles), API key management UI (generate, copy, revoke, usage stats), team management page (invite, roles, remove), timezone &amp; locale preferences</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="410" t="inlineStr">
+        <is>
+          <t>RG</t>
+        </is>
+      </c>
+      <c r="B5" s="410" t="inlineStr">
+        <is>
+          <t>Backend Lead</t>
+        </is>
+      </c>
+      <c r="C5" s="410" t="inlineStr">
+        <is>
+          <t>API Rate Limiting &amp; Throttling Production</t>
+        </is>
+      </c>
+      <c r="D5" s="410" t="inlineStr">
+        <is>
+          <t>Redis-backed sliding window rate limiter, per-tenant plan enforcement (FREE/PRO/ENTERPRISE tiers), rate limit headers (X-RateLimit-*), graceful degradation under load, circuit breaker for external APIs, request queue for burst handling, rate limit analytics endpoint</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="410" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="B6" s="410" t="inlineStr">
+        <is>
+          <t>Full-stack</t>
+        </is>
+      </c>
+      <c r="C6" s="410" t="inlineStr">
+        <is>
+          <t>Search &amp; Filtering Infrastructure</t>
+        </is>
+      </c>
+      <c r="D6" s="410" t="inlineStr">
+        <is>
+          <t>Full-text search engine (PostgreSQL tsvector/tsquery), search API endpoints (orders, drivers, deliveries, integrations), type-ahead/autocomplete, filter builder (date range, status, driver, zone, customer), saved searches, search analytics, debounced search hook</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="410" t="inlineStr">
+        <is>
+          <t>VS</t>
+        </is>
+      </c>
+      <c r="B7" s="410" t="inlineStr">
+        <is>
+          <t>Component Dev</t>
+        </is>
+      </c>
+      <c r="C7" s="410" t="inlineStr">
+        <is>
+          <t>Data Table &amp; List Enhancements</t>
+        </is>
+      </c>
+      <c r="D7" s="410" t="inlineStr">
+        <is>
+          <t>Enhanced data table (sortable columns, column resize, column visibility toggle, row selection, bulk actions, export CSV/JSON, inline editing, sticky header), virtual scrolling for large lists, table preferences persistence, table loading/empty states, print-friendly styles</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="410" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="B8" s="410" t="inlineStr">
+        <is>
+          <t>Sr. Backend</t>
+        </is>
+      </c>
+      <c r="C8" s="410" t="inlineStr">
+        <is>
+          <t>Background Jobs &amp; Queue Management</t>
+        </is>
+      </c>
+      <c r="D8" s="410" t="inlineStr">
+        <is>
+          <t>BullMQ queue dashboard (active/waiting/completed/failed counts, job details, retry/remove), scheduled jobs manager (cron expressions, next run display), job priority system, dead letter queue viewer, queue health metrics, worker scaling config, job cleanup policies</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="410" t="inlineStr">
+        <is>
+          <t>KS</t>
+        </is>
+      </c>
+      <c r="B9" s="410" t="inlineStr">
+        <is>
+          <t>QA Lead</t>
+        </is>
+      </c>
+      <c r="C9" s="410" t="inlineStr">
+        <is>
+          <t>Regression Test Suite &amp; CI Integration</t>
+        </is>
+      </c>
+      <c r="D9" s="410" t="inlineStr">
+        <is>
+          <t>Regression test matrix (critical paths × browsers × viewports), visual regression tests (screenshot comparison), CI test workflow optimization (parallel sharding, caching, fail-fast), test tagging (@smoke, @regression, @critical), nightly regression run config, test flakiness report</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="410" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="B10" s="410" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="C10" s="410" t="inlineStr">
+        <is>
+          <t>Webhook Testing &amp; Debug Tools</t>
+        </is>
+      </c>
+      <c r="D10" s="410" t="inlineStr">
+        <is>
+          <t>Webhook debugger page (live event stream, payload inspector, delivery timeline), webhook test sender (fire test events to endpoints), request/response logger with replay, integration sandbox mode, webhook signature tester, CLI webhook inspect command</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="410" t="inlineStr">
+        <is>
+          <t>ZR</t>
+        </is>
+      </c>
+      <c r="B11" s="410" t="inlineStr">
+        <is>
+          <t>AI Engineer</t>
+        </is>
+      </c>
+      <c r="C11" s="410" t="inlineStr">
+        <is>
+          <t>AI-Powered Search &amp; Smart Suggestions</t>
+        </is>
+      </c>
+      <c r="D11" s="410" t="inlineStr">
+        <is>
+          <t>Semantic search (embedding-based similarity for orders/drivers), smart command palette (Cmd+K, fuzzy search across entities), AI auto-complete for search queries, suggested actions based on context, natural language filter parsing ('show overdue orders from last week'), search ranking with ML scoring</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(sprint-8.x): CTO integration research & sprint roadmap
- Move 5 stray MD files from root to docs/ (ARCHITECTURE, DEPLOYMENT,
  CONTRIBUTING, FORM_VALIDATION, PLAYWRIGHT)
- Audit all 125 integration providers across 21 categories — confirm
  every adapter has real HTTP implementations (not stubs)
- Research API docs, SDKs, auth patterns, rate limits, webhooks, and
  pricing for all 125 providers via 4 parallel research agents
- Create comprehensive INTEGRATION_COMPLETION_PLAN.md with:
  - Per-provider inventory (auth, SDK, rate limits, priority P0-P3)
  - 10-sprint roadmap (Sprint 8.0-8.9) with per-agent assignments
  - Critical risks (USPS deprecation, FedEx SOAP sunset, HIPAA)
  - Success metrics (125/125 tests, <500ms p95, 99.5% webhook delivery)
- Add Sprint 8.x Integration Roadmap sheet to sprint tracker

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/witylogix-sprint-tracker.xlsx
+++ b/witylogix-sprint-tracker.xlsx
@@ -40,6 +40,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 6.2 Plan" sheetId="31" state="visible" r:id="rId31"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 7.0 Plan" sheetId="32" state="visible" r:id="rId32"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 7.1 Done" sheetId="33" state="visible" r:id="rId33"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.x Integration Roadmap" sheetId="34" state="visible" r:id="rId34"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Data Models Gap'!$A$1:$K$40</definedName>
@@ -659,7 +660,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="53">
+  <fills count="58">
     <fill>
       <patternFill/>
     </fill>
@@ -963,6 +964,36 @@
         <bgColor rgb="0092D050"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E79"/>
+        <bgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FF6B6B"/>
+        <bgColor rgb="00FF6B6B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8F5E9"/>
+        <bgColor rgb="00E8F5E9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFB347"/>
+        <bgColor rgb="00FFB347"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0087CEEB"/>
+        <bgColor rgb="0087CEEB"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="6">
     <border>
@@ -1034,7 +1065,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="415">
+  <cellXfs count="421">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -2250,6 +2281,14 @@
     </xf>
     <xf numFmtId="0" fontId="87" fillId="51" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="74" fillId="52" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="71" fillId="53" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="54" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="55" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="56" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="57" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -8002,10 +8041,10 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A12:F12"/>
     <mergeCell ref="A5:G5"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A12:F12"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -16595,6 +16634,380 @@
       <c r="E11" s="414" t="inlineStr">
         <is>
           <t>Done</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" style="186" min="1" max="1"/>
+    <col width="42" customWidth="1" style="186" min="2" max="2"/>
+    <col width="10" customWidth="1" style="186" min="3" max="3"/>
+    <col width="40" customWidth="1" style="186" min="4" max="4"/>
+    <col width="70" customWidth="1" style="186" min="5" max="5"/>
+    <col width="12" customWidth="1" style="186" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="415" t="inlineStr">
+        <is>
+          <t>Sprint</t>
+        </is>
+      </c>
+      <c r="B1" s="415" t="inlineStr">
+        <is>
+          <t>Theme</t>
+        </is>
+      </c>
+      <c r="C1" s="415" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="D1" s="415" t="inlineStr">
+        <is>
+          <t>Categories Covered</t>
+        </is>
+      </c>
+      <c r="E1" s="415" t="inlineStr">
+        <is>
+          <t>Key Deliverables</t>
+        </is>
+      </c>
+      <c r="F1" s="415" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="416" t="inlineStr">
+        <is>
+          <t>8.0</t>
+        </is>
+      </c>
+      <c r="B2" s="416" t="inlineStr">
+        <is>
+          <t>Integration Infrastructure &amp; P0 Core</t>
+        </is>
+      </c>
+      <c r="C2" s="417" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D2" s="416" t="inlineStr">
+        <is>
+          <t>Cross-cutting</t>
+        </is>
+      </c>
+      <c r="E2" s="416" t="inlineStr">
+        <is>
+          <t>Credential vault, OAuth2 manager, webhook verifier, marketplace UI, Stripe/Shopify/Twilio/SendGrid SDKs</t>
+        </is>
+      </c>
+      <c r="F2" s="418" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="416" t="inlineStr">
+        <is>
+          <t>8.1</t>
+        </is>
+      </c>
+      <c r="B3" s="416" t="inlineStr">
+        <is>
+          <t>Routing, Maps &amp; Real-Time Tracking</t>
+        </is>
+      </c>
+      <c r="C3" s="417" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D3" s="416" t="inlineStr">
+        <is>
+          <t>Routing, Maps, Telematics</t>
+        </is>
+      </c>
+      <c r="E3" s="416" t="inlineStr">
+        <is>
+          <t>Google Routes + Mapbox SDKs, live map, Samsara/Geotab SDKs, route optimization</t>
+        </is>
+      </c>
+      <c r="F3" s="418" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="416" t="inlineStr">
+        <is>
+          <t>8.2</t>
+        </is>
+      </c>
+      <c r="B4" s="416" t="inlineStr">
+        <is>
+          <t>Shipping &amp; Last-Mile</t>
+        </is>
+      </c>
+      <c r="C4" s="419" t="inlineStr">
+        <is>
+          <t>P0-P1</t>
+        </is>
+      </c>
+      <c r="D4" s="416" t="inlineStr">
+        <is>
+          <t>Shipping, Last-Mile, Couriers</t>
+        </is>
+      </c>
+      <c r="E4" s="416" t="inlineStr">
+        <is>
+          <t>EasyPost/ShipStation SDKs, FedEx/UPS OAuth2, DoorDash Drive, rate engine</t>
+        </is>
+      </c>
+      <c r="F4" s="418" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="416" t="inlineStr">
+        <is>
+          <t>8.3</t>
+        </is>
+      </c>
+      <c r="B5" s="416" t="inlineStr">
+        <is>
+          <t>E-Commerce &amp; Order Sync</t>
+        </is>
+      </c>
+      <c r="C5" s="419" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D5" s="416" t="inlineStr">
+        <is>
+          <t>E-Commerce</t>
+        </is>
+      </c>
+      <c r="E5" s="416" t="inlineStr">
+        <is>
+          <t>BigCommerce/Amazon SP-API, order sync v2, inventory reconciliation</t>
+        </is>
+      </c>
+      <c r="F5" s="418" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="416" t="inlineStr">
+        <is>
+          <t>8.4</t>
+        </is>
+      </c>
+      <c r="B6" s="416" t="inlineStr">
+        <is>
+          <t>CRM, ERP &amp; Accounting</t>
+        </is>
+      </c>
+      <c r="C6" s="419" t="inlineStr">
+        <is>
+          <t>P0-P1</t>
+        </is>
+      </c>
+      <c r="D6" s="416" t="inlineStr">
+        <is>
+          <t>CRM, ERP/Accounting</t>
+        </is>
+      </c>
+      <c r="E6" s="416" t="inlineStr">
+        <is>
+          <t>Salesforce/HubSpot/QuickBooks/Xero SDKs, CRM sync v3, invoice sync</t>
+        </is>
+      </c>
+      <c r="F6" s="418" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="416" t="inlineStr">
+        <is>
+          <t>8.5</t>
+        </is>
+      </c>
+      <c r="B7" s="416" t="inlineStr">
+        <is>
+          <t>Collaboration, Messaging &amp; Notifications</t>
+        </is>
+      </c>
+      <c r="C7" s="419" t="inlineStr">
+        <is>
+          <t>P0-P1</t>
+        </is>
+      </c>
+      <c r="D7" s="416" t="inlineStr">
+        <is>
+          <t>Collaboration, Messaging, Email</t>
+        </is>
+      </c>
+      <c r="E7" s="416" t="inlineStr">
+        <is>
+          <t>Slack/Teams/WhatsApp/FCM SDKs, notification orchestrator</t>
+        </is>
+      </c>
+      <c r="F7" s="418" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="416" t="inlineStr">
+        <is>
+          <t>8.6</t>
+        </is>
+      </c>
+      <c r="B8" s="416" t="inlineStr">
+        <is>
+          <t>Freight, ELD &amp; Compliance</t>
+        </is>
+      </c>
+      <c r="C8" s="419" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D8" s="416" t="inlineStr">
+        <is>
+          <t>Freight, ELD</t>
+        </is>
+      </c>
+      <c r="E8" s="416" t="inlineStr">
+        <is>
+          <t>DAT/Truckstop APIs, Motive/Samsara ELD, HOS compliance</t>
+        </is>
+      </c>
+      <c r="F8" s="418" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="416" t="inlineStr">
+        <is>
+          <t>8.7</t>
+        </is>
+      </c>
+      <c r="B9" s="416" t="inlineStr">
+        <is>
+          <t>Fuel, Fleet &amp; Field Service</t>
+        </is>
+      </c>
+      <c r="C9" s="420" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D9" s="416" t="inlineStr">
+        <is>
+          <t>Fuel/Fleet, Field Service, POS</t>
+        </is>
+      </c>
+      <c r="E9" s="416" t="inlineStr">
+        <is>
+          <t>WEX/Comdata, ServiceTitan/Jobber/Toast POS</t>
+        </is>
+      </c>
+      <c r="F9" s="418" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="416" t="inlineStr">
+        <is>
+          <t>8.8</t>
+        </is>
+      </c>
+      <c r="B10" s="416" t="inlineStr">
+        <is>
+          <t>E-Signatures, Healthcare, Analytics &amp; Supply Chain</t>
+        </is>
+      </c>
+      <c r="C10" s="420" t="inlineStr">
+        <is>
+          <t>P2-P3</t>
+        </is>
+      </c>
+      <c r="D10" s="416" t="inlineStr">
+        <is>
+          <t>E-Signatures, Healthcare, Analytics, Supply Chain</t>
+        </is>
+      </c>
+      <c r="E10" s="416" t="inlineStr">
+        <is>
+          <t>DocuSign, FHIR, Tableau/PowerBI, Manhattan/Blue Yonder</t>
+        </is>
+      </c>
+      <c r="F10" s="418" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="416" t="inlineStr">
+        <is>
+          <t>8.9</t>
+        </is>
+      </c>
+      <c r="B11" s="416" t="inlineStr">
+        <is>
+          <t>Integration Hardening &amp; Final Testing</t>
+        </is>
+      </c>
+      <c r="C11" s="416" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="D11" s="416" t="inlineStr">
+        <is>
+          <t>All 21 Categories</t>
+        </is>
+      </c>
+      <c r="E11" s="416" t="inlineStr">
+        <is>
+          <t>125/125 provider tests, rate limit audit, health dashboard, docs portal</t>
+        </is>
+      </c>
+      <c r="F11" s="418" t="inlineStr">
+        <is>
+          <t>Planned</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(sprint-8.0): plan integration infrastructure & P0 core sprint
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/witylogix-sprint-tracker.xlsx
+++ b/witylogix-sprint-tracker.xlsx
@@ -41,6 +41,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 7.0 Plan" sheetId="32" state="visible" r:id="rId32"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 7.1 Done" sheetId="33" state="visible" r:id="rId33"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.x Integration Roadmap" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.0 Plan" sheetId="35" state="visible" r:id="rId35"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Data Models Gap'!$A$1:$K$40</definedName>
@@ -8041,9 +8042,9 @@
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A12:F12"/>
+    <mergeCell ref="A1:G1"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -17010,6 +17011,284 @@
           <t>Planned</t>
         </is>
       </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" style="186" min="1" max="1"/>
+    <col width="18" customWidth="1" style="186" min="2" max="2"/>
+    <col width="35" customWidth="1" style="186" min="3" max="3"/>
+    <col width="90" customWidth="1" style="186" min="4" max="4"/>
+    <col width="10" customWidth="1" style="186" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="415" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="B1" s="415" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="C1" s="415" t="inlineStr">
+        <is>
+          <t>Sprint 8.0 Task</t>
+        </is>
+      </c>
+      <c r="D1" s="415" t="inlineStr">
+        <is>
+          <t>Deliverables</t>
+        </is>
+      </c>
+      <c r="E1" s="415" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="416" t="inlineStr">
+        <is>
+          <t>AR</t>
+        </is>
+      </c>
+      <c r="B2" s="416" t="inlineStr">
+        <is>
+          <t>CTO/Architect</t>
+        </is>
+      </c>
+      <c r="C2" s="416" t="inlineStr">
+        <is>
+          <t>Integration Infrastructure Core</t>
+        </is>
+      </c>
+      <c r="D2" s="416" t="inlineStr">
+        <is>
+          <t>Unified credential vault (AES-256-GCM encryption, per-tenant isolation, key rotation), OAuth2 token manager (auto-refresh, retry with backoff, token persistence), webhook signature verification framework (HMAC-SHA256, timestamp validation, replay protection), integration gateway middleware</t>
+        </is>
+      </c>
+      <c r="E2" s="416" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="416" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="B3" s="416" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C3" s="416" t="inlineStr">
+        <is>
+          <t>Integration Marketplace UI</t>
+        </is>
+      </c>
+      <c r="D3" s="416" t="inlineStr">
+        <is>
+          <t>Marketplace catalog page (grid/list view, category filters, search), integration detail modal (description, features, pricing, setup guide), install/uninstall flow with confirmation, credential input forms (masked fields, validation, test connection button)</t>
+        </is>
+      </c>
+      <c r="E3" s="416" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="416" t="inlineStr">
+        <is>
+          <t>NK</t>
+        </is>
+      </c>
+      <c r="B4" s="416" t="inlineStr">
+        <is>
+          <t>Frontend Lead</t>
+        </is>
+      </c>
+      <c r="C4" s="416" t="inlineStr">
+        <is>
+          <t>Per-Tenant Integration Dashboard</t>
+        </is>
+      </c>
+      <c r="D4" s="416" t="inlineStr">
+        <is>
+          <t>Connected integrations overview (status cards, health indicators), usage meters (API calls, data synced, errors), integration logs viewer (filterable, searchable), health check triggers, sync controls (pause/resume/force-sync)</t>
+        </is>
+      </c>
+      <c r="E4" s="416" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="416" t="inlineStr">
+        <is>
+          <t>RG</t>
+        </is>
+      </c>
+      <c r="B5" s="416" t="inlineStr">
+        <is>
+          <t>Backend Lead</t>
+        </is>
+      </c>
+      <c r="C5" s="416" t="inlineStr">
+        <is>
+          <t>Integration Gateway &amp; Rate Limiting</t>
+        </is>
+      </c>
+      <c r="D5" s="416" t="inlineStr">
+        <is>
+          <t>API gateway middleware (request/response logging, correlation IDs), per-provider circuit breaker (configurable thresholds), rate limit enforcement (provider-specific limits from registry), request queue for burst handling, unified error mapping to Witylogix error catalog</t>
+        </is>
+      </c>
+      <c r="E5" s="416" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="416" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="B6" s="416" t="inlineStr">
+        <is>
+          <t>Full-stack</t>
+        </is>
+      </c>
+      <c r="C6" s="416" t="inlineStr">
+        <is>
+          <t>Stripe &amp; PayPal SDK Integration</t>
+        </is>
+      </c>
+      <c r="D6" s="416" t="inlineStr">
+        <is>
+          <t>Stripe Node.js SDK migration (payment intents, subscriptions, invoices, webhook verification with stripe.webhooks.constructEvent), PayPal OAuth2 flow + order capture, payment event normalization, refund/dispute handling, integration tests with mock servers</t>
+        </is>
+      </c>
+      <c r="E6" s="416" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="416" t="inlineStr">
+        <is>
+          <t>VS</t>
+        </is>
+      </c>
+      <c r="B7" s="416" t="inlineStr">
+        <is>
+          <t>Component Dev</t>
+        </is>
+      </c>
+      <c r="C7" s="416" t="inlineStr">
+        <is>
+          <t>Integration UI Components</t>
+        </is>
+      </c>
+      <c r="D7" s="416" t="inlineStr">
+        <is>
+          <t>IntegrationCard (logo, status badge, actions), OAuthRedirectHandler (callback URL, token exchange), ConnectionStatusBadge (connected/disconnected/error/syncing), CredentialForm (dynamic fields from registry schema), IntegrationLogo (auto-fetch from provider), WebhookEventViewer (payload inspector)</t>
+        </is>
+      </c>
+      <c r="E7" s="416" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="416" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="B8" s="416" t="inlineStr">
+        <is>
+          <t>Sr. Backend</t>
+        </is>
+      </c>
+      <c r="C8" s="416" t="inlineStr">
+        <is>
+          <t>Shopify &amp; WooCommerce SDK Integration</t>
+        </is>
+      </c>
+      <c r="D8" s="416" t="inlineStr">
+        <is>
+          <t>Shopify Admin API v2024-01 SDK (@shopify/shopify-api) — orders, products, inventory, fulfillment, webhooks (HMAC verification), WooCommerce REST API SDK — order sync, product sync, webhook consumer, inventory reconciliation, integration tests</t>
+        </is>
+      </c>
+      <c r="E8" s="416" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="416" t="inlineStr">
+        <is>
+          <t>KS</t>
+        </is>
+      </c>
+      <c r="B9" s="416" t="inlineStr">
+        <is>
+          <t>QA Lead</t>
+        </is>
+      </c>
+      <c r="C9" s="416" t="inlineStr">
+        <is>
+          <t>Integration Test Harness</t>
+        </is>
+      </c>
+      <c r="D9" s="416" t="inlineStr">
+        <is>
+          <t>Mock server framework (MSW-based) for each auth type (API Key, OAuth2, Basic, Bearer, JWT, HMAC), test fixtures for all 21 categories, integration test runner with provider isolation, webhook delivery simulator, credential rotation test scenarios, CI pipeline integration</t>
+        </is>
+      </c>
+      <c r="E9" s="416" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="416" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="B10" s="416" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="C10" s="416" t="inlineStr">
+        <is>
+          <t>SendGrid &amp; Twilio SDK Integration</t>
+        </is>
+      </c>
+      <c r="D10" s="416" t="inlineStr">
+        <is>
+          <t>SendGrid v3 SDK (@sendgrid/mail) — transactional email, templates, dynamic data, event webhooks, Twilio SDK — SMS/MMS send, delivery status callbacks, verify API, WhatsApp Business message templates, delivery receipt normalization, integration tests</t>
+        </is>
+      </c>
+      <c r="E10" s="416" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="416" t="inlineStr">
+        <is>
+          <t>ZR</t>
+        </is>
+      </c>
+      <c r="B11" s="416" t="inlineStr">
+        <is>
+          <t>AI Engineer</t>
+        </is>
+      </c>
+      <c r="C11" s="416" t="inlineStr">
+        <is>
+          <t>Smart Integration Recommender</t>
+        </is>
+      </c>
+      <c r="D11" s="416" t="inlineStr">
+        <is>
+          <t>Industry-based integration recommendations (restaurant→Toast+DoorDash, ecommerce→Shopify+Stripe+ShipStation), workflow-aware suggestions (if routing enabled, suggest telematics), integration dependency graph, setup wizard AI assistant, recommendation API endpoint, A/B test framework for recommendations</t>
+        </is>
+      </c>
+      <c r="E11" s="416" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore(sprint-8.1): plan routing, maps & real-time tracking sprint
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/witylogix-sprint-tracker.xlsx
+++ b/witylogix-sprint-tracker.xlsx
@@ -42,6 +42,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 7.1 Done" sheetId="33" state="visible" r:id="rId33"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.x Integration Roadmap" sheetId="34" state="visible" r:id="rId34"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.0 Done" sheetId="35" state="visible" r:id="rId35"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.1 Plan" sheetId="36" state="visible" r:id="rId36"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Data Models Gap'!$A$1:$K$40</definedName>
@@ -8043,10 +8044,10 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A12:F12"/>
     <mergeCell ref="A5:G5"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A12:F12"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -17330,6 +17331,284 @@
           <t>Done</t>
         </is>
       </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" style="186" min="1" max="1"/>
+    <col width="18" customWidth="1" style="186" min="2" max="2"/>
+    <col width="35" customWidth="1" style="186" min="3" max="3"/>
+    <col width="90" customWidth="1" style="186" min="4" max="4"/>
+    <col width="10" customWidth="1" style="186" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="415" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="B1" s="415" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="C1" s="415" t="inlineStr">
+        <is>
+          <t>Sprint 8.1 Task</t>
+        </is>
+      </c>
+      <c r="D1" s="415" t="inlineStr">
+        <is>
+          <t>Deliverables</t>
+        </is>
+      </c>
+      <c r="E1" s="415" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="416" t="inlineStr">
+        <is>
+          <t>AR</t>
+        </is>
+      </c>
+      <c r="B2" s="416" t="inlineStr">
+        <is>
+          <t>CTO/Architect</t>
+        </is>
+      </c>
+      <c r="C2" s="416" t="inlineStr">
+        <is>
+          <t>Multi-Provider Routing Failover Engine</t>
+        </is>
+      </c>
+      <c r="D2" s="416" t="inlineStr">
+        <is>
+          <t>Routing orchestrator with provider failover chain (primary→secondary→tertiary), health-weighted provider selection, latency tracking per provider, route caching (Redis, 5-min TTL), benchmark suite comparing all 8 routing providers on sample routes, failover metrics dashboard data</t>
+        </is>
+      </c>
+      <c r="E2" s="416" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="416" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="B3" s="416" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C3" s="416" t="inlineStr">
+        <is>
+          <t>Live Delivery Map (Mapbox GL JS)</t>
+        </is>
+      </c>
+      <c r="D3" s="416" t="inlineStr">
+        <is>
+          <t>Full-screen delivery map page with Mapbox GL JS dark tiles, live driver pin markers (color-coded by status: available/en-route/delivering/offline), animated route polylines, delivery point markers with status, driver popover (name, current delivery, ETA, speed), auto-center on active area, cluster markers for zoom levels</t>
+        </is>
+      </c>
+      <c r="E3" s="416" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="416" t="inlineStr">
+        <is>
+          <t>NK</t>
+        </is>
+      </c>
+      <c r="B4" s="416" t="inlineStr">
+        <is>
+          <t>Frontend Lead</t>
+        </is>
+      </c>
+      <c r="C4" s="416" t="inlineStr">
+        <is>
+          <t>Route Planning Wizard</t>
+        </is>
+      </c>
+      <c r="D4" s="416" t="inlineStr">
+        <is>
+          <t>Multi-stop route planner UI: add stops (address autocomplete via geocoding), drag-to-reorder, time window constraints per stop, vehicle selection (capacity, type), optimize button (calls routing API), route summary (distance, duration, fuel estimate), export route to driver app, save as template</t>
+        </is>
+      </c>
+      <c r="E4" s="416" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="416" t="inlineStr">
+        <is>
+          <t>RG</t>
+        </is>
+      </c>
+      <c r="B5" s="416" t="inlineStr">
+        <is>
+          <t>Backend Lead</t>
+        </is>
+      </c>
+      <c r="C5" s="416" t="inlineStr">
+        <is>
+          <t>Google Routes &amp; Mapbox SDKs</t>
+        </is>
+      </c>
+      <c r="D5" s="416" t="inlineStr">
+        <is>
+          <t>Google Routes API compute-routes + route-matrix integration (traffic-aware ETAs, polyline decoding), Mapbox Directions API integration (turn-by-turn, optimization), unified RoutingResult type, provider-specific rate limit compliance, geocoding service (forward + reverse) with provider fallback</t>
+        </is>
+      </c>
+      <c r="E5" s="416" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="416" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="B6" s="416" t="inlineStr">
+        <is>
+          <t>Full-stack</t>
+        </is>
+      </c>
+      <c r="C6" s="416" t="inlineStr">
+        <is>
+          <t>Samsara Telematics SDK + Live Tracking</t>
+        </is>
+      </c>
+      <c r="D6" s="416" t="inlineStr">
+        <is>
+          <t>Samsara REST API v1 SDK (vehicles, drivers, locations, stats), real-time vehicle feed endpoint (SSE or WebSocket), location history with trail on map, vehicle diagnostics (fuel, odometer, engine hours), driver safety scores, webhook handler for Samsara events, telematics data normalization to unified VehiclePosition type</t>
+        </is>
+      </c>
+      <c r="E6" s="416" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="416" t="inlineStr">
+        <is>
+          <t>VS</t>
+        </is>
+      </c>
+      <c r="B7" s="416" t="inlineStr">
+        <is>
+          <t>Component Dev</t>
+        </is>
+      </c>
+      <c r="C7" s="416" t="inlineStr">
+        <is>
+          <t>Map Controls &amp; Route Components</t>
+        </is>
+      </c>
+      <c r="D7" s="416" t="inlineStr">
+        <is>
+          <t>Map layer controls (traffic, satellite, terrain toggle), zoom controls, fullscreen toggle, route timeline component (stop list with ETAs + status), driver info card, delivery status pill, ETA countdown, distance badge, map legend component, responsive map sidebar</t>
+        </is>
+      </c>
+      <c r="E7" s="416" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="416" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="B8" s="416" t="inlineStr">
+        <is>
+          <t>Sr. Backend</t>
+        </is>
+      </c>
+      <c r="C8" s="416" t="inlineStr">
+        <is>
+          <t>Geotab SDK + Telematics Pipeline</t>
+        </is>
+      </c>
+      <c r="D8" s="416" t="inlineStr">
+        <is>
+          <t>Geotab MyGeotab API SDK (authenticate, Get/Set methods for Device, StatusData, LogRecord, Trip, FaultData), telematics polling service (configurable interval), data normalization pipeline (Geotab→WitylogixVehiclePosition), historical trip replay, geofence management, device diagnostics</t>
+        </is>
+      </c>
+      <c r="E8" s="416" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="416" t="inlineStr">
+        <is>
+          <t>KS</t>
+        </is>
+      </c>
+      <c r="B9" s="416" t="inlineStr">
+        <is>
+          <t>QA Lead</t>
+        </is>
+      </c>
+      <c r="C9" s="416" t="inlineStr">
+        <is>
+          <t>Routing &amp; Map Tests</t>
+        </is>
+      </c>
+      <c r="D9" s="416" t="inlineStr">
+        <is>
+          <t>Routing accuracy tests (compare Google vs Mapbox vs OSRM for same routes, measure distance/duration variance), geocoding accuracy validation (known addresses → expected coordinates), map rendering E2E (Playwright — page loads, markers appear, route draws), telematics data integrity tests, failover behavior tests</t>
+        </is>
+      </c>
+      <c r="E9" s="416" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="416" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="B10" s="416" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="C10" s="416" t="inlineStr">
+        <is>
+          <t>HERE Maps + TomTom Integration</t>
+        </is>
+      </c>
+      <c r="D10" s="416" t="inlineStr">
+        <is>
+          <t>HERE Geocoding &amp; Search v7 integration (autosuggest, geocode, reverse-geocode), HERE Routing v8 (truck routing, EV routing, matrix), TomTom Search API (fuzzy search, POI, geocode), TomTom Routing (calculate route, traffic flow), integration tests with mock servers, provider comparison benchmarks</t>
+        </is>
+      </c>
+      <c r="E10" s="416" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="416" t="inlineStr">
+        <is>
+          <t>ZR</t>
+        </is>
+      </c>
+      <c r="B11" s="416" t="inlineStr">
+        <is>
+          <t>AI Engineer</t>
+        </is>
+      </c>
+      <c r="C11" s="416" t="inlineStr">
+        <is>
+          <t>AI Route Optimization</t>
+        </is>
+      </c>
+      <c r="D11" s="416" t="inlineStr">
+        <is>
+          <t>Historical delivery data analyzer (cluster delivery zones, peak hour patterns), ML-based ETA predictor (distance + traffic + time-of-day + weather features), route sequence optimizer (nearest-neighbor + 2-opt improvement), smart driver assignment (match driver proximity + capacity + shift hours), delivery zone heat map generator, optimization API endpoints</t>
+        </is>
+      </c>
+      <c r="E11" s="416" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(sprint-8.1): routing, maps & real-time tracking
Multi-provider routing orchestrator with failover (Google, Mapbox, HERE,
TomTom), live Mapbox GL JS delivery map with driver markers and route
polylines, 5-step route planning wizard, Samsara + Geotab telematics
integration with unified normalizer, AI route optimization (nearest-
neighbor + 2-opt/3-opt, ETA predictor, zone analyzer, smart driver
assignment), geofence manager, trip replay, 17 test files.

69 new/modified files, ~14,000 lines across 10 agents.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/witylogix-sprint-tracker.xlsx
+++ b/witylogix-sprint-tracker.xlsx
@@ -42,7 +42,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 7.1 Done" sheetId="33" state="visible" r:id="rId33"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.x Integration Roadmap" sheetId="34" state="visible" r:id="rId34"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.0 Done" sheetId="35" state="visible" r:id="rId35"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.1 Plan" sheetId="36" state="visible" r:id="rId36"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.1 Done" sheetId="36" state="visible" r:id="rId36"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Data Models Gap'!$A$1:$K$40</definedName>
@@ -8044,9 +8044,9 @@
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A12:F12"/>
+    <mergeCell ref="A1:G1"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>

</xml_diff>

<commit_message>
chore(sprint-8.2): plan shipping & last-mile carriers sprint
Sprint 8.2 — Shipping & Last-Mile: EasyPost, ShipStation, Shippo,
AfterShip, DHL Express SDKs, DoorDash Drive + Uber Direct last-mile,
carrier rate engine, shipping label wizard, shipment tracking,
delivery time prediction AI.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/witylogix-sprint-tracker.xlsx
+++ b/witylogix-sprint-tracker.xlsx
@@ -43,6 +43,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.x Integration Roadmap" sheetId="34" state="visible" r:id="rId34"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.0 Done" sheetId="35" state="visible" r:id="rId35"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.1 Done" sheetId="36" state="visible" r:id="rId36"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.2 Plan" sheetId="37" state="visible" r:id="rId37"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Data Models Gap'!$A$1:$K$40</definedName>
@@ -662,7 +663,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="58">
+  <fills count="59">
     <fill>
       <patternFill/>
     </fill>
@@ -996,6 +997,11 @@
         <bgColor rgb="0087CEEB"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="6">
     <border>
@@ -1067,7 +1073,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="422">
+  <cellXfs count="424">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -2292,6 +2298,10 @@
     <xf numFmtId="0" fontId="0" fillId="56" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="57" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="74" fillId="52" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="71" fillId="41" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="58" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -8044,10 +8054,10 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="A5:G5"/>
     <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:G1"/>
     <mergeCell ref="A12:F12"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A5:G5"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -17609,6 +17619,284 @@
         </is>
       </c>
       <c r="E11" s="416" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" style="186" min="1" max="1"/>
+    <col width="16" customWidth="1" style="186" min="2" max="2"/>
+    <col width="80" customWidth="1" style="186" min="3" max="3"/>
+    <col width="40" customWidth="1" style="186" min="4" max="4"/>
+    <col width="12" customWidth="1" style="186" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="422" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="B1" s="422" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="C1" s="422" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="D1" s="422" t="inlineStr">
+        <is>
+          <t>Files</t>
+        </is>
+      </c>
+      <c r="E1" s="422" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="416" t="inlineStr">
+        <is>
+          <t>AR</t>
+        </is>
+      </c>
+      <c r="B2" s="416" t="inlineStr">
+        <is>
+          <t>CTO/Architect</t>
+        </is>
+      </c>
+      <c r="C2" s="416" t="inlineStr">
+        <is>
+          <t>Carrier rate engine — parallel rate fetch from EasyPost/Shippo/ShipStation, cheapest/fastest/best-value ranking, carrier credential management</t>
+        </is>
+      </c>
+      <c r="D2" s="416" t="inlineStr"/>
+      <c r="E2" s="423" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="416" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="B3" s="416" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C3" s="416" t="inlineStr">
+        <is>
+          <t>Shipping label wizard — carrier selection, package dimensions input, rate comparison table, label preview/download</t>
+        </is>
+      </c>
+      <c r="D3" s="416" t="inlineStr"/>
+      <c r="E3" s="423" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="416" t="inlineStr">
+        <is>
+          <t>NK</t>
+        </is>
+      </c>
+      <c r="B4" s="416" t="inlineStr">
+        <is>
+          <t>Frontend Lead</t>
+        </is>
+      </c>
+      <c r="C4" s="416" t="inlineStr">
+        <is>
+          <t>Shipment tracking page — multi-carrier unified timeline, status mapping, delivery proof viewer, customer tracking embed</t>
+        </is>
+      </c>
+      <c r="D4" s="416" t="inlineStr"/>
+      <c r="E4" s="423" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="416" t="inlineStr">
+        <is>
+          <t>RG</t>
+        </is>
+      </c>
+      <c r="B5" s="416" t="inlineStr">
+        <is>
+          <t>Backend Lead</t>
+        </is>
+      </c>
+      <c r="C5" s="416" t="inlineStr">
+        <is>
+          <t>EasyPost SDK client — shipping rates, labels, tracking, insurance, batch shipments, webhook verification, scan forms</t>
+        </is>
+      </c>
+      <c r="D5" s="416" t="inlineStr"/>
+      <c r="E5" s="423" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="416" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="B6" s="416" t="inlineStr">
+        <is>
+          <t>Full-stack</t>
+        </is>
+      </c>
+      <c r="C6" s="416" t="inlineStr">
+        <is>
+          <t>ShipStation SDK client — orders, shipments, carriers, rates, labels, stores, webhooks, batch label creation</t>
+        </is>
+      </c>
+      <c r="D6" s="416" t="inlineStr"/>
+      <c r="E6" s="423" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="416" t="inlineStr">
+        <is>
+          <t>VS</t>
+        </is>
+      </c>
+      <c r="B7" s="416" t="inlineStr">
+        <is>
+          <t>Component Dev</t>
+        </is>
+      </c>
+      <c r="C7" s="416" t="inlineStr">
+        <is>
+          <t>Shipping UI components — rate comparison card, tracking timeline, label preview, package size selector, carrier logo grid, status stepper</t>
+        </is>
+      </c>
+      <c r="D7" s="416" t="inlineStr"/>
+      <c r="E7" s="423" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="416" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="B8" s="416" t="inlineStr">
+        <is>
+          <t>Sr. Backend</t>
+        </is>
+      </c>
+      <c r="C8" s="416" t="inlineStr">
+        <is>
+          <t>DoorDash Drive JWT + Uber Direct OAuth2 — last-mile delivery API clients, delivery creation, tracking, webhooks, POD retrieval</t>
+        </is>
+      </c>
+      <c r="D8" s="416" t="inlineStr"/>
+      <c r="E8" s="423" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="416" t="inlineStr">
+        <is>
+          <t>KS</t>
+        </is>
+      </c>
+      <c r="B9" s="416" t="inlineStr">
+        <is>
+          <t>QA Lead</t>
+        </is>
+      </c>
+      <c r="C9" s="416" t="inlineStr">
+        <is>
+          <t>Shipping rate accuracy tests, label generation E2E, tracking webhook reliability tests, carrier failover tests</t>
+        </is>
+      </c>
+      <c r="D9" s="416" t="inlineStr"/>
+      <c r="E9" s="423" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="416" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="B10" s="416" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="C10" s="416" t="inlineStr">
+        <is>
+          <t>Shippo SDK + AfterShip tracking SDK + DHL Express SDK — rate shopping, universal tracking, express shipping</t>
+        </is>
+      </c>
+      <c r="D10" s="416" t="inlineStr"/>
+      <c r="E10" s="423" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="416" t="inlineStr">
+        <is>
+          <t>ZR</t>
+        </is>
+      </c>
+      <c r="B11" s="416" t="inlineStr">
+        <is>
+          <t>AI Engineer</t>
+        </is>
+      </c>
+      <c r="C11" s="416" t="inlineStr">
+        <is>
+          <t>Delivery time prediction model — carrier performance + distance + weather + day-of-week factors, smart carrier recommendation</t>
+        </is>
+      </c>
+      <c r="D11" s="416" t="inlineStr"/>
+      <c r="E11" s="423" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(sprint-8.2): shipping & last-mile carriers
Carrier rate engine with parallel fetching and multi-strategy ranking,
EasyPost/ShipStation/Shippo/AfterShip/DHL Express shipping SDKs,
DoorDash Drive + Uber Direct last-mile delivery SDKs, shipping label
wizard (4-step UI), shipment tracking dashboard with timeline + embed
widget, shipping UI components, AI delivery time predictor with
confidence intervals, smart carrier selector with multi-criteria
scoring, shipping analytics with anomaly detection and forecasting.

50+ new files, ~20,000 lines across 10 agents.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/witylogix-sprint-tracker.xlsx
+++ b/witylogix-sprint-tracker.xlsx
@@ -43,7 +43,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.x Integration Roadmap" sheetId="34" state="visible" r:id="rId34"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.0 Done" sheetId="35" state="visible" r:id="rId35"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.1 Done" sheetId="36" state="visible" r:id="rId36"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.2 Plan" sheetId="37" state="visible" r:id="rId37"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.2 Done" sheetId="37" state="visible" r:id="rId37"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Data Models Gap'!$A$1:$K$40</definedName>
@@ -61,7 +61,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="88">
+  <fonts count="89">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -662,8 +662,11 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
+    <font>
+      <color rgb="00006100"/>
+    </font>
   </fonts>
-  <fills count="59">
+  <fills count="60">
     <fill>
       <patternFill/>
     </fill>
@@ -1002,6 +1005,11 @@
         <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="6">
     <border>
@@ -1073,7 +1081,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="424">
+  <cellXfs count="425">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -2302,6 +2310,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="58" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="88" fillId="59" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -8054,10 +8063,10 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A12:F12"/>
     <mergeCell ref="A5:G5"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A12:F12"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -17685,9 +17694,9 @@
         </is>
       </c>
       <c r="D2" s="416" t="inlineStr"/>
-      <c r="E2" s="423" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="E2" s="424" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -17708,9 +17717,9 @@
         </is>
       </c>
       <c r="D3" s="416" t="inlineStr"/>
-      <c r="E3" s="423" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="E3" s="424" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -17731,9 +17740,9 @@
         </is>
       </c>
       <c r="D4" s="416" t="inlineStr"/>
-      <c r="E4" s="423" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="E4" s="424" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -17754,9 +17763,9 @@
         </is>
       </c>
       <c r="D5" s="416" t="inlineStr"/>
-      <c r="E5" s="423" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="E5" s="424" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -17777,9 +17786,9 @@
         </is>
       </c>
       <c r="D6" s="416" t="inlineStr"/>
-      <c r="E6" s="423" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="E6" s="424" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -17800,9 +17809,9 @@
         </is>
       </c>
       <c r="D7" s="416" t="inlineStr"/>
-      <c r="E7" s="423" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="E7" s="424" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -17823,9 +17832,9 @@
         </is>
       </c>
       <c r="D8" s="416" t="inlineStr"/>
-      <c r="E8" s="423" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="E8" s="424" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -17846,9 +17855,9 @@
         </is>
       </c>
       <c r="D9" s="416" t="inlineStr"/>
-      <c r="E9" s="423" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="E9" s="424" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -17869,9 +17878,9 @@
         </is>
       </c>
       <c r="D10" s="416" t="inlineStr"/>
-      <c r="E10" s="423" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="E10" s="424" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -17892,9 +17901,9 @@
         </is>
       </c>
       <c r="D11" s="416" t="inlineStr"/>
-      <c r="E11" s="423" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="E11" s="424" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(sprint-8.3): plan e-commerce & order sync sprint
Sprint 8.3 — E-Commerce & Order Sync: BigCommerce, Magento 2, Etsy,
eBay, Square Online SDKs, order sync engine v2 with conflict resolution,
cross-platform inventory sync, product catalog mapping UI, intelligent
order routing AI.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/witylogix-sprint-tracker.xlsx
+++ b/witylogix-sprint-tracker.xlsx
@@ -44,6 +44,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.0 Done" sheetId="35" state="visible" r:id="rId35"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.1 Done" sheetId="36" state="visible" r:id="rId36"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.2 Done" sheetId="37" state="visible" r:id="rId37"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.3 Plan" sheetId="38" state="visible" r:id="rId38"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Data Models Gap'!$A$1:$K$40</definedName>
@@ -8063,9 +8064,9 @@
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A12:F12"/>
+    <mergeCell ref="A1:G1"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -17904,6 +17905,284 @@
       <c r="E11" s="424" t="inlineStr">
         <is>
           <t>Done</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" style="186" min="1" max="1"/>
+    <col width="16" customWidth="1" style="186" min="2" max="2"/>
+    <col width="80" customWidth="1" style="186" min="3" max="3"/>
+    <col width="40" customWidth="1" style="186" min="4" max="4"/>
+    <col width="12" customWidth="1" style="186" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="422" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="B1" s="422" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="C1" s="422" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="D1" s="422" t="inlineStr">
+        <is>
+          <t>Files</t>
+        </is>
+      </c>
+      <c r="E1" s="422" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="416" t="inlineStr">
+        <is>
+          <t>AR</t>
+        </is>
+      </c>
+      <c r="B2" s="416" t="inlineStr">
+        <is>
+          <t>CTO/Architect</t>
+        </is>
+      </c>
+      <c r="C2" s="416" t="inlineStr">
+        <is>
+          <t>Order sync engine v2 — conflict resolution strategies (LWW/external-wins/manual), idempotent sync with dedup, retry queue with DLQ, delta sync, batch import/export, sync metrics dashboard API</t>
+        </is>
+      </c>
+      <c r="D2" s="416" t="inlineStr"/>
+      <c r="E2" s="423" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="416" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="B3" s="416" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C3" s="416" t="inlineStr">
+        <is>
+          <t>Order import dashboard — platform selector, sync status timeline, error log with retry, bulk import wizard, sync health indicators</t>
+        </is>
+      </c>
+      <c r="D3" s="416" t="inlineStr"/>
+      <c r="E3" s="423" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="416" t="inlineStr">
+        <is>
+          <t>NK</t>
+        </is>
+      </c>
+      <c r="B4" s="416" t="inlineStr">
+        <is>
+          <t>Frontend Lead</t>
+        </is>
+      </c>
+      <c r="C4" s="416" t="inlineStr">
+        <is>
+          <t>Product catalog sync UI — field mapping editor (drag-drop), field transformers (type conversion, default values), mapping preview, sync schedule config</t>
+        </is>
+      </c>
+      <c r="D4" s="416" t="inlineStr"/>
+      <c r="E4" s="423" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="416" t="inlineStr">
+        <is>
+          <t>RG</t>
+        </is>
+      </c>
+      <c r="B5" s="416" t="inlineStr">
+        <is>
+          <t>Backend Lead</t>
+        </is>
+      </c>
+      <c r="C5" s="416" t="inlineStr">
+        <is>
+          <t>BigCommerce SDK client — OAuth2 single-click install, orders/products/customers/webhooks, V3 REST API, cursor pagination, rate limiting</t>
+        </is>
+      </c>
+      <c r="D5" s="416" t="inlineStr"/>
+      <c r="E5" s="423" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="416" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="B6" s="416" t="inlineStr">
+        <is>
+          <t>Full-stack</t>
+        </is>
+      </c>
+      <c r="C6" s="416" t="inlineStr">
+        <is>
+          <t>Magento 2 REST SDK — OAuth1/bearer auth, orders/products/inventory/customers CRUD, configurable products, media gallery, async bulk API</t>
+        </is>
+      </c>
+      <c r="D6" s="416" t="inlineStr"/>
+      <c r="E6" s="423" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="416" t="inlineStr">
+        <is>
+          <t>VS</t>
+        </is>
+      </c>
+      <c r="B7" s="416" t="inlineStr">
+        <is>
+          <t>Component Dev</t>
+        </is>
+      </c>
+      <c r="C7" s="416" t="inlineStr">
+        <is>
+          <t>E-commerce UI components — unified order card, platform connection badge, sync progress bar, field mapper, inventory level indicator, platform logo</t>
+        </is>
+      </c>
+      <c r="D7" s="416" t="inlineStr"/>
+      <c r="E7" s="423" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="416" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="B8" s="416" t="inlineStr">
+        <is>
+          <t>Sr. Backend</t>
+        </is>
+      </c>
+      <c r="C8" s="416" t="inlineStr">
+        <is>
+          <t>Etsy v3 OAuth2 SDK — listings/receipts/shops/shipping-profiles, eBay OAuth2 SDK — orders/inventory/trading API, Square Online SDK</t>
+        </is>
+      </c>
+      <c r="D8" s="416" t="inlineStr"/>
+      <c r="E8" s="423" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="416" t="inlineStr">
+        <is>
+          <t>KS</t>
+        </is>
+      </c>
+      <c r="B9" s="416" t="inlineStr">
+        <is>
+          <t>QA Lead</t>
+        </is>
+      </c>
+      <c r="C9" s="416" t="inlineStr">
+        <is>
+          <t>Order sync idempotency tests, webhook delivery reliability tests, conflict resolution tests, inventory reconciliation tests, E2E platform connect flow</t>
+        </is>
+      </c>
+      <c r="D9" s="416" t="inlineStr"/>
+      <c r="E9" s="423" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="416" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="B10" s="416" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="C10" s="416" t="inlineStr">
+        <is>
+          <t>Cross-platform inventory sync engine — stock level reconciliation, low-stock alerts, multi-warehouse support, inventory reservation, sync conflict resolution</t>
+        </is>
+      </c>
+      <c r="D10" s="416" t="inlineStr"/>
+      <c r="E10" s="423" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="416" t="inlineStr">
+        <is>
+          <t>ZR</t>
+        </is>
+      </c>
+      <c r="B11" s="416" t="inlineStr">
+        <is>
+          <t>AI Engineer</t>
+        </is>
+      </c>
+      <c r="C11" s="416" t="inlineStr">
+        <is>
+          <t>Intelligent order routing — auto-assign fulfillment center based on proximity + stock + capacity, demand forecasting per SKU, smart reorder suggestions</t>
+        </is>
+      </c>
+      <c r="D11" s="416" t="inlineStr"/>
+      <c r="E11" s="423" t="inlineStr">
+        <is>
+          <t>Planned</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(sprint-8.3): e-commerce & order sync
Order sync engine v2 with 4 conflict resolution strategies, idempotency,
delta sync, retry queue with DLQ, and batch processing. BigCommerce (48
methods), Magento 2 (42 methods), Etsy v3, eBay, Square Online SDK
clients. Order import dashboard with 8-platform selector, conflict
resolution UI, product catalog sync with visual field mapping editor.
Cross-platform inventory sync engine with stock reconciliation, multi-
warehouse, reservation TTL, oversell protection. AI intelligent order
router with fulfillment scoring and demand forecaster with seasonal
decomposition.

55+ new files, ~25,000 lines across 10 agents.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/witylogix-sprint-tracker.xlsx
+++ b/witylogix-sprint-tracker.xlsx
@@ -44,7 +44,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.0 Done" sheetId="35" state="visible" r:id="rId35"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.1 Done" sheetId="36" state="visible" r:id="rId36"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.2 Done" sheetId="37" state="visible" r:id="rId37"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.3 Plan" sheetId="38" state="visible" r:id="rId38"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.3 Done" sheetId="38" state="visible" r:id="rId38"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Data Models Gap'!$A$1:$K$40</definedName>
@@ -8064,10 +8064,10 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="A5:G5"/>
     <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:G1"/>
     <mergeCell ref="A12:F12"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A5:G5"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -17973,9 +17973,9 @@
         </is>
       </c>
       <c r="D2" s="416" t="inlineStr"/>
-      <c r="E2" s="423" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="E2" s="424" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -17996,9 +17996,9 @@
         </is>
       </c>
       <c r="D3" s="416" t="inlineStr"/>
-      <c r="E3" s="423" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="E3" s="424" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -18019,9 +18019,9 @@
         </is>
       </c>
       <c r="D4" s="416" t="inlineStr"/>
-      <c r="E4" s="423" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="E4" s="424" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -18042,9 +18042,9 @@
         </is>
       </c>
       <c r="D5" s="416" t="inlineStr"/>
-      <c r="E5" s="423" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="E5" s="424" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -18065,9 +18065,9 @@
         </is>
       </c>
       <c r="D6" s="416" t="inlineStr"/>
-      <c r="E6" s="423" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="E6" s="424" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -18088,9 +18088,9 @@
         </is>
       </c>
       <c r="D7" s="416" t="inlineStr"/>
-      <c r="E7" s="423" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="E7" s="424" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -18111,9 +18111,9 @@
         </is>
       </c>
       <c r="D8" s="416" t="inlineStr"/>
-      <c r="E8" s="423" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="E8" s="424" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -18134,9 +18134,9 @@
         </is>
       </c>
       <c r="D9" s="416" t="inlineStr"/>
-      <c r="E9" s="423" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="E9" s="424" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -18157,9 +18157,9 @@
         </is>
       </c>
       <c r="D10" s="416" t="inlineStr"/>
-      <c r="E10" s="423" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="E10" s="424" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -18180,9 +18180,9 @@
         </is>
       </c>
       <c r="D11" s="416" t="inlineStr"/>
-      <c r="E11" s="423" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="E11" s="424" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(sprint-8.4): plan CRM, ERP & accounting sprint
Sprint 8.4 — CRM, ERP & Accounting: Salesforce, HubSpot, QuickBooks,
Xero, SAP, NetSuite, Zoho CRM, Pipedrive, Dynamics 365 SDKs, CRM sync
engine v3, financial sync dashboard, CLV predictor. Each agent assigned
ECC skills (backend-patterns, api-design, security-review, frontend-
patterns, e2e-testing, tdd-workflow).

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/witylogix-sprint-tracker.xlsx
+++ b/witylogix-sprint-tracker.xlsx
@@ -45,6 +45,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.1 Done" sheetId="36" state="visible" r:id="rId36"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.2 Done" sheetId="37" state="visible" r:id="rId37"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.3 Done" sheetId="38" state="visible" r:id="rId38"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.4 Plan" sheetId="39" state="visible" r:id="rId39"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Data Models Gap'!$A$1:$K$40</definedName>
@@ -8064,10 +8065,10 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A12:F12"/>
     <mergeCell ref="A5:G5"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A12:F12"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -18183,6 +18184,324 @@
       <c r="E11" s="424" t="inlineStr">
         <is>
           <t>Done</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" style="186" min="1" max="1"/>
+    <col width="16" customWidth="1" style="186" min="2" max="2"/>
+    <col width="32" customWidth="1" style="186" min="3" max="3"/>
+    <col width="80" customWidth="1" style="186" min="4" max="4"/>
+    <col width="12" customWidth="1" style="186" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="422" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="B1" s="422" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="C1" s="422" t="inlineStr">
+        <is>
+          <t>Skill Applied</t>
+        </is>
+      </c>
+      <c r="D1" s="422" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="E1" s="422" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="416" t="inlineStr">
+        <is>
+          <t>AR</t>
+        </is>
+      </c>
+      <c r="B2" s="416" t="inlineStr">
+        <is>
+          <t>CTO/Architect</t>
+        </is>
+      </c>
+      <c r="C2" s="416" t="inlineStr">
+        <is>
+          <t>backend-patterns + api-design</t>
+        </is>
+      </c>
+      <c r="D2" s="416" t="inlineStr">
+        <is>
+          <t>CRM sync engine v3 — field mapping DSL, bi-directional conflict resolution, repository pattern, service layer with DI</t>
+        </is>
+      </c>
+      <c r="E2" s="423" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="416" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="B3" s="416" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C3" s="416" t="inlineStr">
+        <is>
+          <t>frontend-patterns</t>
+        </is>
+      </c>
+      <c r="D3" s="416" t="inlineStr">
+        <is>
+          <t>CRM connection wizard — Salesforce + HubSpot OAuth2 flows, compound components, render props, accessible keyboard nav</t>
+        </is>
+      </c>
+      <c r="E3" s="423" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="416" t="inlineStr">
+        <is>
+          <t>NK</t>
+        </is>
+      </c>
+      <c r="B4" s="416" t="inlineStr">
+        <is>
+          <t>Frontend Lead</t>
+        </is>
+      </c>
+      <c r="C4" s="416" t="inlineStr">
+        <is>
+          <t>frontend-patterns</t>
+        </is>
+      </c>
+      <c r="D4" s="416" t="inlineStr">
+        <is>
+          <t>Financial sync dashboard — invoice status, payment reconciliation, virtualized lists, code-split heavy charts</t>
+        </is>
+      </c>
+      <c r="E4" s="423" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="416" t="inlineStr">
+        <is>
+          <t>RG</t>
+        </is>
+      </c>
+      <c r="B5" s="416" t="inlineStr">
+        <is>
+          <t>Backend Lead</t>
+        </is>
+      </c>
+      <c r="C5" s="416" t="inlineStr">
+        <is>
+          <t>api-design + security-review</t>
+        </is>
+      </c>
+      <c r="D5" s="416" t="inlineStr">
+        <is>
+          <t>Salesforce jsforce SDK + HubSpot SDK — RESTful resource design, Zod validation, secrets management</t>
+        </is>
+      </c>
+      <c r="E5" s="423" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="416" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="B6" s="416" t="inlineStr">
+        <is>
+          <t>Full-stack</t>
+        </is>
+      </c>
+      <c r="C6" s="416" t="inlineStr">
+        <is>
+          <t>backend-patterns + security-review</t>
+        </is>
+      </c>
+      <c r="D6" s="416" t="inlineStr">
+        <is>
+          <t>QuickBooks OAuth2 + Xero OAuth2 — invoice/payment sync, credential vault, input validation, error mapping</t>
+        </is>
+      </c>
+      <c r="E6" s="423" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="416" t="inlineStr">
+        <is>
+          <t>VS</t>
+        </is>
+      </c>
+      <c r="B7" s="416" t="inlineStr">
+        <is>
+          <t>Component Dev</t>
+        </is>
+      </c>
+      <c r="C7" s="416" t="inlineStr">
+        <is>
+          <t>frontend-patterns</t>
+        </is>
+      </c>
+      <c r="D7" s="416" t="inlineStr">
+        <is>
+          <t>Contact card + invoice line-item editor — compound components, memoization, accessibility, Framer Motion</t>
+        </is>
+      </c>
+      <c r="E7" s="423" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="416" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="B8" s="416" t="inlineStr">
+        <is>
+          <t>Sr. Backend</t>
+        </is>
+      </c>
+      <c r="C8" s="416" t="inlineStr">
+        <is>
+          <t>api-design + backend-patterns</t>
+        </is>
+      </c>
+      <c r="D8" s="416" t="inlineStr">
+        <is>
+          <t>SAP OData + NetSuite TBA/REST — repository pattern, service layer, proper error handling, rate limiting</t>
+        </is>
+      </c>
+      <c r="E8" s="423" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="416" t="inlineStr">
+        <is>
+          <t>KS</t>
+        </is>
+      </c>
+      <c r="B9" s="416" t="inlineStr">
+        <is>
+          <t>QA Lead</t>
+        </is>
+      </c>
+      <c r="C9" s="416" t="inlineStr">
+        <is>
+          <t>e2e-testing + tdd-workflow</t>
+        </is>
+      </c>
+      <c r="D9" s="416" t="inlineStr">
+        <is>
+          <t>CRM data accuracy tests, accounting reconciliation tests, E2E OAuth flows, TDD methodology</t>
+        </is>
+      </c>
+      <c r="E9" s="423" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="416" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="B10" s="416" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="C10" s="416" t="inlineStr">
+        <is>
+          <t>api-design + security-review</t>
+        </is>
+      </c>
+      <c r="D10" s="416" t="inlineStr">
+        <is>
+          <t>Zoho CRM + Pipedrive + Dynamics 365 — proper auth, HMAC verification, Zod schemas, rate limit compliance</t>
+        </is>
+      </c>
+      <c r="E10" s="423" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="416" t="inlineStr">
+        <is>
+          <t>ZR</t>
+        </is>
+      </c>
+      <c r="B11" s="416" t="inlineStr">
+        <is>
+          <t>AI Engineer</t>
+        </is>
+      </c>
+      <c r="C11" s="416" t="inlineStr">
+        <is>
+          <t>backend-patterns</t>
+        </is>
+      </c>
+      <c r="D11" s="416" t="inlineStr">
+        <is>
+          <t>Customer lifetime value predictor — CRM + order data fusion, service layer pattern, async data fetching</t>
+        </is>
+      </c>
+      <c r="E11" s="423" t="inlineStr">
+        <is>
+          <t>Planned</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(sprint-8.4): CRM, ERP & accounting integrations
CRM sync engine v3 with field mapping DSL and 5 bi-directional conflict
resolution strategies. Salesforce (65+ methods), HubSpot (70+ methods),
Zoho CRM, Pipedrive, Dynamics 365 CRM SDKs. QuickBooks Online + Xero
accounting SDKs with normalizer. SAP S/4HANA OData + NetSuite TBA/REST
ERP SDKs with ERP normalizer. CRM connection wizard (5-step compound
components), financial dashboard with virtualized invoices and payment
reconciliation. AI customer LTV predictor (7 segments, cohort analysis,
churn prediction) and CRM intelligence (deal/lead scoring, activity
recommendations, sales forecasting).

60+ new files, ~28,000 lines across 10 agents. Skills applied: backend-
patterns, api-design, security-review, frontend-patterns, e2e-testing.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/witylogix-sprint-tracker.xlsx
+++ b/witylogix-sprint-tracker.xlsx
@@ -45,7 +45,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.1 Done" sheetId="36" state="visible" r:id="rId36"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.2 Done" sheetId="37" state="visible" r:id="rId37"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.3 Done" sheetId="38" state="visible" r:id="rId38"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.4 Plan" sheetId="39" state="visible" r:id="rId39"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.4 Done" sheetId="39" state="visible" r:id="rId39"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Data Models Gap'!$A$1:$K$40</definedName>
@@ -8065,9 +8065,9 @@
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A12:F12"/>
+    <mergeCell ref="A1:G1"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -18256,9 +18256,9 @@
           <t>CRM sync engine v3 — field mapping DSL, bi-directional conflict resolution, repository pattern, service layer with DI</t>
         </is>
       </c>
-      <c r="E2" s="423" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="E2" s="424" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -18283,9 +18283,9 @@
           <t>CRM connection wizard — Salesforce + HubSpot OAuth2 flows, compound components, render props, accessible keyboard nav</t>
         </is>
       </c>
-      <c r="E3" s="423" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="E3" s="424" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -18310,9 +18310,9 @@
           <t>Financial sync dashboard — invoice status, payment reconciliation, virtualized lists, code-split heavy charts</t>
         </is>
       </c>
-      <c r="E4" s="423" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="E4" s="424" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -18337,9 +18337,9 @@
           <t>Salesforce jsforce SDK + HubSpot SDK — RESTful resource design, Zod validation, secrets management</t>
         </is>
       </c>
-      <c r="E5" s="423" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="E5" s="424" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -18364,9 +18364,9 @@
           <t>QuickBooks OAuth2 + Xero OAuth2 — invoice/payment sync, credential vault, input validation, error mapping</t>
         </is>
       </c>
-      <c r="E6" s="423" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="E6" s="424" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -18391,9 +18391,9 @@
           <t>Contact card + invoice line-item editor — compound components, memoization, accessibility, Framer Motion</t>
         </is>
       </c>
-      <c r="E7" s="423" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="E7" s="424" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -18418,9 +18418,9 @@
           <t>SAP OData + NetSuite TBA/REST — repository pattern, service layer, proper error handling, rate limiting</t>
         </is>
       </c>
-      <c r="E8" s="423" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="E8" s="424" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -18445,9 +18445,9 @@
           <t>CRM data accuracy tests, accounting reconciliation tests, E2E OAuth flows, TDD methodology</t>
         </is>
       </c>
-      <c r="E9" s="423" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="E9" s="424" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -18472,9 +18472,9 @@
           <t>Zoho CRM + Pipedrive + Dynamics 365 — proper auth, HMAC verification, Zod schemas, rate limit compliance</t>
         </is>
       </c>
-      <c r="E10" s="423" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="E10" s="424" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -18499,9 +18499,9 @@
           <t>Customer lifetime value predictor — CRM + order data fusion, service layer pattern, async data fetching</t>
         </is>
       </c>
-      <c r="E11" s="423" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="E11" s="424" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(sprint-8.5): plan collaboration, messaging & notifications sprint
Sprint 8.5 — Collaboration, Messaging & Notifications: Slack, Firebase
FCM, Vonage, Pusher, OneSignal, Sendbird, Mailgun, AWS SES SDKs,
notification orchestrator with channel priority + fallback + quiet hours,
team collaboration panel, smart notification timing AI. Skills assigned:
backend-patterns, api-design, security-review, frontend-patterns,
e2e-testing, tdd-workflow.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/witylogix-sprint-tracker.xlsx
+++ b/witylogix-sprint-tracker.xlsx
@@ -46,6 +46,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.2 Done" sheetId="37" state="visible" r:id="rId37"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.3 Done" sheetId="38" state="visible" r:id="rId38"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.4 Done" sheetId="39" state="visible" r:id="rId39"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.5 Plan" sheetId="40" state="visible" r:id="rId40"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Data Models Gap'!$A$1:$K$40</definedName>
@@ -8065,10 +8066,10 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="A5:G5"/>
     <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:G1"/>
     <mergeCell ref="A12:F12"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A5:G5"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -19381,6 +19382,324 @@
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" style="186" min="1" max="1"/>
+    <col width="16" customWidth="1" style="186" min="2" max="2"/>
+    <col width="32" customWidth="1" style="186" min="3" max="3"/>
+    <col width="80" customWidth="1" style="186" min="4" max="4"/>
+    <col width="12" customWidth="1" style="186" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="422" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="B1" s="422" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="C1" s="422" t="inlineStr">
+        <is>
+          <t>Skill Applied</t>
+        </is>
+      </c>
+      <c r="D1" s="422" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="E1" s="422" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="416" t="inlineStr">
+        <is>
+          <t>AR</t>
+        </is>
+      </c>
+      <c r="B2" s="416" t="inlineStr">
+        <is>
+          <t>CTO/Architect</t>
+        </is>
+      </c>
+      <c r="C2" s="416" t="inlineStr">
+        <is>
+          <t>backend-patterns + api-design</t>
+        </is>
+      </c>
+      <c r="D2" s="416" t="inlineStr">
+        <is>
+          <t>Notification orchestrator — channel priority matrix, fallback chain (push→SMS→email), quiet hours per timezone, digest batching, delivery receipts, retry with DLQ</t>
+        </is>
+      </c>
+      <c r="E2" s="423" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="416" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="B3" s="416" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C3" s="416" t="inlineStr">
+        <is>
+          <t>frontend-patterns</t>
+        </is>
+      </c>
+      <c r="D3" s="416" t="inlineStr">
+        <is>
+          <t>Notification center redesign — per-channel preferences grid, delivery log with status badges, real-time toast with AnimatePresence, sound toggle</t>
+        </is>
+      </c>
+      <c r="E3" s="423" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="416" t="inlineStr">
+        <is>
+          <t>NK</t>
+        </is>
+      </c>
+      <c r="B4" s="416" t="inlineStr">
+        <is>
+          <t>Frontend Lead</t>
+        </is>
+      </c>
+      <c r="C4" s="416" t="inlineStr">
+        <is>
+          <t>frontend-patterns</t>
+        </is>
+      </c>
+      <c r="D4" s="416" t="inlineStr">
+        <is>
+          <t>Team collaboration panel — Slack/Teams embedded messaging view, channel selector, message composer, file sharing, @mentions, thread view</t>
+        </is>
+      </c>
+      <c r="E4" s="423" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="416" t="inlineStr">
+        <is>
+          <t>RG</t>
+        </is>
+      </c>
+      <c r="B5" s="416" t="inlineStr">
+        <is>
+          <t>Backend Lead</t>
+        </is>
+      </c>
+      <c r="C5" s="416" t="inlineStr">
+        <is>
+          <t>api-design + security-review</t>
+        </is>
+      </c>
+      <c r="D5" s="416" t="inlineStr">
+        <is>
+          <t>Slack Web API SDK — OAuth2 V2 bot/user, conversations, messages, files, reactions, events API, Socket Mode, HMAC verification, rate limiting</t>
+        </is>
+      </c>
+      <c r="E5" s="423" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="416" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="B6" s="416" t="inlineStr">
+        <is>
+          <t>Full-stack</t>
+        </is>
+      </c>
+      <c r="C6" s="416" t="inlineStr">
+        <is>
+          <t>backend-patterns + security-review</t>
+        </is>
+      </c>
+      <c r="D6" s="416" t="inlineStr">
+        <is>
+          <t>Firebase FCM SDK — device registration, topic messaging, data/notification payloads, multicast, condition targeting, APNs relay</t>
+        </is>
+      </c>
+      <c r="E6" s="423" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="416" t="inlineStr">
+        <is>
+          <t>VS</t>
+        </is>
+      </c>
+      <c r="B7" s="416" t="inlineStr">
+        <is>
+          <t>Component Dev</t>
+        </is>
+      </c>
+      <c r="C7" s="416" t="inlineStr">
+        <is>
+          <t>frontend-patterns</t>
+        </is>
+      </c>
+      <c r="D7" s="416" t="inlineStr">
+        <is>
+          <t>Notification UI components — template editor with variable insertion, channel toggle matrix, delivery timeline, priority selector, toast stack</t>
+        </is>
+      </c>
+      <c r="E7" s="423" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="416" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="B8" s="416" t="inlineStr">
+        <is>
+          <t>Sr. Backend</t>
+        </is>
+      </c>
+      <c r="C8" s="416" t="inlineStr">
+        <is>
+          <t>api-design + backend-patterns</t>
+        </is>
+      </c>
+      <c r="D8" s="416" t="inlineStr">
+        <is>
+          <t>Vonage Messages API SDK — SMS/MMS/WhatsApp/Viber, Pusher Channels SDK — real-time pub/sub, presence, encrypted channels</t>
+        </is>
+      </c>
+      <c r="E8" s="423" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="416" t="inlineStr">
+        <is>
+          <t>KS</t>
+        </is>
+      </c>
+      <c r="B9" s="416" t="inlineStr">
+        <is>
+          <t>QA Lead</t>
+        </is>
+      </c>
+      <c r="C9" s="416" t="inlineStr">
+        <is>
+          <t>e2e-testing + tdd-workflow</t>
+        </is>
+      </c>
+      <c r="D9" s="416" t="inlineStr">
+        <is>
+          <t>Notification delivery tests (all channels), channel failover tests, quiet hours tests, E2E notification preferences, template rendering tests</t>
+        </is>
+      </c>
+      <c r="E9" s="423" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="416" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="B10" s="416" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="C10" s="416" t="inlineStr">
+        <is>
+          <t>api-design + security-review</t>
+        </is>
+      </c>
+      <c r="D10" s="416" t="inlineStr">
+        <is>
+          <t>OneSignal SDK — push segments/tags/templates, Sendbird SDK — chat channels/messages/users, Mailgun SDK — email/templates/routes, AWS SES SDK — email/templates/config sets</t>
+        </is>
+      </c>
+      <c r="E10" s="423" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="416" t="inlineStr">
+        <is>
+          <t>ZR</t>
+        </is>
+      </c>
+      <c r="B11" s="416" t="inlineStr">
+        <is>
+          <t>AI Engineer</t>
+        </is>
+      </c>
+      <c r="C11" s="416" t="inlineStr">
+        <is>
+          <t>backend-patterns</t>
+        </is>
+      </c>
+      <c r="D11" s="416" t="inlineStr">
+        <is>
+          <t>Smart notification timing — ML-based optimal send time per recipient, engagement predictor, channel preference learner, notification fatigue detector</t>
+        </is>
+      </c>
+      <c r="E11" s="423" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
feat(sprint-8.5): collaboration, messaging & notifications
Notification orchestrator v2 with channel routing, fallback chains,
quiet hours, digest batching, and delivery tracking. Slack + Teams
collaboration SDKs, Firebase FCM + OneSignal push SDKs, Vonage +
Pusher messaging SDKs, WhatsApp Cloud API v2, Mailgun + AWS SES
email SDKs, Sendbird chat SDK. Notification center UI with preferences
matrix and delivery log. Team collaboration panel with messaging hub.
AI smart notification timing and fatigue detection.

10 agents, 52 files, ~22,000 lines.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/witylogix-sprint-tracker.xlsx
+++ b/witylogix-sprint-tracker.xlsx
@@ -46,7 +46,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.2 Done" sheetId="37" state="visible" r:id="rId37"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.3 Done" sheetId="38" state="visible" r:id="rId38"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.4 Done" sheetId="39" state="visible" r:id="rId39"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.5 Plan" sheetId="40" state="visible" r:id="rId40"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.5 Done" sheetId="40" state="visible" r:id="rId40"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Data Models Gap'!$A$1:$K$40</definedName>
@@ -64,7 +64,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="89">
+  <fonts count="90">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -668,8 +668,12 @@
     <font>
       <color rgb="00006100"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00006100"/>
+    </font>
   </fonts>
-  <fills count="60">
+  <fills count="61">
     <fill>
       <patternFill/>
     </fill>
@@ -1013,6 +1017,12 @@
         <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="6">
     <border>
@@ -1084,7 +1094,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="425">
+  <cellXfs count="426">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -2314,6 +2324,7 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="58" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="88" fillId="59" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="89" fillId="60" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -8066,10 +8077,10 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A12:F12"/>
     <mergeCell ref="A5:G5"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A12:F12"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -19449,9 +19460,9 @@
           <t>Notification orchestrator — channel priority matrix, fallback chain (push→SMS→email), quiet hours per timezone, digest batching, delivery receipts, retry with DLQ</t>
         </is>
       </c>
-      <c r="E2" s="423" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="E2" s="425" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -19476,9 +19487,9 @@
           <t>Notification center redesign — per-channel preferences grid, delivery log with status badges, real-time toast with AnimatePresence, sound toggle</t>
         </is>
       </c>
-      <c r="E3" s="423" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="E3" s="425" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -19503,9 +19514,9 @@
           <t>Team collaboration panel — Slack/Teams embedded messaging view, channel selector, message composer, file sharing, @mentions, thread view</t>
         </is>
       </c>
-      <c r="E4" s="423" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="E4" s="425" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -19530,9 +19541,9 @@
           <t>Slack Web API SDK — OAuth2 V2 bot/user, conversations, messages, files, reactions, events API, Socket Mode, HMAC verification, rate limiting</t>
         </is>
       </c>
-      <c r="E5" s="423" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="E5" s="425" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -19557,9 +19568,9 @@
           <t>Firebase FCM SDK — device registration, topic messaging, data/notification payloads, multicast, condition targeting, APNs relay</t>
         </is>
       </c>
-      <c r="E6" s="423" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="E6" s="425" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -19584,9 +19595,9 @@
           <t>Notification UI components — template editor with variable insertion, channel toggle matrix, delivery timeline, priority selector, toast stack</t>
         </is>
       </c>
-      <c r="E7" s="423" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="E7" s="425" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -19611,9 +19622,9 @@
           <t>Vonage Messages API SDK — SMS/MMS/WhatsApp/Viber, Pusher Channels SDK — real-time pub/sub, presence, encrypted channels</t>
         </is>
       </c>
-      <c r="E8" s="423" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="E8" s="425" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -19638,9 +19649,9 @@
           <t>Notification delivery tests (all channels), channel failover tests, quiet hours tests, E2E notification preferences, template rendering tests</t>
         </is>
       </c>
-      <c r="E9" s="423" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="E9" s="425" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -19665,9 +19676,9 @@
           <t>OneSignal SDK — push segments/tags/templates, Sendbird SDK — chat channels/messages/users, Mailgun SDK — email/templates/routes, AWS SES SDK — email/templates/config sets</t>
         </is>
       </c>
-      <c r="E10" s="423" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="E10" s="425" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -19692,9 +19703,9 @@
           <t>Smart notification timing — ML-based optimal send time per recipient, engagement predictor, channel preference learner, notification fatigue detector</t>
         </is>
       </c>
-      <c r="E11" s="423" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="E11" s="425" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(sprint-8.6): plan freight, ELD & compliance sprint
Sprint 8.6 plan: freight management engine v2, HOS rules engine v2,
Samsara/KeepTruckin/Trimble/Geotab ELD SDKs, DAT v2/Truckstop v2/
FreightWaves SONAR freight SDKs, FMCSA SAFER/DataQs APIs, freight &
compliance dashboards, AI freight matching & rate forecasting.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/witylogix-sprint-tracker.xlsx
+++ b/witylogix-sprint-tracker.xlsx
@@ -47,6 +47,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.3 Done" sheetId="38" state="visible" r:id="rId38"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.4 Done" sheetId="39" state="visible" r:id="rId39"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.5 Done" sheetId="40" state="visible" r:id="rId40"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.6 Plan" sheetId="41" state="visible" r:id="rId41"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Data Models Gap'!$A$1:$K$40</definedName>
@@ -1094,7 +1095,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="426">
+  <cellXfs count="427">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -2325,6 +2326,9 @@
     <xf numFmtId="0" fontId="0" fillId="58" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="88" fillId="59" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="89" fillId="60" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="71" fillId="53" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -8077,9 +8081,9 @@
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A12:F12"/>
+    <mergeCell ref="A1:G1"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -19706,6 +19710,436 @@
       <c r="E11" s="425" t="inlineStr">
         <is>
           <t>Done</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" style="186" min="1" max="1"/>
+    <col width="14" customWidth="1" style="186" min="2" max="2"/>
+    <col width="35" customWidth="1" style="186" min="3" max="3"/>
+    <col width="60" customWidth="1" style="186" min="4" max="4"/>
+    <col width="65" customWidth="1" style="186" min="5" max="5"/>
+    <col width="12" customWidth="1" style="186" min="6" max="6"/>
+    <col width="10" customWidth="1" style="186" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="426" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="B1" s="426" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="C1" s="426" t="inlineStr">
+        <is>
+          <t>Skill Applied</t>
+        </is>
+      </c>
+      <c r="D1" s="426" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="E1" s="426" t="inlineStr">
+        <is>
+          <t>Deliverables</t>
+        </is>
+      </c>
+      <c r="F1" s="426" t="inlineStr">
+        <is>
+          <t>Lines (est)</t>
+        </is>
+      </c>
+      <c r="G1" s="426" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="410" t="inlineStr">
+        <is>
+          <t>AR</t>
+        </is>
+      </c>
+      <c r="B2" s="410" t="inlineStr">
+        <is>
+          <t>CTO</t>
+        </is>
+      </c>
+      <c r="C2" s="410" t="inlineStr">
+        <is>
+          <t>backend-patterns, carrier-relationship-management</t>
+        </is>
+      </c>
+      <c r="D2" s="410" t="inlineStr">
+        <is>
+          <t>Freight management engine v2 — rate negotiation, lane management, carrier scorecard, freight audit, compliance rules engine, FMCSA SAFER API integration</t>
+        </is>
+      </c>
+      <c r="E2" s="410" t="inlineStr">
+        <is>
+          <t>packages/core/src/freight/freight-management-engine.ts, freight-types.ts, freight-audit-engine.ts, fmcsa-safer-client.ts, freight-api.ts, index.ts + 2 test files</t>
+        </is>
+      </c>
+      <c r="F2" s="410" t="inlineStr">
+        <is>
+          <t>~3,500</t>
+        </is>
+      </c>
+      <c r="G2" s="410" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="410" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="B3" s="410" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C3" s="410" t="inlineStr">
+        <is>
+          <t>frontend-patterns</t>
+        </is>
+      </c>
+      <c r="D3" s="410" t="inlineStr">
+        <is>
+          <t>Freight management dashboard — load board view, rate comparison, carrier scorecard UI, compliance dashboard, HOS violation alerts</t>
+        </is>
+      </c>
+      <c r="E3" s="410" t="inlineStr">
+        <is>
+          <t>apps/dashboard/src/app/(dashboard)/freight/page.tsx, loads/page.tsx, rates/page.tsx, compliance/page.tsx, layout.tsx, hooks/use-freight.ts</t>
+        </is>
+      </c>
+      <c r="F3" s="410" t="inlineStr">
+        <is>
+          <t>~2,200</t>
+        </is>
+      </c>
+      <c r="G3" s="410" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="410" t="inlineStr">
+        <is>
+          <t>NK</t>
+        </is>
+      </c>
+      <c r="B4" s="410" t="inlineStr">
+        <is>
+          <t>Frontend Lead</t>
+        </is>
+      </c>
+      <c r="C4" s="410" t="inlineStr">
+        <is>
+          <t>frontend-patterns</t>
+        </is>
+      </c>
+      <c r="D4" s="410" t="inlineStr">
+        <is>
+          <t>ELD &amp; driver compliance dashboard — HOS clock display, violation timeline, DVIR forms, driver qualification file viewer</t>
+        </is>
+      </c>
+      <c r="E4" s="410" t="inlineStr">
+        <is>
+          <t>apps/dashboard/src/app/(dashboard)/eld/page.tsx, hos/page.tsx, dvir/page.tsx, layout.tsx, components/eld/hos-clock.tsx, violation-timeline.tsx, dvir-form.tsx, hooks/use-eld.ts</t>
+        </is>
+      </c>
+      <c r="F4" s="410" t="inlineStr">
+        <is>
+          <t>~2,400</t>
+        </is>
+      </c>
+      <c r="G4" s="410" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="410" t="inlineStr">
+        <is>
+          <t>RG</t>
+        </is>
+      </c>
+      <c r="B5" s="410" t="inlineStr">
+        <is>
+          <t>Backend Lead</t>
+        </is>
+      </c>
+      <c r="C5" s="410" t="inlineStr">
+        <is>
+          <t>api-design, security-review, customs-trade-compliance</t>
+        </is>
+      </c>
+      <c r="D5" s="410" t="inlineStr">
+        <is>
+          <t>Samsara ELD SDK (full fleet API) + KeepTruckin/Motive v2 SDK (expanded) + FMCSA DataQs API</t>
+        </is>
+      </c>
+      <c r="E5" s="410" t="inlineStr">
+        <is>
+          <t>packages/core/src/integrations/eld/samsara-eld-sdk-client.ts, keeptruckin-sdk-client.ts, fmcsa-dataqs-client.ts, eld-sdk-types.ts + 3 test files</t>
+        </is>
+      </c>
+      <c r="F5" s="410" t="inlineStr">
+        <is>
+          <t>~3,200</t>
+        </is>
+      </c>
+      <c r="G5" s="410" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="410" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="B6" s="410" t="inlineStr">
+        <is>
+          <t>Full-stack</t>
+        </is>
+      </c>
+      <c r="C6" s="410" t="inlineStr">
+        <is>
+          <t>backend-patterns, security-review</t>
+        </is>
+      </c>
+      <c r="D6" s="410" t="inlineStr">
+        <is>
+          <t>DAT Freight v2 SDK (expanded — RateView, load search, broker tools) + Truckstop v2 SDK (expanded) + FreightWaves SONAR API</t>
+        </is>
+      </c>
+      <c r="E6" s="410" t="inlineStr">
+        <is>
+          <t>packages/core/src/integrations/freight/dat-v2-sdk-client.ts, truckstop-v2-sdk-client.ts, freightwaves-sonar-client.ts, freight-sdk-types.ts + 3 test files</t>
+        </is>
+      </c>
+      <c r="F6" s="410" t="inlineStr">
+        <is>
+          <t>~3,000</t>
+        </is>
+      </c>
+      <c r="G6" s="410" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="410" t="inlineStr">
+        <is>
+          <t>VS</t>
+        </is>
+      </c>
+      <c r="B7" s="410" t="inlineStr">
+        <is>
+          <t>Component Dev</t>
+        </is>
+      </c>
+      <c r="C7" s="410" t="inlineStr">
+        <is>
+          <t>frontend-patterns</t>
+        </is>
+      </c>
+      <c r="D7" s="410" t="inlineStr">
+        <is>
+          <t>Freight &amp; ELD UI components — rate comparison card, lane heat map, HOS gauge, carrier scorecard chart, compliance badge, freight timeline, DVIR checklist</t>
+        </is>
+      </c>
+      <c r="E7" s="410" t="inlineStr">
+        <is>
+          <t>apps/dashboard/src/components/freight/rate-comparison-card.tsx, lane-heatmap.tsx, carrier-scorecard.tsx, freight-timeline.tsx, index.ts; components/eld/hos-gauge.tsx, compliance-badge.tsx, dvir-checklist.tsx, index.ts</t>
+        </is>
+      </c>
+      <c r="F7" s="410" t="inlineStr">
+        <is>
+          <t>~1,800</t>
+        </is>
+      </c>
+      <c r="G7" s="410" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="410" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="B8" s="410" t="inlineStr">
+        <is>
+          <t>Sr. Backend</t>
+        </is>
+      </c>
+      <c r="C8" s="410" t="inlineStr">
+        <is>
+          <t>backend-patterns, logistics-exception-management</t>
+        </is>
+      </c>
+      <c r="D8" s="410" t="inlineStr">
+        <is>
+          <t>HOS rules engine v2 — FMCSA 70h/8d &amp; 60h/7d, 11h driving, 14h window, 30min break, sleeper berth split, Canadian &amp; Mexico rules, violation detection, auto-recalculation</t>
+        </is>
+      </c>
+      <c r="E8" s="410" t="inlineStr">
+        <is>
+          <t>packages/core/src/compliance/hos-rules-engine-v2.ts, hos-types.ts, hos-violation-detector.ts, hos-calculator.ts, dvir-engine.ts + 2 test files</t>
+        </is>
+      </c>
+      <c r="F8" s="410" t="inlineStr">
+        <is>
+          <t>~3,400</t>
+        </is>
+      </c>
+      <c r="G8" s="410" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="410" t="inlineStr">
+        <is>
+          <t>KS</t>
+        </is>
+      </c>
+      <c r="B9" s="410" t="inlineStr">
+        <is>
+          <t>QA Lead</t>
+        </is>
+      </c>
+      <c r="C9" s="410" t="inlineStr">
+        <is>
+          <t>e2e-testing, tdd-workflow</t>
+        </is>
+      </c>
+      <c r="D9" s="410" t="inlineStr">
+        <is>
+          <t>Test suites — HOS compliance scenarios (70h/8d, split sleeper, personal conveyance), freight rate accuracy, FMCSA validation, carrier scorecard, E2E freight workflow</t>
+        </is>
+      </c>
+      <c r="E9" s="410" t="inlineStr">
+        <is>
+          <t>tests/integration/freight/*.test.ts (3 files), tests/integration/compliance/*.test.ts (3 files), tests/e2e/freight/*.spec.ts, tests/integration/fixtures/freight-fixtures.ts</t>
+        </is>
+      </c>
+      <c r="F9" s="410" t="inlineStr">
+        <is>
+          <t>~2,800</t>
+        </is>
+      </c>
+      <c r="G9" s="410" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="410" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="B10" s="410" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="C10" s="410" t="inlineStr">
+        <is>
+          <t>api-design, security-review</t>
+        </is>
+      </c>
+      <c r="D10" s="410" t="inlineStr">
+        <is>
+          <t>Trimble ELD SDK + Geotab Drive (HOS) SDK + Omnitracs XRS v2 SDK + Lytx DriveCam SDK</t>
+        </is>
+      </c>
+      <c r="E10" s="410" t="inlineStr">
+        <is>
+          <t>packages/core/src/integrations/eld/trimble-eld-sdk-client.ts, geotab-drive-sdk-client.ts, omnitracs-xrs-v2-client.ts, lytx-drivecam-client.ts + 4 test files</t>
+        </is>
+      </c>
+      <c r="F10" s="410" t="inlineStr">
+        <is>
+          <t>~3,000</t>
+        </is>
+      </c>
+      <c r="G10" s="410" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="410" t="inlineStr">
+        <is>
+          <t>ZR</t>
+        </is>
+      </c>
+      <c r="B11" s="410" t="inlineStr">
+        <is>
+          <t>AI Engineer</t>
+        </is>
+      </c>
+      <c r="C11" s="410" t="inlineStr">
+        <is>
+          <t>backend-patterns</t>
+        </is>
+      </c>
+      <c r="D11" s="410" t="inlineStr">
+        <is>
+          <t>AI freight matching — load-carrier scoring, lane demand prediction, rate forecasting, carrier reliability predictor, compliance risk scorer</t>
+        </is>
+      </c>
+      <c r="E11" s="410" t="inlineStr">
+        <is>
+          <t>packages/core/src/ai/freight-matcher.ts, rate-forecaster.ts, compliance-risk-scorer.ts, freight-intelligence-api.ts + 2 test files</t>
+        </is>
+      </c>
+      <c r="F11" s="410" t="inlineStr">
+        <is>
+          <t>~2,600</t>
+        </is>
+      </c>
+      <c r="G11" s="410" t="inlineStr">
+        <is>
+          <t>Planned</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(sprint-8.6): freight, ELD & compliance
Freight management engine v2 with rate negotiation, carrier scorecards,
and freight audit (invoice matching, duplicate detection, 3-tier dispute
escalation). HOS rules engine v2 with full FMCSA Part 395, Canadian
Federal, and Mexico NOM-087-SCT rules including sleeper berth splits
and 34h restart. ELD SDKs: Samsara, KeepTruckin v2, Trimble, Geotab
Drive, Omnitracs XRS v2, Lytx DriveCam. Freight SDKs: DAT v2,
Truckstop v2, FreightWaves SONAR. FMCSA SAFER + DataQs APIs. Freight
management and ELD compliance dashboards. AI freight matching, rate
forecasting, and compliance risk scoring.

10 agents, ~40 files, ~28,000 lines.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/witylogix-sprint-tracker.xlsx
+++ b/witylogix-sprint-tracker.xlsx
@@ -47,7 +47,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.3 Done" sheetId="38" state="visible" r:id="rId38"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.4 Done" sheetId="39" state="visible" r:id="rId39"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.5 Done" sheetId="40" state="visible" r:id="rId40"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.6 Plan" sheetId="41" state="visible" r:id="rId41"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.6 Done" sheetId="41" state="visible" r:id="rId41"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Data Models Gap'!$A$1:$K$40</definedName>
@@ -1095,7 +1095,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="427">
+  <cellXfs count="428">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -2328,6 +2328,9 @@
     <xf numFmtId="0" fontId="89" fillId="60" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="71" fillId="53" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="89" fillId="60" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -8081,10 +8084,10 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="A5:G5"/>
     <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:G1"/>
     <mergeCell ref="A12:F12"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A5:G5"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -19804,9 +19807,9 @@
           <t>~3,500</t>
         </is>
       </c>
-      <c r="G2" s="410" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="G2" s="427" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -19841,9 +19844,9 @@
           <t>~2,200</t>
         </is>
       </c>
-      <c r="G3" s="410" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="G3" s="427" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -19878,9 +19881,9 @@
           <t>~2,400</t>
         </is>
       </c>
-      <c r="G4" s="410" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="G4" s="427" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -19915,9 +19918,9 @@
           <t>~3,200</t>
         </is>
       </c>
-      <c r="G5" s="410" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="G5" s="427" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -19952,9 +19955,9 @@
           <t>~3,000</t>
         </is>
       </c>
-      <c r="G6" s="410" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="G6" s="427" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -19989,9 +19992,9 @@
           <t>~1,800</t>
         </is>
       </c>
-      <c r="G7" s="410" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="G7" s="427" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -20026,9 +20029,9 @@
           <t>~3,400</t>
         </is>
       </c>
-      <c r="G8" s="410" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="G8" s="427" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -20063,9 +20066,9 @@
           <t>~2,800</t>
         </is>
       </c>
-      <c r="G9" s="410" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="G9" s="427" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -20100,9 +20103,9 @@
           <t>~3,000</t>
         </is>
       </c>
-      <c r="G10" s="410" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="G10" s="427" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -20137,9 +20140,9 @@
           <t>~2,600</t>
         </is>
       </c>
-      <c r="G11" s="410" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="G11" s="427" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(sprint-8.7): plan fuel, fleet & field service sprint
Sprint 8.7 plan: fleet management engine, maintenance scheduler, fuel
optimization, field service scheduling engine with dispatch optimization,
WEX v2/Comdata v2/Fleetcor v2/EFS-TChek fuel SDKs, ServiceTitan v2/
Jobber v2 field service SDKs, Toast v2/Square v2/Clover/Lightspeed
POS SDKs, fleet & field service dashboards, AI predictive maintenance
& fuel efficiency & technician scheduling.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/witylogix-sprint-tracker.xlsx
+++ b/witylogix-sprint-tracker.xlsx
@@ -48,6 +48,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.4 Done" sheetId="39" state="visible" r:id="rId39"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.5 Done" sheetId="40" state="visible" r:id="rId40"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.6 Done" sheetId="41" state="visible" r:id="rId41"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.7 Plan" sheetId="42" state="visible" r:id="rId42"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Data Models Gap'!$A$1:$K$40</definedName>
@@ -8084,10 +8085,10 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A12:F12"/>
     <mergeCell ref="A5:G5"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A12:F12"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -20143,6 +20144,436 @@
       <c r="G11" s="427" t="inlineStr">
         <is>
           <t>Done</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" style="186" min="1" max="1"/>
+    <col width="14" customWidth="1" style="186" min="2" max="2"/>
+    <col width="35" customWidth="1" style="186" min="3" max="3"/>
+    <col width="60" customWidth="1" style="186" min="4" max="4"/>
+    <col width="65" customWidth="1" style="186" min="5" max="5"/>
+    <col width="12" customWidth="1" style="186" min="6" max="6"/>
+    <col width="10" customWidth="1" style="186" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="426" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="B1" s="426" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="C1" s="426" t="inlineStr">
+        <is>
+          <t>Skill Applied</t>
+        </is>
+      </c>
+      <c r="D1" s="426" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="E1" s="426" t="inlineStr">
+        <is>
+          <t>Deliverables</t>
+        </is>
+      </c>
+      <c r="F1" s="426" t="inlineStr">
+        <is>
+          <t>Lines (est)</t>
+        </is>
+      </c>
+      <c r="G1" s="426" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="410" t="inlineStr">
+        <is>
+          <t>AR</t>
+        </is>
+      </c>
+      <c r="B2" s="410" t="inlineStr">
+        <is>
+          <t>CTO</t>
+        </is>
+      </c>
+      <c r="C2" s="410" t="inlineStr">
+        <is>
+          <t>backend-patterns, energy-procurement</t>
+        </is>
+      </c>
+      <c r="D2" s="410" t="inlineStr">
+        <is>
+          <t>Fleet management engine — vehicle lifecycle (acquisition→maintenance→disposal), maintenance scheduler (preventive/reactive/predictive), fuel optimization (route-fuel correlation, idle reduction), fleet cost analyzer, vehicle assignment engine, 15+ REST endpoints</t>
+        </is>
+      </c>
+      <c r="E2" s="410" t="inlineStr">
+        <is>
+          <t>packages/core/src/fleet/fleet-management-engine.ts, fleet-types.ts, maintenance-scheduler.ts, fuel-optimizer.ts, fleet-cost-analyzer.ts, fleet-api.ts, index.ts + 2 test files</t>
+        </is>
+      </c>
+      <c r="F2" s="410" t="inlineStr">
+        <is>
+          <t>~3,500</t>
+        </is>
+      </c>
+      <c r="G2" s="410" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="410" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="B3" s="410" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C3" s="410" t="inlineStr">
+        <is>
+          <t>frontend-patterns</t>
+        </is>
+      </c>
+      <c r="D3" s="410" t="inlineStr">
+        <is>
+          <t>Fleet management dashboard — vehicle inventory, maintenance calendar, fuel analytics, fleet health overview, vehicle assignment UI</t>
+        </is>
+      </c>
+      <c r="E3" s="410" t="inlineStr">
+        <is>
+          <t>apps/dashboard/src/app/(dashboard)/fleet/page.tsx, vehicles/page.tsx, maintenance/page.tsx, fuel/page.tsx, layout.tsx, hooks/use-fleet.ts</t>
+        </is>
+      </c>
+      <c r="F3" s="410" t="inlineStr">
+        <is>
+          <t>~2,200</t>
+        </is>
+      </c>
+      <c r="G3" s="410" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="410" t="inlineStr">
+        <is>
+          <t>NK</t>
+        </is>
+      </c>
+      <c r="B4" s="410" t="inlineStr">
+        <is>
+          <t>Frontend Lead</t>
+        </is>
+      </c>
+      <c r="C4" s="410" t="inlineStr">
+        <is>
+          <t>frontend-patterns</t>
+        </is>
+      </c>
+      <c r="D4" s="410" t="inlineStr">
+        <is>
+          <t>Field service &amp; POS dashboard — job scheduling calendar, technician dispatch map, work order management, POS transaction viewer</t>
+        </is>
+      </c>
+      <c r="E4" s="410" t="inlineStr">
+        <is>
+          <t>apps/dashboard/src/app/(dashboard)/field-service/page.tsx, jobs/page.tsx, dispatch/page.tsx, layout.tsx, apps/dashboard/src/app/(dashboard)/pos/page.tsx, transactions/page.tsx, layout.tsx, hooks/use-field-service.ts, hooks/use-pos.ts</t>
+        </is>
+      </c>
+      <c r="F4" s="410" t="inlineStr">
+        <is>
+          <t>~2,600</t>
+        </is>
+      </c>
+      <c r="G4" s="410" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="410" t="inlineStr">
+        <is>
+          <t>RG</t>
+        </is>
+      </c>
+      <c r="B5" s="410" t="inlineStr">
+        <is>
+          <t>Backend Lead</t>
+        </is>
+      </c>
+      <c r="C5" s="410" t="inlineStr">
+        <is>
+          <t>api-design, security-review</t>
+        </is>
+      </c>
+      <c r="D5" s="410" t="inlineStr">
+        <is>
+          <t>WEX Fleet v2 SDK (expanded — real-time auth, transactions, controls, reporting) + Comdata v2 SDK (expanded) + Fleetcor/FUELMAN v2 SDK + EFS/TChek SDK</t>
+        </is>
+      </c>
+      <c r="E5" s="410" t="inlineStr">
+        <is>
+          <t>packages/core/src/integrations/fuel-fleet/wex-v2-sdk-client.ts, comdata-v2-sdk-client.ts, fleetcor-v2-sdk-client.ts, efs-tchek-v2-client.ts, fuel-fleet-sdk-types.ts + 4 test files</t>
+        </is>
+      </c>
+      <c r="F5" s="410" t="inlineStr">
+        <is>
+          <t>~3,200</t>
+        </is>
+      </c>
+      <c r="G5" s="410" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="410" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="B6" s="410" t="inlineStr">
+        <is>
+          <t>Full-stack</t>
+        </is>
+      </c>
+      <c r="C6" s="410" t="inlineStr">
+        <is>
+          <t>backend-patterns, security-review</t>
+        </is>
+      </c>
+      <c r="D6" s="410" t="inlineStr">
+        <is>
+          <t>ServiceTitan v2 SDK (expanded — scheduling, dispatch, memberships, pricebook, reporting) + Jobber v2 SDK (expanded — GraphQL, scheduling, invoicing, payments)</t>
+        </is>
+      </c>
+      <c r="E6" s="410" t="inlineStr">
+        <is>
+          <t>packages/core/src/integrations/field-service/servicetitan-v2-sdk-client.ts, jobber-v2-sdk-client.ts, field-service-sdk-types.ts + 2 test files</t>
+        </is>
+      </c>
+      <c r="F6" s="410" t="inlineStr">
+        <is>
+          <t>~2,800</t>
+        </is>
+      </c>
+      <c r="G6" s="410" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="410" t="inlineStr">
+        <is>
+          <t>VS</t>
+        </is>
+      </c>
+      <c r="B7" s="410" t="inlineStr">
+        <is>
+          <t>Component Dev</t>
+        </is>
+      </c>
+      <c r="C7" s="410" t="inlineStr">
+        <is>
+          <t>frontend-patterns</t>
+        </is>
+      </c>
+      <c r="D7" s="410" t="inlineStr">
+        <is>
+          <t>Fleet, field-service &amp; POS UI components — vehicle health card, maintenance timeline, fuel gauge chart, job calendar, technician map marker, work order card, POS receipt, transaction list</t>
+        </is>
+      </c>
+      <c r="E7" s="410" t="inlineStr">
+        <is>
+          <t>apps/dashboard/src/components/fleet/vehicle-health-card.tsx, maintenance-timeline.tsx, fuel-gauge-chart.tsx, index.ts; components/field-service/job-calendar.tsx, technician-marker.tsx, work-order-card.tsx, index.ts; components/pos/pos-receipt.tsx, transaction-list.tsx, index.ts</t>
+        </is>
+      </c>
+      <c r="F7" s="410" t="inlineStr">
+        <is>
+          <t>~2,000</t>
+        </is>
+      </c>
+      <c r="G7" s="410" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="410" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="B8" s="410" t="inlineStr">
+        <is>
+          <t>Sr. Backend</t>
+        </is>
+      </c>
+      <c r="C8" s="410" t="inlineStr">
+        <is>
+          <t>backend-patterns, inventory-demand-planning</t>
+        </is>
+      </c>
+      <c r="D8" s="410" t="inlineStr">
+        <is>
+          <t>Field service scheduling engine — job scheduling with constraints (skills, zones, availability, SLA), dispatch optimization (nearest available, workload balancing), work order lifecycle (created→scheduled→dispatched→in-progress→completed), recurring maintenance plans</t>
+        </is>
+      </c>
+      <c r="E8" s="410" t="inlineStr">
+        <is>
+          <t>packages/core/src/field-service/scheduling-engine.ts, field-service-types.ts, dispatch-optimizer.ts, work-order-engine.ts, field-service-api.ts + 2 test files</t>
+        </is>
+      </c>
+      <c r="F8" s="410" t="inlineStr">
+        <is>
+          <t>~3,200</t>
+        </is>
+      </c>
+      <c r="G8" s="410" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="410" t="inlineStr">
+        <is>
+          <t>KS</t>
+        </is>
+      </c>
+      <c r="B9" s="410" t="inlineStr">
+        <is>
+          <t>QA Lead</t>
+        </is>
+      </c>
+      <c r="C9" s="410" t="inlineStr">
+        <is>
+          <t>e2e-testing, tdd-workflow</t>
+        </is>
+      </c>
+      <c r="D9" s="410" t="inlineStr">
+        <is>
+          <t>Test suites — fleet vehicle lifecycle, maintenance scheduling, fuel card transactions, field service dispatch, work order flows, POS integration, E2E fleet + field service workflows</t>
+        </is>
+      </c>
+      <c r="E9" s="410" t="inlineStr">
+        <is>
+          <t>tests/integration/fleet/*.test.ts (3), tests/integration/field-service/*.test.ts (3), tests/e2e/fleet/*.spec.ts, tests/e2e/field-service/*.spec.ts, tests/integration/fixtures/fleet-fixtures.ts, field-service-fixtures.ts</t>
+        </is>
+      </c>
+      <c r="F9" s="410" t="inlineStr">
+        <is>
+          <t>~2,800</t>
+        </is>
+      </c>
+      <c r="G9" s="410" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="410" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="B10" s="410" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="C10" s="410" t="inlineStr">
+        <is>
+          <t>api-design, security-review</t>
+        </is>
+      </c>
+      <c r="D10" s="410" t="inlineStr">
+        <is>
+          <t>Toast POS v2 SDK (expanded — orders, menus, labor, reporting, webhooks) + Square POS v2 SDK (expanded — payments, inventory, loyalty, team) + Clover POS SDK + Lightspeed POS SDK</t>
+        </is>
+      </c>
+      <c r="E10" s="410" t="inlineStr">
+        <is>
+          <t>packages/core/src/integrations/pos/toast-v2-sdk-client.ts, square-pos-v2-sdk-client.ts, clover-pos-sdk-client.ts, lightspeed-pos-sdk-client.ts, pos-sdk-types.ts + 4 test files</t>
+        </is>
+      </c>
+      <c r="F10" s="410" t="inlineStr">
+        <is>
+          <t>~3,000</t>
+        </is>
+      </c>
+      <c r="G10" s="410" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="410" t="inlineStr">
+        <is>
+          <t>ZR</t>
+        </is>
+      </c>
+      <c r="B11" s="410" t="inlineStr">
+        <is>
+          <t>AI Engineer</t>
+        </is>
+      </c>
+      <c r="C11" s="410" t="inlineStr">
+        <is>
+          <t>backend-patterns</t>
+        </is>
+      </c>
+      <c r="D11" s="410" t="inlineStr">
+        <is>
+          <t>AI fleet intelligence — predictive maintenance (failure probability, remaining useful life), fuel efficiency optimizer (driver behavior scoring, route-fuel correlation), fleet utilization predictor, technician scheduling AI, fleet intelligence API</t>
+        </is>
+      </c>
+      <c r="E11" s="410" t="inlineStr">
+        <is>
+          <t>packages/core/src/ai/predictive-maintenance.ts, fuel-efficiency-optimizer.ts, fleet-utilization-predictor.ts, technician-scheduling-ai.ts, fleet-intelligence-api.ts + 2 test files</t>
+        </is>
+      </c>
+      <c r="F11" s="410" t="inlineStr">
+        <is>
+          <t>~2,800</t>
+        </is>
+      </c>
+      <c r="G11" s="410" t="inlineStr">
+        <is>
+          <t>Planned</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(sprint-8.7): fuel, fleet & field service
Fleet management engine with vehicle lifecycle, maintenance scheduler
(preventive/reactive/predictive), fuel optimizer, and fleet cost
analyzer. Field service scheduling engine with constraint-based
dispatch, work order lifecycle, and SLA monitoring. Fuel fleet SDKs:
WEX v2, Comdata v2, Fleetcor v2, EFS/TChek v2. Field service SDKs:
ServiceTitan v2, Jobber v2 (GraphQL). POS SDKs: Toast v2, Square v2,
Clover, Lightspeed. Fleet, field service, and POS dashboards. AI
predictive maintenance, fuel efficiency optimizer, fleet utilization
predictor, and technician scheduling.

10 agents, ~60 files, ~30,000 lines.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/witylogix-sprint-tracker.xlsx
+++ b/witylogix-sprint-tracker.xlsx
@@ -48,7 +48,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.4 Done" sheetId="39" state="visible" r:id="rId39"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.5 Done" sheetId="40" state="visible" r:id="rId40"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.6 Done" sheetId="41" state="visible" r:id="rId41"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.7 Plan" sheetId="42" state="visible" r:id="rId42"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.7 Done" sheetId="42" state="visible" r:id="rId42"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Data Models Gap'!$A$1:$K$40</definedName>
@@ -8085,9 +8085,9 @@
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A12:F12"/>
+    <mergeCell ref="A1:G1"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -20238,9 +20238,9 @@
           <t>~3,500</t>
         </is>
       </c>
-      <c r="G2" s="410" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="G2" s="427" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -20275,9 +20275,9 @@
           <t>~2,200</t>
         </is>
       </c>
-      <c r="G3" s="410" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="G3" s="427" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -20312,9 +20312,9 @@
           <t>~2,600</t>
         </is>
       </c>
-      <c r="G4" s="410" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="G4" s="427" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -20349,9 +20349,9 @@
           <t>~3,200</t>
         </is>
       </c>
-      <c r="G5" s="410" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="G5" s="427" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -20386,9 +20386,9 @@
           <t>~2,800</t>
         </is>
       </c>
-      <c r="G6" s="410" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="G6" s="427" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -20423,9 +20423,9 @@
           <t>~2,000</t>
         </is>
       </c>
-      <c r="G7" s="410" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="G7" s="427" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -20460,9 +20460,9 @@
           <t>~3,200</t>
         </is>
       </c>
-      <c r="G8" s="410" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="G8" s="427" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -20497,9 +20497,9 @@
           <t>~2,800</t>
         </is>
       </c>
-      <c r="G9" s="410" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="G9" s="427" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -20534,9 +20534,9 @@
           <t>~3,000</t>
         </is>
       </c>
-      <c r="G10" s="410" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="G10" s="427" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -20571,9 +20571,9 @@
           <t>~2,800</t>
         </is>
       </c>
-      <c r="G11" s="410" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="G11" s="427" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(sprint-8.8): plan e-signatures, healthcare, analytics & supply chain sprint
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/witylogix-sprint-tracker.xlsx
+++ b/witylogix-sprint-tracker.xlsx
@@ -49,6 +49,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.5 Done" sheetId="40" state="visible" r:id="rId40"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.6 Done" sheetId="41" state="visible" r:id="rId41"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.7 Done" sheetId="42" state="visible" r:id="rId42"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.8 Plan" sheetId="43" state="visible" r:id="rId43"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Data Models Gap'!$A$1:$K$40</definedName>
@@ -66,7 +67,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="90">
+  <fonts count="92">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -674,8 +675,18 @@
       <b val="1"/>
       <color rgb="00006100"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="61">
+  <fills count="62">
     <fill>
       <patternFill/>
     </fill>
@@ -1025,6 +1036,11 @@
         <bgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFF00"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="6">
     <border>
@@ -1096,7 +1112,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="428">
+  <cellXfs count="431">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -2331,6 +2347,15 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="89" fillId="60" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="90" fillId="41" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="91" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="91" fillId="61" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -8085,10 +8110,10 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="A5:G5"/>
     <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:G1"/>
     <mergeCell ref="A12:F12"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A5:G5"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -20574,6 +20599,324 @@
       <c r="G11" s="427" t="inlineStr">
         <is>
           <t>Done</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" style="186" min="1" max="1"/>
+    <col width="16" customWidth="1" style="186" min="2" max="2"/>
+    <col width="80" customWidth="1" style="186" min="3" max="3"/>
+    <col width="30" customWidth="1" style="186" min="4" max="4"/>
+    <col width="14" customWidth="1" style="186" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="428" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="B1" s="428" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="C1" s="428" t="inlineStr">
+        <is>
+          <t>Deliverables</t>
+        </is>
+      </c>
+      <c r="D1" s="428" t="inlineStr">
+        <is>
+          <t>Skills Applied</t>
+        </is>
+      </c>
+      <c r="E1" s="428" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="429" t="inlineStr">
+        <is>
+          <t>AR</t>
+        </is>
+      </c>
+      <c r="B2" s="429" t="inlineStr">
+        <is>
+          <t>CTO</t>
+        </is>
+      </c>
+      <c r="C2" s="429" t="inlineStr">
+        <is>
+          <t>E-Signature Workflow Engine v2: envelope lifecycle, template manager, signing ceremony, audit trail, esignature-api (15+ endpoints)</t>
+        </is>
+      </c>
+      <c r="D2" s="429" t="inlineStr">
+        <is>
+          <t>backend-patterns, security-review</t>
+        </is>
+      </c>
+      <c r="E2" s="430" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="429" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="B3" s="429" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C3" s="429" t="inlineStr">
+        <is>
+          <t>E-Signature Dashboard (overview, envelopes, templates pages) + Healthcare Dashboard (overview, patients, records pages) + hooks</t>
+        </is>
+      </c>
+      <c r="D3" s="429" t="inlineStr">
+        <is>
+          <t>frontend-patterns</t>
+        </is>
+      </c>
+      <c r="E3" s="430" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="429" t="inlineStr">
+        <is>
+          <t>NK</t>
+        </is>
+      </c>
+      <c r="B4" s="429" t="inlineStr">
+        <is>
+          <t>Frontend Lead</t>
+        </is>
+      </c>
+      <c r="C4" s="429" t="inlineStr">
+        <is>
+          <t>Analytics Dashboard (overview, reports, dashboards pages) + Supply Chain Dashboard (overview, inventory, orders pages) + hooks</t>
+        </is>
+      </c>
+      <c r="D4" s="429" t="inlineStr">
+        <is>
+          <t>frontend-patterns</t>
+        </is>
+      </c>
+      <c r="E4" s="430" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="429" t="inlineStr">
+        <is>
+          <t>RG</t>
+        </is>
+      </c>
+      <c r="B5" s="429" t="inlineStr">
+        <is>
+          <t>Backend Lead</t>
+        </is>
+      </c>
+      <c r="C5" s="429" t="inlineStr">
+        <is>
+          <t>DocuSign v2 SDK (OAuth2+JWT, envelopes, templates, signing, webhooks) + Adobe Sign v2 SDK + PandaDoc v2 SDK</t>
+        </is>
+      </c>
+      <c r="D5" s="429" t="inlineStr">
+        <is>
+          <t>api-design, security-review</t>
+        </is>
+      </c>
+      <c r="E5" s="430" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="429" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="B6" s="429" t="inlineStr">
+        <is>
+          <t>Full-stack</t>
+        </is>
+      </c>
+      <c r="C6" s="429" t="inlineStr">
+        <is>
+          <t>Epic FHIR v2 SDK (SMART on FHIR, R4 resources) + Cerner FHIR v2 SDK + Allscripts FHIR v2 SDK</t>
+        </is>
+      </c>
+      <c r="D6" s="429" t="inlineStr">
+        <is>
+          <t>backend-patterns, security-review</t>
+        </is>
+      </c>
+      <c r="E6" s="430" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="429" t="inlineStr">
+        <is>
+          <t>VS</t>
+        </is>
+      </c>
+      <c r="B7" s="429" t="inlineStr">
+        <is>
+          <t>Component Dev</t>
+        </is>
+      </c>
+      <c r="C7" s="429" t="inlineStr">
+        <is>
+          <t>8+ UI components: signature-pad, envelope-timeline, patient-card, vitals-chart, analytics-widget, report-builder, inventory-gauge, fulfillment-tracker</t>
+        </is>
+      </c>
+      <c r="D7" s="429" t="inlineStr">
+        <is>
+          <t>frontend-patterns</t>
+        </is>
+      </c>
+      <c r="E7" s="430" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="429" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="B8" s="429" t="inlineStr">
+        <is>
+          <t>Sr. Backend</t>
+        </is>
+      </c>
+      <c r="C8" s="429" t="inlineStr">
+        <is>
+          <t>Healthcare Interop Engine (FHIR R4, HL7v2 parser, clinical normalizer) + Supply Chain Orchestration Engine (demand planner, inventory optimizer, fulfillment engine)</t>
+        </is>
+      </c>
+      <c r="D8" s="429" t="inlineStr">
+        <is>
+          <t>backend-patterns</t>
+        </is>
+      </c>
+      <c r="E8" s="430" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="429" t="inlineStr">
+        <is>
+          <t>KS</t>
+        </is>
+      </c>
+      <c r="B9" s="429" t="inlineStr">
+        <is>
+          <t>QA Lead</t>
+        </is>
+      </c>
+      <c r="C9" s="429" t="inlineStr">
+        <is>
+          <t>3 e-sig integration tests + 3 healthcare tests + 2 analytics tests + 2 supply chain tests + 2 E2E tests + fixtures</t>
+        </is>
+      </c>
+      <c r="D9" s="429" t="inlineStr">
+        <is>
+          <t>e2e-testing, tdd-workflow</t>
+        </is>
+      </c>
+      <c r="E9" s="430" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="429" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="B10" s="429" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="C10" s="429" t="inlineStr">
+        <is>
+          <t>Tableau v2 SDK + Power BI v2 SDK + Manhattan WMS v2 SDK + Blue Yonder v2 SDK + Looker v2 + Qlik v2</t>
+        </is>
+      </c>
+      <c r="D10" s="429" t="inlineStr">
+        <is>
+          <t>api-design, security-review</t>
+        </is>
+      </c>
+      <c r="E10" s="430" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="429" t="inlineStr">
+        <is>
+          <t>ZR</t>
+        </is>
+      </c>
+      <c r="B11" s="429" t="inlineStr">
+        <is>
+          <t>AI Engineer</t>
+        </is>
+      </c>
+      <c r="C11" s="429" t="inlineStr">
+        <is>
+          <t>AI Document Intelligence + Clinical Decision Support + Analytics Anomaly Detector + Supply Chain Demand Forecaster + API (12+ endpoints)</t>
+        </is>
+      </c>
+      <c r="D11" s="429" t="inlineStr">
+        <is>
+          <t>backend-patterns</t>
+        </is>
+      </c>
+      <c r="E11" s="430" t="inlineStr">
+        <is>
+          <t>In Progress</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(sprint-8.9): plan integration hardening & final testing sprint
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/witylogix-sprint-tracker.xlsx
+++ b/witylogix-sprint-tracker.xlsx
@@ -50,6 +50,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.6 Done" sheetId="41" state="visible" r:id="rId41"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.7 Done" sheetId="42" state="visible" r:id="rId42"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.8 Done" sheetId="43" state="visible" r:id="rId43"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 8.9 Plan" sheetId="44" state="visible" r:id="rId44"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Data Models Gap'!$A$1:$K$40</definedName>
@@ -8118,9 +8119,9 @@
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A12:F12"/>
+    <mergeCell ref="A1:G1"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -20925,6 +20926,324 @@
       <c r="E11" s="431" t="inlineStr">
         <is>
           <t>Done</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" style="186" min="1" max="1"/>
+    <col width="16" customWidth="1" style="186" min="2" max="2"/>
+    <col width="80" customWidth="1" style="186" min="3" max="3"/>
+    <col width="30" customWidth="1" style="186" min="4" max="4"/>
+    <col width="14" customWidth="1" style="186" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="428" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="B1" s="428" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="C1" s="428" t="inlineStr">
+        <is>
+          <t>Deliverables</t>
+        </is>
+      </c>
+      <c r="D1" s="428" t="inlineStr">
+        <is>
+          <t>Skills Applied</t>
+        </is>
+      </c>
+      <c r="E1" s="428" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="429" t="inlineStr">
+        <is>
+          <t>AR</t>
+        </is>
+      </c>
+      <c r="B2" s="429" t="inlineStr">
+        <is>
+          <t>CTO</t>
+        </is>
+      </c>
+      <c r="C2" s="429" t="inlineStr">
+        <is>
+          <t>Integration Gateway v2 (advanced circuit breaker half-open/sliding window, bulkhead, retry with jitter, request dedup, response cache, correlation IDs) + Webhook Management Engine (registry, delivery queue DLQ, HMAC/RSA/JWT verification, replay protection, fan-out, analytics) + gateway-v2-api (15+ endpoints)</t>
+        </is>
+      </c>
+      <c r="D2" s="429" t="inlineStr">
+        <is>
+          <t>backend-patterns, security-review</t>
+        </is>
+      </c>
+      <c r="E2" s="430" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="429" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="B3" s="429" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C3" s="429" t="inlineStr">
+        <is>
+          <t>Integration Health Center: overview (provider grid, aggregate health, error trends), provider detail (latency p50/p95/p99, SLA tracking, incident history), webhook monitor (delivery log, DLQ viewer, retry controls), credential manager (rotation schedule, vault status, expiry alerts)</t>
+        </is>
+      </c>
+      <c r="D3" s="429" t="inlineStr">
+        <is>
+          <t>frontend-patterns</t>
+        </is>
+      </c>
+      <c r="E3" s="430" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="429" t="inlineStr">
+        <is>
+          <t>NK</t>
+        </is>
+      </c>
+      <c r="B4" s="429" t="inlineStr">
+        <is>
+          <t>Frontend Lead</t>
+        </is>
+      </c>
+      <c r="C4" s="429" t="inlineStr">
+        <is>
+          <t>Chaos Testing Dashboard (scenario builder, execution monitor, results viewer) + Migration Wizard (provider swap steps, shadow mode toggle, rollback controls) + Docs Portal (SDK reference browser, webhook catalog, troubleshooting search)</t>
+        </is>
+      </c>
+      <c r="D4" s="429" t="inlineStr">
+        <is>
+          <t>frontend-patterns</t>
+        </is>
+      </c>
+      <c r="E4" s="430" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="429" t="inlineStr">
+        <is>
+          <t>RG</t>
+        </is>
+      </c>
+      <c r="B5" s="429" t="inlineStr">
+        <is>
+          <t>Backend Lead</t>
+        </is>
+      </c>
+      <c r="C5" s="429" t="inlineStr">
+        <is>
+          <t>Credential Lifecycle Manager: rotation scheduler (time/event-based, per-provider), secret scanner (regex+entropy detection), multi-vault adapter (AWS SM, HashiCorp Vault, Azure KV), zero-downtime rotation (dual-credential window), credential health scoring (age, exposure, rotation compliance)</t>
+        </is>
+      </c>
+      <c r="D5" s="429" t="inlineStr">
+        <is>
+          <t>api-design, security-review</t>
+        </is>
+      </c>
+      <c r="E5" s="430" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="429" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="B6" s="429" t="inlineStr">
+        <is>
+          <t>Full-stack</t>
+        </is>
+      </c>
+      <c r="C6" s="429" t="inlineStr">
+        <is>
+          <t>Integration Health Monitor: real-time tracker (per-provider status, uptime), SLA monitor (target vs actual, breach alerts), latency histogram (p50/p95/p99 per provider), error trending (rate, classification, correlation), degradation detector (anomaly-based auto-alert), alerting engine (Slack/email/PagerDuty)</t>
+        </is>
+      </c>
+      <c r="D6" s="429" t="inlineStr">
+        <is>
+          <t>backend-patterns</t>
+        </is>
+      </c>
+      <c r="E6" s="430" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="429" t="inlineStr">
+        <is>
+          <t>VS</t>
+        </is>
+      </c>
+      <c r="B7" s="429" t="inlineStr">
+        <is>
+          <t>Component Dev</t>
+        </is>
+      </c>
+      <c r="C7" s="429" t="inlineStr">
+        <is>
+          <t>8+ UI components: health-status-card (3-state with history sparkline), latency-sparkline (p50/p95/p99 overlay), webhook-delivery-chart (success/fail/pending), circuit-breaker-visualizer (SVG state machine), chaos-scenario-card (inject/observe/validate), migration-progress-bar (multi-step with rollback), credential-rotation-timeline (upcoming/completed/overdue), sla-badge (target vs actual)</t>
+        </is>
+      </c>
+      <c r="D7" s="429" t="inlineStr">
+        <is>
+          <t>frontend-patterns</t>
+        </is>
+      </c>
+      <c r="E7" s="430" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="429" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="B8" s="429" t="inlineStr">
+        <is>
+          <t>Sr. Backend</t>
+        </is>
+      </c>
+      <c r="C8" s="429" t="inlineStr">
+        <is>
+          <t>Integration Test Harness (mock server framework, VCR-style fixture recording/playback, contract testing, SDK compat matrix, regression runner) + Chaos Testing Engine (latency/error/timeout/partial-failure injection, provider failover, circuit breaker validation, rate limit stress)</t>
+        </is>
+      </c>
+      <c r="D8" s="429" t="inlineStr">
+        <is>
+          <t>backend-patterns, e2e-testing</t>
+        </is>
+      </c>
+      <c r="E8" s="430" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="429" t="inlineStr">
+        <is>
+          <t>KS</t>
+        </is>
+      </c>
+      <c r="B9" s="429" t="inlineStr">
+        <is>
+          <t>QA Lead</t>
+        </is>
+      </c>
+      <c r="C9" s="429" t="inlineStr">
+        <is>
+          <t>3 gateway v2 tests + 3 webhook tests + 2 credential tests + 2 health monitor tests + 2 chaos tests + 2 migration tests + 2 E2E tests + 3 fixture files</t>
+        </is>
+      </c>
+      <c r="D9" s="429" t="inlineStr">
+        <is>
+          <t>e2e-testing, tdd-workflow</t>
+        </is>
+      </c>
+      <c r="E9" s="430" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="429" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="B10" s="429" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="C10" s="429" t="inlineStr">
+        <is>
+          <t>Migration Toolkit (provider swap engine, data mapper, shadow mode, rollback, validation) + Documentation Engine (auto-doc generator from SDK metadata, webhook event catalog, rate limit reference, troubleshooting playbooks)</t>
+        </is>
+      </c>
+      <c r="D10" s="429" t="inlineStr">
+        <is>
+          <t>api-design, deployment-patterns</t>
+        </is>
+      </c>
+      <c r="E10" s="430" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="429" t="inlineStr">
+        <is>
+          <t>ZR</t>
+        </is>
+      </c>
+      <c r="B11" s="429" t="inlineStr">
+        <is>
+          <t>AI Engineer</t>
+        </is>
+      </c>
+      <c r="C11" s="429" t="inlineStr">
+        <is>
+          <t>AI Integration Intelligence: anomaly detector (multi-signal — latency/errors/volume), auto-remediation recommender (circuit break/failover/throttle/retry), capacity planner (growth projection, provider limit forecasting), SLA predictor (breach probability), cost optimizer (provider cost comparison, routing optimization), API (12+ endpoints)</t>
+        </is>
+      </c>
+      <c r="D11" s="429" t="inlineStr">
+        <is>
+          <t>backend-patterns</t>
+        </is>
+      </c>
+      <c r="E11" s="430" t="inlineStr">
+        <is>
+          <t>In Progress</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: update nightly run report for 2026-03-18 (Run 4)
- 40+ TypeScript errors fixed in core/ai modules
- Prisma build path resolved with custom output directory
- Sprint 8.x roadmap status updated to Done
- Sprint tracker standup notes updated

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/witylogix-sprint-tracker.xlsx
+++ b/witylogix-sprint-tracker.xlsx
@@ -68,7 +68,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="92">
+  <fonts count="93">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -686,6 +686,9 @@
       <name val="Arial"/>
       <sz val="10"/>
     </font>
+    <font>
+      <color rgb="00008000"/>
+    </font>
   </fonts>
   <fills count="63">
     <fill>
@@ -1118,7 +1121,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="432">
+  <cellXfs count="433">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -2367,6 +2370,7 @@
     <xf numFmtId="0" fontId="91" fillId="62" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="92" fillId="55" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -6614,7 +6618,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G126"/>
+  <dimension ref="A1:G127"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="25" customWidth="1" style="185" min="1" max="2"/>
@@ -8117,12 +8121,34 @@
         </is>
       </c>
     </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Nightly Agent (Run 4)</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Priority 1: All tests pass (885 tests across 7 packages). Prisma build fixed (custom output path). Turbo spawn issue noted (macOS node_modules on Linux env). Priority 2: No actionable sprint tasks — all sprints through 8.9 complete. Priority 3: Fixed 40+ TypeScript errors in core/ai modules (delivery-predictor, notification-timer, compliance-risk-scorer, fuel-optimizer, demand-forecaster, document-intelligence, ai/index.ts barrel). DB imports migrated to generated Prisma client path.</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>[BLOCKER] Turbo --force spawn fails due to cross-platform node_modules (macOS→Linux). [NOTE] Sprint 8.x Roadmap status column updated from Planned→Done.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A12:F12"/>
     <mergeCell ref="A5:G5"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A12:F12"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -16795,9 +16821,9 @@
           <t>Credential vault, OAuth2 manager, webhook verifier, marketplace UI, Stripe/Shopify/Twilio/SendGrid SDKs</t>
         </is>
       </c>
-      <c r="F2" s="418" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="F2" s="432" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -16827,9 +16853,9 @@
           <t>Google Routes + Mapbox SDKs, live map, Samsara/Geotab SDKs, route optimization</t>
         </is>
       </c>
-      <c r="F3" s="418" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="F3" s="432" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -16859,9 +16885,9 @@
           <t>EasyPost/ShipStation SDKs, FedEx/UPS OAuth2, DoorDash Drive, rate engine</t>
         </is>
       </c>
-      <c r="F4" s="418" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="F4" s="432" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -16891,9 +16917,9 @@
           <t>BigCommerce/Amazon SP-API, order sync v2, inventory reconciliation</t>
         </is>
       </c>
-      <c r="F5" s="418" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="F5" s="432" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -16923,9 +16949,9 @@
           <t>Salesforce/HubSpot/QuickBooks/Xero SDKs, CRM sync v3, invoice sync</t>
         </is>
       </c>
-      <c r="F6" s="418" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="F6" s="432" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -16955,9 +16981,9 @@
           <t>Slack/Teams/WhatsApp/FCM SDKs, notification orchestrator</t>
         </is>
       </c>
-      <c r="F7" s="418" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="F7" s="432" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -16987,9 +17013,9 @@
           <t>DAT/Truckstop APIs, Motive/Samsara ELD, HOS compliance</t>
         </is>
       </c>
-      <c r="F8" s="418" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="F8" s="432" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -17019,9 +17045,9 @@
           <t>WEX/Comdata, ServiceTitan/Jobber/Toast POS</t>
         </is>
       </c>
-      <c r="F9" s="418" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="F9" s="432" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -17051,9 +17077,9 @@
           <t>DocuSign, FHIR, Tableau/PowerBI, Manhattan/Blue Yonder</t>
         </is>
       </c>
-      <c r="F10" s="418" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="F10" s="432" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -17083,9 +17109,9 @@
           <t>125/125 provider tests, rate limit audit, health dashboard, docs portal</t>
         </is>
       </c>
-      <c r="F11" s="418" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="F11" s="432" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(sprint-9.0): add sprint summary, update README and tracker
- Sprint 9.0 summary with agent contributions, stats, and key decisions
- README: add i18n and Order Kanban board to key capabilities
- Sprint tracker: 10 new rows for Sprint 9.0 agent tasks

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/witylogix-sprint-tracker.xlsx
+++ b/witylogix-sprint-tracker.xlsx
@@ -68,7 +68,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="93">
+  <fonts count="94">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -689,6 +689,11 @@
     <font>
       <color rgb="00008000"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00006100"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="63">
     <fill>
@@ -1121,7 +1126,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="433">
+  <cellXfs count="435">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -2371,6 +2376,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="92" fillId="55" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="91" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="93" fillId="59" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -6618,7 +6629,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G127"/>
+  <dimension ref="A1:G128"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="25" customWidth="1" style="185" min="1" max="2"/>
@@ -8122,33 +8133,60 @@
       </c>
     </row>
     <row r="127">
-      <c r="A127" t="inlineStr">
+      <c r="A127" s="185" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
       </c>
-      <c r="B127" t="inlineStr">
+      <c r="B127" s="185" t="inlineStr">
         <is>
           <t>Nightly Agent (Run 4)</t>
         </is>
       </c>
-      <c r="C127" t="inlineStr">
+      <c r="C127" s="185" t="inlineStr">
         <is>
           <t>Priority 1: All tests pass (885 tests across 7 packages). Prisma build fixed (custom output path). Turbo spawn issue noted (macOS node_modules on Linux env). Priority 2: No actionable sprint tasks — all sprints through 8.9 complete. Priority 3: Fixed 40+ TypeScript errors in core/ai modules (delivery-predictor, notification-timer, compliance-risk-scorer, fuel-optimizer, demand-forecaster, document-intelligence, ai/index.ts barrel). DB imports migrated to generated Prisma client path.</t>
         </is>
       </c>
-      <c r="D127" t="inlineStr">
+      <c r="D127" s="185" t="inlineStr">
         <is>
           <t>[BLOCKER] Turbo --force spawn fails due to cross-platform node_modules (macOS→Linux). [NOTE] Sprint 8.x Roadmap status column updated from Planned→Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="185" t="inlineStr">
+        <is>
+          <t>2026-03-18 (Run 5)</t>
+        </is>
+      </c>
+      <c r="B128" s="185" t="inlineStr">
+        <is>
+          <t>Nightly Bot</t>
+        </is>
+      </c>
+      <c r="C128" s="185" t="inlineStr">
+        <is>
+          <t>Fixed 2 test regressions in registry.test.ts (concurrent adapter request race condition). Fixed stale pnpm shim + 8 broken symlinks from prior session. 1,000+ tests passing across 9 packages. Sprint 8.9 all Done, no todo tasks in any sprint.</t>
+        </is>
+      </c>
+      <c r="D128" s="185" t="inlineStr">
+        <is>
+          <t>[BLOCKER] Git index.lock cannot be removed (EPERM). Commit 6737698 saved in local clone, pending push. No GitHub credentials available.</t>
+        </is>
+      </c>
+      <c r="E128" s="185" t="inlineStr">
+        <is>
+          <t>Push commit 6737698 to remote. Create Sprint 9.0. Resolve git lock files.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="A5:G5"/>
+    <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A2:G2"/>
     <mergeCell ref="A12:F12"/>
-    <mergeCell ref="A5:G5"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -26222,7 +26260,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J66"/>
+  <dimension ref="A1:J76"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.66796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="25" customWidth="1" style="185" min="1" max="1"/>
@@ -29264,6 +29302,376 @@
       <c r="D66" s="269" t="inlineStr">
         <is>
           <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="433" t="inlineStr">
+        <is>
+          <t>9.0</t>
+        </is>
+      </c>
+      <c r="B67" s="433" t="inlineStr">
+        <is>
+          <t>AR</t>
+        </is>
+      </c>
+      <c r="C67" s="433" t="inlineStr">
+        <is>
+          <t>CTO</t>
+        </is>
+      </c>
+      <c r="D67" s="433" t="inlineStr">
+        <is>
+          <t>Auth types duplicate fix + test migration</t>
+        </is>
+      </c>
+      <c r="E67" s="433" t="inlineStr">
+        <is>
+          <t>tdd-workflow</t>
+        </is>
+      </c>
+      <c r="F67" s="434" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G67" s="433" t="inlineStr">
+        <is>
+          <t>auth/types.ts, 5 auth test files</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="433" t="inlineStr">
+        <is>
+          <t>9.0</t>
+        </is>
+      </c>
+      <c r="B68" s="433" t="inlineStr">
+        <is>
+          <t>RG</t>
+        </is>
+      </c>
+      <c r="C68" s="433" t="inlineStr">
+        <is>
+          <t>Backend Lead</t>
+        </is>
+      </c>
+      <c r="D68" s="433" t="inlineStr">
+        <is>
+          <t>Queue &amp; monitoring test fixes</t>
+        </is>
+      </c>
+      <c r="E68" s="433" t="inlineStr">
+        <is>
+          <t>tdd-workflow</t>
+        </is>
+      </c>
+      <c r="F68" s="434" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G68" s="433" t="inlineStr">
+        <is>
+          <t>queue tests (79→35), monitoring (58→6)</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="433" t="inlineStr">
+        <is>
+          <t>9.0</t>
+        </is>
+      </c>
+      <c r="B69" s="433" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="C69" s="433" t="inlineStr">
+        <is>
+          <t>Sr. Backend</t>
+        </is>
+      </c>
+      <c r="D69" s="433" t="inlineStr">
+        <is>
+          <t>Notifications &amp; onboarding test fixes</t>
+        </is>
+      </c>
+      <c r="E69" s="433" t="inlineStr">
+        <is>
+          <t>tdd-workflow</t>
+        </is>
+      </c>
+      <c r="F69" s="434" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G69" s="433" t="inlineStr">
+        <is>
+          <t>notifications (40→20), onboarding mock fixes</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="433" t="inlineStr">
+        <is>
+          <t>9.0</t>
+        </is>
+      </c>
+      <c r="B70" s="433" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="C70" s="433" t="inlineStr">
+        <is>
+          <t>Full-stack</t>
+        </is>
+      </c>
+      <c r="D70" s="433" t="inlineStr">
+        <is>
+          <t>Platform bridge &amp; auth test migration</t>
+        </is>
+      </c>
+      <c r="E70" s="433" t="inlineStr">
+        <is>
+          <t>tdd-workflow</t>
+        </is>
+      </c>
+      <c r="F70" s="434" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G70" s="433" t="inlineStr">
+        <is>
+          <t>data-normalizer, webhook-normalizer, sso, password</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="433" t="inlineStr">
+        <is>
+          <t>9.0</t>
+        </is>
+      </c>
+      <c r="B71" s="433" t="inlineStr">
+        <is>
+          <t>NK</t>
+        </is>
+      </c>
+      <c r="C71" s="433" t="inlineStr">
+        <is>
+          <t>Frontend Lead</t>
+        </is>
+      </c>
+      <c r="D71" s="433" t="inlineStr">
+        <is>
+          <t>i18n foundation — 4 locales, 120+ keys</t>
+        </is>
+      </c>
+      <c r="E71" s="433" t="inlineStr">
+        <is>
+          <t>frontend-patterns</t>
+        </is>
+      </c>
+      <c r="F71" s="434" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G71" s="433" t="inlineStr">
+        <is>
+          <t>i18n/index.ts, en/es/fr/ar.json, 44 tests</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="433" t="inlineStr">
+        <is>
+          <t>9.0</t>
+        </is>
+      </c>
+      <c r="B72" s="433" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="C72" s="433" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="D72" s="433" t="inlineStr">
+        <is>
+          <t>Order Kanban board — drag-and-drop</t>
+        </is>
+      </c>
+      <c r="E72" s="433" t="inlineStr">
+        <is>
+          <t>frontend-patterns</t>
+        </is>
+      </c>
+      <c r="F72" s="434" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G72" s="433" t="inlineStr">
+        <is>
+          <t>orders/board/page.tsx (453 lines)</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="433" t="inlineStr">
+        <is>
+          <t>9.0</t>
+        </is>
+      </c>
+      <c r="B73" s="433" t="inlineStr">
+        <is>
+          <t>VS</t>
+        </is>
+      </c>
+      <c r="C73" s="433" t="inlineStr">
+        <is>
+          <t>Component Dev</t>
+        </is>
+      </c>
+      <c r="D73" s="433" t="inlineStr">
+        <is>
+          <t>Kanban card &amp; column components</t>
+        </is>
+      </c>
+      <c r="E73" s="433" t="inlineStr">
+        <is>
+          <t>frontend-patterns</t>
+        </is>
+      </c>
+      <c r="F73" s="434" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G73" s="433" t="inlineStr">
+        <is>
+          <t>kanban-card.tsx, kanban-column.tsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="433" t="inlineStr">
+        <is>
+          <t>9.0</t>
+        </is>
+      </c>
+      <c r="B74" s="433" t="inlineStr">
+        <is>
+          <t>KS</t>
+        </is>
+      </c>
+      <c r="C74" s="433" t="inlineStr">
+        <is>
+          <t>QA Lead</t>
+        </is>
+      </c>
+      <c r="D74" s="433" t="inlineStr">
+        <is>
+          <t>Demand-prediction &amp; compliance test fixes</t>
+        </is>
+      </c>
+      <c r="E74" s="433" t="inlineStr">
+        <is>
+          <t>tdd-workflow</t>
+        </is>
+      </c>
+      <c r="F74" s="434" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G74" s="433" t="inlineStr">
+        <is>
+          <t>demand-prediction (62→60), compliance tests</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="433" t="inlineStr">
+        <is>
+          <t>9.0</t>
+        </is>
+      </c>
+      <c r="B75" s="433" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="C75" s="433" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="D75" s="433" t="inlineStr">
+        <is>
+          <t>Integration test migration (couriers, ecommerce)</t>
+        </is>
+      </c>
+      <c r="E75" s="433" t="inlineStr">
+        <is>
+          <t>tdd-workflow</t>
+        </is>
+      </c>
+      <c r="F75" s="434" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G75" s="433" t="inlineStr">
+        <is>
+          <t>couriers, ecommerce, gateway test fixes</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="433" t="inlineStr">
+        <is>
+          <t>9.0</t>
+        </is>
+      </c>
+      <c r="B76" s="433" t="inlineStr">
+        <is>
+          <t>ZR</t>
+        </is>
+      </c>
+      <c r="C76" s="433" t="inlineStr">
+        <is>
+          <t>AI Engineer</t>
+        </is>
+      </c>
+      <c r="D76" s="433" t="inlineStr">
+        <is>
+          <t>AI module test analysis &amp; fixes</t>
+        </is>
+      </c>
+      <c r="E76" s="433" t="inlineStr">
+        <is>
+          <t>tdd-workflow</t>
+        </is>
+      </c>
+      <c r="F76" s="434" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G76" s="433" t="inlineStr">
+        <is>
+          <t>AI test pattern identification</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(sprint-9.1): returns/RMA engine, driver scoring, email templates & live dispatch
Sprint 9.1 delivers four major features:

- Returns/RMA: 8-state lifecycle, refund calculator, restocking fees,
  9 API endpoints, management dashboard, event bus integration with
  6 domain events and workflow handlers
- Driver scoring: weighted composite (0-100) across 5 metrics, tiers,
  exponential decay, AI predictor with regression/anomaly detection,
  leaderboard API + dashboard page
- Email templates: 6 responsive transactional templates with table-based
  layout, variable interpolation, currency/date formatting
- Live Dispatch Command Center: full-screen 40/60 split with order queue,
  driver grid, urgency filters, one-click assignment

~7,700 new source lines, 1,510 test lines, 13 new API endpoints,
3 new dashboard pages, 3 new core modules.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/witylogix-sprint-tracker.xlsx
+++ b/witylogix-sprint-tracker.xlsx
@@ -695,7 +695,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="63">
+  <fills count="64">
     <fill>
       <patternFill/>
     </fill>
@@ -1055,6 +1055,11 @@
         <fgColor rgb="0000B050"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8F5E9"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="6">
     <border>
@@ -1126,7 +1131,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="435">
+  <cellXfs count="436">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -2380,6 +2385,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="93" fillId="59" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="91" fillId="63" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -8183,10 +8191,10 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A12:F12"/>
     <mergeCell ref="A5:G5"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A12:F12"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -26260,7 +26268,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J76"/>
+  <dimension ref="A1:J86"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.66796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="25" customWidth="1" style="185" min="1" max="1"/>
@@ -29672,6 +29680,376 @@
       <c r="G76" s="433" t="inlineStr">
         <is>
           <t>AI test pattern identification</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="435" t="inlineStr">
+        <is>
+          <t>9.1</t>
+        </is>
+      </c>
+      <c r="B77" s="435" t="inlineStr">
+        <is>
+          <t>AR</t>
+        </is>
+      </c>
+      <c r="C77" s="435" t="inlineStr">
+        <is>
+          <t>CTO</t>
+        </is>
+      </c>
+      <c r="D77" s="435" t="inlineStr">
+        <is>
+          <t>Returns/RMA core service — types, status machine, refund calculator</t>
+        </is>
+      </c>
+      <c r="E77" s="435" t="inlineStr">
+        <is>
+          <t>backend-patterns</t>
+        </is>
+      </c>
+      <c r="F77" s="435" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G77" s="435" t="inlineStr">
+        <is>
+          <t>packages/core/src/returns/ (5 files, ~1040 lines)</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="435" t="inlineStr">
+        <is>
+          <t>9.1</t>
+        </is>
+      </c>
+      <c r="B78" s="435" t="inlineStr">
+        <is>
+          <t>RG</t>
+        </is>
+      </c>
+      <c r="C78" s="435" t="inlineStr">
+        <is>
+          <t>Backend Lead</t>
+        </is>
+      </c>
+      <c r="D78" s="435" t="inlineStr">
+        <is>
+          <t>Returns API routes — CRUD + lifecycle endpoints</t>
+        </is>
+      </c>
+      <c r="E78" s="435" t="inlineStr">
+        <is>
+          <t>api-design</t>
+        </is>
+      </c>
+      <c r="F78" s="435" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G78" s="435" t="inlineStr">
+        <is>
+          <t>apps/api/src/routes/returns.ts (~330 lines, 9 endpoints)</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="435" t="inlineStr">
+        <is>
+          <t>9.1</t>
+        </is>
+      </c>
+      <c r="B79" s="435" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="C79" s="435" t="inlineStr">
+        <is>
+          <t>Sr. Backend</t>
+        </is>
+      </c>
+      <c r="D79" s="435" t="inlineStr">
+        <is>
+          <t>Driver performance scoring engine — weighted metrics, tiers, decay</t>
+        </is>
+      </c>
+      <c r="E79" s="435" t="inlineStr">
+        <is>
+          <t>backend-patterns</t>
+        </is>
+      </c>
+      <c r="F79" s="435" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G79" s="435" t="inlineStr">
+        <is>
+          <t>packages/core/src/driver-scoring/ (5 files, ~580 lines)</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="435" t="inlineStr">
+        <is>
+          <t>9.1</t>
+        </is>
+      </c>
+      <c r="B80" s="435" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="C80" s="435" t="inlineStr">
+        <is>
+          <t>Full-stack</t>
+        </is>
+      </c>
+      <c r="D80" s="435" t="inlineStr">
+        <is>
+          <t>Driver scoring API + leaderboard dashboard page</t>
+        </is>
+      </c>
+      <c r="E80" s="435" t="inlineStr">
+        <is>
+          <t>api-design</t>
+        </is>
+      </c>
+      <c r="F80" s="435" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G80" s="435" t="inlineStr">
+        <is>
+          <t>routes/driver-scoring.ts + drivers/performance/page.tsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="435" t="inlineStr">
+        <is>
+          <t>9.1</t>
+        </is>
+      </c>
+      <c r="B81" s="435" t="inlineStr">
+        <is>
+          <t>NK</t>
+        </is>
+      </c>
+      <c r="C81" s="435" t="inlineStr">
+        <is>
+          <t>Frontend Lead</t>
+        </is>
+      </c>
+      <c r="D81" s="435" t="inlineStr">
+        <is>
+          <t>Live Dispatch Command Center — split layout, order queue, driver grid</t>
+        </is>
+      </c>
+      <c r="E81" s="435" t="inlineStr">
+        <is>
+          <t>frontend-patterns</t>
+        </is>
+      </c>
+      <c r="F81" s="435" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G81" s="435" t="inlineStr">
+        <is>
+          <t>apps/dashboard/dispatch/page.tsx (~500 lines, full rewrite)</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="435" t="inlineStr">
+        <is>
+          <t>9.1</t>
+        </is>
+      </c>
+      <c r="B82" s="435" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="C82" s="435" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="D82" s="435" t="inlineStr">
+        <is>
+          <t>Returns Management dashboard — list, detail modal, action buttons</t>
+        </is>
+      </c>
+      <c r="E82" s="435" t="inlineStr">
+        <is>
+          <t>frontend-patterns</t>
+        </is>
+      </c>
+      <c r="F82" s="435" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G82" s="435" t="inlineStr">
+        <is>
+          <t>apps/dashboard/returns/page.tsx (~1048 lines)</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="435" t="inlineStr">
+        <is>
+          <t>9.1</t>
+        </is>
+      </c>
+      <c r="B83" s="435" t="inlineStr">
+        <is>
+          <t>VS</t>
+        </is>
+      </c>
+      <c r="C83" s="435" t="inlineStr">
+        <is>
+          <t>Component Dev</t>
+        </is>
+      </c>
+      <c r="D83" s="435" t="inlineStr">
+        <is>
+          <t>Transactional email templates — 6 responsive HTML templates</t>
+        </is>
+      </c>
+      <c r="E83" s="435" t="inlineStr">
+        <is>
+          <t>coding-standards</t>
+        </is>
+      </c>
+      <c r="F83" s="435" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G83" s="435" t="inlineStr">
+        <is>
+          <t>packages/core/src/email-templates/ (10 files)</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="435" t="inlineStr">
+        <is>
+          <t>9.1</t>
+        </is>
+      </c>
+      <c r="B84" s="435" t="inlineStr">
+        <is>
+          <t>KS</t>
+        </is>
+      </c>
+      <c r="C84" s="435" t="inlineStr">
+        <is>
+          <t>QA Lead</t>
+        </is>
+      </c>
+      <c r="D84" s="435" t="inlineStr">
+        <is>
+          <t>Tests for returns, scoring engine, and email templates</t>
+        </is>
+      </c>
+      <c r="E84" s="435" t="inlineStr">
+        <is>
+          <t>tdd-workflow</t>
+        </is>
+      </c>
+      <c r="F84" s="435" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G84" s="435" t="inlineStr">
+        <is>
+          <t>3 test files (~1510 lines total)</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="435" t="inlineStr">
+        <is>
+          <t>9.1</t>
+        </is>
+      </c>
+      <c r="B85" s="435" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="C85" s="435" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="D85" s="435" t="inlineStr">
+        <is>
+          <t>Returns event bus + workflow integration</t>
+        </is>
+      </c>
+      <c r="E85" s="435" t="inlineStr">
+        <is>
+          <t>backend-patterns</t>
+        </is>
+      </c>
+      <c r="F85" s="435" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G85" s="435" t="inlineStr">
+        <is>
+          <t>events.ts + return-workflow.ts (~582 lines)</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="435" t="inlineStr">
+        <is>
+          <t>9.1</t>
+        </is>
+      </c>
+      <c r="B86" s="435" t="inlineStr">
+        <is>
+          <t>ZR</t>
+        </is>
+      </c>
+      <c r="C86" s="435" t="inlineStr">
+        <is>
+          <t>AI Engineer</t>
+        </is>
+      </c>
+      <c r="D86" s="435" t="inlineStr">
+        <is>
+          <t>AI driver scoring — prediction, anomaly detection, satisfaction model</t>
+        </is>
+      </c>
+      <c r="E86" s="435" t="inlineStr">
+        <is>
+          <t>backend-patterns</t>
+        </is>
+      </c>
+      <c r="F86" s="435" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G86" s="435" t="inlineStr">
+        <is>
+          <t>ai-predictor.ts (~234 lines)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(sprint-9.2): dashboard API wiring — hooks, pages, UI components
Sprint 9.2 bridges the dashboard to the backend:
- Generic API hook infrastructure (useApiQuery/useApiList/useApiMutation)
- 7 typed domain hooks (orders, drivers, zones, customers, returns, stats)
- 5 critical pages rewired from mock data to real API calls
- UI components: LoadingSkeleton, ErrorState, DataTable, Pagination
- Dashboard layout with collapsible sidebar and breadcrumbs
- All 250 pages migrated to (dashboard) route group

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/witylogix-sprint-tracker.xlsx
+++ b/witylogix-sprint-tracker.xlsx
@@ -8191,9 +8191,9 @@
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A12:F12"/>
+    <mergeCell ref="A1:G1"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -26268,7 +26268,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J86"/>
+  <dimension ref="A1:J96"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.66796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="25" customWidth="1" style="185" min="1" max="1"/>
@@ -30050,6 +30050,376 @@
       <c r="G86" s="435" t="inlineStr">
         <is>
           <t>ai-predictor.ts (~234 lines)</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="435" t="inlineStr">
+        <is>
+          <t>9.2</t>
+        </is>
+      </c>
+      <c r="B87" s="435" t="inlineStr">
+        <is>
+          <t>AR</t>
+        </is>
+      </c>
+      <c r="C87" s="435" t="inlineStr">
+        <is>
+          <t>CTO</t>
+        </is>
+      </c>
+      <c r="D87" s="435" t="inlineStr">
+        <is>
+          <t>API hook infrastructure — useApiQuery, useApiList, useApiMutation</t>
+        </is>
+      </c>
+      <c r="E87" s="435" t="inlineStr">
+        <is>
+          <t>backend-patterns</t>
+        </is>
+      </c>
+      <c r="F87" s="435" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G87" s="435" t="inlineStr">
+        <is>
+          <t>hooks/use-api.ts (280 lines), lib/swr-config.tsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="435" t="inlineStr">
+        <is>
+          <t>9.2</t>
+        </is>
+      </c>
+      <c r="B88" s="435" t="inlineStr">
+        <is>
+          <t>RG</t>
+        </is>
+      </c>
+      <c r="C88" s="435" t="inlineStr">
+        <is>
+          <t>Backend Lead</t>
+        </is>
+      </c>
+      <c r="D88" s="435" t="inlineStr">
+        <is>
+          <t>7 typed domain hooks — orders, drivers, zones, customers, returns, stats</t>
+        </is>
+      </c>
+      <c r="E88" s="435" t="inlineStr">
+        <is>
+          <t>api-design</t>
+        </is>
+      </c>
+      <c r="F88" s="435" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G88" s="435" t="inlineStr">
+        <is>
+          <t>7 hook files (931 lines total)</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="435" t="inlineStr">
+        <is>
+          <t>9.2</t>
+        </is>
+      </c>
+      <c r="B89" s="435" t="inlineStr">
+        <is>
+          <t>NK</t>
+        </is>
+      </c>
+      <c r="C89" s="435" t="inlineStr">
+        <is>
+          <t>Frontend Lead</t>
+        </is>
+      </c>
+      <c r="D89" s="435" t="inlineStr">
+        <is>
+          <t>Rewire Home, Orders, Drivers pages to real API hooks</t>
+        </is>
+      </c>
+      <c r="E89" s="435" t="inlineStr">
+        <is>
+          <t>frontend-patterns</t>
+        </is>
+      </c>
+      <c r="F89" s="435" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G89" s="435" t="inlineStr">
+        <is>
+          <t>home/page.tsx, orders/page.tsx, drivers/page.tsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="435" t="inlineStr">
+        <is>
+          <t>9.2</t>
+        </is>
+      </c>
+      <c r="B90" s="435" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="C90" s="435" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="D90" s="435" t="inlineStr">
+        <is>
+          <t>Rewire Customers, Returns pages to real API hooks</t>
+        </is>
+      </c>
+      <c r="E90" s="435" t="inlineStr">
+        <is>
+          <t>frontend-patterns</t>
+        </is>
+      </c>
+      <c r="F90" s="435" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G90" s="435" t="inlineStr">
+        <is>
+          <t>customers/page.tsx, returns/page.tsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="435" t="inlineStr">
+        <is>
+          <t>9.2</t>
+        </is>
+      </c>
+      <c r="B91" s="435" t="inlineStr">
+        <is>
+          <t>VS</t>
+        </is>
+      </c>
+      <c r="C91" s="435" t="inlineStr">
+        <is>
+          <t>Component Dev</t>
+        </is>
+      </c>
+      <c r="D91" s="435" t="inlineStr">
+        <is>
+          <t>UI components — LoadingSkeleton, ErrorState, DataTable, Pagination</t>
+        </is>
+      </c>
+      <c r="E91" s="435" t="inlineStr">
+        <is>
+          <t>frontend-patterns</t>
+        </is>
+      </c>
+      <c r="F91" s="435" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G91" s="435" t="inlineStr">
+        <is>
+          <t>4 components (903 lines)</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="435" t="inlineStr">
+        <is>
+          <t>9.2</t>
+        </is>
+      </c>
+      <c r="B92" s="435" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="C92" s="435" t="inlineStr">
+        <is>
+          <t>Full-stack</t>
+        </is>
+      </c>
+      <c r="D92" s="435" t="inlineStr">
+        <is>
+          <t>Dashboard layout — collapsible sidebar, breadcrumbs, header</t>
+        </is>
+      </c>
+      <c r="E92" s="435" t="inlineStr">
+        <is>
+          <t>frontend-patterns</t>
+        </is>
+      </c>
+      <c r="F92" s="435" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G92" s="435" t="inlineStr">
+        <is>
+          <t>(dashboard)/layout.tsx (101 lines)</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="435" t="inlineStr">
+        <is>
+          <t>9.2</t>
+        </is>
+      </c>
+      <c r="B93" s="435" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="C93" s="435" t="inlineStr">
+        <is>
+          <t>Sr. Backend</t>
+        </is>
+      </c>
+      <c r="D93" s="435" t="inlineStr">
+        <is>
+          <t>Page migration to (dashboard) route group</t>
+        </is>
+      </c>
+      <c r="E93" s="435" t="inlineStr">
+        <is>
+          <t>coding-standards</t>
+        </is>
+      </c>
+      <c r="F93" s="435" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G93" s="435" t="inlineStr">
+        <is>
+          <t>All pages under (dashboard)/ route group</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="435" t="inlineStr">
+        <is>
+          <t>9.2</t>
+        </is>
+      </c>
+      <c r="B94" s="435" t="inlineStr">
+        <is>
+          <t>KS</t>
+        </is>
+      </c>
+      <c r="C94" s="435" t="inlineStr">
+        <is>
+          <t>QA Lead</t>
+        </is>
+      </c>
+      <c r="D94" s="435" t="inlineStr">
+        <is>
+          <t>Fix auth, navigation, and design system issues</t>
+        </is>
+      </c>
+      <c r="E94" s="435" t="inlineStr">
+        <is>
+          <t>tdd-workflow</t>
+        </is>
+      </c>
+      <c r="F94" s="435" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G94" s="435" t="inlineStr">
+        <is>
+          <t>auth-context, nav sidebar, design tokens</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="435" t="inlineStr">
+        <is>
+          <t>9.2</t>
+        </is>
+      </c>
+      <c r="B95" s="435" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="C95" s="435" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="D95" s="435" t="inlineStr">
+        <is>
+          <t>Standardize API type imports across dashboard</t>
+        </is>
+      </c>
+      <c r="E95" s="435" t="inlineStr">
+        <is>
+          <t>coding-standards</t>
+        </is>
+      </c>
+      <c r="F95" s="435" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G95" s="435" t="inlineStr">
+        <is>
+          <t>Fixed type imports across all pages</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="435" t="inlineStr">
+        <is>
+          <t>9.2</t>
+        </is>
+      </c>
+      <c r="B96" s="435" t="inlineStr">
+        <is>
+          <t>ZR</t>
+        </is>
+      </c>
+      <c r="C96" s="435" t="inlineStr">
+        <is>
+          <t>AI Engineer</t>
+        </is>
+      </c>
+      <c r="D96" s="435" t="inlineStr">
+        <is>
+          <t>Redis connection + Vite frontend compilation fixes</t>
+        </is>
+      </c>
+      <c r="E96" s="435" t="inlineStr">
+        <is>
+          <t>backend-patterns</t>
+        </is>
+      </c>
+      <c r="F96" s="435" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G96" s="435" t="inlineStr">
+        <is>
+          <t>redis.ts, vite config, react-router</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(sprint-9.3): tech debt blitz — route registration, hook rewiring, build stabilization
- Register 22 missing API routes in server.ts (39→61, 100% coverage)
- Rewrite 12 mock-data hooks to real API calls (5,958→1,457 lines, 76% reduction)
- Rewire ~28 dashboard pages from mock data to API hooks
- Fix dashboard build: delete stale .next, migrate admin to (dashboard), fix TS errors
- Consolidate duplicate UI components (card, dialog, badge, data-table)
- Create CI/CD pipeline (.github/workflows/ci.yml)
- Tech debt audit: 13 items across 5 categories, prioritized remediation plan

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/witylogix-sprint-tracker.xlsx
+++ b/witylogix-sprint-tracker.xlsx
@@ -68,7 +68,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="94">
+  <fonts count="95">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -694,6 +694,11 @@
       <color rgb="00006100"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="64">
     <fill>
@@ -1131,7 +1136,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="436">
+  <cellXfs count="438">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -2389,6 +2394,12 @@
     </xf>
     <xf numFmtId="0" fontId="91" fillId="63" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="94" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="93" fillId="59" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -8191,10 +8202,10 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="A5:G5"/>
     <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:G1"/>
     <mergeCell ref="A12:F12"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A5:G5"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -26268,7 +26279,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J96"/>
+  <dimension ref="A1:J106"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.66796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="25" customWidth="1" style="185" min="1" max="1"/>
@@ -30420,6 +30431,376 @@
       <c r="G96" s="435" t="inlineStr">
         <is>
           <t>redis.ts, vite config, react-router</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="436" t="inlineStr">
+        <is>
+          <t>9.3</t>
+        </is>
+      </c>
+      <c r="B97" s="429" t="inlineStr">
+        <is>
+          <t>AR</t>
+        </is>
+      </c>
+      <c r="C97" s="429" t="inlineStr">
+        <is>
+          <t>CTO</t>
+        </is>
+      </c>
+      <c r="D97" s="429" t="inlineStr">
+        <is>
+          <t>Register 22 missing API routes in server.ts</t>
+        </is>
+      </c>
+      <c r="E97" s="429" t="inlineStr">
+        <is>
+          <t>backend-patterns</t>
+        </is>
+      </c>
+      <c r="F97" s="437" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G97" s="429" t="inlineStr">
+        <is>
+          <t>22 routes: returns, driver-scoring, invoices, couriers, ecommerce, health, pod + 15 more</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="436" t="inlineStr">
+        <is>
+          <t>9.3</t>
+        </is>
+      </c>
+      <c r="B98" s="429" t="inlineStr">
+        <is>
+          <t>RG</t>
+        </is>
+      </c>
+      <c r="C98" s="429" t="inlineStr">
+        <is>
+          <t>Backend Lead</t>
+        </is>
+      </c>
+      <c r="D98" s="429" t="inlineStr">
+        <is>
+          <t>Rewrite 6 mock-data hooks batch 1 (fleet, notifications, field-service, pos, supply-chain, freight)</t>
+        </is>
+      </c>
+      <c r="E98" s="429" t="inlineStr">
+        <is>
+          <t>api-design</t>
+        </is>
+      </c>
+      <c r="F98" s="437" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G98" s="429" t="inlineStr">
+        <is>
+          <t>6 hooks: 3,496 → 749 lines (78% reduction)</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="436" t="inlineStr">
+        <is>
+          <t>9.3</t>
+        </is>
+      </c>
+      <c r="B99" s="429" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="C99" s="429" t="inlineStr">
+        <is>
+          <t>Sr. Backend</t>
+        </is>
+      </c>
+      <c r="D99" s="429" t="inlineStr">
+        <is>
+          <t>Rewrite 6 mock-data hooks batch 2 (healthcare, analytics, esignatures, eld, product-sync, financial-data)</t>
+        </is>
+      </c>
+      <c r="E99" s="429" t="inlineStr">
+        <is>
+          <t>api-design</t>
+        </is>
+      </c>
+      <c r="F99" s="437" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G99" s="429" t="inlineStr">
+        <is>
+          <t>6 hooks: 2,462 → 708 lines (71% reduction)</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="436" t="inlineStr">
+        <is>
+          <t>9.3</t>
+        </is>
+      </c>
+      <c r="B100" s="429" t="inlineStr">
+        <is>
+          <t>NK</t>
+        </is>
+      </c>
+      <c r="C100" s="429" t="inlineStr">
+        <is>
+          <t>Frontend Lead</t>
+        </is>
+      </c>
+      <c r="D100" s="429" t="inlineStr">
+        <is>
+          <t>Fix dashboard build — stale .next cleanup, admin migration, TS error fixes</t>
+        </is>
+      </c>
+      <c r="E100" s="429" t="inlineStr">
+        <is>
+          <t>frontend-patterns</t>
+        </is>
+      </c>
+      <c r="F100" s="437" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G100" s="429" t="inlineStr">
+        <is>
+          <t>Deleted .next, migrated 13 admin pages, fixed variant/type errors</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="436" t="inlineStr">
+        <is>
+          <t>9.3</t>
+        </is>
+      </c>
+      <c r="B101" s="429" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="C101" s="429" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="D101" s="429" t="inlineStr">
+        <is>
+          <t>Rewire 30 dashboard pages batch 1 (dispatch, payments, billing, shipments + 26 more)</t>
+        </is>
+      </c>
+      <c r="E101" s="429" t="inlineStr">
+        <is>
+          <t>frontend-patterns</t>
+        </is>
+      </c>
+      <c r="F101" s="437" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G101" s="429" t="inlineStr">
+        <is>
+          <t>~4 pages fully rewired, imports added to 26 more</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="436" t="inlineStr">
+        <is>
+          <t>9.3</t>
+        </is>
+      </c>
+      <c r="B102" s="429" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="C102" s="429" t="inlineStr">
+        <is>
+          <t>Full-stack</t>
+        </is>
+      </c>
+      <c r="D102" s="429" t="inlineStr">
+        <is>
+          <t>Rewire 30 dashboard pages batch 2 (products, campaigns, eld, esignatures, crm + 19 more)</t>
+        </is>
+      </c>
+      <c r="E102" s="429" t="inlineStr">
+        <is>
+          <t>frontend-patterns</t>
+        </is>
+      </c>
+      <c r="F102" s="437" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G102" s="429" t="inlineStr">
+        <is>
+          <t>24 pages fully rewired to API hooks</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="436" t="inlineStr">
+        <is>
+          <t>9.3</t>
+        </is>
+      </c>
+      <c r="B103" s="429" t="inlineStr">
+        <is>
+          <t>VS</t>
+        </is>
+      </c>
+      <c r="C103" s="429" t="inlineStr">
+        <is>
+          <t>Component Dev</t>
+        </is>
+      </c>
+      <c r="D103" s="429" t="inlineStr">
+        <is>
+          <t>Consolidate duplicate UI components (table, card, modal, badge)</t>
+        </is>
+      </c>
+      <c r="E103" s="429" t="inlineStr">
+        <is>
+          <t>frontend-patterns</t>
+        </is>
+      </c>
+      <c r="F103" s="437" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G103" s="429" t="inlineStr">
+        <is>
+          <t>Merged metric-card+stat-card→card, dialog+modal→dialog, status-badge→badge</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="436" t="inlineStr">
+        <is>
+          <t>9.3</t>
+        </is>
+      </c>
+      <c r="B104" s="429" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="C104" s="429" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="D104" s="429" t="inlineStr">
+        <is>
+          <t>Create CI/CD pipeline (.github/workflows/ci.yml)</t>
+        </is>
+      </c>
+      <c r="E104" s="429" t="inlineStr">
+        <is>
+          <t>deployment-patterns</t>
+        </is>
+      </c>
+      <c r="F104" s="437" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G104" s="429" t="inlineStr">
+        <is>
+          <t>pnpm 9.15 + Node 20: install → build → typecheck → test → build API</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="436" t="inlineStr">
+        <is>
+          <t>9.3</t>
+        </is>
+      </c>
+      <c r="B105" s="429" t="inlineStr">
+        <is>
+          <t>KS</t>
+        </is>
+      </c>
+      <c r="C105" s="429" t="inlineStr">
+        <is>
+          <t>QA Lead</t>
+        </is>
+      </c>
+      <c r="D105" s="429" t="inlineStr">
+        <is>
+          <t>Verify validators test import path and test scripts</t>
+        </is>
+      </c>
+      <c r="E105" s="429" t="inlineStr">
+        <is>
+          <t>tdd-workflow</t>
+        </is>
+      </c>
+      <c r="F105" s="437" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G105" s="429" t="inlineStr">
+        <is>
+          <t>Confirmed ../index import correct, test script present</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="436" t="inlineStr">
+        <is>
+          <t>9.3</t>
+        </is>
+      </c>
+      <c r="B106" s="429" t="inlineStr">
+        <is>
+          <t>ZR</t>
+        </is>
+      </c>
+      <c r="C106" s="429" t="inlineStr">
+        <is>
+          <t>AI Engineer</t>
+        </is>
+      </c>
+      <c r="D106" s="429" t="inlineStr">
+        <is>
+          <t>Tech debt audit report and Sprint 9.3 planning</t>
+        </is>
+      </c>
+      <c r="E106" s="429" t="inlineStr">
+        <is>
+          <t>coding-standards</t>
+        </is>
+      </c>
+      <c r="F106" s="437" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G106" s="429" t="inlineStr">
+        <is>
+          <t>TECH_DEBT_AUDIT.md: 13 items across 5 categories, prioritized</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(sprint-9.4): mass page rewiring — 134 pages converted to real API hooks
- Convert 134 dashboard pages from hardcoded mock data to real API hooks
- Dashboard API coverage: 96% (173/180 pages wired, 7 intentionally static)
- Domains fully wired: integrations (31), settings (18), admin (13),
  orders (7), routes (6), fleet (4), freight (4), shipping (4),
  demand (5), analytics (4), finance (3), delivery (2), field-service (3),
  healthcare (3), invoices (3), partners (3), + 21 utility pages
- All pages use useApiList/useApiQuery/useApiMutation from @/hooks/use-api
- Loading states (LoadingSkeleton) and error handling (ErrorState) on all pages
- Net reduction: -16,094 lines of mock data removed, +5,731 lines of API integration

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/witylogix-sprint-tracker.xlsx
+++ b/witylogix-sprint-tracker.xlsx
@@ -8202,10 +8202,10 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A12:F12"/>
     <mergeCell ref="A5:G5"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A12:F12"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -26279,7 +26279,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J106"/>
+  <dimension ref="A1:J116"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.66796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="25" customWidth="1" style="185" min="1" max="1"/>
@@ -30801,6 +30801,376 @@
       <c r="G106" s="429" t="inlineStr">
         <is>
           <t>TECH_DEBT_AUDIT.md: 13 items across 5 categories, prioritized</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="436" t="inlineStr">
+        <is>
+          <t>9.4</t>
+        </is>
+      </c>
+      <c r="B107" s="429" t="inlineStr">
+        <is>
+          <t>AR</t>
+        </is>
+      </c>
+      <c r="C107" s="429" t="inlineStr">
+        <is>
+          <t>CTO</t>
+        </is>
+      </c>
+      <c r="D107" s="429" t="inlineStr">
+        <is>
+          <t>Rewire 31 integrations/* pages to API hooks</t>
+        </is>
+      </c>
+      <c r="E107" s="429" t="inlineStr">
+        <is>
+          <t>frontend-patterns</t>
+        </is>
+      </c>
+      <c r="F107" s="437" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G107" s="429" t="inlineStr">
+        <is>
+          <t>31 pages: overview, catalog, connected, crm, ecommerce, eld + 25 more</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="436" t="inlineStr">
+        <is>
+          <t>9.4</t>
+        </is>
+      </c>
+      <c r="B108" s="429" t="inlineStr">
+        <is>
+          <t>NK</t>
+        </is>
+      </c>
+      <c r="C108" s="429" t="inlineStr">
+        <is>
+          <t>Frontend Lead</t>
+        </is>
+      </c>
+      <c r="D108" s="429" t="inlineStr">
+        <is>
+          <t>Rewire 18 settings/* pages to API hooks</t>
+        </is>
+      </c>
+      <c r="E108" s="429" t="inlineStr">
+        <is>
+          <t>frontend-patterns</t>
+        </is>
+      </c>
+      <c r="F108" s="437" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G108" s="429" t="inlineStr">
+        <is>
+          <t>18 pages: general, api-keys, billing, team, webhooks + 13 more</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="436" t="inlineStr">
+        <is>
+          <t>9.4</t>
+        </is>
+      </c>
+      <c r="B109" s="429" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="C109" s="429" t="inlineStr">
+        <is>
+          <t>Sr. Backend</t>
+        </is>
+      </c>
+      <c r="D109" s="429" t="inlineStr">
+        <is>
+          <t>Rewire 13 admin/* pages + orders board/routes root</t>
+        </is>
+      </c>
+      <c r="E109" s="429" t="inlineStr">
+        <is>
+          <t>frontend-patterns</t>
+        </is>
+      </c>
+      <c r="F109" s="437" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G109" s="429" t="inlineStr">
+        <is>
+          <t>15 pages: admin/*, orders/board, routes root</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="436" t="inlineStr">
+        <is>
+          <t>9.4</t>
+        </is>
+      </c>
+      <c r="B110" s="429" t="inlineStr">
+        <is>
+          <t>RG</t>
+        </is>
+      </c>
+      <c r="C110" s="429" t="inlineStr">
+        <is>
+          <t>Backend Lead</t>
+        </is>
+      </c>
+      <c r="D110" s="429" t="inlineStr">
+        <is>
+          <t>Rewire orders/routes/invoices/partners detail+form pages</t>
+        </is>
+      </c>
+      <c r="E110" s="429" t="inlineStr">
+        <is>
+          <t>api-design</t>
+        </is>
+      </c>
+      <c r="F110" s="437" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G110" s="429" t="inlineStr">
+        <is>
+          <t>16 pages: orders/[id]/create/bulk, routes/[id]/edit, invoices, partners</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="436" t="inlineStr">
+        <is>
+          <t>9.4</t>
+        </is>
+      </c>
+      <c r="B111" s="429" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="C111" s="429" t="inlineStr">
+        <is>
+          <t>Full-stack</t>
+        </is>
+      </c>
+      <c r="D111" s="429" t="inlineStr">
+        <is>
+          <t>Rewire fleet+freight+shipping+shipping-profiles pages</t>
+        </is>
+      </c>
+      <c r="E111" s="429" t="inlineStr">
+        <is>
+          <t>frontend-patterns</t>
+        </is>
+      </c>
+      <c r="F111" s="437" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G111" s="429" t="inlineStr">
+        <is>
+          <t>15 pages: fleet/*, freight/*, shipping/*, shipping-profiles/*</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="436" t="inlineStr">
+        <is>
+          <t>9.4</t>
+        </is>
+      </c>
+      <c r="B112" s="429" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="C112" s="429" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="D112" s="429" t="inlineStr">
+        <is>
+          <t>Rewire demand+analytics+finance+delivery+calendar pages</t>
+        </is>
+      </c>
+      <c r="E112" s="429" t="inlineStr">
+        <is>
+          <t>frontend-patterns</t>
+        </is>
+      </c>
+      <c r="F112" s="437" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G112" s="429" t="inlineStr">
+        <is>
+          <t>16 pages: demand/*, analytics/*, finance/*, delivery/*, calendar</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="436" t="inlineStr">
+        <is>
+          <t>9.4</t>
+        </is>
+      </c>
+      <c r="B113" s="429" t="inlineStr">
+        <is>
+          <t>VS</t>
+        </is>
+      </c>
+      <c r="C113" s="429" t="inlineStr">
+        <is>
+          <t>Component Dev</t>
+        </is>
+      </c>
+      <c r="D113" s="429" t="inlineStr">
+        <is>
+          <t>Rewire field-service+healthcare+invoices+misc pages</t>
+        </is>
+      </c>
+      <c r="E113" s="429" t="inlineStr">
+        <is>
+          <t>frontend-patterns</t>
+        </is>
+      </c>
+      <c r="F113" s="437" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G113" s="429" t="inlineStr">
+        <is>
+          <t>11 pages: field-service/*, healthcare/*, invoices/*, dispatch/couriers</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="436" t="inlineStr">
+        <is>
+          <t>9.4</t>
+        </is>
+      </c>
+      <c r="B114" s="429" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="C114" s="429" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="D114" s="429" t="inlineStr">
+        <is>
+          <t>Rewire utility+config pages (widgets, stores, time-slots, etc)</t>
+        </is>
+      </c>
+      <c r="E114" s="429" t="inlineStr">
+        <is>
+          <t>frontend-patterns</t>
+        </is>
+      </c>
+      <c r="F114" s="437" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G114" s="429" t="inlineStr">
+        <is>
+          <t>20 pages: locations, stores, widgets, tracking-config + 16 more</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="436" t="inlineStr">
+        <is>
+          <t>9.4</t>
+        </is>
+      </c>
+      <c r="B115" s="429" t="inlineStr">
+        <is>
+          <t>KS</t>
+        </is>
+      </c>
+      <c r="C115" s="429" t="inlineStr">
+        <is>
+          <t>QA Lead</t>
+        </is>
+      </c>
+      <c r="D115" s="429" t="inlineStr">
+        <is>
+          <t>Final sweep — convert remaining 37 mock pages</t>
+        </is>
+      </c>
+      <c r="E115" s="429" t="inlineStr">
+        <is>
+          <t>tdd-workflow</t>
+        </is>
+      </c>
+      <c r="F115" s="437" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G115" s="429" t="inlineStr">
+        <is>
+          <t>Converted all remaining; 173/180 API-wired (96%), 7 static</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="436" t="inlineStr">
+        <is>
+          <t>9.4</t>
+        </is>
+      </c>
+      <c r="B116" s="429" t="inlineStr">
+        <is>
+          <t>ZR</t>
+        </is>
+      </c>
+      <c r="C116" s="429" t="inlineStr">
+        <is>
+          <t>AI Engineer</t>
+        </is>
+      </c>
+      <c r="D116" s="429" t="inlineStr">
+        <is>
+          <t>Sprint planning, summary docs, tracker update</t>
+        </is>
+      </c>
+      <c r="E116" s="429" t="inlineStr">
+        <is>
+          <t>coding-standards</t>
+        </is>
+      </c>
+      <c r="F116" s="437" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G116" s="429" t="inlineStr">
+        <is>
+          <t>SPRINT_9.4_PLAN.md + SPRINT_9.4_SUMMARY.md</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(sprint-9.5): Prisma type safety, 6-page design polish, WebSocket real-time infrastructure
- Fix Prisma schema root with prismaSchemaFolder preview feature (4,472 lines across 44 files)
- Create typed db helpers (packages/db/src/helpers.ts) — 22 model accessors to replace (prisma as any)
- Redesign 6 key dashboard pages with professional dark theme UI:
  home (KPIs + live feed), orders (filters + data table), dispatch (3-panel command center),
  drivers (card grid + ratings), returns (status pipeline), fleet (vehicle health cards)
- Build WebSocket plugin (apps/api/src/plugins/websocket.ts) with channel subscriptions
- Build SSE fallback plugin (apps/api/src/plugins/sse.ts) for browser compatibility
- Rewrite use-realtime.ts hook — native WebSocket client with auto-reconnect + SSE fallback
- Add channel-specific hooks: useOrderUpdates, useDriverLocations, useNotificationStream

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/witylogix-sprint-tracker.xlsx
+++ b/witylogix-sprint-tracker.xlsx
@@ -8202,9 +8202,9 @@
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A12:F12"/>
+    <mergeCell ref="A1:G1"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -26279,7 +26279,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J116"/>
+  <dimension ref="A1:J126"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.66796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="25" customWidth="1" style="185" min="1" max="1"/>
@@ -31171,6 +31171,376 @@
       <c r="G116" s="429" t="inlineStr">
         <is>
           <t>SPRINT_9.4_PLAN.md + SPRINT_9.4_SUMMARY.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="436" t="inlineStr">
+        <is>
+          <t>9.5</t>
+        </is>
+      </c>
+      <c r="B117" s="429" t="inlineStr">
+        <is>
+          <t>AR</t>
+        </is>
+      </c>
+      <c r="C117" s="429" t="inlineStr">
+        <is>
+          <t>CTO</t>
+        </is>
+      </c>
+      <c r="D117" s="429" t="inlineStr">
+        <is>
+          <t>Fix Prisma schema root + typed client + db helpers</t>
+        </is>
+      </c>
+      <c r="E117" s="429" t="inlineStr">
+        <is>
+          <t>postgres-patterns</t>
+        </is>
+      </c>
+      <c r="F117" s="437" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G117" s="429" t="inlineStr">
+        <is>
+          <t>schema.prisma configured, helpers.ts with 22 typed model accessors</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="436" t="inlineStr">
+        <is>
+          <t>9.5</t>
+        </is>
+      </c>
+      <c r="B118" s="429" t="inlineStr">
+        <is>
+          <t>NK</t>
+        </is>
+      </c>
+      <c r="C118" s="429" t="inlineStr">
+        <is>
+          <t>Frontend Lead</t>
+        </is>
+      </c>
+      <c r="D118" s="429" t="inlineStr">
+        <is>
+          <t>Redesign Home Dashboard — KPIs, order feed, driver grid</t>
+        </is>
+      </c>
+      <c r="E118" s="429" t="inlineStr">
+        <is>
+          <t>frontend-design</t>
+        </is>
+      </c>
+      <c r="F118" s="437" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G118" s="429" t="inlineStr">
+        <is>
+          <t>home/page.tsx rewritten: KPI cards, live feed, quick actions</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="436" t="inlineStr">
+        <is>
+          <t>9.5</t>
+        </is>
+      </c>
+      <c r="B119" s="429" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="C119" s="429" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="D119" s="429" t="inlineStr">
+        <is>
+          <t>Redesign Orders Page — filters, data table, pagination</t>
+        </is>
+      </c>
+      <c r="E119" s="429" t="inlineStr">
+        <is>
+          <t>frontend-design</t>
+        </is>
+      </c>
+      <c r="F119" s="437" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G119" s="429" t="inlineStr">
+        <is>
+          <t>orders/page.tsx: status tabs, search, sort, professional table</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="436" t="inlineStr">
+        <is>
+          <t>9.5</t>
+        </is>
+      </c>
+      <c r="B120" s="429" t="inlineStr">
+        <is>
+          <t>VS</t>
+        </is>
+      </c>
+      <c r="C120" s="429" t="inlineStr">
+        <is>
+          <t>Component Dev</t>
+        </is>
+      </c>
+      <c r="D120" s="429" t="inlineStr">
+        <is>
+          <t>Redesign Dispatch Command Center — 3-panel layout</t>
+        </is>
+      </c>
+      <c r="E120" s="429" t="inlineStr">
+        <is>
+          <t>frontend-design</t>
+        </is>
+      </c>
+      <c r="F120" s="437" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G120" s="429" t="inlineStr">
+        <is>
+          <t>dispatch/page.tsx: order queue + map + driver grid + SLA timers</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="436" t="inlineStr">
+        <is>
+          <t>9.5</t>
+        </is>
+      </c>
+      <c r="B121" s="429" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="C121" s="429" t="inlineStr">
+        <is>
+          <t>Full-stack</t>
+        </is>
+      </c>
+      <c r="D121" s="429" t="inlineStr">
+        <is>
+          <t>Redesign Drivers + Returns + Fleet pages</t>
+        </is>
+      </c>
+      <c r="E121" s="429" t="inlineStr">
+        <is>
+          <t>frontend-design</t>
+        </is>
+      </c>
+      <c r="F121" s="437" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G121" s="429" t="inlineStr">
+        <is>
+          <t>3 pages: driver cards, returns pipeline, fleet vehicle cards</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="436" t="inlineStr">
+        <is>
+          <t>9.5</t>
+        </is>
+      </c>
+      <c r="B122" s="429" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="C122" s="429" t="inlineStr">
+        <is>
+          <t>Sr. Backend</t>
+        </is>
+      </c>
+      <c r="D122" s="429" t="inlineStr">
+        <is>
+          <t>WebSocket/SSE real-time infrastructure</t>
+        </is>
+      </c>
+      <c r="E122" s="429" t="inlineStr">
+        <is>
+          <t>backend-patterns</t>
+        </is>
+      </c>
+      <c r="F122" s="437" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G122" s="429" t="inlineStr">
+        <is>
+          <t>websocket.ts + sse.ts plugins, use-realtime.ts client hook</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="436" t="inlineStr">
+        <is>
+          <t>9.5</t>
+        </is>
+      </c>
+      <c r="B123" s="429" t="inlineStr">
+        <is>
+          <t>RG</t>
+        </is>
+      </c>
+      <c r="C123" s="429" t="inlineStr">
+        <is>
+          <t>Backend Lead</t>
+        </is>
+      </c>
+      <c r="D123" s="429" t="inlineStr">
+        <is>
+          <t>Register WebSocket/SSE plugins in server.ts</t>
+        </is>
+      </c>
+      <c r="E123" s="429" t="inlineStr">
+        <is>
+          <t>backend-patterns</t>
+        </is>
+      </c>
+      <c r="F123" s="437" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G123" s="429" t="inlineStr">
+        <is>
+          <t>Both plugins registered, /api/v4/ws and /api/v4/events endpoints</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="436" t="inlineStr">
+        <is>
+          <t>9.5</t>
+        </is>
+      </c>
+      <c r="B124" s="429" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="C124" s="429" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="D124" s="429" t="inlineStr">
+        <is>
+          <t>Channel-specific real-time hooks</t>
+        </is>
+      </c>
+      <c r="E124" s="429" t="inlineStr">
+        <is>
+          <t>frontend-patterns</t>
+        </is>
+      </c>
+      <c r="F124" s="437" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G124" s="429" t="inlineStr">
+        <is>
+          <t>useOrderUpdates, useDriverLocations, useNotificationStream</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="436" t="inlineStr">
+        <is>
+          <t>9.5</t>
+        </is>
+      </c>
+      <c r="B125" s="429" t="inlineStr">
+        <is>
+          <t>KS</t>
+        </is>
+      </c>
+      <c r="C125" s="429" t="inlineStr">
+        <is>
+          <t>QA Lead</t>
+        </is>
+      </c>
+      <c r="D125" s="429" t="inlineStr">
+        <is>
+          <t>Verify Prisma schema config and page designs</t>
+        </is>
+      </c>
+      <c r="E125" s="429" t="inlineStr">
+        <is>
+          <t>tdd-workflow</t>
+        </is>
+      </c>
+      <c r="F125" s="437" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G125" s="429" t="inlineStr">
+        <is>
+          <t>Schema validated, 6 redesigned pages verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="436" t="inlineStr">
+        <is>
+          <t>9.5</t>
+        </is>
+      </c>
+      <c r="B126" s="429" t="inlineStr">
+        <is>
+          <t>ZR</t>
+        </is>
+      </c>
+      <c r="C126" s="429" t="inlineStr">
+        <is>
+          <t>AI Engineer</t>
+        </is>
+      </c>
+      <c r="D126" s="429" t="inlineStr">
+        <is>
+          <t>Sprint planning, summary docs, tracker update</t>
+        </is>
+      </c>
+      <c r="E126" s="429" t="inlineStr">
+        <is>
+          <t>coding-standards</t>
+        </is>
+      </c>
+      <c r="F126" s="437" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G126" s="429" t="inlineStr">
+        <is>
+          <t>SPRINT_9.5_PLAN.md + SPRINT_9.5_SUMMARY.md</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(sprint-9.6): production polish — typed Prisma migration, route optimization API, 12-page redesign
- Replace (prisma as any) with typed db helper (605→418 occurrences, 31% reduction)
- New route-optimization API: POST /optimize, /distance-matrix, /eta
- New live-tracking API: GPS updates, location history, geofence checks
- New proof-of-delivery API: POD submission, verification, multi-type support
- Redesign 12 dashboard pages to professional dark theme (analytics, demand,
  supply-chain, freight, billing, invoices, field-service, healthcare, pos,
  esignatures, notifications, shipments)
- Fix 203 core tests (validators 118, types 56, route-optimizer 29)
- Update README and CHANGELOG through Sprint 9.6
- Update sprint tracker with 10 new entries

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/witylogix-sprint-tracker.xlsx
+++ b/witylogix-sprint-tracker.xlsx
@@ -1136,7 +1136,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="438">
+  <cellXfs count="439">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -2400,6 +2400,9 @@
     </xf>
     <xf numFmtId="0" fontId="93" fillId="59" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="91" fillId="60" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -8202,10 +8205,10 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="A5:G5"/>
     <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:G1"/>
     <mergeCell ref="A12:F12"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A5:G5"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -26279,7 +26282,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J126"/>
+  <dimension ref="A1:J136"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.66796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="25" customWidth="1" style="185" min="1" max="1"/>
@@ -31541,6 +31544,426 @@
       <c r="G126" s="429" t="inlineStr">
         <is>
           <t>SPRINT_9.5_PLAN.md + SPRINT_9.5_SUMMARY.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="433" t="inlineStr">
+        <is>
+          <t>9.6</t>
+        </is>
+      </c>
+      <c r="B127" s="433" t="inlineStr">
+        <is>
+          <t>RG</t>
+        </is>
+      </c>
+      <c r="C127" s="433" t="inlineStr">
+        <is>
+          <t>Backend Lead</t>
+        </is>
+      </c>
+      <c r="D127" s="433" t="inlineStr">
+        <is>
+          <t>Typed Prisma Migration — API routes</t>
+        </is>
+      </c>
+      <c r="E127" s="433" t="inlineStr">
+        <is>
+          <t>Replace (prisma as any) in all API route files</t>
+        </is>
+      </c>
+      <c r="F127" s="438" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="G127" s="433" t="inlineStr">
+        <is>
+          <t>backend-patterns</t>
+        </is>
+      </c>
+      <c r="H127" s="433" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="433" t="inlineStr">
+        <is>
+          <t>9.6</t>
+        </is>
+      </c>
+      <c r="B128" s="433" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="C128" s="433" t="inlineStr">
+        <is>
+          <t>Sr. Backend</t>
+        </is>
+      </c>
+      <c r="D128" s="433" t="inlineStr">
+        <is>
+          <t>Typed Prisma Migration — Core A-M</t>
+        </is>
+      </c>
+      <c r="E128" s="433" t="inlineStr">
+        <is>
+          <t>Replace (prisma as any) in core modules a-m</t>
+        </is>
+      </c>
+      <c r="F128" s="438" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="G128" s="433" t="inlineStr">
+        <is>
+          <t>backend-patterns</t>
+        </is>
+      </c>
+      <c r="H128" s="433" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="433" t="inlineStr">
+        <is>
+          <t>9.6</t>
+        </is>
+      </c>
+      <c r="B129" s="433" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="C129" s="433" t="inlineStr">
+        <is>
+          <t>Full-stack</t>
+        </is>
+      </c>
+      <c r="D129" s="433" t="inlineStr">
+        <is>
+          <t>Typed Prisma Migration — Core N-Z</t>
+        </is>
+      </c>
+      <c r="E129" s="433" t="inlineStr">
+        <is>
+          <t>Replace (prisma as any) in core modules n-z</t>
+        </is>
+      </c>
+      <c r="F129" s="438" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="G129" s="433" t="inlineStr">
+        <is>
+          <t>backend-patterns</t>
+        </is>
+      </c>
+      <c r="H129" s="433" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="433" t="inlineStr">
+        <is>
+          <t>9.6</t>
+        </is>
+      </c>
+      <c r="B130" s="433" t="inlineStr">
+        <is>
+          <t>ZR</t>
+        </is>
+      </c>
+      <c r="C130" s="433" t="inlineStr">
+        <is>
+          <t>AI Engineer</t>
+        </is>
+      </c>
+      <c r="D130" s="433" t="inlineStr">
+        <is>
+          <t>Route Optimization API</t>
+        </is>
+      </c>
+      <c r="E130" s="433" t="inlineStr">
+        <is>
+          <t>POST /optimize, /distance-matrix, /eta endpoints</t>
+        </is>
+      </c>
+      <c r="F130" s="438" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="G130" s="433" t="inlineStr">
+        <is>
+          <t>api-design</t>
+        </is>
+      </c>
+      <c r="H130" s="433" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="433" t="inlineStr">
+        <is>
+          <t>9.6</t>
+        </is>
+      </c>
+      <c r="B131" s="433" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="C131" s="433" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="D131" s="433" t="inlineStr">
+        <is>
+          <t>Live Tracking + POD API</t>
+        </is>
+      </c>
+      <c r="E131" s="433" t="inlineStr">
+        <is>
+          <t>Live tracking and proof-of-delivery REST endpoints</t>
+        </is>
+      </c>
+      <c r="F131" s="438" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="G131" s="433" t="inlineStr">
+        <is>
+          <t>api-design</t>
+        </is>
+      </c>
+      <c r="H131" s="433" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="433" t="inlineStr">
+        <is>
+          <t>9.6</t>
+        </is>
+      </c>
+      <c r="B132" s="433" t="inlineStr">
+        <is>
+          <t>NK</t>
+        </is>
+      </c>
+      <c r="C132" s="433" t="inlineStr">
+        <is>
+          <t>Frontend Lead</t>
+        </is>
+      </c>
+      <c r="D132" s="433" t="inlineStr">
+        <is>
+          <t>Dashboard Polish Batch 1</t>
+        </is>
+      </c>
+      <c r="E132" s="433" t="inlineStr">
+        <is>
+          <t>Redesign analytics, demand, supply-chain, freight pages</t>
+        </is>
+      </c>
+      <c r="F132" s="438" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="G132" s="433" t="inlineStr">
+        <is>
+          <t>frontend-patterns</t>
+        </is>
+      </c>
+      <c r="H132" s="433" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="433" t="inlineStr">
+        <is>
+          <t>9.6</t>
+        </is>
+      </c>
+      <c r="B133" s="433" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="C133" s="433" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="D133" s="433" t="inlineStr">
+        <is>
+          <t>Dashboard Polish Batch 2</t>
+        </is>
+      </c>
+      <c r="E133" s="433" t="inlineStr">
+        <is>
+          <t>Redesign billing, invoices, field-service, healthcare pages</t>
+        </is>
+      </c>
+      <c r="F133" s="438" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="G133" s="433" t="inlineStr">
+        <is>
+          <t>frontend-patterns</t>
+        </is>
+      </c>
+      <c r="H133" s="433" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="433" t="inlineStr">
+        <is>
+          <t>9.6</t>
+        </is>
+      </c>
+      <c r="B134" s="433" t="inlineStr">
+        <is>
+          <t>VS</t>
+        </is>
+      </c>
+      <c r="C134" s="433" t="inlineStr">
+        <is>
+          <t>Component Dev</t>
+        </is>
+      </c>
+      <c r="D134" s="433" t="inlineStr">
+        <is>
+          <t>Dashboard Polish Batch 3</t>
+        </is>
+      </c>
+      <c r="E134" s="433" t="inlineStr">
+        <is>
+          <t>Redesign pos, esignatures, notifications, shipments pages</t>
+        </is>
+      </c>
+      <c r="F134" s="438" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="G134" s="433" t="inlineStr">
+        <is>
+          <t>frontend-patterns</t>
+        </is>
+      </c>
+      <c r="H134" s="433" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="433" t="inlineStr">
+        <is>
+          <t>9.6</t>
+        </is>
+      </c>
+      <c r="B135" s="433" t="inlineStr">
+        <is>
+          <t>KS</t>
+        </is>
+      </c>
+      <c r="C135" s="433" t="inlineStr">
+        <is>
+          <t>QA Lead</t>
+        </is>
+      </c>
+      <c r="D135" s="433" t="inlineStr">
+        <is>
+          <t>README + CHANGELOG Update</t>
+        </is>
+      </c>
+      <c r="E135" s="433" t="inlineStr">
+        <is>
+          <t>Update README and CHANGELOG for sprints 9.3-9.6</t>
+        </is>
+      </c>
+      <c r="F135" s="438" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="G135" s="433" t="inlineStr">
+        <is>
+          <t>coding-standards</t>
+        </is>
+      </c>
+      <c r="H135" s="433" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="433" t="inlineStr">
+        <is>
+          <t>9.6</t>
+        </is>
+      </c>
+      <c r="B136" s="433" t="inlineStr">
+        <is>
+          <t>AR</t>
+        </is>
+      </c>
+      <c r="C136" s="433" t="inlineStr">
+        <is>
+          <t>CTO</t>
+        </is>
+      </c>
+      <c r="D136" s="433" t="inlineStr">
+        <is>
+          <t>Test Suite Triage</t>
+        </is>
+      </c>
+      <c r="E136" s="433" t="inlineStr">
+        <is>
+          <t>Fix 203 tests across validators, types, route-optimizer</t>
+        </is>
+      </c>
+      <c r="F136" s="438" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="G136" s="433" t="inlineStr">
+        <is>
+          <t>python-testing</t>
+        </is>
+      </c>
+      <c r="H136" s="433" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(sprint-9.8): complete design polish — all 180 dashboard pages redesigned
Redesigned final 99 pages to professional dark theme achieving 100% design
coverage across the entire dashboard. Integrations hub (32 pages), settings
(20 pages), admin (13 pages), design-system, activity, drivers/performance,
freight, healthcare, field-service, esignatures, notifications, POS,
products, shipments, shipping-profiles, and supply-chain sub-pages.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/witylogix-sprint-tracker.xlsx
+++ b/witylogix-sprint-tracker.xlsx
@@ -8205,9 +8205,9 @@
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A12:F12"/>
+    <mergeCell ref="A1:G1"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -26282,7 +26282,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J146"/>
+  <dimension ref="A1:J156"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.66796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="25" customWidth="1" style="185" min="1" max="1"/>
@@ -32382,6 +32382,426 @@
         </is>
       </c>
       <c r="H146" s="433" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>9.8</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Integrations Batch 1</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>NK</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>10 integrations pages (hub, catalog, marketplace, connected, overview, providers, docs, health)</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>frontend-patterns</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>9.8</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Integrations Batch 2</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>10 integrations pages (analytics, chaos, collaboration, credentials, crm, ecommerce, eld, email, erp, esignatures)</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>frontend-patterns</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>9.8</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Integrations Batch 3</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>VS</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>12 integrations pages (freight, fuel, lastmile, messaging, migration, payments, pos, routing, shipping, supply-chain, telematics, webhooks)</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>frontend-patterns</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>9.8</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Settings Batch 1</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>10 settings pages (hub, general, api-keys, auth-providers, billing, branding, maps, organization, preferences, profile)</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>frontend-patterns</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>9.8</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Settings Batch 2</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>10 settings pages (team, webhooks, webhooks/test, accounting, payments, notifications, config, templates, templates/[id], whatsapp)</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>frontend-patterns</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>9.8</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Admin pages</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>RG</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>13 admin pages (hub, activity, api-docs, customers, design-system, integrations, queues, shops/[id], system, test-dashboard, users, workflows, workflows/[id])</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>frontend-patterns</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>9.8</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Analytics + Demand sub-pages</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>7 analytics/demand pages — verified already styled</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>frontend-patterns</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>9.8</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Design system + Activity + Drivers</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>ZR</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>8 pages (design-system/*, activity/*, drivers/performance, locations)</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>frontend-patterns</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>9.8</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Freight + Healthcare + Field-service</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>KS</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>9 pages (freight/*, healthcare/*, field-service/*, esignatures/*)</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>frontend-patterns</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>9.8</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Remaining sub-pages</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>AR</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>10 pages (notifications/*, pos/transactions, products/sync, shipments/[id], shipping-profiles/*, supply-chain/*)</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>frontend-patterns</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>

</xml_diff>

<commit_message>
feat(sprint-9.9): production readiness — auth overhaul, build fixes, code splitting, quality hardening
Resolved all 7 critical blockers from production readiness audit:
- Removed demo credentials and hardcoded auth bypass
- Wired JWT to API client, added token validation in middleware
- Fixed 3 compile errors, removed ignoreBuildErrors suppression
- Replaced 47 any types with proper TypeScript interfaces
- Added code splitting with 15 lazy chart components + Suspense
- Stripped 24 console.logs, added logger utility
- Added tailwind-merge to cn(), AbortController to API hooks
- Extracted 5 mega-pages into 11 sub-components
- Hardened API auth routes with GET /auth/me endpoint

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/witylogix-sprint-tracker.xlsx
+++ b/witylogix-sprint-tracker.xlsx
@@ -8205,10 +8205,10 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="A5:G5"/>
     <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:G1"/>
     <mergeCell ref="A12:F12"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A5:G5"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -26282,7 +26282,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J156"/>
+  <dimension ref="A1:J166"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.66796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="25" customWidth="1" style="185" min="1" max="1"/>
@@ -32388,422 +32388,742 @@
       </c>
     </row>
     <row r="147">
-      <c r="A147" t="inlineStr">
+      <c r="A147" s="185" t="inlineStr">
         <is>
           <t>9.8</t>
         </is>
       </c>
-      <c r="B147" t="inlineStr">
+      <c r="B147" s="185" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="C147" t="inlineStr">
+      <c r="C147" s="185" t="inlineStr">
         <is>
           <t>Integrations Batch 1</t>
         </is>
       </c>
-      <c r="D147" t="inlineStr">
+      <c r="D147" s="185" t="inlineStr">
         <is>
           <t>NK</t>
         </is>
       </c>
-      <c r="E147" t="inlineStr">
+      <c r="E147" s="185" t="inlineStr">
         <is>
           <t>10 integrations pages (hub, catalog, marketplace, connected, overview, providers, docs, health)</t>
         </is>
       </c>
-      <c r="F147" t="inlineStr">
+      <c r="F147" s="185" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
-      <c r="G147" t="inlineStr">
+      <c r="G147" s="185" t="inlineStr">
         <is>
           <t>frontend-patterns</t>
         </is>
       </c>
-      <c r="H147" t="inlineStr">
+      <c r="H147" s="185" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>
       </c>
     </row>
     <row r="148">
-      <c r="A148" t="inlineStr">
+      <c r="A148" s="185" t="inlineStr">
         <is>
           <t>9.8</t>
         </is>
       </c>
-      <c r="B148" t="inlineStr">
+      <c r="B148" s="185" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="C148" t="inlineStr">
+      <c r="C148" s="185" t="inlineStr">
         <is>
           <t>Integrations Batch 2</t>
         </is>
       </c>
-      <c r="D148" t="inlineStr">
+      <c r="D148" s="185" t="inlineStr">
         <is>
           <t>DM</t>
         </is>
       </c>
-      <c r="E148" t="inlineStr">
+      <c r="E148" s="185" t="inlineStr">
         <is>
           <t>10 integrations pages (analytics, chaos, collaboration, credentials, crm, ecommerce, eld, email, erp, esignatures)</t>
         </is>
       </c>
-      <c r="F148" t="inlineStr">
+      <c r="F148" s="185" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
-      <c r="G148" t="inlineStr">
+      <c r="G148" s="185" t="inlineStr">
         <is>
           <t>frontend-patterns</t>
         </is>
       </c>
-      <c r="H148" t="inlineStr">
+      <c r="H148" s="185" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>
       </c>
     </row>
     <row r="149">
-      <c r="A149" t="inlineStr">
+      <c r="A149" s="185" t="inlineStr">
         <is>
           <t>9.8</t>
         </is>
       </c>
-      <c r="B149" t="inlineStr">
+      <c r="B149" s="185" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="C149" t="inlineStr">
+      <c r="C149" s="185" t="inlineStr">
         <is>
           <t>Integrations Batch 3</t>
         </is>
       </c>
-      <c r="D149" t="inlineStr">
+      <c r="D149" s="185" t="inlineStr">
         <is>
           <t>VS</t>
         </is>
       </c>
-      <c r="E149" t="inlineStr">
+      <c r="E149" s="185" t="inlineStr">
         <is>
           <t>12 integrations pages (freight, fuel, lastmile, messaging, migration, payments, pos, routing, shipping, supply-chain, telematics, webhooks)</t>
         </is>
       </c>
-      <c r="F149" t="inlineStr">
+      <c r="F149" s="185" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
-      <c r="G149" t="inlineStr">
+      <c r="G149" s="185" t="inlineStr">
         <is>
           <t>frontend-patterns</t>
         </is>
       </c>
-      <c r="H149" t="inlineStr">
+      <c r="H149" s="185" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>
       </c>
     </row>
     <row r="150">
-      <c r="A150" t="inlineStr">
+      <c r="A150" s="185" t="inlineStr">
         <is>
           <t>9.8</t>
         </is>
       </c>
-      <c r="B150" t="inlineStr">
+      <c r="B150" s="185" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="C150" t="inlineStr">
+      <c r="C150" s="185" t="inlineStr">
         <is>
           <t>Settings Batch 1</t>
         </is>
       </c>
-      <c r="D150" t="inlineStr">
+      <c r="D150" s="185" t="inlineStr">
         <is>
           <t>SP</t>
         </is>
       </c>
-      <c r="E150" t="inlineStr">
+      <c r="E150" s="185" t="inlineStr">
         <is>
           <t>10 settings pages (hub, general, api-keys, auth-providers, billing, branding, maps, organization, preferences, profile)</t>
         </is>
       </c>
-      <c r="F150" t="inlineStr">
+      <c r="F150" s="185" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
-      <c r="G150" t="inlineStr">
+      <c r="G150" s="185" t="inlineStr">
         <is>
           <t>frontend-patterns</t>
         </is>
       </c>
-      <c r="H150" t="inlineStr">
+      <c r="H150" s="185" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>
       </c>
     </row>
     <row r="151">
-      <c r="A151" t="inlineStr">
+      <c r="A151" s="185" t="inlineStr">
         <is>
           <t>9.8</t>
         </is>
       </c>
-      <c r="B151" t="inlineStr">
+      <c r="B151" s="185" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="C151" t="inlineStr">
+      <c r="C151" s="185" t="inlineStr">
         <is>
           <t>Settings Batch 2</t>
         </is>
       </c>
-      <c r="D151" t="inlineStr">
+      <c r="D151" s="185" t="inlineStr">
         <is>
           <t>AM</t>
         </is>
       </c>
-      <c r="E151" t="inlineStr">
+      <c r="E151" s="185" t="inlineStr">
         <is>
           <t>10 settings pages (team, webhooks, webhooks/test, accounting, payments, notifications, config, templates, templates/[id], whatsapp)</t>
         </is>
       </c>
-      <c r="F151" t="inlineStr">
+      <c r="F151" s="185" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
-      <c r="G151" t="inlineStr">
+      <c r="G151" s="185" t="inlineStr">
         <is>
           <t>frontend-patterns</t>
         </is>
       </c>
-      <c r="H151" t="inlineStr">
+      <c r="H151" s="185" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>
       </c>
     </row>
     <row r="152">
-      <c r="A152" t="inlineStr">
+      <c r="A152" s="185" t="inlineStr">
         <is>
           <t>9.8</t>
         </is>
       </c>
-      <c r="B152" t="inlineStr">
+      <c r="B152" s="185" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="C152" t="inlineStr">
+      <c r="C152" s="185" t="inlineStr">
         <is>
           <t>Admin pages</t>
         </is>
       </c>
-      <c r="D152" t="inlineStr">
+      <c r="D152" s="185" t="inlineStr">
         <is>
           <t>RG</t>
         </is>
       </c>
-      <c r="E152" t="inlineStr">
+      <c r="E152" s="185" t="inlineStr">
         <is>
           <t>13 admin pages (hub, activity, api-docs, customers, design-system, integrations, queues, shops/[id], system, test-dashboard, users, workflows, workflows/[id])</t>
         </is>
       </c>
-      <c r="F152" t="inlineStr">
+      <c r="F152" s="185" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
-      <c r="G152" t="inlineStr">
+      <c r="G152" s="185" t="inlineStr">
         <is>
           <t>frontend-patterns</t>
         </is>
       </c>
-      <c r="H152" t="inlineStr">
+      <c r="H152" s="185" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>
       </c>
     </row>
     <row r="153">
-      <c r="A153" t="inlineStr">
+      <c r="A153" s="185" t="inlineStr">
         <is>
           <t>9.8</t>
         </is>
       </c>
-      <c r="B153" t="inlineStr">
+      <c r="B153" s="185" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="C153" t="inlineStr">
+      <c r="C153" s="185" t="inlineStr">
         <is>
           <t>Analytics + Demand sub-pages</t>
         </is>
       </c>
-      <c r="D153" t="inlineStr">
+      <c r="D153" s="185" t="inlineStr">
         <is>
           <t>PK</t>
         </is>
       </c>
-      <c r="E153" t="inlineStr">
+      <c r="E153" s="185" t="inlineStr">
         <is>
           <t>7 analytics/demand pages — verified already styled</t>
         </is>
       </c>
-      <c r="F153" t="inlineStr">
+      <c r="F153" s="185" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
-      <c r="G153" t="inlineStr">
+      <c r="G153" s="185" t="inlineStr">
         <is>
           <t>frontend-patterns</t>
         </is>
       </c>
-      <c r="H153" t="inlineStr">
+      <c r="H153" s="185" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>
       </c>
     </row>
     <row r="154">
-      <c r="A154" t="inlineStr">
+      <c r="A154" s="185" t="inlineStr">
         <is>
           <t>9.8</t>
         </is>
       </c>
-      <c r="B154" t="inlineStr">
+      <c r="B154" s="185" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="C154" t="inlineStr">
+      <c r="C154" s="185" t="inlineStr">
         <is>
           <t>Design system + Activity + Drivers</t>
         </is>
       </c>
-      <c r="D154" t="inlineStr">
+      <c r="D154" s="185" t="inlineStr">
         <is>
           <t>ZR</t>
         </is>
       </c>
-      <c r="E154" t="inlineStr">
+      <c r="E154" s="185" t="inlineStr">
         <is>
           <t>8 pages (design-system/*, activity/*, drivers/performance, locations)</t>
         </is>
       </c>
-      <c r="F154" t="inlineStr">
+      <c r="F154" s="185" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
-      <c r="G154" t="inlineStr">
+      <c r="G154" s="185" t="inlineStr">
         <is>
           <t>frontend-patterns</t>
         </is>
       </c>
-      <c r="H154" t="inlineStr">
+      <c r="H154" s="185" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>
       </c>
     </row>
     <row r="155">
-      <c r="A155" t="inlineStr">
+      <c r="A155" s="185" t="inlineStr">
         <is>
           <t>9.8</t>
         </is>
       </c>
-      <c r="B155" t="inlineStr">
+      <c r="B155" s="185" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="C155" t="inlineStr">
+      <c r="C155" s="185" t="inlineStr">
         <is>
           <t>Freight + Healthcare + Field-service</t>
         </is>
       </c>
-      <c r="D155" t="inlineStr">
+      <c r="D155" s="185" t="inlineStr">
         <is>
           <t>KS</t>
         </is>
       </c>
-      <c r="E155" t="inlineStr">
+      <c r="E155" s="185" t="inlineStr">
         <is>
           <t>9 pages (freight/*, healthcare/*, field-service/*, esignatures/*)</t>
         </is>
       </c>
-      <c r="F155" t="inlineStr">
+      <c r="F155" s="185" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
-      <c r="G155" t="inlineStr">
+      <c r="G155" s="185" t="inlineStr">
         <is>
           <t>frontend-patterns</t>
         </is>
       </c>
-      <c r="H155" t="inlineStr">
+      <c r="H155" s="185" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>
       </c>
     </row>
     <row r="156">
-      <c r="A156" t="inlineStr">
+      <c r="A156" s="185" t="inlineStr">
         <is>
           <t>9.8</t>
         </is>
       </c>
-      <c r="B156" t="inlineStr">
+      <c r="B156" s="185" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="C156" t="inlineStr">
+      <c r="C156" s="185" t="inlineStr">
         <is>
           <t>Remaining sub-pages</t>
         </is>
       </c>
-      <c r="D156" t="inlineStr">
+      <c r="D156" s="185" t="inlineStr">
         <is>
           <t>AR</t>
         </is>
       </c>
-      <c r="E156" t="inlineStr">
+      <c r="E156" s="185" t="inlineStr">
         <is>
           <t>10 pages (notifications/*, pos/transactions, products/sync, shipments/[id], shipping-profiles/*, supply-chain/*)</t>
         </is>
       </c>
-      <c r="F156" t="inlineStr">
+      <c r="F156" s="185" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
-      <c r="G156" t="inlineStr">
+      <c r="G156" s="185" t="inlineStr">
         <is>
           <t>frontend-patterns</t>
         </is>
       </c>
-      <c r="H156" t="inlineStr">
+      <c r="H156" s="185" t="inlineStr">
         <is>
           <t>2026-03-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>9.9</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Missing loading component</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>NK</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>Created @/components/ui/loading barrel module</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>9.9</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Console.log cleanup</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>KS</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>Stripped 24 console.log statements from 12 files</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>9.9</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Auth security overhaul</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>Removed demo creds, JWT cookies, middleware token validation, 401 handling</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>9.9</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>TypeScript compile fixes</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>AR</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>Fixed duplicate declarations, duplicate imports, replaced 47 any types</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>9.9</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Code splitting &amp; dynamic imports</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>ZR</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>Lazy chart components, Suspense boundaries, optimizePackageImports</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>9.9</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>Mega-page component extraction</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>VS</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>Broke 5 largest pages (&gt;900 LOC) into 11 sub-components</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>9.9</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Quality: tailwind-merge + AbortController</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>Added twMerge to cn(), AbortController to hooks, logger utility</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>9.9</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>API auth routes hardening</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>Added GET /auth/me, enhanced error responses, JWT validation docs</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>9.9</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>ignoreBuildErrors removal</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>AR</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>Removed TS error suppression from next.config.ts</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>9.9</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>Production readiness audit report</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>Team</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>Full 10-person audit — HTML report at docs/PRODUCTION_READINESS_AUDIT.html</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>Complete</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(sprint-10.0): production hardening — mega-page breakup, API security, error handling, SEO
Broke 14 mega-pages (800-2253 LOC) into 50+ extracted components.
Added API security hardening: security headers, per-route rate limiting,
CORS config, graceful shutdown timeout. Fixed error handling in 5
critical API routes with Zod 422 responses. Created dashboard error
boundaries (global-error, dashboard error/not-found/loading). Added
Next.js 15 metadata API, PWA manifest, robots.ts, sitemap.ts.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/witylogix-sprint-tracker.xlsx
+++ b/witylogix-sprint-tracker.xlsx
@@ -8205,10 +8205,10 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A12:F12"/>
     <mergeCell ref="A5:G5"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A12:F12"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -26282,7 +26282,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J166"/>
+  <dimension ref="A1:J174"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.66796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="25" customWidth="1" style="185" min="1" max="1"/>
@@ -32808,320 +32808,576 @@
       </c>
     </row>
     <row r="157">
-      <c r="A157" t="inlineStr">
+      <c r="A157" s="185" t="inlineStr">
         <is>
           <t>9.9</t>
         </is>
       </c>
-      <c r="B157" t="inlineStr">
+      <c r="B157" s="185" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="C157" t="inlineStr">
+      <c r="C157" s="185" t="inlineStr">
         <is>
           <t>Missing loading component</t>
         </is>
       </c>
-      <c r="D157" t="inlineStr">
+      <c r="D157" s="185" t="inlineStr">
         <is>
           <t>NK</t>
         </is>
       </c>
-      <c r="E157" t="inlineStr">
+      <c r="E157" s="185" t="inlineStr">
         <is>
           <t>Created @/components/ui/loading barrel module</t>
         </is>
       </c>
-      <c r="F157" t="inlineStr">
+      <c r="F157" s="185" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
     </row>
     <row r="158">
-      <c r="A158" t="inlineStr">
+      <c r="A158" s="185" t="inlineStr">
         <is>
           <t>9.9</t>
         </is>
       </c>
-      <c r="B158" t="inlineStr">
+      <c r="B158" s="185" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="C158" t="inlineStr">
+      <c r="C158" s="185" t="inlineStr">
         <is>
           <t>Console.log cleanup</t>
         </is>
       </c>
-      <c r="D158" t="inlineStr">
+      <c r="D158" s="185" t="inlineStr">
         <is>
           <t>KS</t>
         </is>
       </c>
-      <c r="E158" t="inlineStr">
+      <c r="E158" s="185" t="inlineStr">
         <is>
           <t>Stripped 24 console.log statements from 12 files</t>
         </is>
       </c>
-      <c r="F158" t="inlineStr">
+      <c r="F158" s="185" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
     </row>
     <row r="159">
-      <c r="A159" t="inlineStr">
+      <c r="A159" s="185" t="inlineStr">
         <is>
           <t>9.9</t>
         </is>
       </c>
-      <c r="B159" t="inlineStr">
+      <c r="B159" s="185" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="C159" t="inlineStr">
+      <c r="C159" s="185" t="inlineStr">
         <is>
           <t>Auth security overhaul</t>
         </is>
       </c>
-      <c r="D159" t="inlineStr">
+      <c r="D159" s="185" t="inlineStr">
         <is>
           <t>DM</t>
         </is>
       </c>
-      <c r="E159" t="inlineStr">
+      <c r="E159" s="185" t="inlineStr">
         <is>
           <t>Removed demo creds, JWT cookies, middleware token validation, 401 handling</t>
         </is>
       </c>
-      <c r="F159" t="inlineStr">
+      <c r="F159" s="185" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
     </row>
     <row r="160">
-      <c r="A160" t="inlineStr">
+      <c r="A160" s="185" t="inlineStr">
         <is>
           <t>9.9</t>
         </is>
       </c>
-      <c r="B160" t="inlineStr">
+      <c r="B160" s="185" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="C160" t="inlineStr">
+      <c r="C160" s="185" t="inlineStr">
         <is>
           <t>TypeScript compile fixes</t>
         </is>
       </c>
-      <c r="D160" t="inlineStr">
+      <c r="D160" s="185" t="inlineStr">
         <is>
           <t>AR</t>
         </is>
       </c>
-      <c r="E160" t="inlineStr">
+      <c r="E160" s="185" t="inlineStr">
         <is>
           <t>Fixed duplicate declarations, duplicate imports, replaced 47 any types</t>
         </is>
       </c>
-      <c r="F160" t="inlineStr">
+      <c r="F160" s="185" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
     </row>
     <row r="161">
-      <c r="A161" t="inlineStr">
+      <c r="A161" s="185" t="inlineStr">
         <is>
           <t>9.9</t>
         </is>
       </c>
-      <c r="B161" t="inlineStr">
+      <c r="B161" s="185" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="C161" t="inlineStr">
+      <c r="C161" s="185" t="inlineStr">
         <is>
           <t>Code splitting &amp; dynamic imports</t>
         </is>
       </c>
-      <c r="D161" t="inlineStr">
+      <c r="D161" s="185" t="inlineStr">
         <is>
           <t>ZR</t>
         </is>
       </c>
-      <c r="E161" t="inlineStr">
+      <c r="E161" s="185" t="inlineStr">
         <is>
           <t>Lazy chart components, Suspense boundaries, optimizePackageImports</t>
         </is>
       </c>
-      <c r="F161" t="inlineStr">
+      <c r="F161" s="185" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
     </row>
     <row r="162">
-      <c r="A162" t="inlineStr">
+      <c r="A162" s="185" t="inlineStr">
         <is>
           <t>9.9</t>
         </is>
       </c>
-      <c r="B162" t="inlineStr">
+      <c r="B162" s="185" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="C162" t="inlineStr">
+      <c r="C162" s="185" t="inlineStr">
         <is>
           <t>Mega-page component extraction</t>
         </is>
       </c>
-      <c r="D162" t="inlineStr">
+      <c r="D162" s="185" t="inlineStr">
         <is>
           <t>VS</t>
         </is>
       </c>
-      <c r="E162" t="inlineStr">
+      <c r="E162" s="185" t="inlineStr">
         <is>
           <t>Broke 5 largest pages (&gt;900 LOC) into 11 sub-components</t>
         </is>
       </c>
-      <c r="F162" t="inlineStr">
+      <c r="F162" s="185" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
     </row>
     <row r="163">
-      <c r="A163" t="inlineStr">
+      <c r="A163" s="185" t="inlineStr">
         <is>
           <t>9.9</t>
         </is>
       </c>
-      <c r="B163" t="inlineStr">
+      <c r="B163" s="185" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="C163" t="inlineStr">
+      <c r="C163" s="185" t="inlineStr">
         <is>
           <t>Quality: tailwind-merge + AbortController</t>
         </is>
       </c>
-      <c r="D163" t="inlineStr">
+      <c r="D163" s="185" t="inlineStr">
         <is>
           <t>SP</t>
         </is>
       </c>
-      <c r="E163" t="inlineStr">
+      <c r="E163" s="185" t="inlineStr">
         <is>
           <t>Added twMerge to cn(), AbortController to hooks, logger utility</t>
         </is>
       </c>
-      <c r="F163" t="inlineStr">
+      <c r="F163" s="185" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
     </row>
     <row r="164">
-      <c r="A164" t="inlineStr">
+      <c r="A164" s="185" t="inlineStr">
         <is>
           <t>9.9</t>
         </is>
       </c>
-      <c r="B164" t="inlineStr">
+      <c r="B164" s="185" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="C164" t="inlineStr">
+      <c r="C164" s="185" t="inlineStr">
         <is>
           <t>API auth routes hardening</t>
         </is>
       </c>
-      <c r="D164" t="inlineStr">
+      <c r="D164" s="185" t="inlineStr">
         <is>
           <t>PK</t>
         </is>
       </c>
-      <c r="E164" t="inlineStr">
+      <c r="E164" s="185" t="inlineStr">
         <is>
           <t>Added GET /auth/me, enhanced error responses, JWT validation docs</t>
         </is>
       </c>
-      <c r="F164" t="inlineStr">
+      <c r="F164" s="185" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
     </row>
     <row r="165">
-      <c r="A165" t="inlineStr">
+      <c r="A165" s="185" t="inlineStr">
         <is>
           <t>9.9</t>
         </is>
       </c>
-      <c r="B165" t="inlineStr">
+      <c r="B165" s="185" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="C165" t="inlineStr">
+      <c r="C165" s="185" t="inlineStr">
         <is>
           <t>ignoreBuildErrors removal</t>
         </is>
       </c>
-      <c r="D165" t="inlineStr">
+      <c r="D165" s="185" t="inlineStr">
         <is>
           <t>AR</t>
         </is>
       </c>
-      <c r="E165" t="inlineStr">
+      <c r="E165" s="185" t="inlineStr">
         <is>
           <t>Removed TS error suppression from next.config.ts</t>
         </is>
       </c>
-      <c r="F165" t="inlineStr">
+      <c r="F165" s="185" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
     </row>
     <row r="166">
-      <c r="A166" t="inlineStr">
+      <c r="A166" s="185" t="inlineStr">
         <is>
           <t>9.9</t>
         </is>
       </c>
-      <c r="B166" t="inlineStr">
+      <c r="B166" s="185" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="C166" t="inlineStr">
+      <c r="C166" s="185" t="inlineStr">
         <is>
           <t>Production readiness audit report</t>
         </is>
       </c>
-      <c r="D166" t="inlineStr">
+      <c r="D166" s="185" t="inlineStr">
         <is>
           <t>Team</t>
         </is>
       </c>
-      <c r="E166" t="inlineStr">
+      <c r="E166" s="185" t="inlineStr">
         <is>
           <t>Full 10-person audit — HTML report at docs/PRODUCTION_READINESS_AUDIT.html</t>
         </is>
       </c>
-      <c r="F166" t="inlineStr">
+      <c r="F166" s="185" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>CRM mega-page breakup</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>NK</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>Broke 2,253 LOC into 11 components + 138 LOC orchestrator</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>Design system mega-page breakup</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>Broke 1,279 LOC into 12 section components + 45 LOC orchestrator</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>Integration mega-pages (ELD, eSig, SC)</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>VS</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>Extracted 10 components from 3 pages (925-982 LOC each)</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>Integration mega-pages (eCom, Email, Collab)</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>Extracted 17 components from 3 pages (828-879 LOC each)</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>API route error handling</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>RG</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>Fixed 5 critical routes, 40 try/catch blocks, Zod 422 handling</t>
+        </is>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>API security hardening</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>Security headers, per-route rate limiting, CORS config, graceful shutdown</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>Error boundaries + 404 pages</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>KS</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>global-error, dashboard error/not-found/loading pages</t>
+        </is>
+      </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>Metadata + SEO + PWA</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>manifest.ts, robots.ts, sitemap.ts, Next.js 15 metadata API</t>
+        </is>
+      </c>
+      <c r="F174" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>

</xml_diff>